<commit_message>
AFE: trimmer de 25k en G2 por canal (ganancia por sitio); notas del módulo INA333
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V5Cz1Wb6HSRhqzouEW9mso
</commit_message>
<xml_diff>
--- a/docs/afe-emg/BoM_AFE_AuraVox.xlsx
+++ b/docs/afe-emg/BoM_AFE_AuraVox.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tiendas" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'BoM por modulo'!$A$4:$Q$72</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'BoM por modulo'!$A$4:$Q$73</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -509,7 +509,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q74"/>
+  <dimension ref="A1:Q75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1127,7 +1127,7 @@
       </c>
       <c r="Q13" s="5" t="inlineStr">
         <is>
-          <t>Reemplazar el potenciometro de RG por RGa+RGb y sacar un cable del punto medio al RLD. Respaldo: AD623AN DIP-8 (misma formula de G)</t>
+          <t>Desoldar el trimmer de RG y poner RGa+RGb (2.7k+2.7k) con cable del punto medio al RLD. Alimentar por el pin 3.3V (no VCC) y llevar el pin VREF a tu VREF con buffer. Verificar pines con multimetro. Respaldo: AD623AN DIP-8</t>
         </is>
       </c>
     </row>
@@ -1657,17 +1657,17 @@
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>Resistencia de ganancia</t>
+          <t>Resistencia de ganancia fija</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>10k</t>
+          <t>4.7k</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>10k</t>
+          <t>4.7k</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
@@ -1694,7 +1694,7 @@
       </c>
       <c r="L23" s="5" t="inlineStr">
         <is>
-          <t>resistencia 10k 1%</t>
+          <t>resistencia 4.7k 1%</t>
         </is>
       </c>
       <c r="M23" s="6" t="n"/>
@@ -1718,27 +1718,27 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>Cg</t>
+          <t>RGT</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>Condensador de bloqueo DC (G = 1 en DC)</t>
+          <t>Trimmer de ganancia por sitio de medicion</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>10u</t>
+          <t>25k</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>10u</t>
+          <t>25k multivuelta</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>ceramico X7R o electrolitico 16 V</t>
+          <t>trimmer multivuelta (3296)</t>
         </is>
       </c>
       <c r="G24" s="5" t="n">
@@ -1760,7 +1760,7 @@
       </c>
       <c r="L24" s="5" t="inlineStr">
         <is>
-          <t>condensador 10uF</t>
+          <t>trimmer 25k multivuelta 3296</t>
         </is>
       </c>
       <c r="M24" s="6" t="n"/>
@@ -1774,7 +1774,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="Q24" s="5" t="inlineStr"/>
+      <c r="Q24" s="5" t="inlineStr">
+        <is>
+          <t>G2 = 1 + 240k/(4.7k + RGT): de ~9 (25k) a ~52 (0). Ganancia total ~180-1000. Para G2 = 25: RGT = 5.3k</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
@@ -1784,141 +1788,137 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
+          <t>Cg</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>Condensador de bloqueo DC (G = 1 en DC)</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>10u</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>10u</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>ceramico X7R o electrolitico 16 V</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H25" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="I25" s="5">
+        <f>G25*H25</f>
+        <v/>
+      </c>
+      <c r="J25" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="K25" s="5">
+        <f>I25+J25</f>
+        <v/>
+      </c>
+      <c r="L25" s="5" t="inlineStr">
+        <is>
+          <t>condensador 10uF</t>
+        </is>
+      </c>
+      <c r="M25" s="6" t="n"/>
+      <c r="N25" s="7" t="n"/>
+      <c r="O25" s="8">
+        <f>IF(N25="","",K25*N25)</f>
+        <v/>
+      </c>
+      <c r="P25" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="Q25" s="5" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>5 G2 = 25</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
           <t>XG2</t>
         </is>
       </c>
-      <c r="C25" s="5" t="inlineStr">
+      <c r="C26" s="5" t="inlineStr">
         <is>
           <t>seccion de op-amp</t>
         </is>
       </c>
-      <c r="D25" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E25" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F25" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G25" s="5" t="n"/>
-      <c r="H25" s="5" t="n"/>
-      <c r="I25" s="5" t="n"/>
-      <c r="J25" s="5" t="n"/>
-      <c r="K25" s="5" t="n"/>
-      <c r="L25" s="5" t="inlineStr"/>
-      <c r="M25" s="5" t="n"/>
-      <c r="N25" s="8" t="n"/>
-      <c r="O25" s="8" t="n"/>
-      <c r="P25" s="5" t="n"/>
-      <c r="Q25" s="5" t="inlineStr">
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="n"/>
+      <c r="H26" s="5" t="n"/>
+      <c r="I26" s="5" t="n"/>
+      <c r="J26" s="5" t="n"/>
+      <c r="K26" s="5" t="n"/>
+      <c r="L26" s="5" t="inlineStr"/>
+      <c r="M26" s="5" t="n"/>
+      <c r="N26" s="8" t="n"/>
+      <c r="O26" s="8" t="n"/>
+      <c r="P26" s="5" t="n"/>
+      <c r="Q26" s="5" t="inlineStr">
         <is>
           <t>Contada en el modulo 11 OP-AMPS</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="4" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
         <is>
           <t>6 LPF A 500 Hz (Q 0.541)</t>
         </is>
       </c>
-      <c r="B26" s="4" t="n"/>
-      <c r="C26" s="4" t="inlineStr">
+      <c r="B27" s="4" t="n"/>
+      <c r="C27" s="4" t="inlineStr">
         <is>
           <t>por canal (x4)</t>
         </is>
       </c>
-      <c r="D26" s="4" t="n"/>
-      <c r="E26" s="4" t="n"/>
-      <c r="F26" s="4" t="n"/>
-      <c r="G26" s="4" t="n"/>
-      <c r="H26" s="4" t="n"/>
-      <c r="I26" s="4" t="n"/>
-      <c r="J26" s="4" t="n"/>
-      <c r="K26" s="4" t="n"/>
-      <c r="L26" s="4" t="n"/>
-      <c r="M26" s="4" t="n"/>
-      <c r="N26" s="4" t="n"/>
-      <c r="O26" s="4" t="n"/>
-      <c r="P26" s="4" t="n"/>
-      <c r="Q26" s="4" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="5" t="inlineStr">
-        <is>
-          <t>6 LPF A 500 Hz (Q 0.541)</t>
-        </is>
-      </c>
-      <c r="B27" s="5" t="inlineStr">
-        <is>
-          <t>Rla1, Rla2</t>
-        </is>
-      </c>
-      <c r="C27" s="5" t="inlineStr">
-        <is>
-          <t>Resistencia del LPF A</t>
-        </is>
-      </c>
-      <c r="D27" s="5" t="inlineStr">
-        <is>
-          <t>88.7k</t>
-        </is>
-      </c>
-      <c r="E27" s="5" t="inlineStr">
-        <is>
-          <t>91k</t>
-        </is>
-      </c>
-      <c r="F27" s="5" t="inlineStr">
-        <is>
-          <t>pelicula metalica 1 %</t>
-        </is>
-      </c>
-      <c r="G27" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="H27" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="I27" s="5">
-        <f>G27*H27</f>
-        <v/>
-      </c>
-      <c r="J27" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="K27" s="5">
-        <f>I27+J27</f>
-        <v/>
-      </c>
-      <c r="L27" s="5" t="inlineStr">
-        <is>
-          <t>resistencia 91k 1%</t>
-        </is>
-      </c>
-      <c r="M27" s="6" t="n"/>
-      <c r="N27" s="7" t="n"/>
-      <c r="O27" s="8">
-        <f>IF(N27="","",K27*N27)</f>
-        <v/>
-      </c>
-      <c r="P27" s="6" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="Q27" s="5" t="inlineStr">
-        <is>
-          <t>Con 91k: f0 = 487 Hz</t>
-        </is>
-      </c>
+      <c r="D27" s="4" t="n"/>
+      <c r="E27" s="4" t="n"/>
+      <c r="F27" s="4" t="n"/>
+      <c r="G27" s="4" t="n"/>
+      <c r="H27" s="4" t="n"/>
+      <c r="I27" s="4" t="n"/>
+      <c r="J27" s="4" t="n"/>
+      <c r="K27" s="4" t="n"/>
+      <c r="L27" s="4" t="n"/>
+      <c r="M27" s="4" t="n"/>
+      <c r="N27" s="4" t="n"/>
+      <c r="O27" s="4" t="n"/>
+      <c r="P27" s="4" t="n"/>
+      <c r="Q27" s="4" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
@@ -1928,31 +1928,31 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>C11</t>
+          <t>Rla1, Rla2</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>Condensador de realimentacion</t>
+          <t>Resistencia del LPF A</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>3.9n</t>
+          <t>88.7k</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>3.9n</t>
+          <t>91k</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>poliester 5 % o C0G</t>
+          <t>pelicula metalica 1 %</t>
         </is>
       </c>
       <c r="G28" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H28" s="5" t="n">
         <v>4</v>
@@ -1962,7 +1962,7 @@
         <v/>
       </c>
       <c r="J28" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K28" s="5">
         <f>I28+J28</f>
@@ -1970,7 +1970,7 @@
       </c>
       <c r="L28" s="5" t="inlineStr">
         <is>
-          <t>condensador poliester 3.9nF</t>
+          <t>resistencia 91k 1%</t>
         </is>
       </c>
       <c r="M28" s="6" t="n"/>
@@ -1984,7 +1984,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="Q28" s="5" t="inlineStr"/>
+      <c r="Q28" s="5" t="inlineStr">
+        <is>
+          <t>Con 91k: f0 = 487 Hz</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
@@ -1994,22 +1998,22 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>C12</t>
+          <t>C11</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>Condensador a GND</t>
+          <t>Condensador de realimentacion</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>3.3n</t>
+          <t>3.9n</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>3.3n</t>
+          <t>3.9n</t>
         </is>
       </c>
       <c r="F29" s="5" t="inlineStr">
@@ -2036,7 +2040,7 @@
       </c>
       <c r="L29" s="5" t="inlineStr">
         <is>
-          <t>condensador poliester 3.3nF</t>
+          <t>condensador poliester 3.9nF</t>
         </is>
       </c>
       <c r="M29" s="6" t="n"/>
@@ -2060,141 +2064,137 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
+          <t>C12</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>Condensador a GND</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>3.3n</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>3.3n</t>
+        </is>
+      </c>
+      <c r="F30" s="5" t="inlineStr">
+        <is>
+          <t>poliester 5 % o C0G</t>
+        </is>
+      </c>
+      <c r="G30" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H30" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="I30" s="5">
+        <f>G30*H30</f>
+        <v/>
+      </c>
+      <c r="J30" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="K30" s="5">
+        <f>I30+J30</f>
+        <v/>
+      </c>
+      <c r="L30" s="5" t="inlineStr">
+        <is>
+          <t>condensador poliester 3.3nF</t>
+        </is>
+      </c>
+      <c r="M30" s="6" t="n"/>
+      <c r="N30" s="7" t="n"/>
+      <c r="O30" s="8">
+        <f>IF(N30="","",K30*N30)</f>
+        <v/>
+      </c>
+      <c r="P30" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="Q30" s="5" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>6 LPF A 500 Hz (Q 0.541)</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
           <t>XLA</t>
         </is>
       </c>
-      <c r="C30" s="5" t="inlineStr">
+      <c r="C31" s="5" t="inlineStr">
         <is>
           <t>seccion de op-amp</t>
         </is>
       </c>
-      <c r="D30" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E30" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F30" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G30" s="5" t="n"/>
-      <c r="H30" s="5" t="n"/>
-      <c r="I30" s="5" t="n"/>
-      <c r="J30" s="5" t="n"/>
-      <c r="K30" s="5" t="n"/>
-      <c r="L30" s="5" t="inlineStr"/>
-      <c r="M30" s="5" t="n"/>
-      <c r="N30" s="8" t="n"/>
-      <c r="O30" s="8" t="n"/>
-      <c r="P30" s="5" t="n"/>
-      <c r="Q30" s="5" t="inlineStr">
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F31" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G31" s="5" t="n"/>
+      <c r="H31" s="5" t="n"/>
+      <c r="I31" s="5" t="n"/>
+      <c r="J31" s="5" t="n"/>
+      <c r="K31" s="5" t="n"/>
+      <c r="L31" s="5" t="inlineStr"/>
+      <c r="M31" s="5" t="n"/>
+      <c r="N31" s="8" t="n"/>
+      <c r="O31" s="8" t="n"/>
+      <c r="P31" s="5" t="n"/>
+      <c r="Q31" s="5" t="inlineStr">
         <is>
           <t>Contada en el modulo 11 OP-AMPS</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="4" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
         <is>
           <t>7 LPF B 500 Hz (Q 1.306)</t>
         </is>
       </c>
-      <c r="B31" s="4" t="n"/>
-      <c r="C31" s="4" t="inlineStr">
+      <c r="B32" s="4" t="n"/>
+      <c r="C32" s="4" t="inlineStr">
         <is>
           <t>por canal (x4)</t>
         </is>
       </c>
-      <c r="D31" s="4" t="n"/>
-      <c r="E31" s="4" t="n"/>
-      <c r="F31" s="4" t="n"/>
-      <c r="G31" s="4" t="n"/>
-      <c r="H31" s="4" t="n"/>
-      <c r="I31" s="4" t="n"/>
-      <c r="J31" s="4" t="n"/>
-      <c r="K31" s="4" t="n"/>
-      <c r="L31" s="4" t="n"/>
-      <c r="M31" s="4" t="n"/>
-      <c r="N31" s="4" t="n"/>
-      <c r="O31" s="4" t="n"/>
-      <c r="P31" s="4" t="n"/>
-      <c r="Q31" s="4" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="5" t="inlineStr">
-        <is>
-          <t>7 LPF B 500 Hz (Q 1.306)</t>
-        </is>
-      </c>
-      <c r="B32" s="5" t="inlineStr">
-        <is>
-          <t>Rlb1, Rlb2</t>
-        </is>
-      </c>
-      <c r="C32" s="5" t="inlineStr">
-        <is>
-          <t>Resistencia del LPF B</t>
-        </is>
-      </c>
-      <c r="D32" s="5" t="inlineStr">
-        <is>
-          <t>54.9k</t>
-        </is>
-      </c>
-      <c r="E32" s="5" t="inlineStr">
-        <is>
-          <t>56k</t>
-        </is>
-      </c>
-      <c r="F32" s="5" t="inlineStr">
-        <is>
-          <t>pelicula metalica 1 %</t>
-        </is>
-      </c>
-      <c r="G32" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="H32" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="I32" s="5">
-        <f>G32*H32</f>
-        <v/>
-      </c>
-      <c r="J32" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="K32" s="5">
-        <f>I32+J32</f>
-        <v/>
-      </c>
-      <c r="L32" s="5" t="inlineStr">
-        <is>
-          <t>resistencia 56k 1%</t>
-        </is>
-      </c>
-      <c r="M32" s="6" t="n"/>
-      <c r="N32" s="7" t="n"/>
-      <c r="O32" s="8">
-        <f>IF(N32="","",K32*N32)</f>
-        <v/>
-      </c>
-      <c r="P32" s="6" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="Q32" s="5" t="inlineStr">
-        <is>
-          <t>Con 56k: f0 = 495 Hz</t>
-        </is>
-      </c>
+      <c r="D32" s="4" t="n"/>
+      <c r="E32" s="4" t="n"/>
+      <c r="F32" s="4" t="n"/>
+      <c r="G32" s="4" t="n"/>
+      <c r="H32" s="4" t="n"/>
+      <c r="I32" s="4" t="n"/>
+      <c r="J32" s="4" t="n"/>
+      <c r="K32" s="4" t="n"/>
+      <c r="L32" s="4" t="n"/>
+      <c r="M32" s="4" t="n"/>
+      <c r="N32" s="4" t="n"/>
+      <c r="O32" s="4" t="n"/>
+      <c r="P32" s="4" t="n"/>
+      <c r="Q32" s="4" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
@@ -2204,31 +2204,31 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>C21</t>
+          <t>Rlb1, Rlb2</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>Condensador de realimentacion</t>
+          <t>Resistencia del LPF B</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>15n</t>
+          <t>54.9k</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t>15n</t>
+          <t>56k</t>
         </is>
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>poliester 5 % o C0G</t>
+          <t>pelicula metalica 1 %</t>
         </is>
       </c>
       <c r="G33" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H33" s="5" t="n">
         <v>4</v>
@@ -2238,7 +2238,7 @@
         <v/>
       </c>
       <c r="J33" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K33" s="5">
         <f>I33+J33</f>
@@ -2246,7 +2246,7 @@
       </c>
       <c r="L33" s="5" t="inlineStr">
         <is>
-          <t>condensador poliester 15nF</t>
+          <t>resistencia 56k 1%</t>
         </is>
       </c>
       <c r="M33" s="6" t="n"/>
@@ -2260,7 +2260,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="Q33" s="5" t="inlineStr"/>
+      <c r="Q33" s="5" t="inlineStr">
+        <is>
+          <t>Con 56k: f0 = 495 Hz</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
@@ -2270,22 +2274,22 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>C22</t>
+          <t>C21</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>Condensador a GND</t>
+          <t>Condensador de realimentacion</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>2.2n</t>
+          <t>15n</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>2.2n</t>
+          <t>15n</t>
         </is>
       </c>
       <c r="F34" s="5" t="inlineStr">
@@ -2312,7 +2316,7 @@
       </c>
       <c r="L34" s="5" t="inlineStr">
         <is>
-          <t>condensador poliester 2.2nF</t>
+          <t>condensador poliester 15nF</t>
         </is>
       </c>
       <c r="M34" s="6" t="n"/>
@@ -2336,137 +2340,137 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
+          <t>C22</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>Condensador a GND</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>2.2n</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>2.2n</t>
+        </is>
+      </c>
+      <c r="F35" s="5" t="inlineStr">
+        <is>
+          <t>poliester 5 % o C0G</t>
+        </is>
+      </c>
+      <c r="G35" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H35" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="I35" s="5">
+        <f>G35*H35</f>
+        <v/>
+      </c>
+      <c r="J35" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="K35" s="5">
+        <f>I35+J35</f>
+        <v/>
+      </c>
+      <c r="L35" s="5" t="inlineStr">
+        <is>
+          <t>condensador poliester 2.2nF</t>
+        </is>
+      </c>
+      <c r="M35" s="6" t="n"/>
+      <c r="N35" s="7" t="n"/>
+      <c r="O35" s="8">
+        <f>IF(N35="","",K35*N35)</f>
+        <v/>
+      </c>
+      <c r="P35" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="Q35" s="5" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>7 LPF B 500 Hz (Q 1.306)</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
           <t>XLB</t>
         </is>
       </c>
-      <c r="C35" s="5" t="inlineStr">
+      <c r="C36" s="5" t="inlineStr">
         <is>
           <t>seccion de op-amp</t>
         </is>
       </c>
-      <c r="D35" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E35" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F35" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G35" s="5" t="n"/>
-      <c r="H35" s="5" t="n"/>
-      <c r="I35" s="5" t="n"/>
-      <c r="J35" s="5" t="n"/>
-      <c r="K35" s="5" t="n"/>
-      <c r="L35" s="5" t="inlineStr"/>
-      <c r="M35" s="5" t="n"/>
-      <c r="N35" s="8" t="n"/>
-      <c r="O35" s="8" t="n"/>
-      <c r="P35" s="5" t="n"/>
-      <c r="Q35" s="5" t="inlineStr">
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F36" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G36" s="5" t="n"/>
+      <c r="H36" s="5" t="n"/>
+      <c r="I36" s="5" t="n"/>
+      <c r="J36" s="5" t="n"/>
+      <c r="K36" s="5" t="n"/>
+      <c r="L36" s="5" t="inlineStr"/>
+      <c r="M36" s="5" t="n"/>
+      <c r="N36" s="8" t="n"/>
+      <c r="O36" s="8" t="n"/>
+      <c r="P36" s="5" t="n"/>
+      <c r="Q36" s="5" t="inlineStr">
         <is>
           <t>Contada en el modulo 11 OP-AMPS</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="4" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
         <is>
           <t>8 BUFFER + SALIDA AL ADC</t>
         </is>
       </c>
-      <c r="B36" s="4" t="n"/>
-      <c r="C36" s="4" t="inlineStr">
+      <c r="B37" s="4" t="n"/>
+      <c r="C37" s="4" t="inlineStr">
         <is>
           <t>por canal (x4)</t>
         </is>
       </c>
-      <c r="D36" s="4" t="n"/>
-      <c r="E36" s="4" t="n"/>
-      <c r="F36" s="4" t="n"/>
-      <c r="G36" s="4" t="n"/>
-      <c r="H36" s="4" t="n"/>
-      <c r="I36" s="4" t="n"/>
-      <c r="J36" s="4" t="n"/>
-      <c r="K36" s="4" t="n"/>
-      <c r="L36" s="4" t="n"/>
-      <c r="M36" s="4" t="n"/>
-      <c r="N36" s="4" t="n"/>
-      <c r="O36" s="4" t="n"/>
-      <c r="P36" s="4" t="n"/>
-      <c r="Q36" s="4" t="n"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="5" t="inlineStr">
-        <is>
-          <t>8 BUFFER + SALIDA AL ADC</t>
-        </is>
-      </c>
-      <c r="B37" s="5" t="inlineStr">
-        <is>
-          <t>Rbk</t>
-        </is>
-      </c>
-      <c r="C37" s="5" t="inlineStr">
-        <is>
-          <t>Resistencia del bucket</t>
-        </is>
-      </c>
-      <c r="D37" s="5" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="E37" s="5" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="F37" s="5" t="inlineStr">
-        <is>
-          <t>pelicula metalica 1 %</t>
-        </is>
-      </c>
-      <c r="G37" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="H37" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="I37" s="5">
-        <f>G37*H37</f>
-        <v/>
-      </c>
-      <c r="J37" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="K37" s="5">
-        <f>I37+J37</f>
-        <v/>
-      </c>
-      <c r="L37" s="5" t="inlineStr">
-        <is>
-          <t>resistencia 100 ohm 1%</t>
-        </is>
-      </c>
-      <c r="M37" s="6" t="n"/>
-      <c r="N37" s="7" t="n"/>
-      <c r="O37" s="8">
-        <f>IF(N37="","",K37*N37)</f>
-        <v/>
-      </c>
-      <c r="P37" s="6" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="Q37" s="5" t="inlineStr"/>
+      <c r="D37" s="4" t="n"/>
+      <c r="E37" s="4" t="n"/>
+      <c r="F37" s="4" t="n"/>
+      <c r="G37" s="4" t="n"/>
+      <c r="H37" s="4" t="n"/>
+      <c r="I37" s="4" t="n"/>
+      <c r="J37" s="4" t="n"/>
+      <c r="K37" s="4" t="n"/>
+      <c r="L37" s="4" t="n"/>
+      <c r="M37" s="4" t="n"/>
+      <c r="N37" s="4" t="n"/>
+      <c r="O37" s="4" t="n"/>
+      <c r="P37" s="4" t="n"/>
+      <c r="Q37" s="4" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
@@ -2476,27 +2480,27 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>Cbk</t>
+          <t>Rbk</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>Condensador del bucket</t>
+          <t>Resistencia del bucket</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>1n</t>
+          <t>100</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>1n</t>
+          <t>100</t>
         </is>
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>ceramico C0G/NP0</t>
+          <t>pelicula metalica 1 %</t>
         </is>
       </c>
       <c r="G38" s="5" t="n">
@@ -2518,7 +2522,7 @@
       </c>
       <c r="L38" s="5" t="inlineStr">
         <is>
-          <t>condensador ceramico 1nF NP0</t>
+          <t>resistencia 100 ohm 1%</t>
         </is>
       </c>
       <c r="M38" s="6" t="n"/>
@@ -2542,27 +2546,27 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>ADCk</t>
+          <t>Cbk</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>Cable a Arduino A1..A4 del STM32N6570-DK</t>
+          <t>Condensador del bucket</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1n</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t>jumper Dupont</t>
+          <t>1n</t>
         </is>
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>ceramico C0G/NP0</t>
         </is>
       </c>
       <c r="G39" s="5" t="n">
@@ -2576,7 +2580,7 @@
         <v/>
       </c>
       <c r="J39" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K39" s="5">
         <f>I39+J39</f>
@@ -2584,7 +2588,7 @@
       </c>
       <c r="L39" s="5" t="inlineStr">
         <is>
-          <t>cable dupont macho-macho</t>
+          <t>condensador ceramico 1nF NP0</t>
         </is>
       </c>
       <c r="M39" s="6" t="n"/>
@@ -2598,11 +2602,7 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="Q39" s="5" t="inlineStr">
-        <is>
-          <t>CH1-A1 (PA9), CH2-A2 (PA10), CH3-A3 (PA12), CH4-A4 (PF3). Mas 1 cable de GND. A0 no: comparte ADC con USB1 ISENSE (UM3300)</t>
-        </is>
-      </c>
+      <c r="Q39" s="5" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
@@ -2612,137 +2612,141 @@
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
+          <t>ADCk</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>Cable a Arduino A1..A4 del STM32N6570-DK</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>jumper Dupont</t>
+        </is>
+      </c>
+      <c r="F40" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G40" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H40" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="I40" s="5">
+        <f>G40*H40</f>
+        <v/>
+      </c>
+      <c r="J40" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="K40" s="5">
+        <f>I40+J40</f>
+        <v/>
+      </c>
+      <c r="L40" s="5" t="inlineStr">
+        <is>
+          <t>cable dupont macho-macho</t>
+        </is>
+      </c>
+      <c r="M40" s="6" t="n"/>
+      <c r="N40" s="7" t="n"/>
+      <c r="O40" s="8">
+        <f>IF(N40="","",K40*N40)</f>
+        <v/>
+      </c>
+      <c r="P40" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="Q40" s="5" t="inlineStr">
+        <is>
+          <t>CH1-A1 (PA9), CH2-A2 (PA10), CH3-A3 (PA12), CH4-A4 (PF3). Mas 1 cable de GND. A0 no: comparte ADC con USB1 ISENSE (UM3300)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>8 BUFFER + SALIDA AL ADC</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
           <t>XBF</t>
         </is>
       </c>
-      <c r="C40" s="5" t="inlineStr">
+      <c r="C41" s="5" t="inlineStr">
         <is>
           <t>seccion de op-amp</t>
         </is>
       </c>
-      <c r="D40" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E40" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F40" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G40" s="5" t="n"/>
-      <c r="H40" s="5" t="n"/>
-      <c r="I40" s="5" t="n"/>
-      <c r="J40" s="5" t="n"/>
-      <c r="K40" s="5" t="n"/>
-      <c r="L40" s="5" t="inlineStr"/>
-      <c r="M40" s="5" t="n"/>
-      <c r="N40" s="8" t="n"/>
-      <c r="O40" s="8" t="n"/>
-      <c r="P40" s="5" t="n"/>
-      <c r="Q40" s="5" t="inlineStr">
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F41" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G41" s="5" t="n"/>
+      <c r="H41" s="5" t="n"/>
+      <c r="I41" s="5" t="n"/>
+      <c r="J41" s="5" t="n"/>
+      <c r="K41" s="5" t="n"/>
+      <c r="L41" s="5" t="inlineStr"/>
+      <c r="M41" s="5" t="n"/>
+      <c r="N41" s="8" t="n"/>
+      <c r="O41" s="8" t="n"/>
+      <c r="P41" s="5" t="n"/>
+      <c r="Q41" s="5" t="inlineStr">
         <is>
           <t>Contada en el modulo 11 OP-AMPS</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="4" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
         <is>
           <t>9 VREF 1.65 V (compartido)</t>
         </is>
       </c>
-      <c r="B41" s="4" t="n"/>
-      <c r="C41" s="4" t="inlineStr">
+      <c r="B42" s="4" t="n"/>
+      <c r="C42" s="4" t="inlineStr">
         <is>
           <t>compartido</t>
         </is>
       </c>
-      <c r="D41" s="4" t="n"/>
-      <c r="E41" s="4" t="n"/>
-      <c r="F41" s="4" t="n"/>
-      <c r="G41" s="4" t="n"/>
-      <c r="H41" s="4" t="n"/>
-      <c r="I41" s="4" t="n"/>
-      <c r="J41" s="4" t="n"/>
-      <c r="K41" s="4" t="n"/>
-      <c r="L41" s="4" t="n"/>
-      <c r="M41" s="4" t="n"/>
-      <c r="N41" s="4" t="n"/>
-      <c r="O41" s="4" t="n"/>
-      <c r="P41" s="4" t="n"/>
-      <c r="Q41" s="4" t="n"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="5" t="inlineStr">
-        <is>
-          <t>9 VREF 1.65 V (compartido)</t>
-        </is>
-      </c>
-      <c r="B42" s="5" t="inlineStr">
-        <is>
-          <t>RA1, RA2</t>
-        </is>
-      </c>
-      <c r="C42" s="5" t="inlineStr">
-        <is>
-          <t>Divisor de VREF</t>
-        </is>
-      </c>
-      <c r="D42" s="5" t="inlineStr">
-        <is>
-          <t>100k</t>
-        </is>
-      </c>
-      <c r="E42" s="5" t="inlineStr">
-        <is>
-          <t>100k</t>
-        </is>
-      </c>
-      <c r="F42" s="5" t="inlineStr">
-        <is>
-          <t>pelicula metalica 1 %</t>
-        </is>
-      </c>
-      <c r="G42" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="H42" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="I42" s="5">
-        <f>G42*H42</f>
-        <v/>
-      </c>
-      <c r="J42" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K42" s="5">
-        <f>I42+J42</f>
-        <v/>
-      </c>
-      <c r="L42" s="5" t="inlineStr">
-        <is>
-          <t>resistencia 100k 1%</t>
-        </is>
-      </c>
-      <c r="M42" s="6" t="n"/>
-      <c r="N42" s="7" t="n"/>
-      <c r="O42" s="8">
-        <f>IF(N42="","",K42*N42)</f>
-        <v/>
-      </c>
-      <c r="P42" s="6" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="Q42" s="5" t="inlineStr"/>
+      <c r="D42" s="4" t="n"/>
+      <c r="E42" s="4" t="n"/>
+      <c r="F42" s="4" t="n"/>
+      <c r="G42" s="4" t="n"/>
+      <c r="H42" s="4" t="n"/>
+      <c r="I42" s="4" t="n"/>
+      <c r="J42" s="4" t="n"/>
+      <c r="K42" s="4" t="n"/>
+      <c r="L42" s="4" t="n"/>
+      <c r="M42" s="4" t="n"/>
+      <c r="N42" s="4" t="n"/>
+      <c r="O42" s="4" t="n"/>
+      <c r="P42" s="4" t="n"/>
+      <c r="Q42" s="4" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
@@ -2752,31 +2756,31 @@
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>RA1, RA2</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>Condensador del divisor</t>
+          <t>Divisor de VREF</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>10u</t>
+          <t>100k</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t>10u</t>
+          <t>100k</t>
         </is>
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>ceramico X7R o electrolitico</t>
+          <t>pelicula metalica 1 %</t>
         </is>
       </c>
       <c r="G43" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H43" s="5" t="n">
         <v>1</v>
@@ -2794,7 +2798,7 @@
       </c>
       <c r="L43" s="5" t="inlineStr">
         <is>
-          <t>condensador 10uF</t>
+          <t>resistencia 100k 1%</t>
         </is>
       </c>
       <c r="M43" s="6" t="n"/>
@@ -2818,137 +2822,137 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>Condensador del divisor</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>10u</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t>10u</t>
+        </is>
+      </c>
+      <c r="F44" s="5" t="inlineStr">
+        <is>
+          <t>ceramico X7R o electrolitico</t>
+        </is>
+      </c>
+      <c r="G44" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H44" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I44" s="5">
+        <f>G44*H44</f>
+        <v/>
+      </c>
+      <c r="J44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K44" s="5">
+        <f>I44+J44</f>
+        <v/>
+      </c>
+      <c r="L44" s="5" t="inlineStr">
+        <is>
+          <t>condensador 10uF</t>
+        </is>
+      </c>
+      <c r="M44" s="6" t="n"/>
+      <c r="N44" s="7" t="n"/>
+      <c r="O44" s="8">
+        <f>IF(N44="","",K44*N44)</f>
+        <v/>
+      </c>
+      <c r="P44" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="Q44" s="5" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>9 VREF 1.65 V (compartido)</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
           <t>XVR</t>
         </is>
       </c>
-      <c r="C44" s="5" t="inlineStr">
+      <c r="C45" s="5" t="inlineStr">
         <is>
           <t>seccion de op-amp</t>
         </is>
       </c>
-      <c r="D44" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E44" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F44" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G44" s="5" t="n"/>
-      <c r="H44" s="5" t="n"/>
-      <c r="I44" s="5" t="n"/>
-      <c r="J44" s="5" t="n"/>
-      <c r="K44" s="5" t="n"/>
-      <c r="L44" s="5" t="inlineStr"/>
-      <c r="M44" s="5" t="n"/>
-      <c r="N44" s="8" t="n"/>
-      <c r="O44" s="8" t="n"/>
-      <c r="P44" s="5" t="n"/>
-      <c r="Q44" s="5" t="inlineStr">
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F45" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G45" s="5" t="n"/>
+      <c r="H45" s="5" t="n"/>
+      <c r="I45" s="5" t="n"/>
+      <c r="J45" s="5" t="n"/>
+      <c r="K45" s="5" t="n"/>
+      <c r="L45" s="5" t="inlineStr"/>
+      <c r="M45" s="5" t="n"/>
+      <c r="N45" s="8" t="n"/>
+      <c r="O45" s="8" t="n"/>
+      <c r="P45" s="5" t="n"/>
+      <c r="Q45" s="5" t="inlineStr">
         <is>
           <t>Contada en el modulo 11 OP-AMPS</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="4" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
         <is>
           <t>10 RLD (compartido)</t>
         </is>
       </c>
-      <c r="B45" s="4" t="n"/>
-      <c r="C45" s="4" t="inlineStr">
+      <c r="B46" s="4" t="n"/>
+      <c r="C46" s="4" t="inlineStr">
         <is>
           <t>compartido</t>
         </is>
       </c>
-      <c r="D45" s="4" t="n"/>
-      <c r="E45" s="4" t="n"/>
-      <c r="F45" s="4" t="n"/>
-      <c r="G45" s="4" t="n"/>
-      <c r="H45" s="4" t="n"/>
-      <c r="I45" s="4" t="n"/>
-      <c r="J45" s="4" t="n"/>
-      <c r="K45" s="4" t="n"/>
-      <c r="L45" s="4" t="n"/>
-      <c r="M45" s="4" t="n"/>
-      <c r="N45" s="4" t="n"/>
-      <c r="O45" s="4" t="n"/>
-      <c r="P45" s="4" t="n"/>
-      <c r="Q45" s="4" t="n"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="5" t="inlineStr">
-        <is>
-          <t>10 RLD (compartido)</t>
-        </is>
-      </c>
-      <c r="B46" s="5" t="inlineStr">
-        <is>
-          <t>RSM1..RSM4</t>
-        </is>
-      </c>
-      <c r="C46" s="5" t="inlineStr">
-        <is>
-          <t>Sensado de modo comun (punto medio de RG)</t>
-        </is>
-      </c>
-      <c r="D46" s="5" t="inlineStr">
-        <is>
-          <t>604k</t>
-        </is>
-      </c>
-      <c r="E46" s="5" t="inlineStr">
-        <is>
-          <t>620k</t>
-        </is>
-      </c>
-      <c r="F46" s="5" t="inlineStr">
-        <is>
-          <t>pelicula metalica 1 %</t>
-        </is>
-      </c>
-      <c r="G46" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="H46" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="I46" s="5">
-        <f>G46*H46</f>
-        <v/>
-      </c>
-      <c r="J46" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="K46" s="5">
-        <f>I46+J46</f>
-        <v/>
-      </c>
-      <c r="L46" s="5" t="inlineStr">
-        <is>
-          <t>resistencia 620k 1%</t>
-        </is>
-      </c>
-      <c r="M46" s="6" t="n"/>
-      <c r="N46" s="7" t="n"/>
-      <c r="O46" s="8">
-        <f>IF(N46="","",K46*N46)</f>
-        <v/>
-      </c>
-      <c r="P46" s="6" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="Q46" s="5" t="inlineStr"/>
+      <c r="D46" s="4" t="n"/>
+      <c r="E46" s="4" t="n"/>
+      <c r="F46" s="4" t="n"/>
+      <c r="G46" s="4" t="n"/>
+      <c r="H46" s="4" t="n"/>
+      <c r="I46" s="4" t="n"/>
+      <c r="J46" s="4" t="n"/>
+      <c r="K46" s="4" t="n"/>
+      <c r="L46" s="4" t="n"/>
+      <c r="M46" s="4" t="n"/>
+      <c r="N46" s="4" t="n"/>
+      <c r="O46" s="4" t="n"/>
+      <c r="P46" s="4" t="n"/>
+      <c r="Q46" s="4" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
@@ -2958,31 +2962,31 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>CINT</t>
+          <t>RSM1..RSM4</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>Condensador del integrador</t>
+          <t>Sensado de modo comun (punto medio de RG)</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>1n</t>
+          <t>604k</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t>1n</t>
+          <t>620k</t>
         </is>
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>ceramico C0G/NP0</t>
+          <t>pelicula metalica 1 %</t>
         </is>
       </c>
       <c r="G47" s="5" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H47" s="5" t="n">
         <v>1</v>
@@ -3000,7 +3004,7 @@
       </c>
       <c r="L47" s="5" t="inlineStr">
         <is>
-          <t>condensador ceramico 1nF NP0</t>
+          <t>resistencia 620k 1%</t>
         </is>
       </c>
       <c r="M47" s="6" t="n"/>
@@ -3014,11 +3018,7 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="Q47" s="5" t="inlineStr">
-        <is>
-          <t>Si oscila en banco: 2.2n</t>
-        </is>
-      </c>
+      <c r="Q47" s="5" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
@@ -3028,27 +3028,27 @@
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>RPAR</t>
+          <t>CINT</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>Resistencia en paralelo al integrador</t>
+          <t>Condensador del integrador</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>10M</t>
+          <t>1n</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t>10M</t>
+          <t>1n</t>
         </is>
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>pelicula 5 %</t>
+          <t>ceramico C0G/NP0</t>
         </is>
       </c>
       <c r="G48" s="5" t="n">
@@ -3070,7 +3070,7 @@
       </c>
       <c r="L48" s="5" t="inlineStr">
         <is>
-          <t>resistencia 10M</t>
+          <t>condensador ceramico 1nF NP0</t>
         </is>
       </c>
       <c r="M48" s="6" t="n"/>
@@ -3084,7 +3084,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="Q48" s="5" t="inlineStr"/>
+      <c r="Q48" s="5" t="inlineStr">
+        <is>
+          <t>Si oscila en banco: 2.2n</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
@@ -3094,27 +3098,27 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>RLIM</t>
+          <t>RPAR</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>Resistencia de seguridad al electrodo RLD</t>
+          <t>Resistencia en paralelo al integrador</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>390k</t>
+          <t>10M</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t>390k</t>
+          <t>10M</t>
         </is>
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>pelicula metalica 1 %</t>
+          <t>pelicula 5 %</t>
         </is>
       </c>
       <c r="G49" s="5" t="n">
@@ -3136,7 +3140,7 @@
       </c>
       <c r="L49" s="5" t="inlineStr">
         <is>
-          <t>resistencia 390k 1%</t>
+          <t>resistencia 10M</t>
         </is>
       </c>
       <c r="M49" s="6" t="n"/>
@@ -3150,11 +3154,7 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="Q49" s="5" t="inlineStr">
-        <is>
-          <t>Limita la corriente al paciente</t>
-        </is>
-      </c>
+      <c r="Q49" s="5" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
@@ -3164,147 +3164,141 @@
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
+          <t>RLIM</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>Resistencia de seguridad al electrodo RLD</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>390k</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>390k</t>
+        </is>
+      </c>
+      <c r="F50" s="5" t="inlineStr">
+        <is>
+          <t>pelicula metalica 1 %</t>
+        </is>
+      </c>
+      <c r="G50" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H50" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I50" s="5">
+        <f>G50*H50</f>
+        <v/>
+      </c>
+      <c r="J50" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="K50" s="5">
+        <f>I50+J50</f>
+        <v/>
+      </c>
+      <c r="L50" s="5" t="inlineStr">
+        <is>
+          <t>resistencia 390k 1%</t>
+        </is>
+      </c>
+      <c r="M50" s="6" t="n"/>
+      <c r="N50" s="7" t="n"/>
+      <c r="O50" s="8">
+        <f>IF(N50="","",K50*N50)</f>
+        <v/>
+      </c>
+      <c r="P50" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="Q50" s="5" t="inlineStr">
+        <is>
+          <t>Limita la corriente al paciente</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>10 RLD (compartido)</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
           <t>XRLD</t>
         </is>
       </c>
-      <c r="C50" s="5" t="inlineStr">
+      <c r="C51" s="5" t="inlineStr">
         <is>
           <t>seccion de op-amp</t>
         </is>
       </c>
-      <c r="D50" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E50" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F50" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G50" s="5" t="n"/>
-      <c r="H50" s="5" t="n"/>
-      <c r="I50" s="5" t="n"/>
-      <c r="J50" s="5" t="n"/>
-      <c r="K50" s="5" t="n"/>
-      <c r="L50" s="5" t="inlineStr"/>
-      <c r="M50" s="5" t="n"/>
-      <c r="N50" s="8" t="n"/>
-      <c r="O50" s="8" t="n"/>
-      <c r="P50" s="5" t="n"/>
-      <c r="Q50" s="5" t="inlineStr">
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F51" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G51" s="5" t="n"/>
+      <c r="H51" s="5" t="n"/>
+      <c r="I51" s="5" t="n"/>
+      <c r="J51" s="5" t="n"/>
+      <c r="K51" s="5" t="n"/>
+      <c r="L51" s="5" t="inlineStr"/>
+      <c r="M51" s="5" t="n"/>
+      <c r="N51" s="8" t="n"/>
+      <c r="O51" s="8" t="n"/>
+      <c r="P51" s="5" t="n"/>
+      <c r="Q51" s="5" t="inlineStr">
         <is>
           <t>Contada en el modulo 11 OP-AMPS</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="4" t="inlineStr">
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
         <is>
           <t>11 OP-AMPS (paquetes)</t>
         </is>
       </c>
-      <c r="B51" s="4" t="n"/>
-      <c r="C51" s="4" t="inlineStr">
+      <c r="B52" s="4" t="n"/>
+      <c r="C52" s="4" t="inlineStr">
         <is>
           <t>compartido</t>
         </is>
       </c>
-      <c r="D51" s="4" t="n"/>
-      <c r="E51" s="4" t="n"/>
-      <c r="F51" s="4" t="n"/>
-      <c r="G51" s="4" t="n"/>
-      <c r="H51" s="4" t="n"/>
-      <c r="I51" s="4" t="n"/>
-      <c r="J51" s="4" t="n"/>
-      <c r="K51" s="4" t="n"/>
-      <c r="L51" s="4" t="n"/>
-      <c r="M51" s="4" t="n"/>
-      <c r="N51" s="4" t="n"/>
-      <c r="O51" s="4" t="n"/>
-      <c r="P51" s="4" t="n"/>
-      <c r="Q51" s="4" t="n"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="5" t="inlineStr">
-        <is>
-          <t>11 OP-AMPS (paquetes)</t>
-        </is>
-      </c>
-      <c r="B52" s="5" t="inlineStr">
-        <is>
-          <t>XHP..XBF x4, XRLD, XVR</t>
-        </is>
-      </c>
-      <c r="C52" s="5" t="inlineStr">
-        <is>
-          <t>Op-amp cuadruple MCP6004</t>
-        </is>
-      </c>
-      <c r="D52" s="5" t="inlineStr">
-        <is>
-          <t>MCP6004</t>
-        </is>
-      </c>
-      <c r="E52" s="5" t="inlineStr">
-        <is>
-          <t>MCP6004-I/SL</t>
-        </is>
-      </c>
-      <c r="F52" s="5" t="inlineStr">
-        <is>
-          <t>SOIC-14</t>
-        </is>
-      </c>
-      <c r="G52" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="H52" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="I52" s="5">
-        <f>G52*H52</f>
-        <v/>
-      </c>
-      <c r="J52" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="K52" s="5">
-        <f>I52+J52</f>
-        <v/>
-      </c>
-      <c r="L52" s="5" t="inlineStr">
-        <is>
-          <t>MCP6004-I/SL</t>
-        </is>
-      </c>
-      <c r="M52" s="6" t="inlineStr">
-        <is>
-          <t>RS Chile</t>
-        </is>
-      </c>
-      <c r="N52" s="7" t="n">
-        <v>809</v>
-      </c>
-      <c r="O52" s="8">
-        <f>IF(N52="","",K52*N52)</f>
-        <v/>
-      </c>
-      <c r="P52" s="6" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="Q52" s="5" t="inlineStr">
-        <is>
-          <t>22 secciones = 5 por canal x 4 + RLD + VREF (2 libres). RS Chile vende en paquetes de 10</t>
-        </is>
-      </c>
+      <c r="D52" s="4" t="n"/>
+      <c r="E52" s="4" t="n"/>
+      <c r="F52" s="4" t="n"/>
+      <c r="G52" s="4" t="n"/>
+      <c r="H52" s="4" t="n"/>
+      <c r="I52" s="4" t="n"/>
+      <c r="J52" s="4" t="n"/>
+      <c r="K52" s="4" t="n"/>
+      <c r="L52" s="4" t="n"/>
+      <c r="M52" s="4" t="n"/>
+      <c r="N52" s="4" t="n"/>
+      <c r="O52" s="4" t="n"/>
+      <c r="P52" s="4" t="n"/>
+      <c r="Q52" s="4" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
@@ -3314,27 +3308,27 @@
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>XHP..XBF x4, XRLD, XVR</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>Adaptador SOIC-14 a DIP-14</t>
+          <t>Op-amp cuadruple MCP6004</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>MCP6004</t>
         </is>
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t>SOIC14 a DIP14</t>
+          <t>MCP6004-I/SL</t>
         </is>
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>PCB adaptador</t>
+          <t>SOIC-14</t>
         </is>
       </c>
       <c r="G53" s="5" t="n">
@@ -3348,7 +3342,7 @@
         <v/>
       </c>
       <c r="J53" s="5" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K53" s="5">
         <f>I53+J53</f>
@@ -3356,11 +3350,17 @@
       </c>
       <c r="L53" s="5" t="inlineStr">
         <is>
-          <t>adaptador SOIC14 a DIP14</t>
-        </is>
-      </c>
-      <c r="M53" s="6" t="n"/>
-      <c r="N53" s="7" t="n"/>
+          <t>MCP6004-I/SL</t>
+        </is>
+      </c>
+      <c r="M53" s="6" t="inlineStr">
+        <is>
+          <t>RS Chile</t>
+        </is>
+      </c>
+      <c r="N53" s="7" t="n">
+        <v>809</v>
+      </c>
       <c r="O53" s="8">
         <f>IF(N53="","",K53*N53)</f>
         <v/>
@@ -3372,7 +3372,7 @@
       </c>
       <c r="Q53" s="5" t="inlineStr">
         <is>
-          <t>Para montar el MCP6004-I/SL en perfboard</t>
+          <t>22 secciones = 5 por canal x 4 + RLD + VREF (2 libres). RS Chile vende en paquetes de 10</t>
         </is>
       </c>
     </row>
@@ -3389,7 +3389,7 @@
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>Zocalo DIP-14</t>
+          <t>Adaptador SOIC-14 a DIP-14</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
@@ -3399,12 +3399,12 @@
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t>DIP-14</t>
+          <t>SOIC14 a DIP14</t>
         </is>
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>zocalo</t>
+          <t>PCB adaptador</t>
         </is>
       </c>
       <c r="G54" s="5" t="n">
@@ -3426,7 +3426,7 @@
       </c>
       <c r="L54" s="5" t="inlineStr">
         <is>
-          <t>zocalo DIP 14 pines</t>
+          <t>adaptador SOIC14 a DIP14</t>
         </is>
       </c>
       <c r="M54" s="6" t="n"/>
@@ -3442,7 +3442,7 @@
       </c>
       <c r="Q54" s="5" t="inlineStr">
         <is>
-          <t>Si los op-amps son dobles: 11 zocalos DIP-8</t>
+          <t>Para montar el MCP6004-I/SL en perfboard</t>
         </is>
       </c>
     </row>
@@ -3459,22 +3459,22 @@
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>Desacople de cada op-amp</t>
+          <t>Zocalo DIP-14</t>
         </is>
       </c>
       <c r="D55" s="5" t="inlineStr">
         <is>
-          <t>100n</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t>100n</t>
+          <t>DIP-14</t>
         </is>
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>ceramico X7R</t>
+          <t>zocalo</t>
         </is>
       </c>
       <c r="G55" s="5" t="n">
@@ -3488,7 +3488,7 @@
         <v/>
       </c>
       <c r="J55" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K55" s="5">
         <f>I55+J55</f>
@@ -3496,7 +3496,7 @@
       </c>
       <c r="L55" s="5" t="inlineStr">
         <is>
-          <t>condensador ceramico 100nF</t>
+          <t>zocalo DIP 14 pines</t>
         </is>
       </c>
       <c r="M55" s="6" t="n"/>
@@ -3512,112 +3512,106 @@
       </c>
       <c r="Q55" s="5" t="inlineStr">
         <is>
+          <t>Si los op-amps son dobles: 11 zocalos DIP-8</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>11 OP-AMPS (paquetes)</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>Desacople de cada op-amp</t>
+        </is>
+      </c>
+      <c r="D56" s="5" t="inlineStr">
+        <is>
+          <t>100n</t>
+        </is>
+      </c>
+      <c r="E56" s="5" t="inlineStr">
+        <is>
+          <t>100n</t>
+        </is>
+      </c>
+      <c r="F56" s="5" t="inlineStr">
+        <is>
+          <t>ceramico X7R</t>
+        </is>
+      </c>
+      <c r="G56" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="H56" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I56" s="5">
+        <f>G56*H56</f>
+        <v/>
+      </c>
+      <c r="J56" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="K56" s="5">
+        <f>I56+J56</f>
+        <v/>
+      </c>
+      <c r="L56" s="5" t="inlineStr">
+        <is>
+          <t>condensador ceramico 100nF</t>
+        </is>
+      </c>
+      <c r="M56" s="6" t="n"/>
+      <c r="N56" s="7" t="n"/>
+      <c r="O56" s="8">
+        <f>IF(N56="","",K56*N56)</f>
+        <v/>
+      </c>
+      <c r="P56" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="Q56" s="5" t="inlineStr">
+        <is>
           <t>Pegado al pin de alimentacion</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="4" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
         <is>
           <t>12 ALIMENTACION (a bateria)</t>
         </is>
       </c>
-      <c r="B56" s="4" t="n"/>
-      <c r="C56" s="4" t="inlineStr">
+      <c r="B57" s="4" t="n"/>
+      <c r="C57" s="4" t="inlineStr">
         <is>
           <t>compartido</t>
         </is>
       </c>
-      <c r="D56" s="4" t="n"/>
-      <c r="E56" s="4" t="n"/>
-      <c r="F56" s="4" t="n"/>
-      <c r="G56" s="4" t="n"/>
-      <c r="H56" s="4" t="n"/>
-      <c r="I56" s="4" t="n"/>
-      <c r="J56" s="4" t="n"/>
-      <c r="K56" s="4" t="n"/>
-      <c r="L56" s="4" t="n"/>
-      <c r="M56" s="4" t="n"/>
-      <c r="N56" s="4" t="n"/>
-      <c r="O56" s="4" t="n"/>
-      <c r="P56" s="4" t="n"/>
-      <c r="Q56" s="4" t="n"/>
-    </row>
-    <row r="57">
-      <c r="A57" s="5" t="inlineStr">
-        <is>
-          <t>12 ALIMENTACION (a bateria)</t>
-        </is>
-      </c>
-      <c r="B57" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C57" s="5" t="inlineStr">
-        <is>
-          <t>Regulador LDO 3.3 V</t>
-        </is>
-      </c>
-      <c r="D57" s="5" t="inlineStr">
-        <is>
-          <t>MCP1700-3302E</t>
-        </is>
-      </c>
-      <c r="E57" s="5" t="inlineStr">
-        <is>
-          <t>MCP1700-3302E TO-92</t>
-        </is>
-      </c>
-      <c r="F57" s="5" t="inlineStr">
-        <is>
-          <t>LDO 250 mA</t>
-        </is>
-      </c>
-      <c r="G57" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="H57" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="I57" s="5">
-        <f>G57*H57</f>
-        <v/>
-      </c>
-      <c r="J57" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="K57" s="5">
-        <f>I57+J57</f>
-        <v/>
-      </c>
-      <c r="L57" s="5" t="inlineStr">
-        <is>
-          <t>MCP1700 3.3V TO-92</t>
-        </is>
-      </c>
-      <c r="M57" s="6" t="inlineStr">
-        <is>
-          <t>HUBOT</t>
-        </is>
-      </c>
-      <c r="N57" s="7" t="n">
-        <v>890</v>
-      </c>
-      <c r="O57" s="8">
-        <f>IF(N57="","",K57*N57)</f>
-        <v/>
-      </c>
-      <c r="P57" s="6" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="Q57" s="5" t="inlineStr">
-        <is>
-          <t>EJEMPLO de llenado: CLP 890 c/IVA en hubot.cl (30-sep-2026). Tu LDO de 3.0 V no sirve</t>
-        </is>
-      </c>
+      <c r="D57" s="4" t="n"/>
+      <c r="E57" s="4" t="n"/>
+      <c r="F57" s="4" t="n"/>
+      <c r="G57" s="4" t="n"/>
+      <c r="H57" s="4" t="n"/>
+      <c r="I57" s="4" t="n"/>
+      <c r="J57" s="4" t="n"/>
+      <c r="K57" s="4" t="n"/>
+      <c r="L57" s="4" t="n"/>
+      <c r="M57" s="4" t="n"/>
+      <c r="N57" s="4" t="n"/>
+      <c r="O57" s="4" t="n"/>
+      <c r="P57" s="4" t="n"/>
+      <c r="Q57" s="4" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="5" t="inlineStr">
@@ -3632,26 +3626,26 @@
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>Condensadores del LDO (entrada y salida)</t>
+          <t>Regulador LDO 3.3 V</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>1u</t>
+          <t>MCP1700-3302E</t>
         </is>
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t>1u</t>
+          <t>MCP1700-3302E TO-92</t>
         </is>
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>ceramico X7R</t>
+          <t>LDO 250 mA</t>
         </is>
       </c>
       <c r="G58" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H58" s="5" t="n">
         <v>1</v>
@@ -3669,11 +3663,17 @@
       </c>
       <c r="L58" s="5" t="inlineStr">
         <is>
-          <t>condensador ceramico 1uF</t>
-        </is>
-      </c>
-      <c r="M58" s="6" t="n"/>
-      <c r="N58" s="7" t="n"/>
+          <t>MCP1700 3.3V TO-92</t>
+        </is>
+      </c>
+      <c r="M58" s="6" t="inlineStr">
+        <is>
+          <t>HUBOT</t>
+        </is>
+      </c>
+      <c r="N58" s="7" t="n">
+        <v>890</v>
+      </c>
       <c r="O58" s="8">
         <f>IF(N58="","",K58*N58)</f>
         <v/>
@@ -3685,7 +3685,7 @@
       </c>
       <c r="Q58" s="5" t="inlineStr">
         <is>
-          <t>Ya tienes 2 x 1uF 0402 (SMD): sirven si los sueldas</t>
+          <t>EJEMPLO de llenado: CLP 890 c/IVA en hubot.cl (30-sep-2026). Tu LDO de 3.0 V no sirve</t>
         </is>
       </c>
     </row>
@@ -3702,26 +3702,26 @@
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>Condensador bulk del riel 3.3 V</t>
+          <t>Condensadores del LDO (entrada y salida)</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
-          <t>10u</t>
+          <t>1u</t>
         </is>
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t>10u</t>
+          <t>1u</t>
         </is>
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>ceramico o electrolitico</t>
+          <t>ceramico X7R</t>
         </is>
       </c>
       <c r="G59" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H59" s="5" t="n">
         <v>1</v>
@@ -3739,7 +3739,7 @@
       </c>
       <c r="L59" s="5" t="inlineStr">
         <is>
-          <t>condensador 10uF</t>
+          <t>condensador ceramico 1uF</t>
         </is>
       </c>
       <c r="M59" s="6" t="n"/>
@@ -3753,7 +3753,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="Q59" s="5" t="inlineStr"/>
+      <c r="Q59" s="5" t="inlineStr">
+        <is>
+          <t>Ya tienes 2 x 1uF 0402 (SMD): sirven si los sueldas</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="5" t="inlineStr">
@@ -3768,22 +3772,22 @@
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>Portapilas 3 x AA</t>
+          <t>Condensador bulk del riel 3.3 V</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10u</t>
         </is>
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t>3xAA</t>
+          <t>10u</t>
         </is>
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>ceramico o electrolitico</t>
         </is>
       </c>
       <c r="G60" s="5" t="n">
@@ -3797,7 +3801,7 @@
         <v/>
       </c>
       <c r="J60" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K60" s="5">
         <f>I60+J60</f>
@@ -3805,7 +3809,7 @@
       </c>
       <c r="L60" s="5" t="inlineStr">
         <is>
-          <t>portapilas 3 AA</t>
+          <t>condensador 10uF</t>
         </is>
       </c>
       <c r="M60" s="6" t="n"/>
@@ -3819,11 +3823,7 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="Q60" s="5" t="inlineStr">
-        <is>
-          <t>4.5 V nominal; mantiene el AFE aislado de la red</t>
-        </is>
-      </c>
+      <c r="Q60" s="5" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="5" t="inlineStr">
@@ -3838,7 +3838,7 @@
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>Pilas AA</t>
+          <t>Portapilas 3 x AA</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
@@ -3848,16 +3848,16 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t>AA</t>
+          <t>3xAA</t>
         </is>
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>alcalina</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G61" s="5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H61" s="5" t="n">
         <v>1</v>
@@ -3867,7 +3867,7 @@
         <v/>
       </c>
       <c r="J61" s="5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K61" s="5">
         <f>I61+J61</f>
@@ -3875,7 +3875,7 @@
       </c>
       <c r="L61" s="5" t="inlineStr">
         <is>
-          <t>pila AA</t>
+          <t>portapilas 3 AA</t>
         </is>
       </c>
       <c r="M61" s="6" t="n"/>
@@ -3889,7 +3889,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="Q61" s="5" t="inlineStr"/>
+      <c r="Q61" s="5" t="inlineStr">
+        <is>
+          <t>4.5 V nominal; mantiene el AFE aislado de la red</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="5" t="inlineStr">
@@ -3904,7 +3908,7 @@
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>Interruptor</t>
+          <t>Pilas AA</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
@@ -3914,16 +3918,16 @@
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t>deslizante</t>
+          <t>AA</t>
         </is>
       </c>
       <c r="F62" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>alcalina</t>
         </is>
       </c>
       <c r="G62" s="5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H62" s="5" t="n">
         <v>1</v>
@@ -3933,7 +3937,7 @@
         <v/>
       </c>
       <c r="J62" s="5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K62" s="5">
         <f>I62+J62</f>
@@ -3941,7 +3945,7 @@
       </c>
       <c r="L62" s="5" t="inlineStr">
         <is>
-          <t>interruptor deslizante</t>
+          <t>pila AA</t>
         </is>
       </c>
       <c r="M62" s="6" t="n"/>
@@ -3958,101 +3962,97 @@
       <c r="Q62" s="5" t="inlineStr"/>
     </row>
     <row r="63">
-      <c r="A63" s="4" t="inlineStr">
+      <c r="A63" s="5" t="inlineStr">
+        <is>
+          <t>12 ALIMENTACION (a bateria)</t>
+        </is>
+      </c>
+      <c r="B63" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C63" s="5" t="inlineStr">
+        <is>
+          <t>Interruptor</t>
+        </is>
+      </c>
+      <c r="D63" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E63" s="5" t="inlineStr">
+        <is>
+          <t>deslizante</t>
+        </is>
+      </c>
+      <c r="F63" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G63" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H63" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I63" s="5">
+        <f>G63*H63</f>
+        <v/>
+      </c>
+      <c r="J63" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K63" s="5">
+        <f>I63+J63</f>
+        <v/>
+      </c>
+      <c r="L63" s="5" t="inlineStr">
+        <is>
+          <t>interruptor deslizante</t>
+        </is>
+      </c>
+      <c r="M63" s="6" t="n"/>
+      <c r="N63" s="7" t="n"/>
+      <c r="O63" s="8">
+        <f>IF(N63="","",K63*N63)</f>
+        <v/>
+      </c>
+      <c r="P63" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="Q63" s="5" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="4" t="inlineStr">
         <is>
           <t>13 ELECTRODOS Y CABLES</t>
         </is>
       </c>
-      <c r="B63" s="4" t="n"/>
-      <c r="C63" s="4" t="inlineStr">
+      <c r="B64" s="4" t="n"/>
+      <c r="C64" s="4" t="inlineStr">
         <is>
           <t>compartido</t>
         </is>
       </c>
-      <c r="D63" s="4" t="n"/>
-      <c r="E63" s="4" t="n"/>
-      <c r="F63" s="4" t="n"/>
-      <c r="G63" s="4" t="n"/>
-      <c r="H63" s="4" t="n"/>
-      <c r="I63" s="4" t="n"/>
-      <c r="J63" s="4" t="n"/>
-      <c r="K63" s="4" t="n"/>
-      <c r="L63" s="4" t="n"/>
-      <c r="M63" s="4" t="n"/>
-      <c r="N63" s="4" t="n"/>
-      <c r="O63" s="4" t="n"/>
-      <c r="P63" s="4" t="n"/>
-      <c r="Q63" s="4" t="n"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="5" t="inlineStr">
-        <is>
-          <t>13 ELECTRODOS Y CABLES</t>
-        </is>
-      </c>
-      <c r="B64" s="5" t="inlineStr">
-        <is>
-          <t>XE1P..XE4N, XER</t>
-        </is>
-      </c>
-      <c r="C64" s="5" t="inlineStr">
-        <is>
-          <t>Electrodo Ag/AgCl con broche</t>
-        </is>
-      </c>
-      <c r="D64" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E64" s="5" t="inlineStr">
-        <is>
-          <t>3M Red Dot 2228/2560</t>
-        </is>
-      </c>
-      <c r="F64" s="5" t="inlineStr">
-        <is>
-          <t>desechable</t>
-        </is>
-      </c>
-      <c r="G64" s="5" t="n">
-        <v>9</v>
-      </c>
-      <c r="H64" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="I64" s="5">
-        <f>G64*H64</f>
-        <v/>
-      </c>
-      <c r="J64" s="5" t="n">
-        <v>41</v>
-      </c>
-      <c r="K64" s="5">
-        <f>I64+J64</f>
-        <v/>
-      </c>
-      <c r="L64" s="5" t="inlineStr">
-        <is>
-          <t>electrodo ECG 3M 2228</t>
-        </is>
-      </c>
-      <c r="M64" s="6" t="n"/>
-      <c r="N64" s="7" t="n"/>
-      <c r="O64" s="8">
-        <f>IF(N64="","",K64*N64)</f>
-        <v/>
-      </c>
-      <c r="P64" s="6" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="Q64" s="5" t="inlineStr">
-        <is>
-          <t>9 por sesion (8 de senal + 1 RLD); caja de 50</t>
-        </is>
-      </c>
+      <c r="D64" s="4" t="n"/>
+      <c r="E64" s="4" t="n"/>
+      <c r="F64" s="4" t="n"/>
+      <c r="G64" s="4" t="n"/>
+      <c r="H64" s="4" t="n"/>
+      <c r="I64" s="4" t="n"/>
+      <c r="J64" s="4" t="n"/>
+      <c r="K64" s="4" t="n"/>
+      <c r="L64" s="4" t="n"/>
+      <c r="M64" s="4" t="n"/>
+      <c r="N64" s="4" t="n"/>
+      <c r="O64" s="4" t="n"/>
+      <c r="P64" s="4" t="n"/>
+      <c r="Q64" s="4" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="5" t="inlineStr">
@@ -4062,12 +4062,12 @@
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>XE1P..XE4N, XER</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>Cable con broche (snap) para electrodo</t>
+          <t>Electrodo Ag/AgCl con broche</t>
         </is>
       </c>
       <c r="D65" s="5" t="inlineStr">
@@ -4077,12 +4077,12 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t>broche 4 mm</t>
+          <t>3M Red Dot 2228/2560</t>
         </is>
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>desechable</t>
         </is>
       </c>
       <c r="G65" s="5" t="n">
@@ -4096,7 +4096,7 @@
         <v/>
       </c>
       <c r="J65" s="5" t="n">
-        <v>1</v>
+        <v>41</v>
       </c>
       <c r="K65" s="5">
         <f>I65+J65</f>
@@ -4104,7 +4104,7 @@
       </c>
       <c r="L65" s="5" t="inlineStr">
         <is>
-          <t>cable electrodo broche snap</t>
+          <t>electrodo ECG 3M 2228</t>
         </is>
       </c>
       <c r="M65" s="6" t="n"/>
@@ -4120,7 +4120,7 @@
       </c>
       <c r="Q65" s="5" t="inlineStr">
         <is>
-          <t>O 3 cables ECG de 3 derivaciones</t>
+          <t>9 por sesion (8 de senal + 1 RLD); caja de 50</t>
         </is>
       </c>
     </row>
@@ -4137,7 +4137,7 @@
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>Alcohol isopropilico / gel</t>
+          <t>Cable con broche (snap) para electrodo</t>
         </is>
       </c>
       <c r="D66" s="5" t="inlineStr">
@@ -4147,7 +4147,7 @@
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>broche 4 mm</t>
         </is>
       </c>
       <c r="F66" s="5" t="inlineStr">
@@ -4156,7 +4156,7 @@
         </is>
       </c>
       <c r="G66" s="5" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="H66" s="5" t="n">
         <v>1</v>
@@ -4166,7 +4166,7 @@
         <v/>
       </c>
       <c r="J66" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K66" s="5">
         <f>I66+J66</f>
@@ -4174,7 +4174,7 @@
       </c>
       <c r="L66" s="5" t="inlineStr">
         <is>
-          <t>alcohol isopropilico</t>
+          <t>cable electrodo broche snap</t>
         </is>
       </c>
       <c r="M66" s="6" t="n"/>
@@ -4190,102 +4190,106 @@
       </c>
       <c r="Q66" s="5" t="inlineStr">
         <is>
+          <t>O 3 cables ECG de 3 derivaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="5" t="inlineStr">
+        <is>
+          <t>13 ELECTRODOS Y CABLES</t>
+        </is>
+      </c>
+      <c r="B67" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C67" s="5" t="inlineStr">
+        <is>
+          <t>Alcohol isopropilico / gel</t>
+        </is>
+      </c>
+      <c r="D67" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E67" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F67" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G67" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H67" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I67" s="5">
+        <f>G67*H67</f>
+        <v/>
+      </c>
+      <c r="J67" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K67" s="5">
+        <f>I67+J67</f>
+        <v/>
+      </c>
+      <c r="L67" s="5" t="inlineStr">
+        <is>
+          <t>alcohol isopropilico</t>
+        </is>
+      </c>
+      <c r="M67" s="6" t="n"/>
+      <c r="N67" s="7" t="n"/>
+      <c r="O67" s="8">
+        <f>IF(N67="","",K67*N67)</f>
+        <v/>
+      </c>
+      <c r="P67" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="Q67" s="5" t="inlineStr">
+        <is>
           <t>Preparar la piel</t>
         </is>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" s="4" t="inlineStr">
+    <row r="68">
+      <c r="A68" s="4" t="inlineStr">
         <is>
           <t>14 MECANICA E INTERCONEXION</t>
         </is>
       </c>
-      <c r="B67" s="4" t="n"/>
-      <c r="C67" s="4" t="inlineStr">
+      <c r="B68" s="4" t="n"/>
+      <c r="C68" s="4" t="inlineStr">
         <is>
           <t>compartido</t>
         </is>
       </c>
-      <c r="D67" s="4" t="n"/>
-      <c r="E67" s="4" t="n"/>
-      <c r="F67" s="4" t="n"/>
-      <c r="G67" s="4" t="n"/>
-      <c r="H67" s="4" t="n"/>
-      <c r="I67" s="4" t="n"/>
-      <c r="J67" s="4" t="n"/>
-      <c r="K67" s="4" t="n"/>
-      <c r="L67" s="4" t="n"/>
-      <c r="M67" s="4" t="n"/>
-      <c r="N67" s="4" t="n"/>
-      <c r="O67" s="4" t="n"/>
-      <c r="P67" s="4" t="n"/>
-      <c r="Q67" s="4" t="n"/>
-    </row>
-    <row r="68">
-      <c r="A68" s="5" t="inlineStr">
-        <is>
-          <t>14 MECANICA E INTERCONEXION</t>
-        </is>
-      </c>
-      <c r="B68" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C68" s="5" t="inlineStr">
-        <is>
-          <t>Perfboard</t>
-        </is>
-      </c>
-      <c r="D68" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E68" s="5" t="inlineStr">
-        <is>
-          <t>10 x 15 cm</t>
-        </is>
-      </c>
-      <c r="F68" s="5" t="inlineStr">
-        <is>
-          <t>fibra de vidrio</t>
-        </is>
-      </c>
-      <c r="G68" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="H68" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="I68" s="5">
-        <f>G68*H68</f>
-        <v/>
-      </c>
-      <c r="J68" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="K68" s="5">
-        <f>I68+J68</f>
-        <v/>
-      </c>
-      <c r="L68" s="5" t="inlineStr">
-        <is>
-          <t>placa perforada 10x15</t>
-        </is>
-      </c>
-      <c r="M68" s="6" t="n"/>
-      <c r="N68" s="7" t="n"/>
-      <c r="O68" s="8">
-        <f>IF(N68="","",K68*N68)</f>
-        <v/>
-      </c>
-      <c r="P68" s="6" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="Q68" s="5" t="inlineStr"/>
+      <c r="D68" s="4" t="n"/>
+      <c r="E68" s="4" t="n"/>
+      <c r="F68" s="4" t="n"/>
+      <c r="G68" s="4" t="n"/>
+      <c r="H68" s="4" t="n"/>
+      <c r="I68" s="4" t="n"/>
+      <c r="J68" s="4" t="n"/>
+      <c r="K68" s="4" t="n"/>
+      <c r="L68" s="4" t="n"/>
+      <c r="M68" s="4" t="n"/>
+      <c r="N68" s="4" t="n"/>
+      <c r="O68" s="4" t="n"/>
+      <c r="P68" s="4" t="n"/>
+      <c r="Q68" s="4" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="5" t="inlineStr">
@@ -4300,7 +4304,7 @@
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>Zocalo DIP-8 (INA)</t>
+          <t>Perfboard</t>
         </is>
       </c>
       <c r="D69" s="5" t="inlineStr">
@@ -4310,16 +4314,16 @@
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t>DIP-8</t>
+          <t>10 x 15 cm</t>
         </is>
       </c>
       <c r="F69" s="5" t="inlineStr">
         <is>
-          <t>zocalo</t>
+          <t>fibra de vidrio</t>
         </is>
       </c>
       <c r="G69" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H69" s="5" t="n">
         <v>1</v>
@@ -4329,7 +4333,7 @@
         <v/>
       </c>
       <c r="J69" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K69" s="5">
         <f>I69+J69</f>
@@ -4337,7 +4341,7 @@
       </c>
       <c r="L69" s="5" t="inlineStr">
         <is>
-          <t>zocalo DIP 8 pines</t>
+          <t>placa perforada 10x15</t>
         </is>
       </c>
       <c r="M69" s="6" t="n"/>
@@ -4351,11 +4355,7 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="Q69" s="5" t="inlineStr">
-        <is>
-          <t>Solo si usas el respaldo AD623AN DIP-8</t>
-        </is>
-      </c>
+      <c r="Q69" s="5" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="5" t="inlineStr">
@@ -4370,7 +4370,7 @@
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>Adaptador SOIC/MSOP-8 a DIP-8</t>
+          <t>Zocalo DIP-8 (INA)</t>
         </is>
       </c>
       <c r="D70" s="5" t="inlineStr">
@@ -4380,12 +4380,12 @@
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>DIP-8</t>
         </is>
       </c>
       <c r="F70" s="5" t="inlineStr">
         <is>
-          <t>PCB adaptador</t>
+          <t>zocalo</t>
         </is>
       </c>
       <c r="G70" s="5" t="n">
@@ -4407,7 +4407,7 @@
       </c>
       <c r="L70" s="5" t="inlineStr">
         <is>
-          <t>adaptador SOIC8 a DIP8</t>
+          <t>zocalo DIP 8 pines</t>
         </is>
       </c>
       <c r="M70" s="6" t="n"/>
@@ -4423,7 +4423,7 @@
       </c>
       <c r="Q70" s="5" t="inlineStr">
         <is>
-          <t>Solo si compras el INA333 suelto (SMD)</t>
+          <t>Solo si usas el respaldo AD623AN DIP-8</t>
         </is>
       </c>
     </row>
@@ -4440,7 +4440,7 @@
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>Tira de headers macho/hembra</t>
+          <t>Adaptador SOIC/MSOP-8 a DIP-8</t>
         </is>
       </c>
       <c r="D71" s="5" t="inlineStr">
@@ -4450,16 +4450,16 @@
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t>2.54 mm</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F71" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>PCB adaptador</t>
         </is>
       </c>
       <c r="G71" s="5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H71" s="5" t="n">
         <v>1</v>
@@ -4469,7 +4469,7 @@
         <v/>
       </c>
       <c r="J71" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K71" s="5">
         <f>I71+J71</f>
@@ -4477,7 +4477,7 @@
       </c>
       <c r="L71" s="5" t="inlineStr">
         <is>
-          <t>header 2.54mm 40 pines</t>
+          <t>adaptador SOIC8 a DIP8</t>
         </is>
       </c>
       <c r="M71" s="6" t="n"/>
@@ -4491,7 +4491,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="Q71" s="5" t="inlineStr"/>
+      <c r="Q71" s="5" t="inlineStr">
+        <is>
+          <t>Solo si compras el INA333 suelto (SMD)</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="5" t="inlineStr">
@@ -4506,7 +4510,7 @@
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>Cable para puentes</t>
+          <t>Tira de headers macho/hembra</t>
         </is>
       </c>
       <c r="D72" s="5" t="inlineStr">
@@ -4516,7 +4520,7 @@
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t>24 AWG rigido</t>
+          <t>2.54 mm</t>
         </is>
       </c>
       <c r="F72" s="5" t="inlineStr">
@@ -4525,7 +4529,7 @@
         </is>
       </c>
       <c r="G72" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H72" s="5" t="n">
         <v>1</v>
@@ -4535,7 +4539,7 @@
         <v/>
       </c>
       <c r="J72" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K72" s="5">
         <f>I72+J72</f>
@@ -4543,7 +4547,7 @@
       </c>
       <c r="L72" s="5" t="inlineStr">
         <is>
-          <t>cable rigido 24 AWG</t>
+          <t>header 2.54mm 40 pines</t>
         </is>
       </c>
       <c r="M72" s="6" t="n"/>
@@ -4559,21 +4563,87 @@
       </c>
       <c r="Q72" s="5" t="inlineStr"/>
     </row>
-    <row r="74">
-      <c r="N74" s="9" t="inlineStr">
+    <row r="73">
+      <c r="A73" s="5" t="inlineStr">
+        <is>
+          <t>14 MECANICA E INTERCONEXION</t>
+        </is>
+      </c>
+      <c r="B73" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C73" s="5" t="inlineStr">
+        <is>
+          <t>Cable para puentes</t>
+        </is>
+      </c>
+      <c r="D73" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E73" s="5" t="inlineStr">
+        <is>
+          <t>24 AWG rigido</t>
+        </is>
+      </c>
+      <c r="F73" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G73" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H73" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I73" s="5">
+        <f>G73*H73</f>
+        <v/>
+      </c>
+      <c r="J73" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K73" s="5">
+        <f>I73+J73</f>
+        <v/>
+      </c>
+      <c r="L73" s="5" t="inlineStr">
+        <is>
+          <t>cable rigido 24 AWG</t>
+        </is>
+      </c>
+      <c r="M73" s="6" t="n"/>
+      <c r="N73" s="7" t="n"/>
+      <c r="O73" s="8">
+        <f>IF(N73="","",K73*N73)</f>
+        <v/>
+      </c>
+      <c r="P73" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="Q73" s="5" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="N75" s="9" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="O74" s="10">
-        <f>SUM(O5:O72)</f>
+      <c r="O75" s="10">
+        <f>SUM(O5:O73)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:Q72"/>
+  <autoFilter ref="A4:Q73"/>
   <dataValidations count="1">
-    <dataValidation sqref="P6 P7 P9 P10 P11 P13 P14 P15 P17 P18 P19 P22 P23 P24 P27 P28 P29 P32 P33 P34 P37 P38 P39 P42 P43 P46 P47 P48 P49 P52 P53 P54 P55 P57 P58 P59 P60 P61 P62 P64 P65 P66 P68 P69 P70 P71 P72" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="P6 P7 P9 P10 P11 P13 P14 P15 P17 P18 P19 P22 P23 P24 P25 P28 P29 P30 P33 P34 P35 P38 P39 P40 P43 P44 P47 P48 P49 P50 P53 P54 P55 P56 P58 P59 P60 P61 P62 P63 P65 P66 P67 P69 P70 P71 P72 P73" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pendiente,Comprado,No hay,No aplica"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4632,15 +4702,15 @@
         </is>
       </c>
       <c r="B4" s="11">
-        <f>COUNTIFS('BoM por modulo'!$A$5:$A$72,A4,'BoM por modulo'!$P$5:$P$72,"&lt;&gt;")</f>
+        <f>COUNTIFS('BoM por modulo'!$A$5:$A$73,A4,'BoM por modulo'!$P$5:$P$73,"&lt;&gt;")</f>
         <v/>
       </c>
       <c r="C4" s="11">
-        <f>COUNTIFS('BoM por modulo'!$A$5:$A$72,A4,'BoM por modulo'!$P$5:$P$72,"Pendiente")</f>
+        <f>COUNTIFS('BoM por modulo'!$A$5:$A$73,A4,'BoM por modulo'!$P$5:$P$73,"Pendiente")</f>
         <v/>
       </c>
       <c r="D4" s="12">
-        <f>SUMIF('BoM por modulo'!$A$5:$A$72,A4,'BoM por modulo'!$O$5:$O$72)</f>
+        <f>SUMIF('BoM por modulo'!$A$5:$A$73,A4,'BoM por modulo'!$O$5:$O$73)</f>
         <v/>
       </c>
     </row>
@@ -4651,15 +4721,15 @@
         </is>
       </c>
       <c r="B5" s="11">
-        <f>COUNTIFS('BoM por modulo'!$A$5:$A$72,A5,'BoM por modulo'!$P$5:$P$72,"&lt;&gt;")</f>
+        <f>COUNTIFS('BoM por modulo'!$A$5:$A$73,A5,'BoM por modulo'!$P$5:$P$73,"&lt;&gt;")</f>
         <v/>
       </c>
       <c r="C5" s="11">
-        <f>COUNTIFS('BoM por modulo'!$A$5:$A$72,A5,'BoM por modulo'!$P$5:$P$72,"Pendiente")</f>
+        <f>COUNTIFS('BoM por modulo'!$A$5:$A$73,A5,'BoM por modulo'!$P$5:$P$73,"Pendiente")</f>
         <v/>
       </c>
       <c r="D5" s="12">
-        <f>SUMIF('BoM por modulo'!$A$5:$A$72,A5,'BoM por modulo'!$O$5:$O$72)</f>
+        <f>SUMIF('BoM por modulo'!$A$5:$A$73,A5,'BoM por modulo'!$O$5:$O$73)</f>
         <v/>
       </c>
     </row>
@@ -4670,15 +4740,15 @@
         </is>
       </c>
       <c r="B6" s="11">
-        <f>COUNTIFS('BoM por modulo'!$A$5:$A$72,A6,'BoM por modulo'!$P$5:$P$72,"&lt;&gt;")</f>
+        <f>COUNTIFS('BoM por modulo'!$A$5:$A$73,A6,'BoM por modulo'!$P$5:$P$73,"&lt;&gt;")</f>
         <v/>
       </c>
       <c r="C6" s="11">
-        <f>COUNTIFS('BoM por modulo'!$A$5:$A$72,A6,'BoM por modulo'!$P$5:$P$72,"Pendiente")</f>
+        <f>COUNTIFS('BoM por modulo'!$A$5:$A$73,A6,'BoM por modulo'!$P$5:$P$73,"Pendiente")</f>
         <v/>
       </c>
       <c r="D6" s="12">
-        <f>SUMIF('BoM por modulo'!$A$5:$A$72,A6,'BoM por modulo'!$O$5:$O$72)</f>
+        <f>SUMIF('BoM por modulo'!$A$5:$A$73,A6,'BoM por modulo'!$O$5:$O$73)</f>
         <v/>
       </c>
     </row>
@@ -4689,15 +4759,15 @@
         </is>
       </c>
       <c r="B7" s="11">
-        <f>COUNTIFS('BoM por modulo'!$A$5:$A$72,A7,'BoM por modulo'!$P$5:$P$72,"&lt;&gt;")</f>
+        <f>COUNTIFS('BoM por modulo'!$A$5:$A$73,A7,'BoM por modulo'!$P$5:$P$73,"&lt;&gt;")</f>
         <v/>
       </c>
       <c r="C7" s="11">
-        <f>COUNTIFS('BoM por modulo'!$A$5:$A$72,A7,'BoM por modulo'!$P$5:$P$72,"Pendiente")</f>
+        <f>COUNTIFS('BoM por modulo'!$A$5:$A$73,A7,'BoM por modulo'!$P$5:$P$73,"Pendiente")</f>
         <v/>
       </c>
       <c r="D7" s="12">
-        <f>SUMIF('BoM por modulo'!$A$5:$A$72,A7,'BoM por modulo'!$O$5:$O$72)</f>
+        <f>SUMIF('BoM por modulo'!$A$5:$A$73,A7,'BoM por modulo'!$O$5:$O$73)</f>
         <v/>
       </c>
     </row>
@@ -4708,15 +4778,15 @@
         </is>
       </c>
       <c r="B8" s="11">
-        <f>COUNTIFS('BoM por modulo'!$A$5:$A$72,A8,'BoM por modulo'!$P$5:$P$72,"&lt;&gt;")</f>
+        <f>COUNTIFS('BoM por modulo'!$A$5:$A$73,A8,'BoM por modulo'!$P$5:$P$73,"&lt;&gt;")</f>
         <v/>
       </c>
       <c r="C8" s="11">
-        <f>COUNTIFS('BoM por modulo'!$A$5:$A$72,A8,'BoM por modulo'!$P$5:$P$72,"Pendiente")</f>
+        <f>COUNTIFS('BoM por modulo'!$A$5:$A$73,A8,'BoM por modulo'!$P$5:$P$73,"Pendiente")</f>
         <v/>
       </c>
       <c r="D8" s="12">
-        <f>SUMIF('BoM por modulo'!$A$5:$A$72,A8,'BoM por modulo'!$O$5:$O$72)</f>
+        <f>SUMIF('BoM por modulo'!$A$5:$A$73,A8,'BoM por modulo'!$O$5:$O$73)</f>
         <v/>
       </c>
     </row>
@@ -4727,15 +4797,15 @@
         </is>
       </c>
       <c r="B9" s="11">
-        <f>COUNTIFS('BoM por modulo'!$A$5:$A$72,A9,'BoM por modulo'!$P$5:$P$72,"&lt;&gt;")</f>
+        <f>COUNTIFS('BoM por modulo'!$A$5:$A$73,A9,'BoM por modulo'!$P$5:$P$73,"&lt;&gt;")</f>
         <v/>
       </c>
       <c r="C9" s="11">
-        <f>COUNTIFS('BoM por modulo'!$A$5:$A$72,A9,'BoM por modulo'!$P$5:$P$72,"Pendiente")</f>
+        <f>COUNTIFS('BoM por modulo'!$A$5:$A$73,A9,'BoM por modulo'!$P$5:$P$73,"Pendiente")</f>
         <v/>
       </c>
       <c r="D9" s="12">
-        <f>SUMIF('BoM por modulo'!$A$5:$A$72,A9,'BoM por modulo'!$O$5:$O$72)</f>
+        <f>SUMIF('BoM por modulo'!$A$5:$A$73,A9,'BoM por modulo'!$O$5:$O$73)</f>
         <v/>
       </c>
     </row>
@@ -4746,15 +4816,15 @@
         </is>
       </c>
       <c r="B10" s="11">
-        <f>COUNTIFS('BoM por modulo'!$A$5:$A$72,A10,'BoM por modulo'!$P$5:$P$72,"&lt;&gt;")</f>
+        <f>COUNTIFS('BoM por modulo'!$A$5:$A$73,A10,'BoM por modulo'!$P$5:$P$73,"&lt;&gt;")</f>
         <v/>
       </c>
       <c r="C10" s="11">
-        <f>COUNTIFS('BoM por modulo'!$A$5:$A$72,A10,'BoM por modulo'!$P$5:$P$72,"Pendiente")</f>
+        <f>COUNTIFS('BoM por modulo'!$A$5:$A$73,A10,'BoM por modulo'!$P$5:$P$73,"Pendiente")</f>
         <v/>
       </c>
       <c r="D10" s="12">
-        <f>SUMIF('BoM por modulo'!$A$5:$A$72,A10,'BoM por modulo'!$O$5:$O$72)</f>
+        <f>SUMIF('BoM por modulo'!$A$5:$A$73,A10,'BoM por modulo'!$O$5:$O$73)</f>
         <v/>
       </c>
     </row>
@@ -4765,15 +4835,15 @@
         </is>
       </c>
       <c r="B11" s="11">
-        <f>COUNTIFS('BoM por modulo'!$A$5:$A$72,A11,'BoM por modulo'!$P$5:$P$72,"&lt;&gt;")</f>
+        <f>COUNTIFS('BoM por modulo'!$A$5:$A$73,A11,'BoM por modulo'!$P$5:$P$73,"&lt;&gt;")</f>
         <v/>
       </c>
       <c r="C11" s="11">
-        <f>COUNTIFS('BoM por modulo'!$A$5:$A$72,A11,'BoM por modulo'!$P$5:$P$72,"Pendiente")</f>
+        <f>COUNTIFS('BoM por modulo'!$A$5:$A$73,A11,'BoM por modulo'!$P$5:$P$73,"Pendiente")</f>
         <v/>
       </c>
       <c r="D11" s="12">
-        <f>SUMIF('BoM por modulo'!$A$5:$A$72,A11,'BoM por modulo'!$O$5:$O$72)</f>
+        <f>SUMIF('BoM por modulo'!$A$5:$A$73,A11,'BoM por modulo'!$O$5:$O$73)</f>
         <v/>
       </c>
     </row>
@@ -4784,15 +4854,15 @@
         </is>
       </c>
       <c r="B12" s="11">
-        <f>COUNTIFS('BoM por modulo'!$A$5:$A$72,A12,'BoM por modulo'!$P$5:$P$72,"&lt;&gt;")</f>
+        <f>COUNTIFS('BoM por modulo'!$A$5:$A$73,A12,'BoM por modulo'!$P$5:$P$73,"&lt;&gt;")</f>
         <v/>
       </c>
       <c r="C12" s="11">
-        <f>COUNTIFS('BoM por modulo'!$A$5:$A$72,A12,'BoM por modulo'!$P$5:$P$72,"Pendiente")</f>
+        <f>COUNTIFS('BoM por modulo'!$A$5:$A$73,A12,'BoM por modulo'!$P$5:$P$73,"Pendiente")</f>
         <v/>
       </c>
       <c r="D12" s="12">
-        <f>SUMIF('BoM por modulo'!$A$5:$A$72,A12,'BoM por modulo'!$O$5:$O$72)</f>
+        <f>SUMIF('BoM por modulo'!$A$5:$A$73,A12,'BoM por modulo'!$O$5:$O$73)</f>
         <v/>
       </c>
     </row>
@@ -4803,15 +4873,15 @@
         </is>
       </c>
       <c r="B13" s="11">
-        <f>COUNTIFS('BoM por modulo'!$A$5:$A$72,A13,'BoM por modulo'!$P$5:$P$72,"&lt;&gt;")</f>
+        <f>COUNTIFS('BoM por modulo'!$A$5:$A$73,A13,'BoM por modulo'!$P$5:$P$73,"&lt;&gt;")</f>
         <v/>
       </c>
       <c r="C13" s="11">
-        <f>COUNTIFS('BoM por modulo'!$A$5:$A$72,A13,'BoM por modulo'!$P$5:$P$72,"Pendiente")</f>
+        <f>COUNTIFS('BoM por modulo'!$A$5:$A$73,A13,'BoM por modulo'!$P$5:$P$73,"Pendiente")</f>
         <v/>
       </c>
       <c r="D13" s="12">
-        <f>SUMIF('BoM por modulo'!$A$5:$A$72,A13,'BoM por modulo'!$O$5:$O$72)</f>
+        <f>SUMIF('BoM por modulo'!$A$5:$A$73,A13,'BoM por modulo'!$O$5:$O$73)</f>
         <v/>
       </c>
     </row>
@@ -4822,15 +4892,15 @@
         </is>
       </c>
       <c r="B14" s="11">
-        <f>COUNTIFS('BoM por modulo'!$A$5:$A$72,A14,'BoM por modulo'!$P$5:$P$72,"&lt;&gt;")</f>
+        <f>COUNTIFS('BoM por modulo'!$A$5:$A$73,A14,'BoM por modulo'!$P$5:$P$73,"&lt;&gt;")</f>
         <v/>
       </c>
       <c r="C14" s="11">
-        <f>COUNTIFS('BoM por modulo'!$A$5:$A$72,A14,'BoM por modulo'!$P$5:$P$72,"Pendiente")</f>
+        <f>COUNTIFS('BoM por modulo'!$A$5:$A$73,A14,'BoM por modulo'!$P$5:$P$73,"Pendiente")</f>
         <v/>
       </c>
       <c r="D14" s="12">
-        <f>SUMIF('BoM por modulo'!$A$5:$A$72,A14,'BoM por modulo'!$O$5:$O$72)</f>
+        <f>SUMIF('BoM por modulo'!$A$5:$A$73,A14,'BoM por modulo'!$O$5:$O$73)</f>
         <v/>
       </c>
     </row>
@@ -4841,15 +4911,15 @@
         </is>
       </c>
       <c r="B15" s="11">
-        <f>COUNTIFS('BoM por modulo'!$A$5:$A$72,A15,'BoM por modulo'!$P$5:$P$72,"&lt;&gt;")</f>
+        <f>COUNTIFS('BoM por modulo'!$A$5:$A$73,A15,'BoM por modulo'!$P$5:$P$73,"&lt;&gt;")</f>
         <v/>
       </c>
       <c r="C15" s="11">
-        <f>COUNTIFS('BoM por modulo'!$A$5:$A$72,A15,'BoM por modulo'!$P$5:$P$72,"Pendiente")</f>
+        <f>COUNTIFS('BoM por modulo'!$A$5:$A$73,A15,'BoM por modulo'!$P$5:$P$73,"Pendiente")</f>
         <v/>
       </c>
       <c r="D15" s="12">
-        <f>SUMIF('BoM por modulo'!$A$5:$A$72,A15,'BoM por modulo'!$O$5:$O$72)</f>
+        <f>SUMIF('BoM por modulo'!$A$5:$A$73,A15,'BoM por modulo'!$O$5:$O$73)</f>
         <v/>
       </c>
     </row>
@@ -4860,15 +4930,15 @@
         </is>
       </c>
       <c r="B16" s="11">
-        <f>COUNTIFS('BoM por modulo'!$A$5:$A$72,A16,'BoM por modulo'!$P$5:$P$72,"&lt;&gt;")</f>
+        <f>COUNTIFS('BoM por modulo'!$A$5:$A$73,A16,'BoM por modulo'!$P$5:$P$73,"&lt;&gt;")</f>
         <v/>
       </c>
       <c r="C16" s="11">
-        <f>COUNTIFS('BoM por modulo'!$A$5:$A$72,A16,'BoM por modulo'!$P$5:$P$72,"Pendiente")</f>
+        <f>COUNTIFS('BoM por modulo'!$A$5:$A$73,A16,'BoM por modulo'!$P$5:$P$73,"Pendiente")</f>
         <v/>
       </c>
       <c r="D16" s="12">
-        <f>SUMIF('BoM por modulo'!$A$5:$A$72,A16,'BoM por modulo'!$O$5:$O$72)</f>
+        <f>SUMIF('BoM por modulo'!$A$5:$A$73,A16,'BoM por modulo'!$O$5:$O$73)</f>
         <v/>
       </c>
     </row>
@@ -4879,15 +4949,15 @@
         </is>
       </c>
       <c r="B17" s="11">
-        <f>COUNTIFS('BoM por modulo'!$A$5:$A$72,A17,'BoM por modulo'!$P$5:$P$72,"&lt;&gt;")</f>
+        <f>COUNTIFS('BoM por modulo'!$A$5:$A$73,A17,'BoM por modulo'!$P$5:$P$73,"&lt;&gt;")</f>
         <v/>
       </c>
       <c r="C17" s="11">
-        <f>COUNTIFS('BoM por modulo'!$A$5:$A$72,A17,'BoM por modulo'!$P$5:$P$72,"Pendiente")</f>
+        <f>COUNTIFS('BoM por modulo'!$A$5:$A$73,A17,'BoM por modulo'!$P$5:$P$73,"Pendiente")</f>
         <v/>
       </c>
       <c r="D17" s="12">
-        <f>SUMIF('BoM por modulo'!$A$5:$A$72,A17,'BoM por modulo'!$O$5:$O$72)</f>
+        <f>SUMIF('BoM por modulo'!$A$5:$A$73,A17,'BoM por modulo'!$O$5:$O$73)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
AFE: 3 canales (submentoniano, labio, laringe) con TS922 y LPF MFB+SK
- Canal de 7 etapas: HPF SK + LPF MFB x25 + LPF SK (4o orden), sin G2 ni buffer.
- 11 secciones de op-amp = 6 TS922 (stock en Chile). Modelo TS922 conductual.
- Hoja AuraVox_AFE.asc de 3 canales; BoM xlsx actualizada.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V5Cz1Wb6HSRhqzouEW9mso
</commit_message>
<xml_diff>
--- a/docs/afe-emg/BoM_AFE_AuraVox.xlsx
+++ b/docs/afe-emg/BoM_AFE_AuraVox.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tiendas" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'BoM por modulo'!$A$4:$Q$73</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'BoM por modulo'!$A$4:$Q$68</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -509,7 +509,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q75"/>
+  <dimension ref="A1:Q70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -534,7 +534,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>BoM AFE sEMG AuraVox: 4 canales, 9 electrodos, RLD. Ordenada por modulo, igual que los recuadros del esquematico LTspice (sim/ltspice).</t>
+          <t>BoM AFE sEMG AuraVox: 3 canales (submentoniano, labio inferior, laringe), 7 electrodos, RLD. Ordenada por modulo, igual que los recuadros del esquematico LTspice (sim/ltspice).</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
       <c r="B5" s="4" t="n"/>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>por canal (x4)</t>
+          <t>por canal (x3)</t>
         </is>
       </c>
       <c r="D5" s="4" t="n"/>
@@ -694,7 +694,7 @@
         <v>2</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I6" s="5">
         <f>G6*H6</f>
@@ -764,7 +764,7 @@
         <v>4</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I7" s="5">
         <f>G7*H7</f>
@@ -808,7 +808,7 @@
       <c r="B8" s="4" t="n"/>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>por canal (x4)</t>
+          <t>por canal (x3)</t>
         </is>
       </c>
       <c r="D8" s="4" t="n"/>
@@ -861,7 +861,7 @@
         <v>2</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I9" s="5">
         <f>G9*H9</f>
@@ -927,7 +927,7 @@
         <v>2</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I10" s="5">
         <f>G10*H10</f>
@@ -997,7 +997,7 @@
         <v>1</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I11" s="5">
         <f>G11*H11</f>
@@ -1037,7 +1037,7 @@
       <c r="B12" s="4" t="n"/>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>por canal (x4)</t>
+          <t>por canal (x3)</t>
         </is>
       </c>
       <c r="D12" s="4" t="n"/>
@@ -1090,7 +1090,7 @@
         <v>1</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I13" s="5">
         <f>G13*H13</f>
@@ -1166,7 +1166,7 @@
         <v>2</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I14" s="5">
         <f>G14*H14</f>
@@ -1236,7 +1236,7 @@
         <v>1</v>
       </c>
       <c r="H15" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I15" s="5">
         <f>G15*H15</f>
@@ -1280,7 +1280,7 @@
       <c r="B16" s="4" t="n"/>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>por canal (x4)</t>
+          <t>por canal (x3)</t>
         </is>
       </c>
       <c r="D16" s="4" t="n"/>
@@ -1333,7 +1333,7 @@
         <v>2</v>
       </c>
       <c r="H17" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I17" s="5">
         <f>G17*H17</f>
@@ -1403,7 +1403,7 @@
         <v>1</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I18" s="5">
         <f>G18*H18</f>
@@ -1473,7 +1473,7 @@
         <v>1</v>
       </c>
       <c r="H19" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I19" s="5">
         <f>G19*H19</f>
@@ -1554,13 +1554,13 @@
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>5 G2 = 25</t>
+          <t>5 LPF MFB 500 Hz x25 (Q 0.54)</t>
         </is>
       </c>
       <c r="B21" s="4" t="n"/>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>por canal (x4)</t>
+          <t>por canal (x3)</t>
         </is>
       </c>
       <c r="D21" s="4" t="n"/>
@@ -1581,27 +1581,27 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>5 G2 = 25</t>
+          <t>5 LPF MFB 500 Hz x25 (Q 0.54)</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Rf</t>
+          <t>Rm1</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Resistencia de realimentacion</t>
+          <t>Resistencia de entrada (fija la ganancia)</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>240k</t>
+          <t>3k</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>240k</t>
+          <t>3k</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
@@ -1613,7 +1613,7 @@
         <v>1</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I22" s="5">
         <f>G22*H22</f>
@@ -1628,7 +1628,7 @@
       </c>
       <c r="L22" s="5" t="inlineStr">
         <is>
-          <t>resistencia 240k 1%</t>
+          <t>resistencia 3k 1%</t>
         </is>
       </c>
       <c r="M22" s="6" t="n"/>
@@ -1642,32 +1642,36 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="Q22" s="5" t="inlineStr"/>
+      <c r="Q22" s="5" t="inlineStr">
+        <is>
+          <t>Ganancia = Rm2/Rm1 = 25. No poner trimmer aqui: cambia el Q del filtro</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>5 G2 = 25</t>
+          <t>5 LPF MFB 500 Hz x25 (Q 0.54)</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>Rg</t>
+          <t>Rm2</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>Resistencia de ganancia fija</t>
+          <t>Resistencia de realimentacion</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>4.7k</t>
+          <t>75k</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>4.7k</t>
+          <t>75k</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
@@ -1679,7 +1683,7 @@
         <v>1</v>
       </c>
       <c r="H23" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I23" s="5">
         <f>G23*H23</f>
@@ -1694,7 +1698,7 @@
       </c>
       <c r="L23" s="5" t="inlineStr">
         <is>
-          <t>resistencia 4.7k 1%</t>
+          <t>resistencia 75k 1%</t>
         </is>
       </c>
       <c r="M23" s="6" t="n"/>
@@ -1713,39 +1717,39 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>5 G2 = 25</t>
+          <t>5 LPF MFB 500 Hz x25 (Q 0.54)</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>RGT</t>
+          <t>Rm3</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>Trimmer de ganancia por sitio de medicion</t>
+          <t>Resistencia a la entrada inversora</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>25k</t>
+          <t>20k</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>25k multivuelta</t>
+          <t>20k</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>trimmer multivuelta (3296)</t>
+          <t>pelicula metalica 1 %</t>
         </is>
       </c>
       <c r="G24" s="5" t="n">
         <v>1</v>
       </c>
       <c r="H24" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I24" s="5">
         <f>G24*H24</f>
@@ -1760,7 +1764,7 @@
       </c>
       <c r="L24" s="5" t="inlineStr">
         <is>
-          <t>trimmer 25k multivuelta 3296</t>
+          <t>resistencia 20k 1%</t>
         </is>
       </c>
       <c r="M24" s="6" t="n"/>
@@ -1774,48 +1778,44 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="Q24" s="5" t="inlineStr">
-        <is>
-          <t>G2 = 1 + 240k/(4.7k + RGT): de ~9 (25k) a ~52 (0). Ganancia total ~180-1000. Para G2 = 25: RGT = 5.3k</t>
-        </is>
-      </c>
+      <c r="Q24" s="5" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>5 G2 = 25</t>
+          <t>5 LPF MFB 500 Hz x25 (Q 0.54)</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>Cg</t>
+          <t>Cm1</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Condensador de bloqueo DC (G = 1 en DC)</t>
+          <t>Condensador a GND</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>10u</t>
+          <t>68n</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>10u</t>
+          <t>68n</t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>ceramico X7R o electrolitico 16 V</t>
+          <t>poliester 5 %</t>
         </is>
       </c>
       <c r="G25" s="5" t="n">
         <v>1</v>
       </c>
       <c r="H25" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I25" s="5">
         <f>G25*H25</f>
@@ -1830,7 +1830,7 @@
       </c>
       <c r="L25" s="5" t="inlineStr">
         <is>
-          <t>condensador 10uF</t>
+          <t>condensador poliester 68nF</t>
         </is>
       </c>
       <c r="M25" s="6" t="n"/>
@@ -1849,190 +1849,186 @@
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>5 G2 = 25</t>
+          <t>5 LPF MFB 500 Hz x25 (Q 0.54)</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>XG2</t>
+          <t>Cm2</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
+          <t>Condensador de realimentacion</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>1n</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>1n</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>ceramico C0G/NP0</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H26" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="I26" s="5">
+        <f>G26*H26</f>
+        <v/>
+      </c>
+      <c r="J26" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="K26" s="5">
+        <f>I26+J26</f>
+        <v/>
+      </c>
+      <c r="L26" s="5" t="inlineStr">
+        <is>
+          <t>condensador ceramico 1nF NP0</t>
+        </is>
+      </c>
+      <c r="M26" s="6" t="n"/>
+      <c r="N26" s="7" t="n"/>
+      <c r="O26" s="8">
+        <f>IF(N26="","",K26*N26)</f>
+        <v/>
+      </c>
+      <c r="P26" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="Q26" s="5" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>5 LPF MFB 500 Hz x25 (Q 0.54)</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>XMF</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
           <t>seccion de op-amp</t>
         </is>
       </c>
-      <c r="D26" s="5" t="inlineStr">
+      <c r="D27" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E26" s="5" t="inlineStr">
+      <c r="E27" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F26" s="5" t="inlineStr">
+      <c r="F27" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G26" s="5" t="n"/>
-      <c r="H26" s="5" t="n"/>
-      <c r="I26" s="5" t="n"/>
-      <c r="J26" s="5" t="n"/>
-      <c r="K26" s="5" t="n"/>
-      <c r="L26" s="5" t="inlineStr"/>
-      <c r="M26" s="5" t="n"/>
-      <c r="N26" s="8" t="n"/>
-      <c r="O26" s="8" t="n"/>
-      <c r="P26" s="5" t="n"/>
-      <c r="Q26" s="5" t="inlineStr">
+      <c r="G27" s="5" t="n"/>
+      <c r="H27" s="5" t="n"/>
+      <c r="I27" s="5" t="n"/>
+      <c r="J27" s="5" t="n"/>
+      <c r="K27" s="5" t="n"/>
+      <c r="L27" s="5" t="inlineStr"/>
+      <c r="M27" s="5" t="n"/>
+      <c r="N27" s="8" t="n"/>
+      <c r="O27" s="8" t="n"/>
+      <c r="P27" s="5" t="n"/>
+      <c r="Q27" s="5" t="inlineStr">
         <is>
           <t>Contada en el modulo 11 OP-AMPS</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="4" t="inlineStr">
-        <is>
-          <t>6 LPF A 500 Hz (Q 0.541)</t>
-        </is>
-      </c>
-      <c r="B27" s="4" t="n"/>
-      <c r="C27" s="4" t="inlineStr">
-        <is>
-          <t>por canal (x4)</t>
-        </is>
-      </c>
-      <c r="D27" s="4" t="n"/>
-      <c r="E27" s="4" t="n"/>
-      <c r="F27" s="4" t="n"/>
-      <c r="G27" s="4" t="n"/>
-      <c r="H27" s="4" t="n"/>
-      <c r="I27" s="4" t="n"/>
-      <c r="J27" s="4" t="n"/>
-      <c r="K27" s="4" t="n"/>
-      <c r="L27" s="4" t="n"/>
-      <c r="M27" s="4" t="n"/>
-      <c r="N27" s="4" t="n"/>
-      <c r="O27" s="4" t="n"/>
-      <c r="P27" s="4" t="n"/>
-      <c r="Q27" s="4" t="n"/>
-    </row>
     <row r="28">
-      <c r="A28" s="5" t="inlineStr">
-        <is>
-          <t>6 LPF A 500 Hz (Q 0.541)</t>
-        </is>
-      </c>
-      <c r="B28" s="5" t="inlineStr">
-        <is>
-          <t>Rla1, Rla2</t>
-        </is>
-      </c>
-      <c r="C28" s="5" t="inlineStr">
-        <is>
-          <t>Resistencia del LPF A</t>
-        </is>
-      </c>
-      <c r="D28" s="5" t="inlineStr">
-        <is>
-          <t>88.7k</t>
-        </is>
-      </c>
-      <c r="E28" s="5" t="inlineStr">
-        <is>
-          <t>91k</t>
-        </is>
-      </c>
-      <c r="F28" s="5" t="inlineStr">
-        <is>
-          <t>pelicula metalica 1 %</t>
-        </is>
-      </c>
-      <c r="G28" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="H28" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="I28" s="5">
-        <f>G28*H28</f>
-        <v/>
-      </c>
-      <c r="J28" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="K28" s="5">
-        <f>I28+J28</f>
-        <v/>
-      </c>
-      <c r="L28" s="5" t="inlineStr">
-        <is>
-          <t>resistencia 91k 1%</t>
-        </is>
-      </c>
-      <c r="M28" s="6" t="n"/>
-      <c r="N28" s="7" t="n"/>
-      <c r="O28" s="8">
-        <f>IF(N28="","",K28*N28)</f>
-        <v/>
-      </c>
-      <c r="P28" s="6" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="Q28" s="5" t="inlineStr">
-        <is>
-          <t>Con 91k: f0 = 487 Hz</t>
-        </is>
-      </c>
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>6 LPF Sallen-Key 500 Hz (Q 1.31)</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="n"/>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>por canal (x3)</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="n"/>
+      <c r="E28" s="4" t="n"/>
+      <c r="F28" s="4" t="n"/>
+      <c r="G28" s="4" t="n"/>
+      <c r="H28" s="4" t="n"/>
+      <c r="I28" s="4" t="n"/>
+      <c r="J28" s="4" t="n"/>
+      <c r="K28" s="4" t="n"/>
+      <c r="L28" s="4" t="n"/>
+      <c r="M28" s="4" t="n"/>
+      <c r="N28" s="4" t="n"/>
+      <c r="O28" s="4" t="n"/>
+      <c r="P28" s="4" t="n"/>
+      <c r="Q28" s="4" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>6 LPF A 500 Hz (Q 0.541)</t>
+          <t>6 LPF Sallen-Key 500 Hz (Q 1.31)</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>C11</t>
+          <t>Rlb1, Rlb2</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>Condensador de realimentacion</t>
+          <t>Resistencia del LPF B</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>3.9n</t>
+          <t>54.9k</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>3.9n</t>
+          <t>56k</t>
         </is>
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>poliester 5 % o C0G</t>
+          <t>pelicula metalica 1 %</t>
         </is>
       </c>
       <c r="G29" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H29" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I29" s="5">
         <f>G29*H29</f>
         <v/>
       </c>
       <c r="J29" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K29" s="5">
         <f>I29+J29</f>
@@ -2040,7 +2036,7 @@
       </c>
       <c r="L29" s="5" t="inlineStr">
         <is>
-          <t>condensador poliester 3.9nF</t>
+          <t>resistencia 56k 1%</t>
         </is>
       </c>
       <c r="M29" s="6" t="n"/>
@@ -2054,32 +2050,36 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="Q29" s="5" t="inlineStr"/>
+      <c r="Q29" s="5" t="inlineStr">
+        <is>
+          <t>Con 56k: f0 = 495 Hz</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>6 LPF A 500 Hz (Q 0.541)</t>
+          <t>6 LPF Sallen-Key 500 Hz (Q 1.31)</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>C12</t>
+          <t>C21</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>Condensador a GND</t>
+          <t>Condensador de realimentacion</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>3.3n</t>
+          <t>15n</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>3.3n</t>
+          <t>15n</t>
         </is>
       </c>
       <c r="F30" s="5" t="inlineStr">
@@ -2091,7 +2091,7 @@
         <v>1</v>
       </c>
       <c r="H30" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I30" s="5">
         <f>G30*H30</f>
@@ -2106,7 +2106,7 @@
       </c>
       <c r="L30" s="5" t="inlineStr">
         <is>
-          <t>condensador poliester 3.3nF</t>
+          <t>condensador poliester 15nF</t>
         </is>
       </c>
       <c r="M30" s="6" t="n"/>
@@ -2125,183 +2125,179 @@
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>6 LPF A 500 Hz (Q 0.541)</t>
+          <t>6 LPF Sallen-Key 500 Hz (Q 1.31)</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>XLA</t>
+          <t>C22</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
+          <t>Condensador a GND</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>2.2n</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>2.2n</t>
+        </is>
+      </c>
+      <c r="F31" s="5" t="inlineStr">
+        <is>
+          <t>poliester 5 % o C0G</t>
+        </is>
+      </c>
+      <c r="G31" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H31" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="I31" s="5">
+        <f>G31*H31</f>
+        <v/>
+      </c>
+      <c r="J31" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="K31" s="5">
+        <f>I31+J31</f>
+        <v/>
+      </c>
+      <c r="L31" s="5" t="inlineStr">
+        <is>
+          <t>condensador poliester 2.2nF</t>
+        </is>
+      </c>
+      <c r="M31" s="6" t="n"/>
+      <c r="N31" s="7" t="n"/>
+      <c r="O31" s="8">
+        <f>IF(N31="","",K31*N31)</f>
+        <v/>
+      </c>
+      <c r="P31" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="Q31" s="5" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>6 LPF Sallen-Key 500 Hz (Q 1.31)</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>XLB</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
           <t>seccion de op-amp</t>
         </is>
       </c>
-      <c r="D31" s="5" t="inlineStr">
+      <c r="D32" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E31" s="5" t="inlineStr">
+      <c r="E32" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F31" s="5" t="inlineStr">
+      <c r="F32" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G31" s="5" t="n"/>
-      <c r="H31" s="5" t="n"/>
-      <c r="I31" s="5" t="n"/>
-      <c r="J31" s="5" t="n"/>
-      <c r="K31" s="5" t="n"/>
-      <c r="L31" s="5" t="inlineStr"/>
-      <c r="M31" s="5" t="n"/>
-      <c r="N31" s="8" t="n"/>
-      <c r="O31" s="8" t="n"/>
-      <c r="P31" s="5" t="n"/>
-      <c r="Q31" s="5" t="inlineStr">
+      <c r="G32" s="5" t="n"/>
+      <c r="H32" s="5" t="n"/>
+      <c r="I32" s="5" t="n"/>
+      <c r="J32" s="5" t="n"/>
+      <c r="K32" s="5" t="n"/>
+      <c r="L32" s="5" t="inlineStr"/>
+      <c r="M32" s="5" t="n"/>
+      <c r="N32" s="8" t="n"/>
+      <c r="O32" s="8" t="n"/>
+      <c r="P32" s="5" t="n"/>
+      <c r="Q32" s="5" t="inlineStr">
         <is>
           <t>Contada en el modulo 11 OP-AMPS</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="4" t="inlineStr">
-        <is>
-          <t>7 LPF B 500 Hz (Q 1.306)</t>
-        </is>
-      </c>
-      <c r="B32" s="4" t="n"/>
-      <c r="C32" s="4" t="inlineStr">
-        <is>
-          <t>por canal (x4)</t>
-        </is>
-      </c>
-      <c r="D32" s="4" t="n"/>
-      <c r="E32" s="4" t="n"/>
-      <c r="F32" s="4" t="n"/>
-      <c r="G32" s="4" t="n"/>
-      <c r="H32" s="4" t="n"/>
-      <c r="I32" s="4" t="n"/>
-      <c r="J32" s="4" t="n"/>
-      <c r="K32" s="4" t="n"/>
-      <c r="L32" s="4" t="n"/>
-      <c r="M32" s="4" t="n"/>
-      <c r="N32" s="4" t="n"/>
-      <c r="O32" s="4" t="n"/>
-      <c r="P32" s="4" t="n"/>
-      <c r="Q32" s="4" t="n"/>
-    </row>
     <row r="33">
-      <c r="A33" s="5" t="inlineStr">
-        <is>
-          <t>7 LPF B 500 Hz (Q 1.306)</t>
-        </is>
-      </c>
-      <c r="B33" s="5" t="inlineStr">
-        <is>
-          <t>Rlb1, Rlb2</t>
-        </is>
-      </c>
-      <c r="C33" s="5" t="inlineStr">
-        <is>
-          <t>Resistencia del LPF B</t>
-        </is>
-      </c>
-      <c r="D33" s="5" t="inlineStr">
-        <is>
-          <t>54.9k</t>
-        </is>
-      </c>
-      <c r="E33" s="5" t="inlineStr">
-        <is>
-          <t>56k</t>
-        </is>
-      </c>
-      <c r="F33" s="5" t="inlineStr">
-        <is>
-          <t>pelicula metalica 1 %</t>
-        </is>
-      </c>
-      <c r="G33" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="H33" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="I33" s="5">
-        <f>G33*H33</f>
-        <v/>
-      </c>
-      <c r="J33" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="K33" s="5">
-        <f>I33+J33</f>
-        <v/>
-      </c>
-      <c r="L33" s="5" t="inlineStr">
-        <is>
-          <t>resistencia 56k 1%</t>
-        </is>
-      </c>
-      <c r="M33" s="6" t="n"/>
-      <c r="N33" s="7" t="n"/>
-      <c r="O33" s="8">
-        <f>IF(N33="","",K33*N33)</f>
-        <v/>
-      </c>
-      <c r="P33" s="6" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="Q33" s="5" t="inlineStr">
-        <is>
-          <t>Con 56k: f0 = 495 Hz</t>
-        </is>
-      </c>
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>7 BUCKET + SALIDA AL ADC</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="n"/>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>por canal (x3)</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="n"/>
+      <c r="E33" s="4" t="n"/>
+      <c r="F33" s="4" t="n"/>
+      <c r="G33" s="4" t="n"/>
+      <c r="H33" s="4" t="n"/>
+      <c r="I33" s="4" t="n"/>
+      <c r="J33" s="4" t="n"/>
+      <c r="K33" s="4" t="n"/>
+      <c r="L33" s="4" t="n"/>
+      <c r="M33" s="4" t="n"/>
+      <c r="N33" s="4" t="n"/>
+      <c r="O33" s="4" t="n"/>
+      <c r="P33" s="4" t="n"/>
+      <c r="Q33" s="4" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>7 LPF B 500 Hz (Q 1.306)</t>
+          <t>7 BUCKET + SALIDA AL ADC</t>
         </is>
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>C21</t>
+          <t>Rbk</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>Condensador de realimentacion</t>
+          <t>Resistencia del bucket</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>15n</t>
+          <t>100</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>15n</t>
+          <t>100</t>
         </is>
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>poliester 5 % o C0G</t>
+          <t>pelicula metalica 1 %</t>
         </is>
       </c>
       <c r="G34" s="5" t="n">
         <v>1</v>
       </c>
       <c r="H34" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I34" s="5">
         <f>G34*H34</f>
@@ -2316,7 +2312,7 @@
       </c>
       <c r="L34" s="5" t="inlineStr">
         <is>
-          <t>condensador poliester 15nF</t>
+          <t>resistencia 100 ohm 1%</t>
         </is>
       </c>
       <c r="M34" s="6" t="n"/>
@@ -2335,39 +2331,39 @@
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>7 LPF B 500 Hz (Q 1.306)</t>
+          <t>7 BUCKET + SALIDA AL ADC</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>C22</t>
+          <t>Cbk</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>Condensador a GND</t>
+          <t>Condensador del bucket</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>2.2n</t>
+          <t>1n</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t>2.2n</t>
+          <t>1n</t>
         </is>
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>poliester 5 % o C0G</t>
+          <t>ceramico C0G/NP0</t>
         </is>
       </c>
       <c r="G35" s="5" t="n">
         <v>1</v>
       </c>
       <c r="H35" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I35" s="5">
         <f>G35*H35</f>
@@ -2382,7 +2378,7 @@
       </c>
       <c r="L35" s="5" t="inlineStr">
         <is>
-          <t>condensador poliester 2.2nF</t>
+          <t>condensador ceramico 1nF NP0</t>
         </is>
       </c>
       <c r="M35" s="6" t="n"/>
@@ -2401,17 +2397,17 @@
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>7 LPF B 500 Hz (Q 1.306)</t>
+          <t>7 BUCKET + SALIDA AL ADC</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>XLB</t>
+          <t>ADCk</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>seccion de op-amp</t>
+          <t>Cable a Arduino A1..A3 del STM32N6570-DK</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
@@ -2421,40 +2417,63 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
+          <t>jumper Dupont</t>
+        </is>
+      </c>
+      <c r="F36" s="5" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F36" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G36" s="5" t="n"/>
-      <c r="H36" s="5" t="n"/>
-      <c r="I36" s="5" t="n"/>
-      <c r="J36" s="5" t="n"/>
-      <c r="K36" s="5" t="n"/>
-      <c r="L36" s="5" t="inlineStr"/>
-      <c r="M36" s="5" t="n"/>
-      <c r="N36" s="8" t="n"/>
-      <c r="O36" s="8" t="n"/>
-      <c r="P36" s="5" t="n"/>
+      <c r="G36" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H36" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="I36" s="5">
+        <f>G36*H36</f>
+        <v/>
+      </c>
+      <c r="J36" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="K36" s="5">
+        <f>I36+J36</f>
+        <v/>
+      </c>
+      <c r="L36" s="5" t="inlineStr">
+        <is>
+          <t>cable dupont macho-macho</t>
+        </is>
+      </c>
+      <c r="M36" s="6" t="n"/>
+      <c r="N36" s="7" t="n"/>
+      <c r="O36" s="8">
+        <f>IF(N36="","",K36*N36)</f>
+        <v/>
+      </c>
+      <c r="P36" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
       <c r="Q36" s="5" t="inlineStr">
         <is>
-          <t>Contada en el modulo 11 OP-AMPS</t>
+          <t>CH1-A1 (PA9), CH2-A2 (PA10), CH3-A3 (PA12). Mas 1 cable de GND. A0 no: comparte ADC con USB1 ISENSE (UM3300)</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>8 BUFFER + SALIDA AL ADC</t>
+          <t>9 VREF 1.65 V (compartido)</t>
         </is>
       </c>
       <c r="B37" s="4" t="n"/>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>por canal (x4)</t>
+          <t>compartido</t>
         </is>
       </c>
       <c r="D37" s="4" t="n"/>
@@ -2475,27 +2494,27 @@
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t>8 BUFFER + SALIDA AL ADC</t>
+          <t>9 VREF 1.65 V (compartido)</t>
         </is>
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>Rbk</t>
+          <t>RA1, RA2</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>Resistencia del bucket</t>
+          <t>Divisor de VREF</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>100k</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>100k</t>
         </is>
       </c>
       <c r="F38" s="5" t="inlineStr">
@@ -2504,17 +2523,17 @@
         </is>
       </c>
       <c r="G38" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H38" s="5" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I38" s="5">
         <f>G38*H38</f>
         <v/>
       </c>
       <c r="J38" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K38" s="5">
         <f>I38+J38</f>
@@ -2522,7 +2541,7 @@
       </c>
       <c r="L38" s="5" t="inlineStr">
         <is>
-          <t>resistencia 100 ohm 1%</t>
+          <t>resistencia 100k 1%</t>
         </is>
       </c>
       <c r="M38" s="6" t="n"/>
@@ -2541,46 +2560,46 @@
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t>8 BUFFER + SALIDA AL ADC</t>
+          <t>9 VREF 1.65 V (compartido)</t>
         </is>
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>Cbk</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>Condensador del bucket</t>
+          <t>Condensador del divisor</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>1n</t>
+          <t>10u</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t>1n</t>
+          <t>10u</t>
         </is>
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>ceramico C0G/NP0</t>
+          <t>ceramico X7R o electrolitico</t>
         </is>
       </c>
       <c r="G39" s="5" t="n">
         <v>1</v>
       </c>
       <c r="H39" s="5" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I39" s="5">
         <f>G39*H39</f>
         <v/>
       </c>
       <c r="J39" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K39" s="5">
         <f>I39+J39</f>
@@ -2588,7 +2607,7 @@
       </c>
       <c r="L39" s="5" t="inlineStr">
         <is>
-          <t>condensador ceramico 1nF NP0</t>
+          <t>condensador 10uF</t>
         </is>
       </c>
       <c r="M39" s="6" t="n"/>
@@ -2607,17 +2626,17 @@
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
-          <t>8 BUFFER + SALIDA AL ADC</t>
+          <t>9 VREF 1.65 V (compartido)</t>
         </is>
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>ADCk</t>
+          <t>XVR</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>Cable a Arduino A1..A4 del STM32N6570-DK</t>
+          <t>seccion de op-amp</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
@@ -2627,7 +2646,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t>jumper Dupont</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F40" s="5" t="inlineStr">
@@ -2635,152 +2654,148 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G40" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="H40" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="I40" s="5">
-        <f>G40*H40</f>
-        <v/>
-      </c>
-      <c r="J40" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="K40" s="5">
-        <f>I40+J40</f>
-        <v/>
-      </c>
-      <c r="L40" s="5" t="inlineStr">
-        <is>
-          <t>cable dupont macho-macho</t>
-        </is>
-      </c>
-      <c r="M40" s="6" t="n"/>
-      <c r="N40" s="7" t="n"/>
-      <c r="O40" s="8">
-        <f>IF(N40="","",K40*N40)</f>
-        <v/>
-      </c>
-      <c r="P40" s="6" t="inlineStr">
+      <c r="G40" s="5" t="n"/>
+      <c r="H40" s="5" t="n"/>
+      <c r="I40" s="5" t="n"/>
+      <c r="J40" s="5" t="n"/>
+      <c r="K40" s="5" t="n"/>
+      <c r="L40" s="5" t="inlineStr"/>
+      <c r="M40" s="5" t="n"/>
+      <c r="N40" s="8" t="n"/>
+      <c r="O40" s="8" t="n"/>
+      <c r="P40" s="5" t="n"/>
+      <c r="Q40" s="5" t="inlineStr">
+        <is>
+          <t>Contada en el modulo 11 OP-AMPS</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>10 RLD (compartido)</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="n"/>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>compartido</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="n"/>
+      <c r="E41" s="4" t="n"/>
+      <c r="F41" s="4" t="n"/>
+      <c r="G41" s="4" t="n"/>
+      <c r="H41" s="4" t="n"/>
+      <c r="I41" s="4" t="n"/>
+      <c r="J41" s="4" t="n"/>
+      <c r="K41" s="4" t="n"/>
+      <c r="L41" s="4" t="n"/>
+      <c r="M41" s="4" t="n"/>
+      <c r="N41" s="4" t="n"/>
+      <c r="O41" s="4" t="n"/>
+      <c r="P41" s="4" t="n"/>
+      <c r="Q41" s="4" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>10 RLD (compartido)</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>RSM1..RSM3</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>Sensado de modo comun (punto medio de RG)</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>604k</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>620k</t>
+        </is>
+      </c>
+      <c r="F42" s="5" t="inlineStr">
+        <is>
+          <t>pelicula metalica 1 %</t>
+        </is>
+      </c>
+      <c r="G42" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="H42" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I42" s="5">
+        <f>G42*H42</f>
+        <v/>
+      </c>
+      <c r="J42" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="K42" s="5">
+        <f>I42+J42</f>
+        <v/>
+      </c>
+      <c r="L42" s="5" t="inlineStr">
+        <is>
+          <t>resistencia 620k 1%</t>
+        </is>
+      </c>
+      <c r="M42" s="6" t="n"/>
+      <c r="N42" s="7" t="n"/>
+      <c r="O42" s="8">
+        <f>IF(N42="","",K42*N42)</f>
+        <v/>
+      </c>
+      <c r="P42" s="6" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="Q40" s="5" t="inlineStr">
-        <is>
-          <t>CH1-A1 (PA9), CH2-A2 (PA10), CH3-A3 (PA12), CH4-A4 (PF3). Mas 1 cable de GND. A0 no: comparte ADC con USB1 ISENSE (UM3300)</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="5" t="inlineStr">
-        <is>
-          <t>8 BUFFER + SALIDA AL ADC</t>
-        </is>
-      </c>
-      <c r="B41" s="5" t="inlineStr">
-        <is>
-          <t>XBF</t>
-        </is>
-      </c>
-      <c r="C41" s="5" t="inlineStr">
-        <is>
-          <t>seccion de op-amp</t>
-        </is>
-      </c>
-      <c r="D41" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E41" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F41" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G41" s="5" t="n"/>
-      <c r="H41" s="5" t="n"/>
-      <c r="I41" s="5" t="n"/>
-      <c r="J41" s="5" t="n"/>
-      <c r="K41" s="5" t="n"/>
-      <c r="L41" s="5" t="inlineStr"/>
-      <c r="M41" s="5" t="n"/>
-      <c r="N41" s="8" t="n"/>
-      <c r="O41" s="8" t="n"/>
-      <c r="P41" s="5" t="n"/>
-      <c r="Q41" s="5" t="inlineStr">
-        <is>
-          <t>Contada en el modulo 11 OP-AMPS</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="4" t="inlineStr">
-        <is>
-          <t>9 VREF 1.65 V (compartido)</t>
-        </is>
-      </c>
-      <c r="B42" s="4" t="n"/>
-      <c r="C42" s="4" t="inlineStr">
-        <is>
-          <t>compartido</t>
-        </is>
-      </c>
-      <c r="D42" s="4" t="n"/>
-      <c r="E42" s="4" t="n"/>
-      <c r="F42" s="4" t="n"/>
-      <c r="G42" s="4" t="n"/>
-      <c r="H42" s="4" t="n"/>
-      <c r="I42" s="4" t="n"/>
-      <c r="J42" s="4" t="n"/>
-      <c r="K42" s="4" t="n"/>
-      <c r="L42" s="4" t="n"/>
-      <c r="M42" s="4" t="n"/>
-      <c r="N42" s="4" t="n"/>
-      <c r="O42" s="4" t="n"/>
-      <c r="P42" s="4" t="n"/>
-      <c r="Q42" s="4" t="n"/>
+      <c r="Q42" s="5" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
         <is>
-          <t>9 VREF 1.65 V (compartido)</t>
+          <t>10 RLD (compartido)</t>
         </is>
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>RA1, RA2</t>
+          <t>CINT</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>Divisor de VREF</t>
+          <t>Condensador del integrador</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>100k</t>
+          <t>1n</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t>100k</t>
+          <t>1n</t>
         </is>
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>pelicula metalica 1 %</t>
+          <t>ceramico C0G/NP0</t>
         </is>
       </c>
       <c r="G43" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H43" s="5" t="n">
         <v>1</v>
@@ -2790,7 +2805,7 @@
         <v/>
       </c>
       <c r="J43" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K43" s="5">
         <f>I43+J43</f>
@@ -2798,7 +2813,7 @@
       </c>
       <c r="L43" s="5" t="inlineStr">
         <is>
-          <t>resistencia 100k 1%</t>
+          <t>condensador ceramico 1nF NP0</t>
         </is>
       </c>
       <c r="M43" s="6" t="n"/>
@@ -2812,37 +2827,41 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="Q43" s="5" t="inlineStr"/>
+      <c r="Q43" s="5" t="inlineStr">
+        <is>
+          <t>Si oscila en banco: 2.2n</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
         <is>
-          <t>9 VREF 1.65 V (compartido)</t>
+          <t>10 RLD (compartido)</t>
         </is>
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>RPAR</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>Condensador del divisor</t>
+          <t>Resistencia en paralelo al integrador</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>10u</t>
+          <t>10M</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t>10u</t>
+          <t>10M</t>
         </is>
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>ceramico X7R o electrolitico</t>
+          <t>pelicula 5 %</t>
         </is>
       </c>
       <c r="G44" s="5" t="n">
@@ -2856,7 +2875,7 @@
         <v/>
       </c>
       <c r="J44" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K44" s="5">
         <f>I44+J44</f>
@@ -2864,7 +2883,7 @@
       </c>
       <c r="L44" s="5" t="inlineStr">
         <is>
-          <t>condensador 10uF</t>
+          <t>resistencia 10M</t>
         </is>
       </c>
       <c r="M44" s="6" t="n"/>
@@ -2883,176 +2902,180 @@
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
         <is>
-          <t>9 VREF 1.65 V (compartido)</t>
+          <t>10 RLD (compartido)</t>
         </is>
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>XVR</t>
+          <t>RLIM</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
+          <t>Resistencia de seguridad al electrodo RLD</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>390k</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>390k</t>
+        </is>
+      </c>
+      <c r="F45" s="5" t="inlineStr">
+        <is>
+          <t>pelicula metalica 1 %</t>
+        </is>
+      </c>
+      <c r="G45" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H45" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I45" s="5">
+        <f>G45*H45</f>
+        <v/>
+      </c>
+      <c r="J45" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="K45" s="5">
+        <f>I45+J45</f>
+        <v/>
+      </c>
+      <c r="L45" s="5" t="inlineStr">
+        <is>
+          <t>resistencia 390k 1%</t>
+        </is>
+      </c>
+      <c r="M45" s="6" t="n"/>
+      <c r="N45" s="7" t="n"/>
+      <c r="O45" s="8">
+        <f>IF(N45="","",K45*N45)</f>
+        <v/>
+      </c>
+      <c r="P45" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="Q45" s="5" t="inlineStr">
+        <is>
+          <t>Limita la corriente al paciente</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>10 RLD (compartido)</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>XRLD</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
           <t>seccion de op-amp</t>
         </is>
       </c>
-      <c r="D45" s="5" t="inlineStr">
+      <c r="D46" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E45" s="5" t="inlineStr">
+      <c r="E46" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F45" s="5" t="inlineStr">
+      <c r="F46" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G45" s="5" t="n"/>
-      <c r="H45" s="5" t="n"/>
-      <c r="I45" s="5" t="n"/>
-      <c r="J45" s="5" t="n"/>
-      <c r="K45" s="5" t="n"/>
-      <c r="L45" s="5" t="inlineStr"/>
-      <c r="M45" s="5" t="n"/>
-      <c r="N45" s="8" t="n"/>
-      <c r="O45" s="8" t="n"/>
-      <c r="P45" s="5" t="n"/>
-      <c r="Q45" s="5" t="inlineStr">
+      <c r="G46" s="5" t="n"/>
+      <c r="H46" s="5" t="n"/>
+      <c r="I46" s="5" t="n"/>
+      <c r="J46" s="5" t="n"/>
+      <c r="K46" s="5" t="n"/>
+      <c r="L46" s="5" t="inlineStr"/>
+      <c r="M46" s="5" t="n"/>
+      <c r="N46" s="8" t="n"/>
+      <c r="O46" s="8" t="n"/>
+      <c r="P46" s="5" t="n"/>
+      <c r="Q46" s="5" t="inlineStr">
         <is>
           <t>Contada en el modulo 11 OP-AMPS</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="4" t="inlineStr">
-        <is>
-          <t>10 RLD (compartido)</t>
-        </is>
-      </c>
-      <c r="B46" s="4" t="n"/>
-      <c r="C46" s="4" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>11 OP-AMPS (paquetes)</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="n"/>
+      <c r="C47" s="4" t="inlineStr">
         <is>
           <t>compartido</t>
         </is>
       </c>
-      <c r="D46" s="4" t="n"/>
-      <c r="E46" s="4" t="n"/>
-      <c r="F46" s="4" t="n"/>
-      <c r="G46" s="4" t="n"/>
-      <c r="H46" s="4" t="n"/>
-      <c r="I46" s="4" t="n"/>
-      <c r="J46" s="4" t="n"/>
-      <c r="K46" s="4" t="n"/>
-      <c r="L46" s="4" t="n"/>
-      <c r="M46" s="4" t="n"/>
-      <c r="N46" s="4" t="n"/>
-      <c r="O46" s="4" t="n"/>
-      <c r="P46" s="4" t="n"/>
-      <c r="Q46" s="4" t="n"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="5" t="inlineStr">
-        <is>
-          <t>10 RLD (compartido)</t>
-        </is>
-      </c>
-      <c r="B47" s="5" t="inlineStr">
-        <is>
-          <t>RSM1..RSM4</t>
-        </is>
-      </c>
-      <c r="C47" s="5" t="inlineStr">
-        <is>
-          <t>Sensado de modo comun (punto medio de RG)</t>
-        </is>
-      </c>
-      <c r="D47" s="5" t="inlineStr">
-        <is>
-          <t>604k</t>
-        </is>
-      </c>
-      <c r="E47" s="5" t="inlineStr">
-        <is>
-          <t>620k</t>
-        </is>
-      </c>
-      <c r="F47" s="5" t="inlineStr">
-        <is>
-          <t>pelicula metalica 1 %</t>
-        </is>
-      </c>
-      <c r="G47" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="H47" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="I47" s="5">
-        <f>G47*H47</f>
-        <v/>
-      </c>
-      <c r="J47" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="K47" s="5">
-        <f>I47+J47</f>
-        <v/>
-      </c>
-      <c r="L47" s="5" t="inlineStr">
-        <is>
-          <t>resistencia 620k 1%</t>
-        </is>
-      </c>
-      <c r="M47" s="6" t="n"/>
-      <c r="N47" s="7" t="n"/>
-      <c r="O47" s="8">
-        <f>IF(N47="","",K47*N47)</f>
-        <v/>
-      </c>
-      <c r="P47" s="6" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="Q47" s="5" t="inlineStr"/>
+      <c r="D47" s="4" t="n"/>
+      <c r="E47" s="4" t="n"/>
+      <c r="F47" s="4" t="n"/>
+      <c r="G47" s="4" t="n"/>
+      <c r="H47" s="4" t="n"/>
+      <c r="I47" s="4" t="n"/>
+      <c r="J47" s="4" t="n"/>
+      <c r="K47" s="4" t="n"/>
+      <c r="L47" s="4" t="n"/>
+      <c r="M47" s="4" t="n"/>
+      <c r="N47" s="4" t="n"/>
+      <c r="O47" s="4" t="n"/>
+      <c r="P47" s="4" t="n"/>
+      <c r="Q47" s="4" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
         <is>
-          <t>10 RLD (compartido)</t>
+          <t>11 OP-AMPS (paquetes)</t>
         </is>
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>CINT</t>
+          <t>XHP, XMF, XLB x3, XRLD, XVR</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>Condensador del integrador</t>
+          <t>Op-amp doble TS922 (rail-to-rail, 4 MHz)</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>1n</t>
+          <t>TS922</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t>1n</t>
+          <t>TS922AIYDT</t>
         </is>
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>ceramico C0G/NP0</t>
+          <t>SOIC-8</t>
         </is>
       </c>
       <c r="G48" s="5" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="H48" s="5" t="n">
         <v>1</v>
@@ -3062,7 +3085,7 @@
         <v/>
       </c>
       <c r="J48" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K48" s="5">
         <f>I48+J48</f>
@@ -3070,7 +3093,7 @@
       </c>
       <c r="L48" s="5" t="inlineStr">
         <is>
-          <t>condensador ceramico 1nF NP0</t>
+          <t>TS922AIYDT</t>
         </is>
       </c>
       <c r="M48" s="6" t="n"/>
@@ -3086,43 +3109,43 @@
       </c>
       <c r="Q48" s="5" t="inlineStr">
         <is>
-          <t>Si oscila en banco: 2.2n</t>
+          <t>11 secciones = 3 por canal x 3 + RLD + VREF (1 libre). Solo habia 6 en stock</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t>10 RLD (compartido)</t>
+          <t>11 OP-AMPS (paquetes)</t>
         </is>
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>RPAR</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>Resistencia en paralelo al integrador</t>
+          <t>Adaptador SOIC-8 a DIP-8</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>10M</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t>10M</t>
+          <t>SOIC8 a DIP8</t>
         </is>
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>pelicula 5 %</t>
+          <t>PCB adaptador</t>
         </is>
       </c>
       <c r="G49" s="5" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="H49" s="5" t="n">
         <v>1</v>
@@ -3140,7 +3163,7 @@
       </c>
       <c r="L49" s="5" t="inlineStr">
         <is>
-          <t>resistencia 10M</t>
+          <t>adaptador SOIC8 a DIP8</t>
         </is>
       </c>
       <c r="M49" s="6" t="n"/>
@@ -3154,41 +3177,45 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="Q49" s="5" t="inlineStr"/>
+      <c r="Q49" s="5" t="inlineStr">
+        <is>
+          <t>Soldar el TS922 al adaptador y probarlo antes de montarlo</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
         <is>
-          <t>10 RLD (compartido)</t>
+          <t>11 OP-AMPS (paquetes)</t>
         </is>
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>RLIM</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>Resistencia de seguridad al electrodo RLD</t>
+          <t>Zocalo DIP-8</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>390k</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E50" s="5" t="inlineStr">
         <is>
-          <t>390k</t>
+          <t>DIP-8</t>
         </is>
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>pelicula metalica 1 %</t>
+          <t>zocalo</t>
         </is>
       </c>
       <c r="G50" s="5" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="H50" s="5" t="n">
         <v>1</v>
@@ -3206,7 +3233,7 @@
       </c>
       <c r="L50" s="5" t="inlineStr">
         <is>
-          <t>resistencia 390k 1%</t>
+          <t>zocalo DIP 8 pines</t>
         </is>
       </c>
       <c r="M50" s="6" t="n"/>
@@ -3220,63 +3247,82 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="Q50" s="5" t="inlineStr">
-        <is>
-          <t>Limita la corriente al paciente</t>
-        </is>
-      </c>
+      <c r="Q50" s="5" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>10 RLD (compartido)</t>
+          <t>11 OP-AMPS (paquetes)</t>
         </is>
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>XRLD</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>seccion de op-amp</t>
+          <t>Desacople de cada op-amp</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>100n</t>
         </is>
       </c>
       <c r="E51" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>100n</t>
         </is>
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G51" s="5" t="n"/>
-      <c r="H51" s="5" t="n"/>
-      <c r="I51" s="5" t="n"/>
-      <c r="J51" s="5" t="n"/>
-      <c r="K51" s="5" t="n"/>
-      <c r="L51" s="5" t="inlineStr"/>
-      <c r="M51" s="5" t="n"/>
-      <c r="N51" s="8" t="n"/>
-      <c r="O51" s="8" t="n"/>
-      <c r="P51" s="5" t="n"/>
+          <t>ceramico X7R</t>
+        </is>
+      </c>
+      <c r="G51" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="H51" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I51" s="5">
+        <f>G51*H51</f>
+        <v/>
+      </c>
+      <c r="J51" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="K51" s="5">
+        <f>I51+J51</f>
+        <v/>
+      </c>
+      <c r="L51" s="5" t="inlineStr">
+        <is>
+          <t>condensador ceramico 100nF</t>
+        </is>
+      </c>
+      <c r="M51" s="6" t="n"/>
+      <c r="N51" s="7" t="n"/>
+      <c r="O51" s="8">
+        <f>IF(N51="","",K51*N51)</f>
+        <v/>
+      </c>
+      <c r="P51" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
       <c r="Q51" s="5" t="inlineStr">
         <is>
-          <t>Contada en el modulo 11 OP-AMPS</t>
+          <t>Pegado al pin de alimentacion</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
         <is>
-          <t>11 OP-AMPS (paquetes)</t>
+          <t>12 ALIMENTACION (a bateria)</t>
         </is>
       </c>
       <c r="B52" s="4" t="n"/>
@@ -3303,36 +3349,36 @@
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
         <is>
-          <t>11 OP-AMPS (paquetes)</t>
+          <t>12 ALIMENTACION (a bateria)</t>
         </is>
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>XHP..XBF x4, XRLD, XVR</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>Op-amp cuadruple MCP6004</t>
+          <t>Regulador LDO 3.3 V</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>MCP6004</t>
+          <t>MCP1700-3302E</t>
         </is>
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t>MCP6004-I/SL</t>
+          <t>MCP1700-3302E TO-92</t>
         </is>
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>SOIC-14</t>
+          <t>LDO 250 mA</t>
         </is>
       </c>
       <c r="G53" s="5" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="H53" s="5" t="n">
         <v>1</v>
@@ -3342,7 +3388,7 @@
         <v/>
       </c>
       <c r="J53" s="5" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K53" s="5">
         <f>I53+J53</f>
@@ -3350,16 +3396,16 @@
       </c>
       <c r="L53" s="5" t="inlineStr">
         <is>
-          <t>MCP6004-I/SL</t>
+          <t>MCP1700 3.3V TO-92</t>
         </is>
       </c>
       <c r="M53" s="6" t="inlineStr">
         <is>
-          <t>RS Chile</t>
+          <t>HUBOT</t>
         </is>
       </c>
       <c r="N53" s="7" t="n">
-        <v>809</v>
+        <v>890</v>
       </c>
       <c r="O53" s="8">
         <f>IF(N53="","",K53*N53)</f>
@@ -3372,14 +3418,14 @@
       </c>
       <c r="Q53" s="5" t="inlineStr">
         <is>
-          <t>22 secciones = 5 por canal x 4 + RLD + VREF (2 libres). RS Chile vende en paquetes de 10</t>
+          <t>EJEMPLO de llenado: CLP 890 c/IVA en hubot.cl (30-sep-2026). Tu LDO de 3.0 V no sirve</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="5" t="inlineStr">
         <is>
-          <t>11 OP-AMPS (paquetes)</t>
+          <t>12 ALIMENTACION (a bateria)</t>
         </is>
       </c>
       <c r="B54" s="5" t="inlineStr">
@@ -3389,26 +3435,26 @@
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>Adaptador SOIC-14 a DIP-14</t>
+          <t>Condensadores del LDO (entrada y salida)</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1u</t>
         </is>
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t>SOIC14 a DIP14</t>
+          <t>1u</t>
         </is>
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>PCB adaptador</t>
+          <t>ceramico X7R</t>
         </is>
       </c>
       <c r="G54" s="5" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="H54" s="5" t="n">
         <v>1</v>
@@ -3426,7 +3472,7 @@
       </c>
       <c r="L54" s="5" t="inlineStr">
         <is>
-          <t>adaptador SOIC14 a DIP14</t>
+          <t>condensador ceramico 1uF</t>
         </is>
       </c>
       <c r="M54" s="6" t="n"/>
@@ -3442,14 +3488,14 @@
       </c>
       <c r="Q54" s="5" t="inlineStr">
         <is>
-          <t>Para montar el MCP6004-I/SL en perfboard</t>
+          <t>Ya tienes 2 x 1uF 0402 (SMD): sirven si los sueldas</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="5" t="inlineStr">
         <is>
-          <t>11 OP-AMPS (paquetes)</t>
+          <t>12 ALIMENTACION (a bateria)</t>
         </is>
       </c>
       <c r="B55" s="5" t="inlineStr">
@@ -3459,26 +3505,26 @@
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>Zocalo DIP-14</t>
+          <t>Condensador bulk del riel 3.3 V</t>
         </is>
       </c>
       <c r="D55" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10u</t>
         </is>
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t>DIP-14</t>
+          <t>10u</t>
         </is>
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>zocalo</t>
+          <t>ceramico o electrolitico</t>
         </is>
       </c>
       <c r="G55" s="5" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="H55" s="5" t="n">
         <v>1</v>
@@ -3496,7 +3542,7 @@
       </c>
       <c r="L55" s="5" t="inlineStr">
         <is>
-          <t>zocalo DIP 14 pines</t>
+          <t>condensador 10uF</t>
         </is>
       </c>
       <c r="M55" s="6" t="n"/>
@@ -3510,16 +3556,12 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="Q55" s="5" t="inlineStr">
-        <is>
-          <t>Si los op-amps son dobles: 11 zocalos DIP-8</t>
-        </is>
-      </c>
+      <c r="Q55" s="5" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="5" t="inlineStr">
         <is>
-          <t>11 OP-AMPS (paquetes)</t>
+          <t>12 ALIMENTACION (a bateria)</t>
         </is>
       </c>
       <c r="B56" s="5" t="inlineStr">
@@ -3529,26 +3571,26 @@
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>Desacople de cada op-amp</t>
+          <t>Portapilas 3 x AA</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>100n</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t>100n</t>
+          <t>3xAA</t>
         </is>
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>ceramico X7R</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G56" s="5" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="H56" s="5" t="n">
         <v>1</v>
@@ -3558,7 +3600,7 @@
         <v/>
       </c>
       <c r="J56" s="5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K56" s="5">
         <f>I56+J56</f>
@@ -3566,7 +3608,7 @@
       </c>
       <c r="L56" s="5" t="inlineStr">
         <is>
-          <t>condensador ceramico 100nF</t>
+          <t>portapilas 3 AA</t>
         </is>
       </c>
       <c r="M56" s="6" t="n"/>
@@ -3582,36 +3624,75 @@
       </c>
       <c r="Q56" s="5" t="inlineStr">
         <is>
-          <t>Pegado al pin de alimentacion</t>
+          <t>4.5 V nominal; mantiene el AFE aislado de la red</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="4" t="inlineStr">
+      <c r="A57" s="5" t="inlineStr">
         <is>
           <t>12 ALIMENTACION (a bateria)</t>
         </is>
       </c>
-      <c r="B57" s="4" t="n"/>
-      <c r="C57" s="4" t="inlineStr">
-        <is>
-          <t>compartido</t>
-        </is>
-      </c>
-      <c r="D57" s="4" t="n"/>
-      <c r="E57" s="4" t="n"/>
-      <c r="F57" s="4" t="n"/>
-      <c r="G57" s="4" t="n"/>
-      <c r="H57" s="4" t="n"/>
-      <c r="I57" s="4" t="n"/>
-      <c r="J57" s="4" t="n"/>
-      <c r="K57" s="4" t="n"/>
-      <c r="L57" s="4" t="n"/>
-      <c r="M57" s="4" t="n"/>
-      <c r="N57" s="4" t="n"/>
-      <c r="O57" s="4" t="n"/>
-      <c r="P57" s="4" t="n"/>
-      <c r="Q57" s="4" t="n"/>
+      <c r="B57" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>Pilas AA</t>
+        </is>
+      </c>
+      <c r="D57" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E57" s="5" t="inlineStr">
+        <is>
+          <t>AA</t>
+        </is>
+      </c>
+      <c r="F57" s="5" t="inlineStr">
+        <is>
+          <t>alcalina</t>
+        </is>
+      </c>
+      <c r="G57" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="H57" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I57" s="5">
+        <f>G57*H57</f>
+        <v/>
+      </c>
+      <c r="J57" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="K57" s="5">
+        <f>I57+J57</f>
+        <v/>
+      </c>
+      <c r="L57" s="5" t="inlineStr">
+        <is>
+          <t>pila AA</t>
+        </is>
+      </c>
+      <c r="M57" s="6" t="n"/>
+      <c r="N57" s="7" t="n"/>
+      <c r="O57" s="8">
+        <f>IF(N57="","",K57*N57)</f>
+        <v/>
+      </c>
+      <c r="P57" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="Q57" s="5" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="5" t="inlineStr">
@@ -3626,22 +3707,22 @@
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>Regulador LDO 3.3 V</t>
+          <t>Interruptor</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>MCP1700-3302E</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t>MCP1700-3302E TO-92</t>
+          <t>deslizante</t>
         </is>
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>LDO 250 mA</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G58" s="5" t="n">
@@ -3655,7 +3736,7 @@
         <v/>
       </c>
       <c r="J58" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K58" s="5">
         <f>I58+J58</f>
@@ -3663,17 +3744,11 @@
       </c>
       <c r="L58" s="5" t="inlineStr">
         <is>
-          <t>MCP1700 3.3V TO-92</t>
-        </is>
-      </c>
-      <c r="M58" s="6" t="inlineStr">
-        <is>
-          <t>HUBOT</t>
-        </is>
-      </c>
-      <c r="N58" s="7" t="n">
-        <v>890</v>
-      </c>
+          <t>interruptor deslizante</t>
+        </is>
+      </c>
+      <c r="M58" s="6" t="n"/>
+      <c r="N58" s="7" t="n"/>
       <c r="O58" s="8">
         <f>IF(N58="","",K58*N58)</f>
         <v/>
@@ -3683,115 +3758,68 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="Q58" s="5" t="inlineStr">
-        <is>
-          <t>EJEMPLO de llenado: CLP 890 c/IVA en hubot.cl (30-sep-2026). Tu LDO de 3.0 V no sirve</t>
-        </is>
-      </c>
+      <c r="Q58" s="5" t="inlineStr"/>
     </row>
     <row r="59">
-      <c r="A59" s="5" t="inlineStr">
-        <is>
-          <t>12 ALIMENTACION (a bateria)</t>
-        </is>
-      </c>
-      <c r="B59" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C59" s="5" t="inlineStr">
-        <is>
-          <t>Condensadores del LDO (entrada y salida)</t>
-        </is>
-      </c>
-      <c r="D59" s="5" t="inlineStr">
-        <is>
-          <t>1u</t>
-        </is>
-      </c>
-      <c r="E59" s="5" t="inlineStr">
-        <is>
-          <t>1u</t>
-        </is>
-      </c>
-      <c r="F59" s="5" t="inlineStr">
-        <is>
-          <t>ceramico X7R</t>
-        </is>
-      </c>
-      <c r="G59" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="H59" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="I59" s="5">
-        <f>G59*H59</f>
-        <v/>
-      </c>
-      <c r="J59" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="K59" s="5">
-        <f>I59+J59</f>
-        <v/>
-      </c>
-      <c r="L59" s="5" t="inlineStr">
-        <is>
-          <t>condensador ceramico 1uF</t>
-        </is>
-      </c>
-      <c r="M59" s="6" t="n"/>
-      <c r="N59" s="7" t="n"/>
-      <c r="O59" s="8">
-        <f>IF(N59="","",K59*N59)</f>
-        <v/>
-      </c>
-      <c r="P59" s="6" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="Q59" s="5" t="inlineStr">
-        <is>
-          <t>Ya tienes 2 x 1uF 0402 (SMD): sirven si los sueldas</t>
-        </is>
-      </c>
+      <c r="A59" s="4" t="inlineStr">
+        <is>
+          <t>13 ELECTRODOS Y CABLES</t>
+        </is>
+      </c>
+      <c r="B59" s="4" t="n"/>
+      <c r="C59" s="4" t="inlineStr">
+        <is>
+          <t>compartido</t>
+        </is>
+      </c>
+      <c r="D59" s="4" t="n"/>
+      <c r="E59" s="4" t="n"/>
+      <c r="F59" s="4" t="n"/>
+      <c r="G59" s="4" t="n"/>
+      <c r="H59" s="4" t="n"/>
+      <c r="I59" s="4" t="n"/>
+      <c r="J59" s="4" t="n"/>
+      <c r="K59" s="4" t="n"/>
+      <c r="L59" s="4" t="n"/>
+      <c r="M59" s="4" t="n"/>
+      <c r="N59" s="4" t="n"/>
+      <c r="O59" s="4" t="n"/>
+      <c r="P59" s="4" t="n"/>
+      <c r="Q59" s="4" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="5" t="inlineStr">
         <is>
-          <t>12 ALIMENTACION (a bateria)</t>
+          <t>13 ELECTRODOS Y CABLES</t>
         </is>
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
+          <t>XE1P..XE3N, XER</t>
+        </is>
+      </c>
+      <c r="C60" s="5" t="inlineStr">
+        <is>
+          <t>Electrodo Ag/AgCl con broche</t>
+        </is>
+      </c>
+      <c r="D60" s="5" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="C60" s="5" t="inlineStr">
-        <is>
-          <t>Condensador bulk del riel 3.3 V</t>
-        </is>
-      </c>
-      <c r="D60" s="5" t="inlineStr">
-        <is>
-          <t>10u</t>
-        </is>
-      </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t>10u</t>
+          <t>3M Red Dot 2228/2560</t>
         </is>
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>ceramico o electrolitico</t>
+          <t>desechable</t>
         </is>
       </c>
       <c r="G60" s="5" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="H60" s="5" t="n">
         <v>1</v>
@@ -3801,7 +3829,7 @@
         <v/>
       </c>
       <c r="J60" s="5" t="n">
-        <v>1</v>
+        <v>43</v>
       </c>
       <c r="K60" s="5">
         <f>I60+J60</f>
@@ -3809,7 +3837,7 @@
       </c>
       <c r="L60" s="5" t="inlineStr">
         <is>
-          <t>condensador 10uF</t>
+          <t>electrodo ECG 3M 2228</t>
         </is>
       </c>
       <c r="M60" s="6" t="n"/>
@@ -3823,12 +3851,16 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="Q60" s="5" t="inlineStr"/>
+      <c r="Q60" s="5" t="inlineStr">
+        <is>
+          <t>7 por sesion (6 de senal + 1 RLD); caja de 50</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="5" t="inlineStr">
         <is>
-          <t>12 ALIMENTACION (a bateria)</t>
+          <t>13 ELECTRODOS Y CABLES</t>
         </is>
       </c>
       <c r="B61" s="5" t="inlineStr">
@@ -3838,7 +3870,7 @@
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>Portapilas 3 x AA</t>
+          <t>Cable con broche (snap) para electrodo</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
@@ -3848,7 +3880,7 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t>3xAA</t>
+          <t>broche 4 mm</t>
         </is>
       </c>
       <c r="F61" s="5" t="inlineStr">
@@ -3857,7 +3889,7 @@
         </is>
       </c>
       <c r="G61" s="5" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="H61" s="5" t="n">
         <v>1</v>
@@ -3867,7 +3899,7 @@
         <v/>
       </c>
       <c r="J61" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K61" s="5">
         <f>I61+J61</f>
@@ -3875,7 +3907,7 @@
       </c>
       <c r="L61" s="5" t="inlineStr">
         <is>
-          <t>portapilas 3 AA</t>
+          <t>cable electrodo broche snap</t>
         </is>
       </c>
       <c r="M61" s="6" t="n"/>
@@ -3891,14 +3923,14 @@
       </c>
       <c r="Q61" s="5" t="inlineStr">
         <is>
-          <t>4.5 V nominal; mantiene el AFE aislado de la red</t>
+          <t>O 3 cables ECG de 3 derivaciones</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="5" t="inlineStr">
         <is>
-          <t>12 ALIMENTACION (a bateria)</t>
+          <t>13 ELECTRODOS Y CABLES</t>
         </is>
       </c>
       <c r="B62" s="5" t="inlineStr">
@@ -3908,7 +3940,7 @@
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>Pilas AA</t>
+          <t>Alcohol isopropilico / gel</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
@@ -3918,16 +3950,16 @@
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t>AA</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F62" s="5" t="inlineStr">
         <is>
-          <t>alcalina</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G62" s="5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H62" s="5" t="n">
         <v>1</v>
@@ -3937,7 +3969,7 @@
         <v/>
       </c>
       <c r="J62" s="5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K62" s="5">
         <f>I62+J62</f>
@@ -3945,7 +3977,7 @@
       </c>
       <c r="L62" s="5" t="inlineStr">
         <is>
-          <t>pila AA</t>
+          <t>alcohol isopropilico</t>
         </is>
       </c>
       <c r="M62" s="6" t="n"/>
@@ -3959,115 +3991,119 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="Q62" s="5" t="inlineStr"/>
+      <c r="Q62" s="5" t="inlineStr">
+        <is>
+          <t>Preparar la piel</t>
+        </is>
+      </c>
     </row>
     <row r="63">
-      <c r="A63" s="5" t="inlineStr">
-        <is>
-          <t>12 ALIMENTACION (a bateria)</t>
-        </is>
-      </c>
-      <c r="B63" s="5" t="inlineStr">
+      <c r="A63" s="4" t="inlineStr">
+        <is>
+          <t>14 MECANICA E INTERCONEXION</t>
+        </is>
+      </c>
+      <c r="B63" s="4" t="n"/>
+      <c r="C63" s="4" t="inlineStr">
+        <is>
+          <t>compartido</t>
+        </is>
+      </c>
+      <c r="D63" s="4" t="n"/>
+      <c r="E63" s="4" t="n"/>
+      <c r="F63" s="4" t="n"/>
+      <c r="G63" s="4" t="n"/>
+      <c r="H63" s="4" t="n"/>
+      <c r="I63" s="4" t="n"/>
+      <c r="J63" s="4" t="n"/>
+      <c r="K63" s="4" t="n"/>
+      <c r="L63" s="4" t="n"/>
+      <c r="M63" s="4" t="n"/>
+      <c r="N63" s="4" t="n"/>
+      <c r="O63" s="4" t="n"/>
+      <c r="P63" s="4" t="n"/>
+      <c r="Q63" s="4" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="5" t="inlineStr">
+        <is>
+          <t>14 MECANICA E INTERCONEXION</t>
+        </is>
+      </c>
+      <c r="B64" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="C63" s="5" t="inlineStr">
-        <is>
-          <t>Interruptor</t>
-        </is>
-      </c>
-      <c r="D63" s="5" t="inlineStr">
+      <c r="C64" s="5" t="inlineStr">
+        <is>
+          <t>Perfboard</t>
+        </is>
+      </c>
+      <c r="D64" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E63" s="5" t="inlineStr">
-        <is>
-          <t>deslizante</t>
-        </is>
-      </c>
-      <c r="F63" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G63" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="H63" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="I63" s="5">
-        <f>G63*H63</f>
-        <v/>
-      </c>
-      <c r="J63" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K63" s="5">
-        <f>I63+J63</f>
-        <v/>
-      </c>
-      <c r="L63" s="5" t="inlineStr">
-        <is>
-          <t>interruptor deslizante</t>
-        </is>
-      </c>
-      <c r="M63" s="6" t="n"/>
-      <c r="N63" s="7" t="n"/>
-      <c r="O63" s="8">
-        <f>IF(N63="","",K63*N63)</f>
-        <v/>
-      </c>
-      <c r="P63" s="6" t="inlineStr">
+      <c r="E64" s="5" t="inlineStr">
+        <is>
+          <t>10 x 15 cm</t>
+        </is>
+      </c>
+      <c r="F64" s="5" t="inlineStr">
+        <is>
+          <t>fibra de vidrio</t>
+        </is>
+      </c>
+      <c r="G64" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H64" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I64" s="5">
+        <f>G64*H64</f>
+        <v/>
+      </c>
+      <c r="J64" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="K64" s="5">
+        <f>I64+J64</f>
+        <v/>
+      </c>
+      <c r="L64" s="5" t="inlineStr">
+        <is>
+          <t>placa perforada 10x15</t>
+        </is>
+      </c>
+      <c r="M64" s="6" t="n"/>
+      <c r="N64" s="7" t="n"/>
+      <c r="O64" s="8">
+        <f>IF(N64="","",K64*N64)</f>
+        <v/>
+      </c>
+      <c r="P64" s="6" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="Q63" s="5" t="inlineStr"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="4" t="inlineStr">
-        <is>
-          <t>13 ELECTRODOS Y CABLES</t>
-        </is>
-      </c>
-      <c r="B64" s="4" t="n"/>
-      <c r="C64" s="4" t="inlineStr">
-        <is>
-          <t>compartido</t>
-        </is>
-      </c>
-      <c r="D64" s="4" t="n"/>
-      <c r="E64" s="4" t="n"/>
-      <c r="F64" s="4" t="n"/>
-      <c r="G64" s="4" t="n"/>
-      <c r="H64" s="4" t="n"/>
-      <c r="I64" s="4" t="n"/>
-      <c r="J64" s="4" t="n"/>
-      <c r="K64" s="4" t="n"/>
-      <c r="L64" s="4" t="n"/>
-      <c r="M64" s="4" t="n"/>
-      <c r="N64" s="4" t="n"/>
-      <c r="O64" s="4" t="n"/>
-      <c r="P64" s="4" t="n"/>
-      <c r="Q64" s="4" t="n"/>
+      <c r="Q64" s="5" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="5" t="inlineStr">
         <is>
-          <t>13 ELECTRODOS Y CABLES</t>
+          <t>14 MECANICA E INTERCONEXION</t>
         </is>
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>XE1P..XE4N, XER</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>Electrodo Ag/AgCl con broche</t>
+          <t>Zocalo DIP-8 (INA)</t>
         </is>
       </c>
       <c r="D65" s="5" t="inlineStr">
@@ -4077,16 +4113,16 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t>3M Red Dot 2228/2560</t>
+          <t xml:space="preserve">DIP-8 </t>
         </is>
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
-          <t>desechable</t>
+          <t>zocalo</t>
         </is>
       </c>
       <c r="G65" s="5" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H65" s="5" t="n">
         <v>1</v>
@@ -4096,7 +4132,7 @@
         <v/>
       </c>
       <c r="J65" s="5" t="n">
-        <v>41</v>
+        <v>0</v>
       </c>
       <c r="K65" s="5">
         <f>I65+J65</f>
@@ -4104,7 +4140,7 @@
       </c>
       <c r="L65" s="5" t="inlineStr">
         <is>
-          <t>electrodo ECG 3M 2228</t>
+          <t>zocalo DIP 8 pines</t>
         </is>
       </c>
       <c r="M65" s="6" t="n"/>
@@ -4120,14 +4156,14 @@
       </c>
       <c r="Q65" s="5" t="inlineStr">
         <is>
-          <t>9 por sesion (8 de senal + 1 RLD); caja de 50</t>
+          <t>Solo si usas el respaldo AD623AN DIP-8</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="5" t="inlineStr">
         <is>
-          <t>13 ELECTRODOS Y CABLES</t>
+          <t>14 MECANICA E INTERCONEXION</t>
         </is>
       </c>
       <c r="B66" s="5" t="inlineStr">
@@ -4137,7 +4173,7 @@
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>Cable con broche (snap) para electrodo</t>
+          <t>Adaptador SOIC/MSOP-8 a DIP-8</t>
         </is>
       </c>
       <c r="D66" s="5" t="inlineStr">
@@ -4147,16 +4183,16 @@
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t>broche 4 mm</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F66" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>PCB adaptador</t>
         </is>
       </c>
       <c r="G66" s="5" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H66" s="5" t="n">
         <v>1</v>
@@ -4166,7 +4202,7 @@
         <v/>
       </c>
       <c r="J66" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K66" s="5">
         <f>I66+J66</f>
@@ -4174,7 +4210,7 @@
       </c>
       <c r="L66" s="5" t="inlineStr">
         <is>
-          <t>cable electrodo broche snap</t>
+          <t>adaptador SOIC8 a DIP8</t>
         </is>
       </c>
       <c r="M66" s="6" t="n"/>
@@ -4190,14 +4226,14 @@
       </c>
       <c r="Q66" s="5" t="inlineStr">
         <is>
-          <t>O 3 cables ECG de 3 derivaciones</t>
+          <t>Solo si compras el INA333 suelto (SMD)</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="5" t="inlineStr">
         <is>
-          <t>13 ELECTRODOS Y CABLES</t>
+          <t>14 MECANICA E INTERCONEXION</t>
         </is>
       </c>
       <c r="B67" s="5" t="inlineStr">
@@ -4207,7 +4243,7 @@
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>Alcohol isopropilico / gel</t>
+          <t>Tira de headers macho/hembra</t>
         </is>
       </c>
       <c r="D67" s="5" t="inlineStr">
@@ -4217,16 +4253,16 @@
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
+          <t>2.54 mm</t>
+        </is>
+      </c>
+      <c r="F67" s="5" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F67" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="G67" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H67" s="5" t="n">
         <v>1</v>
@@ -4236,7 +4272,7 @@
         <v/>
       </c>
       <c r="J67" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K67" s="5">
         <f>I67+J67</f>
@@ -4244,7 +4280,7 @@
       </c>
       <c r="L67" s="5" t="inlineStr">
         <is>
-          <t>alcohol isopropilico</t>
+          <t>header 2.54mm 40 pines</t>
         </is>
       </c>
       <c r="M67" s="6" t="n"/>
@@ -4258,392 +4294,89 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="Q67" s="5" t="inlineStr">
-        <is>
-          <t>Preparar la piel</t>
-        </is>
-      </c>
+      <c r="Q67" s="5" t="inlineStr"/>
     </row>
     <row r="68">
-      <c r="A68" s="4" t="inlineStr">
+      <c r="A68" s="5" t="inlineStr">
         <is>
           <t>14 MECANICA E INTERCONEXION</t>
         </is>
       </c>
-      <c r="B68" s="4" t="n"/>
-      <c r="C68" s="4" t="inlineStr">
-        <is>
-          <t>compartido</t>
-        </is>
-      </c>
-      <c r="D68" s="4" t="n"/>
-      <c r="E68" s="4" t="n"/>
-      <c r="F68" s="4" t="n"/>
-      <c r="G68" s="4" t="n"/>
-      <c r="H68" s="4" t="n"/>
-      <c r="I68" s="4" t="n"/>
-      <c r="J68" s="4" t="n"/>
-      <c r="K68" s="4" t="n"/>
-      <c r="L68" s="4" t="n"/>
-      <c r="M68" s="4" t="n"/>
-      <c r="N68" s="4" t="n"/>
-      <c r="O68" s="4" t="n"/>
-      <c r="P68" s="4" t="n"/>
-      <c r="Q68" s="4" t="n"/>
-    </row>
-    <row r="69">
-      <c r="A69" s="5" t="inlineStr">
-        <is>
-          <t>14 MECANICA E INTERCONEXION</t>
-        </is>
-      </c>
-      <c r="B69" s="5" t="inlineStr">
+      <c r="B68" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="C69" s="5" t="inlineStr">
-        <is>
-          <t>Perfboard</t>
-        </is>
-      </c>
-      <c r="D69" s="5" t="inlineStr">
+      <c r="C68" s="5" t="inlineStr">
+        <is>
+          <t>Cable para puentes</t>
+        </is>
+      </c>
+      <c r="D68" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E69" s="5" t="inlineStr">
-        <is>
-          <t>10 x 15 cm</t>
-        </is>
-      </c>
-      <c r="F69" s="5" t="inlineStr">
-        <is>
-          <t>fibra de vidrio</t>
-        </is>
-      </c>
-      <c r="G69" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="H69" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="I69" s="5">
-        <f>G69*H69</f>
-        <v/>
-      </c>
-      <c r="J69" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="K69" s="5">
-        <f>I69+J69</f>
-        <v/>
-      </c>
-      <c r="L69" s="5" t="inlineStr">
-        <is>
-          <t>placa perforada 10x15</t>
-        </is>
-      </c>
-      <c r="M69" s="6" t="n"/>
-      <c r="N69" s="7" t="n"/>
-      <c r="O69" s="8">
-        <f>IF(N69="","",K69*N69)</f>
-        <v/>
-      </c>
-      <c r="P69" s="6" t="inlineStr">
+      <c r="E68" s="5" t="inlineStr">
+        <is>
+          <t>24 AWG rigido</t>
+        </is>
+      </c>
+      <c r="F68" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G68" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H68" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I68" s="5">
+        <f>G68*H68</f>
+        <v/>
+      </c>
+      <c r="J68" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K68" s="5">
+        <f>I68+J68</f>
+        <v/>
+      </c>
+      <c r="L68" s="5" t="inlineStr">
+        <is>
+          <t>cable rigido 24 AWG</t>
+        </is>
+      </c>
+      <c r="M68" s="6" t="n"/>
+      <c r="N68" s="7" t="n"/>
+      <c r="O68" s="8">
+        <f>IF(N68="","",K68*N68)</f>
+        <v/>
+      </c>
+      <c r="P68" s="6" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="Q69" s="5" t="inlineStr"/>
+      <c r="Q68" s="5" t="inlineStr"/>
     </row>
     <row r="70">
-      <c r="A70" s="5" t="inlineStr">
-        <is>
-          <t>14 MECANICA E INTERCONEXION</t>
-        </is>
-      </c>
-      <c r="B70" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C70" s="5" t="inlineStr">
-        <is>
-          <t>Zocalo DIP-8 (INA)</t>
-        </is>
-      </c>
-      <c r="D70" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E70" s="5" t="inlineStr">
-        <is>
-          <t>DIP-8</t>
-        </is>
-      </c>
-      <c r="F70" s="5" t="inlineStr">
-        <is>
-          <t>zocalo</t>
-        </is>
-      </c>
-      <c r="G70" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H70" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="I70" s="5">
-        <f>G70*H70</f>
-        <v/>
-      </c>
-      <c r="J70" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K70" s="5">
-        <f>I70+J70</f>
-        <v/>
-      </c>
-      <c r="L70" s="5" t="inlineStr">
-        <is>
-          <t>zocalo DIP 8 pines</t>
-        </is>
-      </c>
-      <c r="M70" s="6" t="n"/>
-      <c r="N70" s="7" t="n"/>
-      <c r="O70" s="8">
-        <f>IF(N70="","",K70*N70)</f>
-        <v/>
-      </c>
-      <c r="P70" s="6" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="Q70" s="5" t="inlineStr">
-        <is>
-          <t>Solo si usas el respaldo AD623AN DIP-8</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="5" t="inlineStr">
-        <is>
-          <t>14 MECANICA E INTERCONEXION</t>
-        </is>
-      </c>
-      <c r="B71" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C71" s="5" t="inlineStr">
-        <is>
-          <t>Adaptador SOIC/MSOP-8 a DIP-8</t>
-        </is>
-      </c>
-      <c r="D71" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E71" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F71" s="5" t="inlineStr">
-        <is>
-          <t>PCB adaptador</t>
-        </is>
-      </c>
-      <c r="G71" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H71" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="I71" s="5">
-        <f>G71*H71</f>
-        <v/>
-      </c>
-      <c r="J71" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K71" s="5">
-        <f>I71+J71</f>
-        <v/>
-      </c>
-      <c r="L71" s="5" t="inlineStr">
-        <is>
-          <t>adaptador SOIC8 a DIP8</t>
-        </is>
-      </c>
-      <c r="M71" s="6" t="n"/>
-      <c r="N71" s="7" t="n"/>
-      <c r="O71" s="8">
-        <f>IF(N71="","",K71*N71)</f>
-        <v/>
-      </c>
-      <c r="P71" s="6" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="Q71" s="5" t="inlineStr">
-        <is>
-          <t>Solo si compras el INA333 suelto (SMD)</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="5" t="inlineStr">
-        <is>
-          <t>14 MECANICA E INTERCONEXION</t>
-        </is>
-      </c>
-      <c r="B72" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C72" s="5" t="inlineStr">
-        <is>
-          <t>Tira de headers macho/hembra</t>
-        </is>
-      </c>
-      <c r="D72" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E72" s="5" t="inlineStr">
-        <is>
-          <t>2.54 mm</t>
-        </is>
-      </c>
-      <c r="F72" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G72" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="H72" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="I72" s="5">
-        <f>G72*H72</f>
-        <v/>
-      </c>
-      <c r="J72" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="K72" s="5">
-        <f>I72+J72</f>
-        <v/>
-      </c>
-      <c r="L72" s="5" t="inlineStr">
-        <is>
-          <t>header 2.54mm 40 pines</t>
-        </is>
-      </c>
-      <c r="M72" s="6" t="n"/>
-      <c r="N72" s="7" t="n"/>
-      <c r="O72" s="8">
-        <f>IF(N72="","",K72*N72)</f>
-        <v/>
-      </c>
-      <c r="P72" s="6" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="Q72" s="5" t="inlineStr"/>
-    </row>
-    <row r="73">
-      <c r="A73" s="5" t="inlineStr">
-        <is>
-          <t>14 MECANICA E INTERCONEXION</t>
-        </is>
-      </c>
-      <c r="B73" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C73" s="5" t="inlineStr">
-        <is>
-          <t>Cable para puentes</t>
-        </is>
-      </c>
-      <c r="D73" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E73" s="5" t="inlineStr">
-        <is>
-          <t>24 AWG rigido</t>
-        </is>
-      </c>
-      <c r="F73" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G73" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="H73" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="I73" s="5">
-        <f>G73*H73</f>
-        <v/>
-      </c>
-      <c r="J73" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K73" s="5">
-        <f>I73+J73</f>
-        <v/>
-      </c>
-      <c r="L73" s="5" t="inlineStr">
-        <is>
-          <t>cable rigido 24 AWG</t>
-        </is>
-      </c>
-      <c r="M73" s="6" t="n"/>
-      <c r="N73" s="7" t="n"/>
-      <c r="O73" s="8">
-        <f>IF(N73="","",K73*N73)</f>
-        <v/>
-      </c>
-      <c r="P73" s="6" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="Q73" s="5" t="inlineStr"/>
-    </row>
-    <row r="75">
-      <c r="N75" s="9" t="inlineStr">
+      <c r="N70" s="9" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="O75" s="10">
-        <f>SUM(O5:O73)</f>
+      <c r="O70" s="10">
+        <f>SUM(O5:O68)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:Q73"/>
+  <autoFilter ref="A4:Q68"/>
   <dataValidations count="1">
-    <dataValidation sqref="P6 P7 P9 P10 P11 P13 P14 P15 P17 P18 P19 P22 P23 P24 P25 P28 P29 P30 P33 P34 P35 P38 P39 P40 P43 P44 P47 P48 P49 P50 P53 P54 P55 P56 P58 P59 P60 P61 P62 P63 P65 P66 P67 P69 P70 P71 P72 P73" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="P6 P7 P9 P10 P11 P13 P14 P15 P17 P18 P19 P22 P23 P24 P25 P26 P29 P30 P31 P34 P35 P36 P38 P39 P42 P43 P44 P45 P48 P49 P50 P51 P53 P54 P55 P56 P57 P58 P60 P61 P62 P64 P65 P66 P67 P68" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pendiente,Comprado,No hay,No aplica"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4657,7 +4390,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -4702,15 +4435,15 @@
         </is>
       </c>
       <c r="B4" s="11">
-        <f>COUNTIFS('BoM por modulo'!$A$5:$A$73,A4,'BoM por modulo'!$P$5:$P$73,"&lt;&gt;")</f>
+        <f>COUNTIFS('BoM por modulo'!$A$5:$A$68,A4,'BoM por modulo'!$P$5:$P$68,"&lt;&gt;")</f>
         <v/>
       </c>
       <c r="C4" s="11">
-        <f>COUNTIFS('BoM por modulo'!$A$5:$A$73,A4,'BoM por modulo'!$P$5:$P$73,"Pendiente")</f>
+        <f>COUNTIFS('BoM por modulo'!$A$5:$A$68,A4,'BoM por modulo'!$P$5:$P$68,"Pendiente")</f>
         <v/>
       </c>
       <c r="D4" s="12">
-        <f>SUMIF('BoM por modulo'!$A$5:$A$73,A4,'BoM por modulo'!$O$5:$O$73)</f>
+        <f>SUMIF('BoM por modulo'!$A$5:$A$68,A4,'BoM por modulo'!$O$5:$O$68)</f>
         <v/>
       </c>
     </row>
@@ -4721,15 +4454,15 @@
         </is>
       </c>
       <c r="B5" s="11">
-        <f>COUNTIFS('BoM por modulo'!$A$5:$A$73,A5,'BoM por modulo'!$P$5:$P$73,"&lt;&gt;")</f>
+        <f>COUNTIFS('BoM por modulo'!$A$5:$A$68,A5,'BoM por modulo'!$P$5:$P$68,"&lt;&gt;")</f>
         <v/>
       </c>
       <c r="C5" s="11">
-        <f>COUNTIFS('BoM por modulo'!$A$5:$A$73,A5,'BoM por modulo'!$P$5:$P$73,"Pendiente")</f>
+        <f>COUNTIFS('BoM por modulo'!$A$5:$A$68,A5,'BoM por modulo'!$P$5:$P$68,"Pendiente")</f>
         <v/>
       </c>
       <c r="D5" s="12">
-        <f>SUMIF('BoM por modulo'!$A$5:$A$73,A5,'BoM por modulo'!$O$5:$O$73)</f>
+        <f>SUMIF('BoM por modulo'!$A$5:$A$68,A5,'BoM por modulo'!$O$5:$O$68)</f>
         <v/>
       </c>
     </row>
@@ -4740,15 +4473,15 @@
         </is>
       </c>
       <c r="B6" s="11">
-        <f>COUNTIFS('BoM por modulo'!$A$5:$A$73,A6,'BoM por modulo'!$P$5:$P$73,"&lt;&gt;")</f>
+        <f>COUNTIFS('BoM por modulo'!$A$5:$A$68,A6,'BoM por modulo'!$P$5:$P$68,"&lt;&gt;")</f>
         <v/>
       </c>
       <c r="C6" s="11">
-        <f>COUNTIFS('BoM por modulo'!$A$5:$A$73,A6,'BoM por modulo'!$P$5:$P$73,"Pendiente")</f>
+        <f>COUNTIFS('BoM por modulo'!$A$5:$A$68,A6,'BoM por modulo'!$P$5:$P$68,"Pendiente")</f>
         <v/>
       </c>
       <c r="D6" s="12">
-        <f>SUMIF('BoM por modulo'!$A$5:$A$73,A6,'BoM por modulo'!$O$5:$O$73)</f>
+        <f>SUMIF('BoM por modulo'!$A$5:$A$68,A6,'BoM por modulo'!$O$5:$O$68)</f>
         <v/>
       </c>
     </row>
@@ -4759,229 +4492,210 @@
         </is>
       </c>
       <c r="B7" s="11">
-        <f>COUNTIFS('BoM por modulo'!$A$5:$A$73,A7,'BoM por modulo'!$P$5:$P$73,"&lt;&gt;")</f>
+        <f>COUNTIFS('BoM por modulo'!$A$5:$A$68,A7,'BoM por modulo'!$P$5:$P$68,"&lt;&gt;")</f>
         <v/>
       </c>
       <c r="C7" s="11">
-        <f>COUNTIFS('BoM por modulo'!$A$5:$A$73,A7,'BoM por modulo'!$P$5:$P$73,"Pendiente")</f>
+        <f>COUNTIFS('BoM por modulo'!$A$5:$A$68,A7,'BoM por modulo'!$P$5:$P$68,"Pendiente")</f>
         <v/>
       </c>
       <c r="D7" s="12">
-        <f>SUMIF('BoM por modulo'!$A$5:$A$73,A7,'BoM por modulo'!$O$5:$O$73)</f>
+        <f>SUMIF('BoM por modulo'!$A$5:$A$68,A7,'BoM por modulo'!$O$5:$O$68)</f>
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
         <is>
-          <t>5 G2 = 25</t>
+          <t>5 LPF MFB 500 Hz x25 (Q 0.54)</t>
         </is>
       </c>
       <c r="B8" s="11">
-        <f>COUNTIFS('BoM por modulo'!$A$5:$A$73,A8,'BoM por modulo'!$P$5:$P$73,"&lt;&gt;")</f>
+        <f>COUNTIFS('BoM por modulo'!$A$5:$A$68,A8,'BoM por modulo'!$P$5:$P$68,"&lt;&gt;")</f>
         <v/>
       </c>
       <c r="C8" s="11">
-        <f>COUNTIFS('BoM por modulo'!$A$5:$A$73,A8,'BoM por modulo'!$P$5:$P$73,"Pendiente")</f>
+        <f>COUNTIFS('BoM por modulo'!$A$5:$A$68,A8,'BoM por modulo'!$P$5:$P$68,"Pendiente")</f>
         <v/>
       </c>
       <c r="D8" s="12">
-        <f>SUMIF('BoM por modulo'!$A$5:$A$73,A8,'BoM por modulo'!$O$5:$O$73)</f>
+        <f>SUMIF('BoM por modulo'!$A$5:$A$68,A8,'BoM por modulo'!$O$5:$O$68)</f>
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="11" t="inlineStr">
         <is>
-          <t>6 LPF A 500 Hz (Q 0.541)</t>
+          <t>6 LPF Sallen-Key 500 Hz (Q 1.31)</t>
         </is>
       </c>
       <c r="B9" s="11">
-        <f>COUNTIFS('BoM por modulo'!$A$5:$A$73,A9,'BoM por modulo'!$P$5:$P$73,"&lt;&gt;")</f>
+        <f>COUNTIFS('BoM por modulo'!$A$5:$A$68,A9,'BoM por modulo'!$P$5:$P$68,"&lt;&gt;")</f>
         <v/>
       </c>
       <c r="C9" s="11">
-        <f>COUNTIFS('BoM por modulo'!$A$5:$A$73,A9,'BoM por modulo'!$P$5:$P$73,"Pendiente")</f>
+        <f>COUNTIFS('BoM por modulo'!$A$5:$A$68,A9,'BoM por modulo'!$P$5:$P$68,"Pendiente")</f>
         <v/>
       </c>
       <c r="D9" s="12">
-        <f>SUMIF('BoM por modulo'!$A$5:$A$73,A9,'BoM por modulo'!$O$5:$O$73)</f>
+        <f>SUMIF('BoM por modulo'!$A$5:$A$68,A9,'BoM por modulo'!$O$5:$O$68)</f>
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>7 LPF B 500 Hz (Q 1.306)</t>
+          <t>7 BUCKET + SALIDA AL ADC</t>
         </is>
       </c>
       <c r="B10" s="11">
-        <f>COUNTIFS('BoM por modulo'!$A$5:$A$73,A10,'BoM por modulo'!$P$5:$P$73,"&lt;&gt;")</f>
+        <f>COUNTIFS('BoM por modulo'!$A$5:$A$68,A10,'BoM por modulo'!$P$5:$P$68,"&lt;&gt;")</f>
         <v/>
       </c>
       <c r="C10" s="11">
-        <f>COUNTIFS('BoM por modulo'!$A$5:$A$73,A10,'BoM por modulo'!$P$5:$P$73,"Pendiente")</f>
+        <f>COUNTIFS('BoM por modulo'!$A$5:$A$68,A10,'BoM por modulo'!$P$5:$P$68,"Pendiente")</f>
         <v/>
       </c>
       <c r="D10" s="12">
-        <f>SUMIF('BoM por modulo'!$A$5:$A$73,A10,'BoM por modulo'!$O$5:$O$73)</f>
+        <f>SUMIF('BoM por modulo'!$A$5:$A$68,A10,'BoM por modulo'!$O$5:$O$68)</f>
         <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="11" t="inlineStr">
         <is>
-          <t>8 BUFFER + SALIDA AL ADC</t>
+          <t>9 VREF 1.65 V (compartido)</t>
         </is>
       </c>
       <c r="B11" s="11">
-        <f>COUNTIFS('BoM por modulo'!$A$5:$A$73,A11,'BoM por modulo'!$P$5:$P$73,"&lt;&gt;")</f>
+        <f>COUNTIFS('BoM por modulo'!$A$5:$A$68,A11,'BoM por modulo'!$P$5:$P$68,"&lt;&gt;")</f>
         <v/>
       </c>
       <c r="C11" s="11">
-        <f>COUNTIFS('BoM por modulo'!$A$5:$A$73,A11,'BoM por modulo'!$P$5:$P$73,"Pendiente")</f>
+        <f>COUNTIFS('BoM por modulo'!$A$5:$A$68,A11,'BoM por modulo'!$P$5:$P$68,"Pendiente")</f>
         <v/>
       </c>
       <c r="D11" s="12">
-        <f>SUMIF('BoM por modulo'!$A$5:$A$73,A11,'BoM por modulo'!$O$5:$O$73)</f>
+        <f>SUMIF('BoM por modulo'!$A$5:$A$68,A11,'BoM por modulo'!$O$5:$O$68)</f>
         <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>9 VREF 1.65 V (compartido)</t>
+          <t>10 RLD (compartido)</t>
         </is>
       </c>
       <c r="B12" s="11">
-        <f>COUNTIFS('BoM por modulo'!$A$5:$A$73,A12,'BoM por modulo'!$P$5:$P$73,"&lt;&gt;")</f>
+        <f>COUNTIFS('BoM por modulo'!$A$5:$A$68,A12,'BoM por modulo'!$P$5:$P$68,"&lt;&gt;")</f>
         <v/>
       </c>
       <c r="C12" s="11">
-        <f>COUNTIFS('BoM por modulo'!$A$5:$A$73,A12,'BoM por modulo'!$P$5:$P$73,"Pendiente")</f>
+        <f>COUNTIFS('BoM por modulo'!$A$5:$A$68,A12,'BoM por modulo'!$P$5:$P$68,"Pendiente")</f>
         <v/>
       </c>
       <c r="D12" s="12">
-        <f>SUMIF('BoM por modulo'!$A$5:$A$73,A12,'BoM por modulo'!$O$5:$O$73)</f>
+        <f>SUMIF('BoM por modulo'!$A$5:$A$68,A12,'BoM por modulo'!$O$5:$O$68)</f>
         <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="11" t="inlineStr">
         <is>
-          <t>10 RLD (compartido)</t>
+          <t>11 OP-AMPS (paquetes)</t>
         </is>
       </c>
       <c r="B13" s="11">
-        <f>COUNTIFS('BoM por modulo'!$A$5:$A$73,A13,'BoM por modulo'!$P$5:$P$73,"&lt;&gt;")</f>
+        <f>COUNTIFS('BoM por modulo'!$A$5:$A$68,A13,'BoM por modulo'!$P$5:$P$68,"&lt;&gt;")</f>
         <v/>
       </c>
       <c r="C13" s="11">
-        <f>COUNTIFS('BoM por modulo'!$A$5:$A$73,A13,'BoM por modulo'!$P$5:$P$73,"Pendiente")</f>
+        <f>COUNTIFS('BoM por modulo'!$A$5:$A$68,A13,'BoM por modulo'!$P$5:$P$68,"Pendiente")</f>
         <v/>
       </c>
       <c r="D13" s="12">
-        <f>SUMIF('BoM por modulo'!$A$5:$A$73,A13,'BoM por modulo'!$O$5:$O$73)</f>
+        <f>SUMIF('BoM por modulo'!$A$5:$A$68,A13,'BoM por modulo'!$O$5:$O$68)</f>
         <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="11" t="inlineStr">
         <is>
-          <t>11 OP-AMPS (paquetes)</t>
+          <t>12 ALIMENTACION (a bateria)</t>
         </is>
       </c>
       <c r="B14" s="11">
-        <f>COUNTIFS('BoM por modulo'!$A$5:$A$73,A14,'BoM por modulo'!$P$5:$P$73,"&lt;&gt;")</f>
+        <f>COUNTIFS('BoM por modulo'!$A$5:$A$68,A14,'BoM por modulo'!$P$5:$P$68,"&lt;&gt;")</f>
         <v/>
       </c>
       <c r="C14" s="11">
-        <f>COUNTIFS('BoM por modulo'!$A$5:$A$73,A14,'BoM por modulo'!$P$5:$P$73,"Pendiente")</f>
+        <f>COUNTIFS('BoM por modulo'!$A$5:$A$68,A14,'BoM por modulo'!$P$5:$P$68,"Pendiente")</f>
         <v/>
       </c>
       <c r="D14" s="12">
-        <f>SUMIF('BoM por modulo'!$A$5:$A$73,A14,'BoM por modulo'!$O$5:$O$73)</f>
+        <f>SUMIF('BoM por modulo'!$A$5:$A$68,A14,'BoM por modulo'!$O$5:$O$68)</f>
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="11" t="inlineStr">
         <is>
-          <t>12 ALIMENTACION (a bateria)</t>
+          <t>13 ELECTRODOS Y CABLES</t>
         </is>
       </c>
       <c r="B15" s="11">
-        <f>COUNTIFS('BoM por modulo'!$A$5:$A$73,A15,'BoM por modulo'!$P$5:$P$73,"&lt;&gt;")</f>
+        <f>COUNTIFS('BoM por modulo'!$A$5:$A$68,A15,'BoM por modulo'!$P$5:$P$68,"&lt;&gt;")</f>
         <v/>
       </c>
       <c r="C15" s="11">
-        <f>COUNTIFS('BoM por modulo'!$A$5:$A$73,A15,'BoM por modulo'!$P$5:$P$73,"Pendiente")</f>
+        <f>COUNTIFS('BoM por modulo'!$A$5:$A$68,A15,'BoM por modulo'!$P$5:$P$68,"Pendiente")</f>
         <v/>
       </c>
       <c r="D15" s="12">
-        <f>SUMIF('BoM por modulo'!$A$5:$A$73,A15,'BoM por modulo'!$O$5:$O$73)</f>
+        <f>SUMIF('BoM por modulo'!$A$5:$A$68,A15,'BoM por modulo'!$O$5:$O$68)</f>
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="11" t="inlineStr">
         <is>
-          <t>13 ELECTRODOS Y CABLES</t>
+          <t>14 MECANICA E INTERCONEXION</t>
         </is>
       </c>
       <c r="B16" s="11">
-        <f>COUNTIFS('BoM por modulo'!$A$5:$A$73,A16,'BoM por modulo'!$P$5:$P$73,"&lt;&gt;")</f>
+        <f>COUNTIFS('BoM por modulo'!$A$5:$A$68,A16,'BoM por modulo'!$P$5:$P$68,"&lt;&gt;")</f>
         <v/>
       </c>
       <c r="C16" s="11">
-        <f>COUNTIFS('BoM por modulo'!$A$5:$A$73,A16,'BoM por modulo'!$P$5:$P$73,"Pendiente")</f>
+        <f>COUNTIFS('BoM por modulo'!$A$5:$A$68,A16,'BoM por modulo'!$P$5:$P$68,"Pendiente")</f>
         <v/>
       </c>
       <c r="D16" s="12">
-        <f>SUMIF('BoM por modulo'!$A$5:$A$73,A16,'BoM por modulo'!$O$5:$O$73)</f>
+        <f>SUMIF('BoM por modulo'!$A$5:$A$68,A16,'BoM por modulo'!$O$5:$O$68)</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="11" t="inlineStr">
-        <is>
-          <t>14 MECANICA E INTERCONEXION</t>
-        </is>
-      </c>
-      <c r="B17" s="11">
-        <f>COUNTIFS('BoM por modulo'!$A$5:$A$73,A17,'BoM por modulo'!$P$5:$P$73,"&lt;&gt;")</f>
-        <v/>
-      </c>
-      <c r="C17" s="11">
-        <f>COUNTIFS('BoM por modulo'!$A$5:$A$73,A17,'BoM por modulo'!$P$5:$P$73,"Pendiente")</f>
-        <v/>
-      </c>
-      <c r="D17" s="12">
-        <f>SUMIF('BoM por modulo'!$A$5:$A$73,A17,'BoM por modulo'!$O$5:$O$73)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="13" t="inlineStr">
+      <c r="A17" s="13" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B18" s="13">
-        <f>SUM(B4:B17)</f>
-        <v/>
-      </c>
-      <c r="C18" s="13">
-        <f>SUM(C4:C17)</f>
-        <v/>
-      </c>
-      <c r="D18" s="14">
-        <f>SUM(D4:D17)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+      <c r="B17" s="13">
+        <f>SUM(B4:B16)</f>
+        <v/>
+      </c>
+      <c r="C17" s="13">
+        <f>SUM(C4:C16)</f>
+        <v/>
+      </c>
+      <c r="D17" s="14">
+        <f>SUM(D4:D16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>El total solo suma las filas con precio. Llena el precio en la hoja BoM por modulo.</t>
         </is>

</xml_diff>

<commit_message>
BoM: adaptadores SOP8/TSSOP8 doble cara, Cm0 ceramico o bipolar, aviso del terminal del cable de electrodo
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V5Cz1Wb6HSRhqzouEW9mso
</commit_message>
<xml_diff>
--- a/docs/afe-emg/BoM_AFE_AuraVox.xlsx
+++ b/docs/afe-emg/BoM_AFE_AuraVox.xlsx
@@ -1606,7 +1606,7 @@
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>ceramico X7R o electrolitico 16 V</t>
+          <t>ceramico X7R 16 V o electrolitico BIPOLAR (NP)</t>
         </is>
       </c>
       <c r="G22" s="5" t="n">
@@ -1628,7 +1628,7 @@
       </c>
       <c r="L22" s="5" t="inlineStr">
         <is>
-          <t>condensador 10uF</t>
+          <t>condensador ceramico 10uF X7R / electrolitico bipolar 10uF</t>
         </is>
       </c>
       <c r="M22" s="6" t="n"/>
@@ -1644,7 +1644,7 @@
       </c>
       <c r="Q22" s="5" t="inlineStr">
         <is>
-          <t>Sin el, la corriente de polarizacion del TS922 por Ra (110k) x 25 deja +0.3 V de offset</t>
+          <t>NO usar electrolitico polarizado: ambos lados quedan en ~1.65 V y la senal lo invierte. Sin Cm0, Ib del TS922 x Ra (110k) x G2 desplaza la salida</t>
         </is>
       </c>
     </row>
@@ -3204,7 +3204,7 @@
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>Adaptador SOIC-8 a DIP-8</t>
+          <t>Adaptador SOP8/TSSOP8 a DIP8 doble cara (SOIC-8 1.27 mm + MSOP/TSSOP-8 0.65 mm)</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
@@ -3214,12 +3214,12 @@
       </c>
       <c r="E50" s="5" t="inlineStr">
         <is>
-          <t>SOIC8 a DIP8</t>
+          <t>SOP8/TSSOP8 a DIP8</t>
         </is>
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>PCB adaptador</t>
+          <t>PCB adaptador doble cara</t>
         </is>
       </c>
       <c r="G50" s="5" t="n">
@@ -3233,7 +3233,7 @@
         <v/>
       </c>
       <c r="J50" s="5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K50" s="5">
         <f>I50+J50</f>
@@ -3241,7 +3241,7 @@
       </c>
       <c r="L50" s="5" t="inlineStr">
         <is>
-          <t>adaptador SOIC8 a DIP8</t>
+          <t>adaptador SOP8 TSSOP8 a DIP8</t>
         </is>
       </c>
       <c r="M50" s="6" t="n"/>
@@ -3257,7 +3257,7 @@
       </c>
       <c r="Q50" s="5" t="inlineStr">
         <is>
-          <t>Soldar el TS922 al adaptador y probarlo antes de montarlo</t>
+          <t>Cara SOIC-8: TS922. Cara MSOP-8: INA333 si hay que desoldarlo del modulo (3 extra). Soldar con flux y probar antes de montar</t>
         </is>
       </c>
     </row>
@@ -3921,7 +3921,7 @@
       </c>
       <c r="L61" s="5" t="inlineStr">
         <is>
-          <t>cable electrodo broche snap</t>
+          <t>cable electrodo snap 4 mm / cable ECG broche</t>
         </is>
       </c>
       <c r="M61" s="6" t="n"/>
@@ -3937,7 +3937,7 @@
       </c>
       <c r="Q61" s="5" t="inlineStr">
         <is>
-          <t>Uno por electrodo; trenzar los dos de cada par</t>
+          <t>Uno por electrodo; trenzar los dos de cada par. REVISAR EL TERMINAL antes de comprar: debe calzar en header hembra 2.54 mm. Si termina en DIN 1.5 mm touchproof (DIN 42802), cortar y crimpar terminal Dupont hembra o comprar bases touchproof. Alternativa: cable de 3 electrodos con jack 3.5 mm (el de los kits AD8232) + jack hembra 3.5 mm TRS en la placa</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
BoM: Cm1 (100n+47n poliester), C21 15n poliester y 1 uF MLCC del LDO, por agregar en Global
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V5Cz1Wb6HSRhqzouEW9mso
</commit_message>
<xml_diff>
--- a/docs/afe-emg/BoM_AFE_AuraVox.xlsx
+++ b/docs/afe-emg/BoM_AFE_AuraVox.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="801" uniqueCount="449">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="807" uniqueCount="457">
   <si>
     <t xml:space="preserve">BoM AFE sEMG AuraVox: 3 canales (submentoniano, labio inferior, laringe), 7 electrodos, RLD. Ordenada por modulo, igual que los recuadros del esquematico LTspice (sim/ltspice).</t>
   </si>
@@ -430,435 +430,450 @@
     <t xml:space="preserve">condensador poliester 150nF</t>
   </si>
   <si>
+    <t xml:space="preserve">2A104K poliester 100nF 100V + 2A473J poliester 47nF 100V, en paralelo (par)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Pendiente</t>
   </si>
   <si>
+    <t xml:space="preserve">AGREGAR AL CARRITO DE GLOBAL. No hay 150 nF en Global: 100n + 47n en paralelo = 147 nF (f0 +1 %, Q -1 %). Precio = el par ($70 + $60)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cm2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Condensador de realimentacion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1n</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ceramico C0G/NP0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">condensador ceramico 1nF NP0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RPE110X7R102K050V MLCC X7R 1nF 50V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">X7R en vez de C0G: aceptado para la demo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">XMF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6 LPF Sallen-Key 500 Hz (Q 1.31)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rlb1, Rlb2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resistencia del LPF B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">54.9k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Con 56k: f0 = 495 Hz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15n</t>
+  </si>
+  <si>
+    <t xml:space="preserve">poliester 5 % o C0G</t>
+  </si>
+  <si>
+    <t xml:space="preserve">condensador poliester 15nF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2A153J poliester 15nF 100V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AGREGAR AL CARRITO DE GLOBAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.2n</t>
+  </si>
+  <si>
+    <t xml:space="preserve">condensador poliester 2.2nF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C222NPO05D disco NPO 2.2nF 50V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">XLB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7 BUCKET + SALIDA AL ADC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rbk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resistencia del bucket</t>
+  </si>
+  <si>
+    <t xml:space="preserve">100</t>
+  </si>
+  <si>
+    <t xml:space="preserve">resistencia 100 ohm 1%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R1W100 carbon 1 W 100 ohm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cbk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Condensador del bucket</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ADCk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cable a Arduino A1..A3 del STM32N6570-DK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">jumper Dupont M-H</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cable dupont macho-hembra (tira de 40)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FALTA EN EL CARRITO. CH1-A1 (PA9), CH2-A2 (PA10), CH3-A3 (PA12). Mas 1 cable de GND. A0 no: comparte ADC con USB1 ISENSE (UM3300)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8 VREF 1.65 V (compartido)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">compartido</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RA1, RA2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Divisor de VREF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">resistencia 100k 1%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Condensador del divisor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ceramico X7R o electrolitico</t>
+  </si>
+  <si>
+    <t xml:space="preserve">condensador 10uF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">XVR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9 RLD (compartido)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RSM1..RSM3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sensado de modo comun (punto medio de RG)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">604k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">620k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">resistencia 620k 1%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">291-620K carbon 1/4 W 5 %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CINT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Condensador del integrador</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Si oscila en banco: 2.2n</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RPAR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resistencia en paralelo al integrador</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pelicula 5 %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">resistencia 10M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">291-10M carbon 1/4 W 5 %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RLIM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resistencia de seguridad al electrodo RLD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">390k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">resistencia 390k 1%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">293-390K carbon 1/2 W 5 %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Limita la corriente al paciente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">XRLD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10 OP-AMPS (paquetes)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">XHP, XMF, XLB x3, XRLD, XVR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Op-amp doble TS922AIYDT (Global 001-TS922)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TS922</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TS922AIYDT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SOIC-8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11 secciones = 3 por canal x 3 + RLD + VREF (1 libre). Solo habia 6 en stock</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adaptador SOIC-8 a DIP-8 (S08D8, Global; trae PCB y 2 headers de 4)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S08D8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PCB adaptador</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S08D8 adaptador SOIC 8 a DIP 8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">En el carrito hay 12; bastan 7 (sobran 5 = $1.250). Solo para los TS922 (SOIC-8, 1.27 mm). NO sirve para el TLV757 (SOT-23) ni para el INA333 (MSOP). Soldar con flux y probar antes de montar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zocalo DIP-8 (opcional)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DIP-8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">zocalo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">zocalo DIP 8 pines</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Opcional: soldar los pines del S08D8 directo a la perfboard, o usar tira hembra 2.54 como zocalo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Desacople de cada op-amp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11 ALIMENTACION (5 V USB / powerbank -&gt; 3.3 V)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">XLDO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Regulador LDO 3.3 V TLV75733PDBVR (Global 014-75733)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TLV75733P</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TLV75733PDBVR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SOT-23-5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entrada 5 V desde el pin +5V del STM32N6570-DK (Arduino CN8). EN unido a IN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Montaje del TLV757 sin adaptador (dead bug)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pegado boca arriba en la perfboard, hilo fino a cada pata. Pines: 1 IN, 2 GND, 3 EN (a IN), 4 NC, 5 OUT. El SOT23S3 de Global es de 3 pines: no sirve</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CLDOI, CLDOO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Condensadores del LDO (entrada y salida)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1u</t>
+  </si>
+  <si>
+    <t xml:space="preserve">condensador ceramico 1uF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CE50102 electrolitico 1uF 50V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ver la fila CLDOO cer.: a la salida hace falta ademas un ceramico. Pegados a los pines del LDO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CLDOO cer.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Condensador ceramico de salida del LDO (en paralelo con el electrolitico)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1u X7R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MLCC X7R 16 V o mas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MLCC THD 1uF X7R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CM105 MLCC THD 1uF 50V X7R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AGREGAR AL CARRITO DE GLOBAL. El TLV757 esta pensado para ceramico a la salida (&gt;= 0.47 uF efectivos); un electrolitico solo puede oscilar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CBULK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Condensador bulk del riel 3.3 V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ceramico o electrolitico</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cable 5 V y GND desde el DK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cable dupont macho-hembra</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FALTA EN EL CARRITO. Usar powerbank o PC a bateria mientras haya electrodos puestos (ver Notas de seguridad)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12 ELECTRODOS Y CONECTORES (7)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">XE1P..XE3N, XER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Electrodo Ag/AgCl con broche 4 mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Skintact FS-RG1/10 32x41</t>
+  </si>
+  <si>
+    <t xml:space="preserve">desechable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Skintact FS-RG1/10 / Kendall Arbo H124SG 24 mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FALTA EN EL CARRITO. 7 por sesion (6 de senal + 1 RLD); caja de 50. Skintact para CH1, CH3 y RLD. CH2: Arbo H124SG (24 mm) o par sobre el menton. ISIMED 55x55 solo como RLD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cable de electrodo con broche (snap) 4 mm, idealmente apantallado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">broche 4 mm a pin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cable electrodo snap 4 mm / cable ECG broche</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FALTA EN EL CARRITO. Uno por electrodo; trenzar los dos de cada par. REVISAR EL TERMINAL antes de comprar: debe calzar en header hembra 2.54 mm. Si termina en DIN 1.5 mm touchproof (DIN 42802), cortar y crimpar terminal Dupont hembra o comprar bases touchproof. Alternativa: cable de 3 electrodos con jack 3.5 mm (el de los kits AD8232) + jack hembra 3.5 mm TRS en la placa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Conector de la placa para los 7 electrodos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hembra 2x8 2.54 THT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1105-8X2 conector hembra doble fila 16 vias</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1105-8X2 hembra doble fila 16 vias 2.54</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Una fila: CH1+ CH1- CH2+ CH2- CH3+ CH3- RLD GND(malla). Se enchufa el bus Dupont macho</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bus de 8 cables Dupont macho (separado de una tira de 40)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">jumper Dupont M-M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cable dupont macho-macho 20 cm tira 40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FALTA EN EL CARRITO. Lado macho al conector 2x8; el otro extremo se une a los cables de electrodo (soldado + termorretractil o enchufado)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alcohol isopropilico / gel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">alcohol isopropilico</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FALTA EN EL CARRITO. Preparar la piel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13 MECANICA E INTERCONEXION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Perfboard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10 x 15 cm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fibra de vidrio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">placa perforada 10x15</t>
+  </si>
+  <si>
     <t xml:space="preserve">FALTA EN EL CARRITO</t>
   </si>
   <si>
-    <t xml:space="preserve">Cm2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Condensador de realimentacion</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1n</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ceramico C0G/NP0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">condensador ceramico 1nF NP0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RPE110X7R102K050V MLCC X7R 1nF 50V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">X7R en vez de C0G: aceptado para la demo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">XMF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6 LPF Sallen-Key 500 Hz (Q 1.31)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rlb1, Rlb2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Resistencia del LPF B</t>
-  </si>
-  <si>
-    <t xml:space="preserve">54.9k</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Con 56k: f0 = 495 Hz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C21</t>
-  </si>
-  <si>
-    <t xml:space="preserve">15n</t>
-  </si>
-  <si>
-    <t xml:space="preserve">poliester 5 % o C0G</t>
-  </si>
-  <si>
-    <t xml:space="preserve">condensador poliester 15nF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C22</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.2n</t>
-  </si>
-  <si>
-    <t xml:space="preserve">condensador poliester 2.2nF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C222NPO05D disco NPO 2.2nF 50V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">XLB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7 BUCKET + SALIDA AL ADC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rbk</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Resistencia del bucket</t>
-  </si>
-  <si>
-    <t xml:space="preserve">100</t>
-  </si>
-  <si>
-    <t xml:space="preserve">resistencia 100 ohm 1%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R1W100 carbon 1 W 100 ohm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cbk</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Condensador del bucket</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ADCk</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cable a Arduino A1..A3 del STM32N6570-DK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">jumper Dupont M-H</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cable dupont macho-hembra (tira de 40)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FALTA EN EL CARRITO. CH1-A1 (PA9), CH2-A2 (PA10), CH3-A3 (PA12). Mas 1 cable de GND. A0 no: comparte ADC con USB1 ISENSE (UM3300)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8 VREF 1.65 V (compartido)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">compartido</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RA1, RA2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Divisor de VREF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">resistencia 100k 1%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Condensador del divisor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ceramico X7R o electrolitico</t>
-  </si>
-  <si>
-    <t xml:space="preserve">condensador 10uF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">XVR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9 RLD (compartido)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RSM1..RSM3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sensado de modo comun (punto medio de RG)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">604k</t>
-  </si>
-  <si>
-    <t xml:space="preserve">620k</t>
-  </si>
-  <si>
-    <t xml:space="preserve">resistencia 620k 1%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">291-620K carbon 1/4 W 5 %</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CINT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Condensador del integrador</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Si oscila en banco: 2.2n</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RPAR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Resistencia en paralelo al integrador</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10M</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pelicula 5 %</t>
-  </si>
-  <si>
-    <t xml:space="preserve">resistencia 10M</t>
-  </si>
-  <si>
-    <t xml:space="preserve">291-10M carbon 1/4 W 5 %</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RLIM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Resistencia de seguridad al electrodo RLD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">390k</t>
-  </si>
-  <si>
-    <t xml:space="preserve">resistencia 390k 1%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">293-390K carbon 1/2 W 5 %</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Limita la corriente al paciente</t>
-  </si>
-  <si>
-    <t xml:space="preserve">XRLD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10 OP-AMPS (paquetes)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">XHP, XMF, XLB x3, XRLD, XVR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Op-amp doble TS922AIYDT (Global 001-TS922)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TS922</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TS922AIYDT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SOIC-8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">11 secciones = 3 por canal x 3 + RLD + VREF (1 libre). Solo habia 6 en stock</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Adaptador SOIC-8 a DIP-8 (S08D8, Global; trae PCB y 2 headers de 4)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S08D8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PCB adaptador</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S08D8 adaptador SOIC 8 a DIP 8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">En el carrito hay 12; bastan 7 (sobran 5 = $1.250). Solo para los TS922 (SOIC-8, 1.27 mm). NO sirve para el TLV757 (SOT-23) ni para el INA333 (MSOP). Soldar con flux y probar antes de montar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Zocalo DIP-8 (opcional)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DIP-8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">zocalo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">zocalo DIP 8 pines</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Opcional: soldar los pines del S08D8 directo a la perfboard, o usar tira hembra 2.54 como zocalo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Desacople de cada op-amp</t>
-  </si>
-  <si>
-    <t xml:space="preserve">11 ALIMENTACION (5 V USB / powerbank -&gt; 3.3 V)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">XLDO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Regulador LDO 3.3 V TLV75733PDBVR (Global 014-75733)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TLV75733P</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TLV75733PDBVR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SOT-23-5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Entrada 5 V desde el pin +5V del STM32N6570-DK (Arduino CN8). EN unido a IN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Montaje del TLV757 sin adaptador (dead bug)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pegado boca arriba en la perfboard, hilo fino a cada pata. Pines: 1 IN, 2 GND, 3 EN (a IN), 4 NC, 5 OUT. El SOT23S3 de Global es de 3 pines: no sirve</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CLDOI, CLDOO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Condensadores del LDO (entrada y salida)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1u</t>
-  </si>
-  <si>
-    <t xml:space="preserve">condensador ceramico 1uF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CE50102 electrolitico 1uF 50V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ver la fila CLDOO cer.: a la salida hace falta ademas un ceramico. Pegados a los pines del LDO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CLDOO cer.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Condensador ceramico de salida del LDO (en paralelo con el electrolitico)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1u X7R</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MLCC X7R 16 V o mas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MLCC THD 1uF X7R</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FALTA EN EL CARRITO. El TLV757 esta pensado para ceramico a la salida (&gt;= 0.47 uF efectivos); un electrolitico solo puede oscilar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBULK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Condensador bulk del riel 3.3 V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ceramico o electrolitico</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cable 5 V y GND desde el DK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cable dupont macho-hembra</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FALTA EN EL CARRITO. Usar powerbank o PC a bateria mientras haya electrodos puestos (ver Notas de seguridad)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">12 ELECTRODOS Y CONECTORES (7)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">XE1P..XE3N, XER</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Electrodo Ag/AgCl con broche 4 mm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Skintact FS-RG1/10 32x41</t>
-  </si>
-  <si>
-    <t xml:space="preserve">desechable</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Skintact FS-RG1/10 / Kendall Arbo H124SG 24 mm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FALTA EN EL CARRITO. 7 por sesion (6 de senal + 1 RLD); caja de 50. Skintact para CH1, CH3 y RLD. CH2: Arbo H124SG (24 mm) o par sobre el menton. ISIMED 55x55 solo como RLD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cable de electrodo con broche (snap) 4 mm, idealmente apantallado</t>
-  </si>
-  <si>
-    <t xml:space="preserve">broche 4 mm a pin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cable electrodo snap 4 mm / cable ECG broche</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FALTA EN EL CARRITO. Uno por electrodo; trenzar los dos de cada par. REVISAR EL TERMINAL antes de comprar: debe calzar en header hembra 2.54 mm. Si termina en DIN 1.5 mm touchproof (DIN 42802), cortar y crimpar terminal Dupont hembra o comprar bases touchproof. Alternativa: cable de 3 electrodos con jack 3.5 mm (el de los kits AD8232) + jack hembra 3.5 mm TRS en la placa</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Conector de la placa para los 7 electrodos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">hembra 2x8 2.54 THT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1105-8X2 conector hembra doble fila 16 vias</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1105-8X2 hembra doble fila 16 vias 2.54</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Una fila: CH1+ CH1- CH2+ CH2- CH3+ CH3- RLD GND(malla). Se enchufa el bus Dupont macho</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bus de 8 cables Dupont macho (separado de una tira de 40)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">jumper Dupont M-M</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cable dupont macho-macho 20 cm tira 40</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FALTA EN EL CARRITO. Lado macho al conector 2x8; el otro extremo se une a los cables de electrodo (soldado + termorretractil o enchufado)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alcohol isopropilico / gel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">alcohol isopropilico</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FALTA EN EL CARRITO. Preparar la piel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">13 MECANICA E INTERCONEXION</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Perfboard</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10 x 15 cm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fibra de vidrio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">placa perforada 10x15</t>
-  </si>
-  <si>
     <t xml:space="preserve">Tira de headers 1x40 2.54 THT (1 macho + 1 hembra)</t>
   </si>
   <si>
@@ -901,10 +916,10 @@
     <t xml:space="preserve">modulo microfono INMP441</t>
   </si>
   <si>
-    <t xml:space="preserve">INMP411 sensor microfono omnidireccional (pagina 5044)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VERIFICAR: el titulo dice INMP411. Debe ser el INMP441 I2S (pines SCK, WS, SD, L/R). El INMP411 es otro microfono, de salida analogica, y no sirve para el SAI. A SAI/I2S del STM32N6570-DK (pines por definir en CubeMX). Alternativa sin cableado: microfono MEMS PDM que trae el DK (U13)</t>
+    <t xml:space="preserve">INMP441 sensor microfono omnidireccional (pagina 5044)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A SAI/I2S del STM32N6570-DK (pines por definir en CubeMX). Alternativa sin cableado: microfono MEMS PDM que trae el DK (U13)</t>
   </si>
   <si>
     <t xml:space="preserve">Cables Dupont para el microfono</t>
@@ -925,7 +940,10 @@
     <t xml:space="preserve">Pendientes</t>
   </si>
   <si>
-    <t xml:space="preserve">Subtotal en carrito (CLP)</t>
+    <t xml:space="preserve">En carrito (CLP)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Por agregar (CLP)</t>
   </si>
   <si>
     <t xml:space="preserve">Faltan en los carritos</t>
@@ -934,15 +952,24 @@
     <t xml:space="preserve">4 x 150n  Condensador a GND</t>
   </si>
   <si>
+    <t xml:space="preserve">Global: 2A104K poliester 100nF 100V + 2A473J poliester 47nF 100V, en paralelo (par)</t>
+  </si>
+  <si>
     <t xml:space="preserve">4 x 15n  Condensador de realimentacion</t>
   </si>
   <si>
+    <t xml:space="preserve">Global: 2A153J poliester 15nF 100V</t>
+  </si>
+  <si>
     <t xml:space="preserve">5 x jumper Dupont M-H  Cable a Arduino A1..A3 del STM32N6570-DK</t>
   </si>
   <si>
     <t xml:space="preserve">2 x 1u X7R  Condensador ceramico de salida del LDO (en paralelo con el electrolitico)</t>
   </si>
   <si>
+    <t xml:space="preserve">Global: CM105 MLCC THD 1uF 50V X7R</t>
+  </si>
+  <si>
     <t xml:space="preserve">3 x jumper Dupont M-H  Cable 5 V y GND desde el DK</t>
   </si>
   <si>
@@ -970,13 +997,10 @@
     <t xml:space="preserve">Avisos de la compra</t>
   </si>
   <si>
-    <t xml:space="preserve">FALTAN en los carritos: Cm1 150 nF x4 (MFB) y C21 15 nF x4 (LPF Sallen-Key). Sin ellos el canal no funciona.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FALTAN: 1 uF ceramico X7R x2 para la salida del LDO; electrodos, cables de electrodo, jumpers Dupont (tira M-H y tira M-M), perfboard, tiras de header 1x40 y alcohol.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VERIFICAR el microfono: el carrito dice INMP411; el diseno usa el INMP441 (I2S).</t>
+    <t xml:space="preserve">AGREGAR al carrito de Global: 4 x 2A104K (100n poliester) + 4 x 2A473J (47n poliester) para Cm1 (100n + 47n en paralelo = 147 nF); 4 x 2A153J (15n poliester) para C21; 2 x CM105 (1 uF MLCC X7R) para la salida del LDO.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pendiente (otra tienda): electrodos, cables de electrodo, jumpers Dupont (tira M-H y tira M-M), perfboard, tiras de header 1x40 y alcohol.</t>
   </si>
   <si>
     <t xml:space="preserve">Resistencias de carbon 5 % en vez de pelicula metalica 1 %: aceptado para la demo (ganancia por canal +-7 %, se normaliza en firmware). Para produccion: 1 %.</t>
@@ -3169,19 +3193,27 @@
       <c r="L26" s="5" t="s">
         <v>133</v>
       </c>
-      <c r="M26" s="6"/>
-      <c r="N26" s="6"/>
-      <c r="O26" s="6"/>
-      <c r="P26" s="7"/>
-      <c r="Q26" s="8" t="str">
+      <c r="M26" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="N26" s="6" t="s">
+        <v>134</v>
+      </c>
+      <c r="O26" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="P26" s="7" t="n">
+        <v>130</v>
+      </c>
+      <c r="Q26" s="8" t="n">
         <f aca="false">IF(P26="","",IF(O26="",K26,O26)*P26)</f>
-        <v/>
+        <v>520</v>
       </c>
       <c r="R26" s="9" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="S26" s="5" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3189,19 +3221,19 @@
         <v>105</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="G27" s="5" t="n">
         <v>1</v>
@@ -3221,13 +3253,13 @@
         <v>4</v>
       </c>
       <c r="L27" s="5" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="M27" s="6" t="s">
         <v>28</v>
       </c>
       <c r="N27" s="6" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="O27" s="6" t="n">
         <v>4</v>
@@ -3243,7 +3275,7 @@
         <v>30</v>
       </c>
       <c r="S27" s="5" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3251,7 +3283,7 @@
         <v>105</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C28" s="5" t="s">
         <v>101</v>
@@ -3285,7 +3317,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B29" s="4"/>
       <c r="C29" s="4" t="s">
@@ -3310,16 +3342,16 @@
     </row>
     <row r="30" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="5" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E30" s="5" t="s">
         <v>90</v>
@@ -3367,27 +3399,27 @@
         <v>30</v>
       </c>
       <c r="S30" s="5" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="5" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="F31" s="5" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="G31" s="5" t="n">
         <v>1</v>
@@ -3407,41 +3439,49 @@
         <v>4</v>
       </c>
       <c r="L31" s="5" t="s">
-        <v>152</v>
-      </c>
-      <c r="M31" s="6"/>
-      <c r="N31" s="6"/>
-      <c r="O31" s="6"/>
-      <c r="P31" s="7"/>
-      <c r="Q31" s="8" t="str">
+        <v>153</v>
+      </c>
+      <c r="M31" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="N31" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="O31" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="P31" s="7" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q31" s="8" t="n">
         <f aca="false">IF(P31="","",IF(O31="",K31,O31)*P31)</f>
-        <v/>
+        <v>240</v>
       </c>
       <c r="R31" s="9" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="S31" s="5" t="s">
-        <v>135</v>
+        <v>155</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="5" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="C32" s="5" t="s">
         <v>130</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="F32" s="5" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="G32" s="5" t="n">
         <v>1</v>
@@ -3461,13 +3501,13 @@
         <v>4</v>
       </c>
       <c r="L32" s="5" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="M32" s="6" t="s">
         <v>28</v>
       </c>
       <c r="N32" s="6" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="O32" s="6" t="n">
         <v>4</v>
@@ -3486,10 +3526,10 @@
     </row>
     <row r="33" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="5" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="C33" s="5" t="s">
         <v>101</v>
@@ -3523,7 +3563,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="B34" s="4"/>
       <c r="C34" s="4" t="s">
@@ -3548,19 +3588,19 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="5" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="F35" s="5" t="s">
         <v>41</v>
@@ -3583,13 +3623,13 @@
         <v>4</v>
       </c>
       <c r="L35" s="5" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="M35" s="6" t="s">
         <v>28</v>
       </c>
       <c r="N35" s="6" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="O35" s="6" t="n">
         <v>6</v>
@@ -3608,22 +3648,22 @@
     </row>
     <row r="36" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="5" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="E36" s="5" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F36" s="5" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="G36" s="5" t="n">
         <v>1</v>
@@ -3643,13 +3683,13 @@
         <v>4</v>
       </c>
       <c r="L36" s="5" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="M36" s="6" t="s">
         <v>28</v>
       </c>
       <c r="N36" s="6" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="O36" s="6" t="n">
         <v>4</v>
@@ -3668,19 +3708,19 @@
     </row>
     <row r="37" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="5" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="D37" s="5" t="s">
         <v>102</v>
       </c>
       <c r="E37" s="5" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="F37" s="5" t="s">
         <v>102</v>
@@ -3703,7 +3743,7 @@
         <v>5</v>
       </c>
       <c r="L37" s="5" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="M37" s="6"/>
       <c r="N37" s="6"/>
@@ -3714,19 +3754,19 @@
         <v/>
       </c>
       <c r="R37" s="9" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="S37" s="5" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="4" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="B38" s="4"/>
       <c r="C38" s="4" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="D38" s="4"/>
       <c r="E38" s="4"/>
@@ -3747,13 +3787,13 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="5" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="D39" s="5" t="s">
         <v>25</v>
@@ -3782,7 +3822,7 @@
         <v>2</v>
       </c>
       <c r="L39" s="5" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="M39" s="6" t="s">
         <v>28</v>
@@ -3807,13 +3847,13 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="5" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="D40" s="5" t="s">
         <v>108</v>
@@ -3822,7 +3862,7 @@
         <v>108</v>
       </c>
       <c r="F40" s="5" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="G40" s="5" t="n">
         <v>1</v>
@@ -3842,7 +3882,7 @@
         <v>1</v>
       </c>
       <c r="L40" s="5" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="M40" s="6" t="s">
         <v>28</v>
@@ -3867,10 +3907,10 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="5" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="C41" s="5" t="s">
         <v>101</v>
@@ -3904,11 +3944,11 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="4" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="B42" s="4"/>
       <c r="C42" s="4" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="D42" s="4"/>
       <c r="E42" s="4"/>
@@ -3929,19 +3969,19 @@
     </row>
     <row r="43" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="5" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="D43" s="5" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="E43" s="5" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="F43" s="5" t="s">
         <v>41</v>
@@ -3964,13 +4004,13 @@
         <v>4</v>
       </c>
       <c r="L43" s="5" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="M43" s="6" t="s">
         <v>28</v>
       </c>
       <c r="N43" s="6" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="O43" s="6" t="n">
         <v>6</v>
@@ -3989,22 +4029,22 @@
     </row>
     <row r="44" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="5" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="D44" s="5" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="E44" s="5" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F44" s="5" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="G44" s="5" t="n">
         <v>1</v>
@@ -4024,13 +4064,13 @@
         <v>2</v>
       </c>
       <c r="L44" s="5" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="M44" s="6" t="s">
         <v>28</v>
       </c>
       <c r="N44" s="6" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="O44" s="6" t="n">
         <v>2</v>
@@ -4046,27 +4086,27 @@
         <v>30</v>
       </c>
       <c r="S44" s="5" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="5" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="D45" s="5" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="E45" s="5" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="F45" s="5" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="G45" s="5" t="n">
         <v>1</v>
@@ -4086,13 +4126,13 @@
         <v>2</v>
       </c>
       <c r="L45" s="5" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="M45" s="6" t="s">
         <v>28</v>
       </c>
       <c r="N45" s="6" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="O45" s="6" t="n">
         <v>4</v>
@@ -4111,19 +4151,19 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="5" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="D46" s="5" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="E46" s="5" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="F46" s="5" t="s">
         <v>41</v>
@@ -4146,13 +4186,13 @@
         <v>2</v>
       </c>
       <c r="L46" s="5" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="M46" s="6" t="s">
         <v>28</v>
       </c>
       <c r="N46" s="6" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="O46" s="6" t="n">
         <v>4</v>
@@ -4168,15 +4208,15 @@
         <v>30</v>
       </c>
       <c r="S46" s="5" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="5" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="B47" s="5" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="C47" s="5" t="s">
         <v>101</v>
@@ -4210,11 +4250,11 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="4" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="B48" s="4"/>
       <c r="C48" s="4" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="D48" s="4"/>
       <c r="E48" s="4"/>
@@ -4235,22 +4275,22 @@
     </row>
     <row r="49" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="5" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="B49" s="5" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="C49" s="5" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="D49" s="5" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="E49" s="5" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="F49" s="5" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="G49" s="5" t="n">
         <v>6</v>
@@ -4270,13 +4310,13 @@
         <v>6</v>
       </c>
       <c r="L49" s="5" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="M49" s="6" t="s">
         <v>28</v>
       </c>
       <c r="N49" s="6" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="O49" s="6" t="n">
         <v>6</v>
@@ -4292,27 +4332,27 @@
         <v>30</v>
       </c>
       <c r="S49" s="5" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="5" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="B50" s="5" t="s">
         <v>102</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="D50" s="5" t="s">
         <v>102</v>
       </c>
       <c r="E50" s="5" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="F50" s="5" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="G50" s="5" t="n">
         <v>6</v>
@@ -4332,13 +4372,13 @@
         <v>7</v>
       </c>
       <c r="L50" s="5" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="M50" s="6" t="s">
         <v>28</v>
       </c>
       <c r="N50" s="6" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="O50" s="6" t="n">
         <v>12</v>
@@ -4354,27 +4394,27 @@
         <v>30</v>
       </c>
       <c r="S50" s="5" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="5" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="B51" s="5" t="s">
         <v>102</v>
       </c>
       <c r="C51" s="5" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="D51" s="5" t="s">
         <v>102</v>
       </c>
       <c r="E51" s="5" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="F51" s="5" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="G51" s="5"/>
       <c r="H51" s="5"/>
@@ -4382,7 +4422,7 @@
       <c r="J51" s="5"/>
       <c r="K51" s="5"/>
       <c r="L51" s="5" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="M51" s="5"/>
       <c r="N51" s="5"/>
@@ -4393,18 +4433,18 @@
         <v>103</v>
       </c>
       <c r="S51" s="5" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="5" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="B52" s="5" t="s">
         <v>102</v>
       </c>
       <c r="C52" s="5" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="D52" s="5" t="s">
         <v>76</v>
@@ -4460,11 +4500,11 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="4" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="B53" s="4"/>
       <c r="C53" s="4" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="D53" s="4"/>
       <c r="E53" s="4"/>
@@ -4485,22 +4525,22 @@
     </row>
     <row r="54" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="5" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="B54" s="5" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="C54" s="5" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="D54" s="5" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="E54" s="5" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="F54" s="5" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="G54" s="5" t="n">
         <v>1</v>
@@ -4520,13 +4560,13 @@
         <v>2</v>
       </c>
       <c r="L54" s="5" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="M54" s="6" t="s">
         <v>28</v>
       </c>
       <c r="N54" s="6" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="O54" s="6" t="n">
         <v>2</v>
@@ -4542,18 +4582,18 @@
         <v>30</v>
       </c>
       <c r="S54" s="5" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="5" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="B55" s="5" t="s">
         <v>102</v>
       </c>
       <c r="C55" s="5" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="D55" s="5" t="s">
         <v>102</v>
@@ -4579,24 +4619,24 @@
         <v>103</v>
       </c>
       <c r="S55" s="5" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="5" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="B56" s="5" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="C56" s="5" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="D56" s="5" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="E56" s="5" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="F56" s="5" t="s">
         <v>77</v>
@@ -4619,13 +4659,13 @@
         <v>3</v>
       </c>
       <c r="L56" s="5" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="M56" s="6" t="s">
         <v>28</v>
       </c>
       <c r="N56" s="6" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="O56" s="6" t="n">
         <v>3</v>
@@ -4641,27 +4681,27 @@
         <v>30</v>
       </c>
       <c r="S56" s="5" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="5" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="B57" s="5" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="C57" s="5" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="D57" s="5" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="E57" s="5" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="F57" s="5" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="G57" s="5" t="n">
         <v>1</v>
@@ -4681,32 +4721,40 @@
         <v>2</v>
       </c>
       <c r="L57" s="5" t="s">
-        <v>241</v>
-      </c>
-      <c r="M57" s="6"/>
-      <c r="N57" s="6"/>
-      <c r="O57" s="6"/>
-      <c r="P57" s="7"/>
-      <c r="Q57" s="8" t="str">
+        <v>244</v>
+      </c>
+      <c r="M57" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="N57" s="6" t="s">
+        <v>245</v>
+      </c>
+      <c r="O57" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="P57" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="Q57" s="8" t="n">
         <f aca="false">IF(P57="","",IF(O57="",K57,O57)*P57)</f>
-        <v/>
+        <v>100</v>
       </c>
       <c r="R57" s="9" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="S57" s="5" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="5" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="B58" s="5" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="C58" s="5" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="D58" s="5" t="s">
         <v>108</v>
@@ -4715,7 +4763,7 @@
         <v>108</v>
       </c>
       <c r="F58" s="5" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="G58" s="5" t="n">
         <v>1</v>
@@ -4735,7 +4783,7 @@
         <v>2</v>
       </c>
       <c r="L58" s="5" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="M58" s="6" t="s">
         <v>28</v>
@@ -4760,19 +4808,19 @@
     </row>
     <row r="59" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="5" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="B59" s="5" t="s">
         <v>102</v>
       </c>
       <c r="C59" s="5" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="D59" s="5" t="s">
         <v>102</v>
       </c>
       <c r="E59" s="5" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="F59" s="5" t="s">
         <v>102</v>
@@ -4795,7 +4843,7 @@
         <v>3</v>
       </c>
       <c r="L59" s="5" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="M59" s="6"/>
       <c r="N59" s="6"/>
@@ -4806,19 +4854,19 @@
         <v/>
       </c>
       <c r="R59" s="9" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="S59" s="5" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="4" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="B60" s="4"/>
       <c r="C60" s="4" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="D60" s="4"/>
       <c r="E60" s="4"/>
@@ -4839,22 +4887,22 @@
     </row>
     <row r="61" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="5" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="B61" s="5" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
       <c r="C61" s="5" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="D61" s="5" t="s">
         <v>102</v>
       </c>
       <c r="E61" s="5" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="F61" s="5" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
       <c r="G61" s="5" t="n">
         <v>7</v>
@@ -4874,7 +4922,7 @@
         <v>50</v>
       </c>
       <c r="L61" s="5" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
       <c r="M61" s="6"/>
       <c r="N61" s="6"/>
@@ -4885,27 +4933,27 @@
         <v/>
       </c>
       <c r="R61" s="9" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="S61" s="5" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="5" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="B62" s="5" t="s">
         <v>102</v>
       </c>
       <c r="C62" s="5" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
       <c r="D62" s="5" t="s">
         <v>102</v>
       </c>
       <c r="E62" s="5" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="F62" s="5" t="s">
         <v>102</v>
@@ -4928,7 +4976,7 @@
         <v>8</v>
       </c>
       <c r="L62" s="5" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
       <c r="M62" s="6"/>
       <c r="N62" s="6"/>
@@ -4939,27 +4987,27 @@
         <v/>
       </c>
       <c r="R62" s="9" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="S62" s="5" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="5" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="B63" s="5" t="s">
         <v>102</v>
       </c>
       <c r="C63" s="5" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="D63" s="5" t="s">
         <v>102</v>
       </c>
       <c r="E63" s="5" t="s">
-        <v>261</v>
+        <v>265</v>
       </c>
       <c r="F63" s="5" t="s">
         <v>102</v>
@@ -4982,13 +5030,13 @@
         <v>2</v>
       </c>
       <c r="L63" s="5" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="M63" s="6" t="s">
         <v>28</v>
       </c>
       <c r="N63" s="6" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="O63" s="6" t="n">
         <v>2</v>
@@ -5004,24 +5052,24 @@
         <v>30</v>
       </c>
       <c r="S63" s="5" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="5" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="B64" s="5" t="s">
         <v>102</v>
       </c>
       <c r="C64" s="5" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="D64" s="5" t="s">
         <v>102</v>
       </c>
       <c r="E64" s="5" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="F64" s="5" t="s">
         <v>102</v>
@@ -5044,7 +5092,7 @@
         <v>8</v>
       </c>
       <c r="L64" s="5" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
       <c r="M64" s="6"/>
       <c r="N64" s="6"/>
@@ -5055,21 +5103,21 @@
         <v/>
       </c>
       <c r="R64" s="9" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="S64" s="5" t="s">
-        <v>268</v>
+        <v>272</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="5" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="B65" s="5" t="s">
         <v>102</v>
       </c>
       <c r="C65" s="5" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
       <c r="D65" s="5" t="s">
         <v>102</v>
@@ -5098,7 +5146,7 @@
         <v>1</v>
       </c>
       <c r="L65" s="5" t="s">
-        <v>270</v>
+        <v>274</v>
       </c>
       <c r="M65" s="6"/>
       <c r="N65" s="6"/>
@@ -5109,19 +5157,19 @@
         <v/>
       </c>
       <c r="R65" s="9" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="S65" s="5" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="4" t="s">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="B66" s="4"/>
       <c r="C66" s="4" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="D66" s="4"/>
       <c r="E66" s="4"/>
@@ -5142,22 +5190,22 @@
     </row>
     <row r="67" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="5" t="s">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="B67" s="5" t="s">
         <v>102</v>
       </c>
       <c r="C67" s="5" t="s">
-        <v>273</v>
+        <v>277</v>
       </c>
       <c r="D67" s="5" t="s">
         <v>102</v>
       </c>
       <c r="E67" s="5" t="s">
-        <v>274</v>
+        <v>278</v>
       </c>
       <c r="F67" s="5" t="s">
-        <v>275</v>
+        <v>279</v>
       </c>
       <c r="G67" s="5" t="n">
         <v>1</v>
@@ -5177,7 +5225,7 @@
         <v>2</v>
       </c>
       <c r="L67" s="5" t="s">
-        <v>276</v>
+        <v>280</v>
       </c>
       <c r="M67" s="6"/>
       <c r="N67" s="6"/>
@@ -5188,27 +5236,27 @@
         <v/>
       </c>
       <c r="R67" s="9" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="S67" s="5" t="s">
-        <v>135</v>
+        <v>281</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="5" t="s">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="B68" s="5" t="s">
         <v>102</v>
       </c>
       <c r="C68" s="5" t="s">
-        <v>277</v>
+        <v>282</v>
       </c>
       <c r="D68" s="5" t="s">
         <v>102</v>
       </c>
       <c r="E68" s="5" t="s">
-        <v>278</v>
+        <v>283</v>
       </c>
       <c r="F68" s="5" t="s">
         <v>102</v>
@@ -5231,7 +5279,7 @@
         <v>3</v>
       </c>
       <c r="L68" s="5" t="s">
-        <v>279</v>
+        <v>284</v>
       </c>
       <c r="M68" s="6"/>
       <c r="N68" s="6"/>
@@ -5242,27 +5290,27 @@
         <v/>
       </c>
       <c r="R68" s="9" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="S68" s="5" t="s">
-        <v>280</v>
+        <v>285</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="5" t="s">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="B69" s="5" t="s">
         <v>102</v>
       </c>
       <c r="C69" s="5" t="s">
-        <v>281</v>
+        <v>286</v>
       </c>
       <c r="D69" s="5" t="s">
         <v>102</v>
       </c>
       <c r="E69" s="5" t="s">
-        <v>282</v>
+        <v>287</v>
       </c>
       <c r="F69" s="5" t="s">
         <v>102</v>
@@ -5285,13 +5333,13 @@
         <v>1</v>
       </c>
       <c r="L69" s="5" t="s">
-        <v>283</v>
+        <v>288</v>
       </c>
       <c r="M69" s="6" t="s">
         <v>28</v>
       </c>
       <c r="N69" s="6" t="s">
-        <v>284</v>
+        <v>289</v>
       </c>
       <c r="O69" s="6" t="n">
         <v>3</v>
@@ -5307,16 +5355,16 @@
         <v>30</v>
       </c>
       <c r="S69" s="5" t="s">
-        <v>285</v>
+        <v>290</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="4" t="s">
-        <v>286</v>
+        <v>291</v>
       </c>
       <c r="B70" s="4"/>
       <c r="C70" s="4" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="D70" s="4"/>
       <c r="E70" s="4"/>
@@ -5335,24 +5383,24 @@
       <c r="R70" s="4"/>
       <c r="S70" s="4"/>
     </row>
-    <row r="71" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="71" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="5" t="s">
-        <v>286</v>
+        <v>291</v>
       </c>
       <c r="B71" s="5" t="s">
         <v>102</v>
       </c>
       <c r="C71" s="5" t="s">
-        <v>287</v>
+        <v>292</v>
       </c>
       <c r="D71" s="5" t="s">
         <v>102</v>
       </c>
       <c r="E71" s="5" t="s">
-        <v>288</v>
+        <v>293</v>
       </c>
       <c r="F71" s="5" t="s">
-        <v>289</v>
+        <v>294</v>
       </c>
       <c r="G71" s="5" t="n">
         <v>1</v>
@@ -5372,13 +5420,13 @@
         <v>2</v>
       </c>
       <c r="L71" s="5" t="s">
-        <v>290</v>
+        <v>295</v>
       </c>
       <c r="M71" s="6" t="s">
         <v>28</v>
       </c>
       <c r="N71" s="6" t="s">
-        <v>291</v>
+        <v>296</v>
       </c>
       <c r="O71" s="6" t="n">
         <v>1</v>
@@ -5394,24 +5442,24 @@
         <v>30</v>
       </c>
       <c r="S71" s="5" t="s">
-        <v>292</v>
+        <v>297</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="5" t="s">
-        <v>286</v>
+        <v>291</v>
       </c>
       <c r="B72" s="5" t="s">
         <v>102</v>
       </c>
       <c r="C72" s="5" t="s">
-        <v>293</v>
+        <v>298</v>
       </c>
       <c r="D72" s="5" t="s">
         <v>102</v>
       </c>
       <c r="E72" s="5" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="F72" s="5" t="s">
         <v>102</v>
@@ -5434,7 +5482,7 @@
         <v>6</v>
       </c>
       <c r="L72" s="5" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="M72" s="6"/>
       <c r="N72" s="6"/>
@@ -5445,19 +5493,19 @@
         <v/>
       </c>
       <c r="R72" s="9" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="S72" s="5" t="s">
-        <v>294</v>
+        <v>299</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="P74" s="10" t="s">
-        <v>295</v>
+        <v>300</v>
       </c>
       <c r="Q74" s="11" t="n">
         <f aca="false">SUM(Q5:Q72)</f>
-        <v>65643</v>
+        <v>66503</v>
       </c>
     </row>
   </sheetData>
@@ -5484,7 +5532,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D44"/>
+  <dimension ref="A1:D43"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="70"/>
@@ -5495,7 +5543,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>296</v>
+        <v>301</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5503,10 +5551,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>297</v>
+        <v>302</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>298</v>
+        <v>303</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>18</v>
@@ -5594,12 +5642,12 @@
       </c>
       <c r="D8" s="13" t="n">
         <f aca="false">SUMIF('BoM por modulo'!$A$5:$A$72,A8,'BoM por modulo'!$Q$5:$Q$72)</f>
-        <v>805</v>
+        <v>1325</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="12" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B9" s="12" t="n">
         <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$72,A9,'BoM por modulo'!$R$5:$R$72,"&lt;&gt;No aplica",'BoM por modulo'!$R$5:$R$72,"&lt;&gt;")</f>
@@ -5611,12 +5659,12 @@
       </c>
       <c r="D9" s="13" t="n">
         <f aca="false">SUMIF('BoM por modulo'!$A$5:$A$72,A9,'BoM por modulo'!$Q$5:$Q$72)</f>
-        <v>320</v>
+        <v>560</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="12" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="B10" s="12" t="n">
         <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$72,A10,'BoM por modulo'!$R$5:$R$72,"&lt;&gt;No aplica",'BoM por modulo'!$R$5:$R$72,"&lt;&gt;")</f>
@@ -5633,7 +5681,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="12" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="B11" s="12" t="n">
         <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$72,A11,'BoM por modulo'!$R$5:$R$72,"&lt;&gt;No aplica",'BoM por modulo'!$R$5:$R$72,"&lt;&gt;")</f>
@@ -5650,7 +5698,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="12" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="B12" s="12" t="n">
         <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$72,A12,'BoM por modulo'!$R$5:$R$72,"&lt;&gt;No aplica",'BoM por modulo'!$R$5:$R$72,"&lt;&gt;")</f>
@@ -5667,7 +5715,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="12" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="B13" s="12" t="n">
         <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$72,A13,'BoM por modulo'!$R$5:$R$72,"&lt;&gt;No aplica",'BoM por modulo'!$R$5:$R$72,"&lt;&gt;")</f>
@@ -5684,7 +5732,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="12" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="B14" s="12" t="n">
         <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$72,A14,'BoM por modulo'!$R$5:$R$72,"&lt;&gt;No aplica",'BoM por modulo'!$R$5:$R$72,"&lt;&gt;")</f>
@@ -5696,12 +5744,12 @@
       </c>
       <c r="D14" s="13" t="n">
         <f aca="false">SUMIF('BoM por modulo'!$A$5:$A$72,A14,'BoM por modulo'!$Q$5:$Q$72)</f>
-        <v>2270</v>
+        <v>2370</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="12" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="B15" s="12" t="n">
         <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$72,A15,'BoM por modulo'!$R$5:$R$72,"&lt;&gt;No aplica",'BoM por modulo'!$R$5:$R$72,"&lt;&gt;")</f>
@@ -5718,7 +5766,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="12" t="s">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="B16" s="12" t="n">
         <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$72,A16,'BoM por modulo'!$R$5:$R$72,"&lt;&gt;No aplica",'BoM por modulo'!$R$5:$R$72,"&lt;&gt;")</f>
@@ -5735,7 +5783,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="12" t="s">
-        <v>286</v>
+        <v>291</v>
       </c>
       <c r="B17" s="12" t="n">
         <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$72,A17,'BoM por modulo'!$R$5:$R$72,"&lt;&gt;No aplica",'BoM por modulo'!$R$5:$R$72,"&lt;&gt;")</f>
@@ -5752,7 +5800,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="14" t="s">
-        <v>295</v>
+        <v>300</v>
       </c>
       <c r="B18" s="14" t="n">
         <f aca="false">SUM(B4:B17)</f>
@@ -5764,17 +5812,19 @@
       </c>
       <c r="D18" s="15" t="n">
         <f aca="false">SUM(D4:D17)</f>
-        <v>65643</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>66503</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
         <v>14</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>299</v>
-      </c>
-      <c r="C20" s="3"/>
+        <v>304</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>305</v>
+      </c>
       <c r="D20" s="3"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5782,8 +5832,12 @@
         <v>28</v>
       </c>
       <c r="B21" s="17" t="n">
-        <f aca="false">SUMIF('BoM por modulo'!$M$5:$M$72,A21,'BoM por modulo'!$Q$5:$Q$72)</f>
+        <f aca="false">SUMIFS('BoM por modulo'!$Q$5:$Q$72,'BoM por modulo'!$M$5:$M$72,A21,'BoM por modulo'!$R$5:$R$72,"En carrito")</f>
         <v>37683</v>
+      </c>
+      <c r="C21" s="17" t="n">
+        <f aca="false">SUMIFS('BoM por modulo'!$Q$5:$Q$72,'BoM por modulo'!$M$5:$M$72,A21,'BoM por modulo'!$R$5:$R$72,"Pendiente")</f>
+        <v>860</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5791,144 +5845,143 @@
         <v>43</v>
       </c>
       <c r="B22" s="17" t="n">
-        <f aca="false">SUMIF('BoM por modulo'!$M$5:$M$72,A22,'BoM por modulo'!$Q$5:$Q$72)</f>
+        <f aca="false">SUMIFS('BoM por modulo'!$Q$5:$Q$72,'BoM por modulo'!$M$5:$M$72,A22,'BoM por modulo'!$R$5:$R$72,"En carrito")</f>
         <v>27960</v>
+      </c>
+      <c r="C22" s="17" t="n">
+        <f aca="false">SUMIFS('BoM por modulo'!$Q$5:$Q$72,'BoM por modulo'!$M$5:$M$72,A22,'BoM por modulo'!$R$5:$R$72,"Pendiente")</f>
+        <v>0</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="18" t="s">
-        <v>300</v>
+        <v>306</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="16" t="s">
-        <v>301</v>
+        <v>307</v>
       </c>
       <c r="B25" s="19" t="s">
-        <v>133</v>
+        <v>308</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="16" t="s">
-        <v>302</v>
+        <v>309</v>
       </c>
       <c r="B26" s="19" t="s">
-        <v>152</v>
+        <v>310</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="16" t="s">
-        <v>303</v>
+        <v>311</v>
       </c>
       <c r="B27" s="19" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="16" t="s">
-        <v>304</v>
+        <v>312</v>
       </c>
       <c r="B28" s="19" t="s">
-        <v>241</v>
+        <v>313</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="16" t="s">
-        <v>305</v>
+        <v>314</v>
       </c>
       <c r="B29" s="19" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="16" t="s">
-        <v>306</v>
+        <v>315</v>
       </c>
       <c r="B30" s="19" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="16" t="s">
-        <v>307</v>
+        <v>316</v>
       </c>
       <c r="B31" s="19" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="16" t="s">
-        <v>308</v>
+        <v>317</v>
       </c>
       <c r="B32" s="19" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="16" t="s">
-        <v>309</v>
+        <v>318</v>
       </c>
       <c r="B33" s="19" t="s">
-        <v>270</v>
+        <v>274</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="16" t="s">
-        <v>310</v>
+        <v>319</v>
       </c>
       <c r="B34" s="19" t="s">
-        <v>276</v>
+        <v>280</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="16" t="s">
-        <v>311</v>
+        <v>320</v>
       </c>
       <c r="B35" s="19" t="s">
-        <v>279</v>
+        <v>284</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="16" t="s">
-        <v>312</v>
+        <v>321</v>
       </c>
       <c r="B36" s="19" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="10" t="s">
-        <v>313</v>
+        <v>322</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="16" t="s">
-        <v>314</v>
+        <v>323</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="16" t="s">
-        <v>315</v>
+        <v>324</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="16" t="s">
-        <v>316</v>
+        <v>325</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="16" t="s">
-        <v>317</v>
+        <v>326</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="16" t="s">
-        <v>318</v>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="16" t="s">
-        <v>319</v>
+        <v>327</v>
       </c>
     </row>
   </sheetData>
@@ -5957,396 +6010,396 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>320</v>
+        <v>328</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>321</v>
+        <v>329</v>
       </c>
       <c r="B3" s="4"/>
       <c r="C3" s="4"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>322</v>
+        <v>330</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>323</v>
+        <v>331</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>324</v>
+        <v>332</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="20" t="s">
-        <v>325</v>
+        <v>333</v>
       </c>
       <c r="B5" s="21" t="s">
-        <v>326</v>
+        <v>334</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>327</v>
+        <v>335</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="20" t="s">
-        <v>328</v>
+        <v>336</v>
       </c>
       <c r="B6" s="21" t="s">
-        <v>329</v>
+        <v>337</v>
       </c>
       <c r="C6" s="21" t="s">
-        <v>330</v>
+        <v>338</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="20" t="s">
-        <v>331</v>
+        <v>339</v>
       </c>
       <c r="B7" s="21" t="s">
-        <v>332</v>
+        <v>340</v>
       </c>
       <c r="C7" s="21" t="s">
-        <v>333</v>
+        <v>341</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="20" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>335</v>
+        <v>343</v>
       </c>
       <c r="C8" s="21" t="s">
-        <v>336</v>
+        <v>344</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="20" t="s">
-        <v>337</v>
+        <v>345</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>338</v>
+        <v>346</v>
       </c>
       <c r="C9" s="21" t="s">
-        <v>339</v>
+        <v>347</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="20" t="s">
-        <v>340</v>
+        <v>348</v>
       </c>
       <c r="B10" s="21" t="s">
-        <v>341</v>
+        <v>349</v>
       </c>
       <c r="C10" s="21" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="20" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="B11" s="21" t="s">
-        <v>344</v>
+        <v>352</v>
       </c>
       <c r="C11" s="21" t="s">
-        <v>345</v>
+        <v>353</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="20" t="s">
-        <v>346</v>
+        <v>354</v>
       </c>
       <c r="B12" s="21" t="s">
-        <v>347</v>
+        <v>355</v>
       </c>
       <c r="C12" s="21" t="s">
-        <v>348</v>
+        <v>356</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="20" t="s">
-        <v>349</v>
+        <v>357</v>
       </c>
       <c r="B13" s="21" t="s">
-        <v>350</v>
+        <v>358</v>
       </c>
       <c r="C13" s="21" t="s">
-        <v>351</v>
+        <v>359</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="20" t="s">
-        <v>352</v>
+        <v>360</v>
       </c>
       <c r="B14" s="21" t="s">
-        <v>353</v>
+        <v>361</v>
       </c>
       <c r="C14" s="21" t="s">
-        <v>273</v>
+        <v>277</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="20" t="s">
-        <v>354</v>
+        <v>362</v>
       </c>
       <c r="B15" s="21" t="s">
-        <v>355</v>
+        <v>363</v>
       </c>
       <c r="C15" s="21"/>
     </row>
     <row r="16" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="20" t="s">
-        <v>356</v>
+        <v>364</v>
       </c>
       <c r="B16" s="21" t="s">
-        <v>357</v>
+        <v>365</v>
       </c>
       <c r="C16" s="21"/>
     </row>
     <row r="17" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="20" t="s">
-        <v>358</v>
+        <v>366</v>
       </c>
       <c r="B17" s="21" t="s">
-        <v>359</v>
+        <v>367</v>
       </c>
       <c r="C17" s="21"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>360</v>
+        <v>368</v>
       </c>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>322</v>
+        <v>330</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>323</v>
+        <v>331</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>324</v>
+        <v>332</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="20" t="s">
-        <v>325</v>
+        <v>333</v>
       </c>
       <c r="B21" s="21" t="s">
-        <v>361</v>
+        <v>369</v>
       </c>
       <c r="C21" s="21" t="s">
-        <v>362</v>
+        <v>370</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="20" t="s">
-        <v>363</v>
+        <v>371</v>
       </c>
       <c r="B22" s="21" t="s">
-        <v>364</v>
+        <v>372</v>
       </c>
       <c r="C22" s="21" t="s">
-        <v>365</v>
+        <v>373</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="20" t="s">
-        <v>331</v>
+        <v>339</v>
       </c>
       <c r="B23" s="21" t="s">
-        <v>366</v>
+        <v>374</v>
       </c>
       <c r="C23" s="21" t="s">
-        <v>367</v>
+        <v>375</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="20" t="s">
-        <v>368</v>
+        <v>376</v>
       </c>
       <c r="B24" s="21" t="s">
-        <v>369</v>
+        <v>377</v>
       </c>
       <c r="C24" s="21" t="s">
-        <v>370</v>
+        <v>378</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="20" t="s">
-        <v>371</v>
+        <v>379</v>
       </c>
       <c r="B25" s="21" t="s">
-        <v>372</v>
+        <v>380</v>
       </c>
       <c r="C25" s="21" t="s">
-        <v>373</v>
+        <v>381</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="20" t="s">
-        <v>374</v>
+        <v>382</v>
       </c>
       <c r="B26" s="21" t="s">
-        <v>375</v>
+        <v>383</v>
       </c>
       <c r="C26" s="21" t="s">
-        <v>376</v>
+        <v>384</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="20" t="s">
-        <v>340</v>
+        <v>348</v>
       </c>
       <c r="B27" s="21" t="s">
-        <v>377</v>
+        <v>385</v>
       </c>
       <c r="C27" s="21" t="s">
-        <v>378</v>
+        <v>386</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="20" t="s">
-        <v>346</v>
+        <v>354</v>
       </c>
       <c r="B28" s="21" t="s">
-        <v>379</v>
+        <v>387</v>
       </c>
       <c r="C28" s="21" t="s">
-        <v>380</v>
+        <v>388</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="20" t="s">
-        <v>381</v>
+        <v>389</v>
       </c>
       <c r="B29" s="21" t="s">
-        <v>382</v>
+        <v>390</v>
       </c>
       <c r="C29" s="21" t="s">
-        <v>383</v>
+        <v>391</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="20" t="s">
-        <v>352</v>
+        <v>360</v>
       </c>
       <c r="B30" s="21" t="s">
-        <v>384</v>
+        <v>392</v>
       </c>
       <c r="C30" s="21" t="s">
-        <v>273</v>
+        <v>277</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="20" t="s">
-        <v>354</v>
+        <v>362</v>
       </c>
       <c r="B31" s="21" t="s">
-        <v>385</v>
+        <v>393</v>
       </c>
       <c r="C31" s="21"/>
     </row>
     <row r="32" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="20" t="s">
-        <v>356</v>
+        <v>364</v>
       </c>
       <c r="B32" s="21" t="s">
-        <v>386</v>
+        <v>394</v>
       </c>
       <c r="C32" s="21" t="s">
-        <v>387</v>
+        <v>395</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="20" t="s">
-        <v>358</v>
+        <v>366</v>
       </c>
       <c r="B33" s="21" t="s">
-        <v>388</v>
+        <v>396</v>
       </c>
       <c r="C33" s="21"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="s">
-        <v>389</v>
+        <v>397</v>
       </c>
       <c r="B35" s="4"/>
       <c r="C35" s="4"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="3" t="s">
-        <v>322</v>
+        <v>330</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>323</v>
+        <v>331</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>324</v>
+        <v>332</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="20" t="s">
-        <v>363</v>
+        <v>371</v>
       </c>
       <c r="B37" s="21" t="s">
-        <v>390</v>
+        <v>398</v>
       </c>
       <c r="C37" s="21" t="s">
-        <v>391</v>
+        <v>399</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="20" t="s">
-        <v>392</v>
+        <v>400</v>
       </c>
       <c r="B38" s="21" t="s">
-        <v>393</v>
+        <v>401</v>
       </c>
       <c r="C38" s="21" t="s">
-        <v>394</v>
+        <v>402</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="20" t="s">
-        <v>395</v>
+        <v>403</v>
       </c>
       <c r="B39" s="21" t="s">
-        <v>396</v>
+        <v>404</v>
       </c>
       <c r="C39" s="21"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="20" t="s">
-        <v>354</v>
+        <v>362</v>
       </c>
       <c r="B40" s="21" t="s">
-        <v>397</v>
+        <v>405</v>
       </c>
       <c r="C40" s="21" t="s">
-        <v>398</v>
+        <v>406</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="20" t="s">
-        <v>356</v>
+        <v>364</v>
       </c>
       <c r="B41" s="21" t="s">
-        <v>399</v>
+        <v>407</v>
       </c>
       <c r="C41" s="21"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="20" t="s">
-        <v>400</v>
+        <v>408</v>
       </c>
       <c r="B42" s="21" t="s">
-        <v>401</v>
+        <v>409</v>
       </c>
       <c r="C42" s="21"/>
     </row>
@@ -6378,7 +6431,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>402</v>
+        <v>410</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6386,16 +6439,16 @@
         <v>14</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>403</v>
+        <v>411</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>404</v>
+        <v>412</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>405</v>
+        <v>413</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>406</v>
+        <v>414</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6403,84 +6456,84 @@
         <v>28</v>
       </c>
       <c r="B4" s="21" t="s">
-        <v>407</v>
+        <v>415</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>408</v>
+        <v>416</v>
       </c>
       <c r="D4" s="21" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>410</v>
+        <v>418</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="21" t="s">
-        <v>411</v>
+        <v>419</v>
       </c>
       <c r="B5" s="21" t="s">
-        <v>412</v>
+        <v>420</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>413</v>
+        <v>421</v>
       </c>
       <c r="D5" s="21" t="s">
-        <v>414</v>
+        <v>422</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>415</v>
+        <v>423</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="21" t="s">
-        <v>416</v>
+        <v>424</v>
       </c>
       <c r="B6" s="21" t="s">
-        <v>407</v>
+        <v>415</v>
       </c>
       <c r="C6" s="21" t="s">
-        <v>417</v>
+        <v>425</v>
       </c>
       <c r="D6" s="21" t="s">
-        <v>418</v>
+        <v>426</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>419</v>
+        <v>427</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="21" t="s">
-        <v>420</v>
+        <v>428</v>
       </c>
       <c r="B7" s="21" t="s">
-        <v>407</v>
+        <v>415</v>
       </c>
       <c r="C7" s="21" t="s">
-        <v>421</v>
+        <v>429</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>422</v>
+        <v>430</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>423</v>
+        <v>431</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="21" t="s">
-        <v>424</v>
+        <v>432</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>407</v>
+        <v>415</v>
       </c>
       <c r="C8" s="21" t="s">
-        <v>425</v>
+        <v>433</v>
       </c>
       <c r="D8" s="21" t="s">
-        <v>426</v>
+        <v>434</v>
       </c>
       <c r="E8" s="21" t="s">
-        <v>427</v>
+        <v>435</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6488,84 +6541,84 @@
         <v>43</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>428</v>
+        <v>436</v>
       </c>
       <c r="C9" s="21" t="s">
-        <v>429</v>
+        <v>437</v>
       </c>
       <c r="D9" s="21" t="s">
-        <v>430</v>
+        <v>438</v>
       </c>
       <c r="E9" s="21" t="s">
-        <v>431</v>
+        <v>439</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="21" t="s">
-        <v>432</v>
+        <v>440</v>
       </c>
       <c r="B10" s="21" t="s">
         <v>102</v>
       </c>
       <c r="C10" s="21" t="s">
-        <v>433</v>
+        <v>441</v>
       </c>
       <c r="D10" s="21" t="s">
-        <v>434</v>
+        <v>442</v>
       </c>
       <c r="E10" s="21" t="s">
-        <v>435</v>
+        <v>443</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="21" t="s">
-        <v>436</v>
+        <v>444</v>
       </c>
       <c r="B11" s="21" t="s">
         <v>102</v>
       </c>
       <c r="C11" s="21" t="s">
-        <v>437</v>
+        <v>445</v>
       </c>
       <c r="D11" s="21" t="s">
-        <v>438</v>
+        <v>446</v>
       </c>
       <c r="E11" s="21" t="s">
-        <v>439</v>
+        <v>447</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="21" t="s">
-        <v>440</v>
+        <v>448</v>
       </c>
       <c r="B12" s="21" t="s">
-        <v>407</v>
+        <v>415</v>
       </c>
       <c r="C12" s="21" t="s">
-        <v>441</v>
+        <v>449</v>
       </c>
       <c r="D12" s="21" t="s">
-        <v>442</v>
+        <v>450</v>
       </c>
       <c r="E12" s="21" t="s">
-        <v>443</v>
+        <v>451</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="21" t="s">
-        <v>444</v>
+        <v>452</v>
       </c>
       <c r="B13" s="21" t="s">
-        <v>445</v>
+        <v>453</v>
       </c>
       <c r="C13" s="21" t="s">
-        <v>446</v>
+        <v>454</v>
       </c>
       <c r="D13" s="21" t="s">
-        <v>447</v>
+        <v>455</v>
       </c>
       <c r="E13" s="21" t="s">
-        <v>448</v>
+        <v>456</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
BoM: carrito actualizado (tiras de header, Cm1 100n+47n, 1 uF MLCC), C21 = 10n + 4.7n (15n agotado), lista FALTA COMPRAR al final
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V5Cz1Wb6HSRhqzouEW9mso
</commit_message>
<xml_diff>
--- a/docs/afe-emg/BoM_AFE_AuraVox.xlsx
+++ b/docs/afe-emg/BoM_AFE_AuraVox.xlsx
@@ -14,7 +14,7 @@
     <sheet name="Tiendas" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'BoM por modulo'!$A$4:$S$72</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'BoM por modulo'!$A$4:$S$73</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="807" uniqueCount="457">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="871" uniqueCount="501">
   <si>
     <t xml:space="preserve">BoM AFE sEMG AuraVox: 3 canales (submentoniano, labio inferior, laringe), 7 electrodos, RLD. Ordenada por modulo, igual que los recuadros del esquematico LTspice (sim/ltspice).</t>
   </si>
@@ -433,67 +433,67 @@
     <t xml:space="preserve">2A104K poliester 100nF 100V + 2A473J poliester 47nF 100V, en paralelo (par)</t>
   </si>
   <si>
+    <t xml:space="preserve">No hay 150 nF en Global: 100n + 47n en paralelo = 147 nF (f0 +1 %, Q -1 %). Cantidad en pares; precio del par ($70 + $60)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cm2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Condensador de realimentacion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1n</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ceramico C0G/NP0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">condensador ceramico 1nF NP0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RPE110X7R102K050V MLCC X7R 1nF 50V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">X7R en vez de C0G: aceptado para la demo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">XMF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6 LPF Sallen-Key 500 Hz (Q 1.31)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rlb1, Rlb2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resistencia del LPF B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">54.9k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Con 56k: f0 = 495 Hz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15n</t>
+  </si>
+  <si>
+    <t xml:space="preserve">poliester 5 % o C0G</t>
+  </si>
+  <si>
+    <t xml:space="preserve">condensador poliester 15nF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2A103J poliester 10nF 100V + 2A472K poliester 4.7nF 100V, en paralelo (par)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Pendiente</t>
   </si>
   <si>
-    <t xml:space="preserve">AGREGAR AL CARRITO DE GLOBAL. No hay 150 nF en Global: 100n + 47n en paralelo = 147 nF (f0 +1 %, Q -1 %). Precio = el par ($70 + $60)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cm2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Condensador de realimentacion</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1n</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ceramico C0G/NP0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">condensador ceramico 1nF NP0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RPE110X7R102K050V MLCC X7R 1nF 50V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">X7R en vez de C0G: aceptado para la demo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">XMF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6 LPF Sallen-Key 500 Hz (Q 1.31)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rlb1, Rlb2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Resistencia del LPF B</t>
-  </si>
-  <si>
-    <t xml:space="preserve">54.9k</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Con 56k: f0 = 495 Hz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C21</t>
-  </si>
-  <si>
-    <t xml:space="preserve">15n</t>
-  </si>
-  <si>
-    <t xml:space="preserve">poliester 5 % o C0G</t>
-  </si>
-  <si>
-    <t xml:space="preserve">condensador poliester 15nF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2A153J poliester 15nF 100V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AGREGAR AL CARRITO DE GLOBAL</t>
+    <t xml:space="preserve">AGREGAR AL CARRITO DE GLOBAL. 15 nF agotado (2A153J en Global; tampoco en MechatronicStore): 10n + 4.7n en paralelo = 14.7 nF (f0 +1 %, Q -1 %). Stock al 4-oct: 2A103J 22 u, 2A472K 122 u. Cantidad en pares; precio del par ($50 + $60)</t>
   </si>
   <si>
     <t xml:space="preserve">C22</t>
@@ -766,7 +766,7 @@
     <t xml:space="preserve">CM105 MLCC THD 1uF 50V X7R</t>
   </si>
   <si>
-    <t xml:space="preserve">AGREGAR AL CARRITO DE GLOBAL. El TLV757 esta pensado para ceramico a la salida (&gt;= 0.47 uF efectivos); un electrolitico solo puede oscilar</t>
+    <t xml:space="preserve">El TLV757 esta pensado para ceramico a la salida (&gt;= 0.47 uF efectivos); un electrolitico solo puede oscilar</t>
   </si>
   <si>
     <t xml:space="preserve">CBULK</t>
@@ -874,16 +874,34 @@
     <t xml:space="preserve">FALTA EN EL CARRITO</t>
   </si>
   <si>
-    <t xml:space="preserve">Tira de headers 1x40 2.54 THT (1 macho + 1 hembra)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.54 mm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tira header macho 1x40 / tira hembra 1x40</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FALTA EN EL CARRITO. Macho: salidas A1-A3, GND, 5 V y microfono. Hembra: zocalo de los modulos INA333</t>
+    <t xml:space="preserve">Tira de header macho 1x40 2.54 THT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">macho 1x40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tira poste recto una fila 40 pines</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1109-40L tira poste recto una fila 40 pines, pin largo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Salidas A1-A3 + GND, 5 V/GND y microfono</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tira de header hembra 1x40 2.54 THT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hembra 1x40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tira 40 pines header hembra 2.54</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fila de 40 pines header hembra 2.54 (GD2-3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zocalo de los 3 modulos INA333 (se cambian sin desoldar)</t>
   </si>
   <si>
     <t xml:space="preserve">Cable para puentes</t>
@@ -931,6 +949,135 @@
     <t xml:space="preserve">TOTAL</t>
   </si>
   <si>
+    <t xml:space="preserve">FALTA COMPRAR (no esta en los carritos del 4-oct-2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cant.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Que</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Donde</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15n Condensador de realimentacion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Global (agregar al carrito)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15 nF agotado (2A153J en Global; tampoco en MechatronicStore): 10n + 4.7n en paralelo = 14.7 nF (f0 +1 %, Q -1 %). Stock al 4-oct: 2A103J 22 u, 2A472K 122 u. Cantidad en pares; precio del par ($50 + $60)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">jumper Dupont M-H Cable a Arduino A1..A3 del STM32N6570-DK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MechatronicStore / Global. 1 tira de 40 M-H cubre las 3 filas M-H (14 cables)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CH1-A1 (PA9), CH2-A2 (PA10), CH3-A3 (PA12). Mas 1 cable de GND. A0 no: comparte ADC con USB1 ISENSE (UM3300)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">jumper Dupont M-H Cable 5 V y GND desde el DK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MechatronicStore / Global (misma tira M-H)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Usar powerbank o PC a bateria mientras haya electrodos puestos (ver Notas de seguridad)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Skintact FS-RG1/10 32x41 Electrodo Ag/AgCl con broche 4 mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiendas de insumos medicos / Mercado Libre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7 por sesion (6 de senal + 1 RLD); caja de 50. Skintact para CH1, CH3 y RLD. CH2: Arbo H124SG (24 mm) o par sobre el menton. ISIMED 55x55 solo como RLD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">broche 4 mm a pin Cable de electrodo con broche (snap) 4 mm, idealmente apantallado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MechatronicStore ("cable de electrodos AD8232") / tiendas medicas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Uno por electrodo; trenzar los dos de cada par. REVISAR EL TERMINAL antes de comprar: debe calzar en header hembra 2.54 mm. Si termina en DIN 1.5 mm touchproof (DIN 42802), cortar y crimpar terminal Dupont hembra o comprar bases touchproof. Alternativa: cable de 3 electrodos con jack 3.5 mm (el de los kits AD8232) + jack hembra 3.5 mm TRS en la placa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">jumper Dupont M-M Bus de 8 cables Dupont macho (separado de una tira de 40)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MechatronicStore / Global. 1 tira de 40 M-M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lado macho al conector 2x8; el otro extremo se une a los cables de electrodo (soldado + termorretractil o enchufado)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Farmacia / ferreteria</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Preparar la piel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10 x 15 cm Perfboard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Global (tarjetas para prototipos) / MechatronicStore</t>
+  </si>
+  <si>
+    <t xml:space="preserve">jumper Dupont M-H Cables Dupont para el microfono</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VDD 3.3V, GND, SCK, WS, SD, L/R (L/R a GND)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estano 0.5-0.8 mm con nucleo de flux</t>
+  </si>
+  <si>
+    <t xml:space="preserve">soldadura estano 0.8 mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Global (soldadura)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">insumo, no esta en el esquematico</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flux (lapiz o pasta)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">flux</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Global (flux y mallas)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Imprescindible para soldar los TS922 en los S08D8 (insumo, no esta en el esquematico)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Malla desoldadora</t>
+  </si>
+  <si>
+    <t xml:space="preserve">malla desoldadora</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Para sacar los trimmers de los modulos INA333 (insumo, no esta en el esquematico)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Termorretractil 2-3 mm (surtido)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tubo termo retractil</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Global</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Uniones bus Dupont - cable de electrodo (insumo, no esta en el esquematico)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Resumen por modulo</t>
   </si>
   <si>
@@ -949,27 +1096,15 @@
     <t xml:space="preserve">Faltan en los carritos</t>
   </si>
   <si>
-    <t xml:space="preserve">4 x 150n  Condensador a GND</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Global: 2A104K poliester 100nF 100V + 2A473J poliester 47nF 100V, en paralelo (par)</t>
-  </si>
-  <si>
     <t xml:space="preserve">4 x 15n  Condensador de realimentacion</t>
   </si>
   <si>
-    <t xml:space="preserve">Global: 2A153J poliester 15nF 100V</t>
+    <t xml:space="preserve">Global: 2A103J poliester 10nF 100V + 2A472K poliester 4.7nF 100V, en paralelo (par)</t>
   </si>
   <si>
     <t xml:space="preserve">5 x jumper Dupont M-H  Cable a Arduino A1..A3 del STM32N6570-DK</t>
   </si>
   <si>
-    <t xml:space="preserve">2 x 1u X7R  Condensador ceramico de salida del LDO (en paralelo con el electrolitico)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Global: CM105 MLCC THD 1uF 50V X7R</t>
-  </si>
-  <si>
     <t xml:space="preserve">3 x jumper Dupont M-H  Cable 5 V y GND desde el DK</t>
   </si>
   <si>
@@ -988,16 +1123,13 @@
     <t xml:space="preserve">2 x 10 x 15 cm  Perfboard</t>
   </si>
   <si>
-    <t xml:space="preserve">3 x 2.54 mm  Tira de headers 1x40 2.54 THT (1 macho + 1 hembra)</t>
-  </si>
-  <si>
     <t xml:space="preserve">6 x jumper Dupont M-H  Cables Dupont para el microfono</t>
   </si>
   <si>
     <t xml:space="preserve">Avisos de la compra</t>
   </si>
   <si>
-    <t xml:space="preserve">AGREGAR al carrito de Global: 4 x 2A104K (100n poliester) + 4 x 2A473J (47n poliester) para Cm1 (100n + 47n en paralelo = 147 nF); 4 x 2A153J (15n poliester) para C21; 2 x CM105 (1 uF MLCC X7R) para la salida del LDO.</t>
+    <t xml:space="preserve">AGREGAR al carrito de Global: 4 x 2A103J (10n poliester) + 4 x 2A472K (4.7n poliester) para C21 (10n + 4.7n en paralelo = 14.7 nF; el 15 nF esta agotado).</t>
   </si>
   <si>
     <t xml:space="preserve">Pendiente (otra tienda): electrodos, cables de electrodo, jumpers Dupont (tira M-H y tira M-M), perfboard, tiras de header 1x40 y alcohol.</t>
@@ -1407,7 +1539,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="\$#,##0;&quot;($&quot;#,##0\);\-"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1476,6 +1608,14 @@
     <font>
       <b val="true"/>
       <sz val="11"/>
+      <color rgb="FFC00000"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="12"/>
       <color rgb="FFC00000"/>
       <name val="Arial"/>
       <family val="0"/>
@@ -1570,7 +1710,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1619,11 +1759,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1635,7 +1783,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1647,15 +1795,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1980,7 +2124,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:S74"/>
+  <dimension ref="A1:S91"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
@@ -3209,11 +3353,11 @@
         <f aca="false">IF(P26="","",IF(O26="",K26,O26)*P26)</f>
         <v>520</v>
       </c>
-      <c r="R26" s="9" t="s">
+      <c r="R26" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="S26" s="5" t="s">
         <v>135</v>
-      </c>
-      <c r="S26" s="5" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3221,19 +3365,19 @@
         <v>105</v>
       </c>
       <c r="B27" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="C27" s="5" t="s">
         <v>137</v>
       </c>
-      <c r="C27" s="5" t="s">
+      <c r="D27" s="5" t="s">
         <v>138</v>
       </c>
-      <c r="D27" s="5" t="s">
+      <c r="E27" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="F27" s="5" t="s">
         <v>139</v>
-      </c>
-      <c r="E27" s="5" t="s">
-        <v>139</v>
-      </c>
-      <c r="F27" s="5" t="s">
-        <v>140</v>
       </c>
       <c r="G27" s="5" t="n">
         <v>1</v>
@@ -3253,13 +3397,13 @@
         <v>4</v>
       </c>
       <c r="L27" s="5" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="M27" s="6" t="s">
         <v>28</v>
       </c>
       <c r="N27" s="6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="O27" s="6" t="n">
         <v>4</v>
@@ -3275,7 +3419,7 @@
         <v>30</v>
       </c>
       <c r="S27" s="5" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3283,7 +3427,7 @@
         <v>105</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C28" s="5" t="s">
         <v>101</v>
@@ -3317,7 +3461,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B29" s="4"/>
       <c r="C29" s="4" t="s">
@@ -3342,16 +3486,16 @@
     </row>
     <row r="30" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="B30" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="B30" s="5" t="s">
+      <c r="C30" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="C30" s="5" t="s">
+      <c r="D30" s="5" t="s">
         <v>147</v>
-      </c>
-      <c r="D30" s="5" t="s">
-        <v>148</v>
       </c>
       <c r="E30" s="5" t="s">
         <v>90</v>
@@ -3399,27 +3543,27 @@
         <v>30</v>
       </c>
       <c r="S30" s="5" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="B31" s="5" t="s">
         <v>149</v>
       </c>
-    </row>
-    <row r="31" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="5" t="s">
-        <v>145</v>
-      </c>
-      <c r="B31" s="5" t="s">
+      <c r="C31" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="D31" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="C31" s="5" t="s">
-        <v>138</v>
-      </c>
-      <c r="D31" s="5" t="s">
+      <c r="E31" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="F31" s="5" t="s">
         <v>151</v>
-      </c>
-      <c r="E31" s="5" t="s">
-        <v>151</v>
-      </c>
-      <c r="F31" s="5" t="s">
-        <v>152</v>
       </c>
       <c r="G31" s="5" t="n">
         <v>1</v>
@@ -3439,26 +3583,26 @@
         <v>4</v>
       </c>
       <c r="L31" s="5" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="M31" s="6" t="s">
         <v>28</v>
       </c>
       <c r="N31" s="6" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="O31" s="6" t="n">
         <v>4</v>
       </c>
       <c r="P31" s="7" t="n">
-        <v>60</v>
+        <v>110</v>
       </c>
       <c r="Q31" s="8" t="n">
         <f aca="false">IF(P31="","",IF(O31="",K31,O31)*P31)</f>
-        <v>240</v>
+        <v>440</v>
       </c>
       <c r="R31" s="9" t="s">
-        <v>135</v>
+        <v>154</v>
       </c>
       <c r="S31" s="5" t="s">
         <v>155</v>
@@ -3466,7 +3610,7 @@
     </row>
     <row r="32" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="5" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B32" s="5" t="s">
         <v>156</v>
@@ -3481,7 +3625,7 @@
         <v>157</v>
       </c>
       <c r="F32" s="5" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="G32" s="5" t="n">
         <v>1</v>
@@ -3526,7 +3670,7 @@
     </row>
     <row r="33" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="5" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B33" s="5" t="s">
         <v>160</v>
@@ -3657,13 +3801,13 @@
         <v>168</v>
       </c>
       <c r="D36" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="E36" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="F36" s="5" t="s">
         <v>139</v>
-      </c>
-      <c r="E36" s="5" t="s">
-        <v>139</v>
-      </c>
-      <c r="F36" s="5" t="s">
-        <v>140</v>
       </c>
       <c r="G36" s="5" t="n">
         <v>1</v>
@@ -3683,13 +3827,13 @@
         <v>4</v>
       </c>
       <c r="L36" s="5" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="M36" s="6" t="s">
         <v>28</v>
       </c>
       <c r="N36" s="6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="O36" s="6" t="n">
         <v>4</v>
@@ -3754,7 +3898,7 @@
         <v/>
       </c>
       <c r="R37" s="9" t="s">
-        <v>135</v>
+        <v>154</v>
       </c>
       <c r="S37" s="5" t="s">
         <v>173</v>
@@ -4038,13 +4182,13 @@
         <v>192</v>
       </c>
       <c r="D44" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="E44" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="F44" s="5" t="s">
         <v>139</v>
-      </c>
-      <c r="E44" s="5" t="s">
-        <v>139</v>
-      </c>
-      <c r="F44" s="5" t="s">
-        <v>140</v>
       </c>
       <c r="G44" s="5" t="n">
         <v>1</v>
@@ -4064,13 +4208,13 @@
         <v>2</v>
       </c>
       <c r="L44" s="5" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="M44" s="6" t="s">
         <v>28</v>
       </c>
       <c r="N44" s="6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="O44" s="6" t="n">
         <v>2</v>
@@ -4739,8 +4883,8 @@
         <f aca="false">IF(P57="","",IF(O57="",K57,O57)*P57)</f>
         <v>100</v>
       </c>
-      <c r="R57" s="9" t="s">
-        <v>135</v>
+      <c r="R57" s="6" t="s">
+        <v>30</v>
       </c>
       <c r="S57" s="5" t="s">
         <v>246</v>
@@ -4854,7 +4998,7 @@
         <v/>
       </c>
       <c r="R59" s="9" t="s">
-        <v>135</v>
+        <v>154</v>
       </c>
       <c r="S59" s="5" t="s">
         <v>252</v>
@@ -4933,7 +5077,7 @@
         <v/>
       </c>
       <c r="R61" s="9" t="s">
-        <v>135</v>
+        <v>154</v>
       </c>
       <c r="S61" s="5" t="s">
         <v>259</v>
@@ -4987,7 +5131,7 @@
         <v/>
       </c>
       <c r="R62" s="9" t="s">
-        <v>135</v>
+        <v>154</v>
       </c>
       <c r="S62" s="5" t="s">
         <v>263</v>
@@ -5103,7 +5247,7 @@
         <v/>
       </c>
       <c r="R64" s="9" t="s">
-        <v>135</v>
+        <v>154</v>
       </c>
       <c r="S64" s="5" t="s">
         <v>272</v>
@@ -5157,7 +5301,7 @@
         <v/>
       </c>
       <c r="R65" s="9" t="s">
-        <v>135</v>
+        <v>154</v>
       </c>
       <c r="S65" s="5" t="s">
         <v>275</v>
@@ -5236,7 +5380,7 @@
         <v/>
       </c>
       <c r="R67" s="9" t="s">
-        <v>135</v>
+        <v>154</v>
       </c>
       <c r="S67" s="5" t="s">
         <v>281</v>
@@ -5262,38 +5406,46 @@
         <v>102</v>
       </c>
       <c r="G68" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H68" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I68" s="5" t="n">
         <f aca="false">G68*H68</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J68" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K68" s="5" t="n">
         <f aca="false">I68+J68</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L68" s="5" t="s">
         <v>284</v>
       </c>
-      <c r="M68" s="6"/>
-      <c r="N68" s="6"/>
-      <c r="O68" s="6"/>
-      <c r="P68" s="7"/>
-      <c r="Q68" s="8" t="str">
+      <c r="M68" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="N68" s="6" t="s">
+        <v>285</v>
+      </c>
+      <c r="O68" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="P68" s="7" t="n">
+        <v>490</v>
+      </c>
+      <c r="Q68" s="8" t="n">
         <f aca="false">IF(P68="","",IF(O68="",K68,O68)*P68)</f>
-        <v/>
-      </c>
-      <c r="R68" s="9" t="s">
-        <v>135</v>
+        <v>490</v>
+      </c>
+      <c r="R68" s="6" t="s">
+        <v>30</v>
       </c>
       <c r="S68" s="5" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5304,13 +5456,13 @@
         <v>102</v>
       </c>
       <c r="C69" s="5" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="D69" s="5" t="s">
         <v>102</v>
       </c>
       <c r="E69" s="5" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="F69" s="5" t="s">
         <v>102</v>
@@ -5333,121 +5485,121 @@
         <v>1</v>
       </c>
       <c r="L69" s="5" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="M69" s="6" t="s">
-        <v>28</v>
+        <v>43</v>
       </c>
       <c r="N69" s="6" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="O69" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="P69" s="7" t="n">
-        <v>300</v>
+        <v>490</v>
       </c>
       <c r="Q69" s="8" t="n">
         <f aca="false">IF(P69="","",IF(O69="",K69,O69)*P69)</f>
-        <v>900</v>
+        <v>490</v>
       </c>
       <c r="R69" s="6" t="s">
         <v>30</v>
       </c>
       <c r="S69" s="5" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="4" t="s">
         <v>291</v>
       </c>
-      <c r="B70" s="4"/>
-      <c r="C70" s="4" t="s">
+    </row>
+    <row r="70" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="5" t="s">
+        <v>276</v>
+      </c>
+      <c r="B70" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="C70" s="5" t="s">
+        <v>292</v>
+      </c>
+      <c r="D70" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="E70" s="5" t="s">
+        <v>293</v>
+      </c>
+      <c r="F70" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="G70" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H70" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I70" s="5" t="n">
+        <f aca="false">G70*H70</f>
+        <v>1</v>
+      </c>
+      <c r="J70" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K70" s="5" t="n">
+        <f aca="false">I70+J70</f>
+        <v>1</v>
+      </c>
+      <c r="L70" s="5" t="s">
+        <v>294</v>
+      </c>
+      <c r="M70" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="N70" s="6" t="s">
+        <v>295</v>
+      </c>
+      <c r="O70" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="P70" s="7" t="n">
+        <v>300</v>
+      </c>
+      <c r="Q70" s="8" t="n">
+        <f aca="false">IF(P70="","",IF(O70="",K70,O70)*P70)</f>
+        <v>900</v>
+      </c>
+      <c r="R70" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="S70" s="5" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="4" t="s">
+        <v>297</v>
+      </c>
+      <c r="B71" s="4"/>
+      <c r="C71" s="4" t="s">
         <v>175</v>
       </c>
-      <c r="D70" s="4"/>
-      <c r="E70" s="4"/>
-      <c r="F70" s="4"/>
-      <c r="G70" s="4"/>
-      <c r="H70" s="4"/>
-      <c r="I70" s="4"/>
-      <c r="J70" s="4"/>
-      <c r="K70" s="4"/>
-      <c r="L70" s="4"/>
-      <c r="M70" s="4"/>
-      <c r="N70" s="4"/>
-      <c r="O70" s="4"/>
-      <c r="P70" s="4"/>
-      <c r="Q70" s="4"/>
-      <c r="R70" s="4"/>
-      <c r="S70" s="4"/>
-    </row>
-    <row r="71" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="5" t="s">
-        <v>291</v>
-      </c>
-      <c r="B71" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="C71" s="5" t="s">
-        <v>292</v>
-      </c>
-      <c r="D71" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="E71" s="5" t="s">
-        <v>293</v>
-      </c>
-      <c r="F71" s="5" t="s">
-        <v>294</v>
-      </c>
-      <c r="G71" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="H71" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="I71" s="5" t="n">
-        <f aca="false">G71*H71</f>
-        <v>1</v>
-      </c>
-      <c r="J71" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="K71" s="5" t="n">
-        <f aca="false">I71+J71</f>
-        <v>2</v>
-      </c>
-      <c r="L71" s="5" t="s">
-        <v>295</v>
-      </c>
-      <c r="M71" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="N71" s="6" t="s">
-        <v>296</v>
-      </c>
-      <c r="O71" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="P71" s="7" t="n">
-        <v>7790</v>
-      </c>
-      <c r="Q71" s="8" t="n">
-        <f aca="false">IF(P71="","",IF(O71="",K71,O71)*P71)</f>
-        <v>7790</v>
-      </c>
-      <c r="R71" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="S71" s="5" t="s">
-        <v>297</v>
-      </c>
+      <c r="D71" s="4"/>
+      <c r="E71" s="4"/>
+      <c r="F71" s="4"/>
+      <c r="G71" s="4"/>
+      <c r="H71" s="4"/>
+      <c r="I71" s="4"/>
+      <c r="J71" s="4"/>
+      <c r="K71" s="4"/>
+      <c r="L71" s="4"/>
+      <c r="M71" s="4"/>
+      <c r="N71" s="4"/>
+      <c r="O71" s="4"/>
+      <c r="P71" s="4"/>
+      <c r="Q71" s="4"/>
+      <c r="R71" s="4"/>
+      <c r="S71" s="4"/>
     </row>
     <row r="72" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="5" t="s">
-        <v>291</v>
+        <v>297</v>
       </c>
       <c r="B72" s="5" t="s">
         <v>102</v>
@@ -5459,59 +5611,362 @@
         <v>102</v>
       </c>
       <c r="E72" s="5" t="s">
-        <v>171</v>
+        <v>299</v>
       </c>
       <c r="F72" s="5" t="s">
-        <v>102</v>
+        <v>300</v>
       </c>
       <c r="G72" s="5" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="H72" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I72" s="5" t="n">
         <f aca="false">G72*H72</f>
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="J72" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K72" s="5" t="n">
         <f aca="false">I72+J72</f>
+        <v>2</v>
+      </c>
+      <c r="L72" s="5" t="s">
+        <v>301</v>
+      </c>
+      <c r="M72" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="N72" s="6" t="s">
+        <v>302</v>
+      </c>
+      <c r="O72" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="P72" s="7" t="n">
+        <v>7790</v>
+      </c>
+      <c r="Q72" s="8" t="n">
+        <f aca="false">IF(P72="","",IF(O72="",K72,O72)*P72)</f>
+        <v>7790</v>
+      </c>
+      <c r="R72" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="S72" s="5" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="5" t="s">
+        <v>297</v>
+      </c>
+      <c r="B73" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="C73" s="5" t="s">
+        <v>304</v>
+      </c>
+      <c r="D73" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="E73" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="F73" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="G73" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="L72" s="5" t="s">
+      <c r="H73" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I73" s="5" t="n">
+        <f aca="false">G73*H73</f>
+        <v>6</v>
+      </c>
+      <c r="J73" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K73" s="5" t="n">
+        <f aca="false">I73+J73</f>
+        <v>6</v>
+      </c>
+      <c r="L73" s="5" t="s">
         <v>251</v>
       </c>
-      <c r="M72" s="6"/>
-      <c r="N72" s="6"/>
-      <c r="O72" s="6"/>
-      <c r="P72" s="7"/>
-      <c r="Q72" s="8" t="str">
-        <f aca="false">IF(P72="","",IF(O72="",K72,O72)*P72)</f>
+      <c r="M73" s="6"/>
+      <c r="N73" s="6"/>
+      <c r="O73" s="6"/>
+      <c r="P73" s="7"/>
+      <c r="Q73" s="8" t="str">
+        <f aca="false">IF(P73="","",IF(O73="",K73,O73)*P73)</f>
         <v/>
       </c>
-      <c r="R72" s="9" t="s">
-        <v>135</v>
-      </c>
-      <c r="S72" s="5" t="s">
-        <v>299</v>
-      </c>
-    </row>
-    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="P74" s="10" t="s">
-        <v>300</v>
-      </c>
-      <c r="Q74" s="11" t="n">
-        <f aca="false">SUM(Q5:Q72)</f>
-        <v>66503</v>
+      <c r="R73" s="9" t="s">
+        <v>154</v>
+      </c>
+      <c r="S73" s="5" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P75" s="10" t="s">
+        <v>306</v>
+      </c>
+      <c r="Q75" s="11" t="n">
+        <f aca="false">SUM(Q5:Q73)</f>
+        <v>67683</v>
+      </c>
+    </row>
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A77" s="12" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="3" t="s">
+        <v>308</v>
+      </c>
+      <c r="B78" s="3" t="s">
+        <v>309</v>
+      </c>
+      <c r="C78" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D78" s="3" t="s">
+        <v>310</v>
+      </c>
+      <c r="E78" s="3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="79" customFormat="false" ht="115.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="B79" s="13" t="s">
+        <v>311</v>
+      </c>
+      <c r="C79" s="13" t="s">
+        <v>153</v>
+      </c>
+      <c r="D79" s="13" t="s">
+        <v>312</v>
+      </c>
+      <c r="E79" s="13" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="80" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="B80" s="13" t="s">
+        <v>314</v>
+      </c>
+      <c r="C80" s="13" t="s">
+        <v>172</v>
+      </c>
+      <c r="D80" s="13" t="s">
+        <v>315</v>
+      </c>
+      <c r="E80" s="13" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="81" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="B81" s="13" t="s">
+        <v>317</v>
+      </c>
+      <c r="C81" s="13" t="s">
+        <v>251</v>
+      </c>
+      <c r="D81" s="13" t="s">
+        <v>318</v>
+      </c>
+      <c r="E81" s="13" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="82" customFormat="false" ht="90.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A82" s="13" t="n">
+        <v>50</v>
+      </c>
+      <c r="B82" s="13" t="s">
+        <v>320</v>
+      </c>
+      <c r="C82" s="13" t="s">
+        <v>258</v>
+      </c>
+      <c r="D82" s="13" t="s">
+        <v>321</v>
+      </c>
+      <c r="E82" s="13" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="83" customFormat="false" ht="191.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A83" s="13" t="n">
+        <v>8</v>
+      </c>
+      <c r="B83" s="13" t="s">
+        <v>323</v>
+      </c>
+      <c r="C83" s="13" t="s">
+        <v>262</v>
+      </c>
+      <c r="D83" s="13" t="s">
+        <v>324</v>
+      </c>
+      <c r="E83" s="13" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="84" customFormat="false" ht="77.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="13" t="n">
+        <v>8</v>
+      </c>
+      <c r="B84" s="13" t="s">
+        <v>326</v>
+      </c>
+      <c r="C84" s="13" t="s">
+        <v>271</v>
+      </c>
+      <c r="D84" s="13" t="s">
+        <v>327</v>
+      </c>
+      <c r="E84" s="13" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="85" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A85" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="B85" s="13" t="s">
+        <v>273</v>
+      </c>
+      <c r="C85" s="13" t="s">
+        <v>274</v>
+      </c>
+      <c r="D85" s="13" t="s">
+        <v>329</v>
+      </c>
+      <c r="E85" s="13" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="86" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A86" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="B86" s="13" t="s">
+        <v>331</v>
+      </c>
+      <c r="C86" s="13" t="s">
+        <v>280</v>
+      </c>
+      <c r="D86" s="13" t="s">
+        <v>332</v>
+      </c>
+      <c r="E86" s="13"/>
+    </row>
+    <row r="87" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A87" s="13" t="n">
+        <v>6</v>
+      </c>
+      <c r="B87" s="13" t="s">
+        <v>333</v>
+      </c>
+      <c r="C87" s="13" t="s">
+        <v>251</v>
+      </c>
+      <c r="D87" s="13" t="s">
+        <v>318</v>
+      </c>
+      <c r="E87" s="13" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="88" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A88" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="B88" s="13" t="s">
+        <v>335</v>
+      </c>
+      <c r="C88" s="13" t="s">
+        <v>336</v>
+      </c>
+      <c r="D88" s="13" t="s">
+        <v>337</v>
+      </c>
+      <c r="E88" s="13" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="89" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A89" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="B89" s="13" t="s">
+        <v>339</v>
+      </c>
+      <c r="C89" s="13" t="s">
+        <v>340</v>
+      </c>
+      <c r="D89" s="13" t="s">
+        <v>341</v>
+      </c>
+      <c r="E89" s="13" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="90" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A90" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="B90" s="13" t="s">
+        <v>343</v>
+      </c>
+      <c r="C90" s="13" t="s">
+        <v>344</v>
+      </c>
+      <c r="D90" s="13" t="s">
+        <v>341</v>
+      </c>
+      <c r="E90" s="13" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="91" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A91" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="B91" s="13" t="s">
+        <v>346</v>
+      </c>
+      <c r="C91" s="13" t="s">
+        <v>347</v>
+      </c>
+      <c r="D91" s="13" t="s">
+        <v>348</v>
+      </c>
+      <c r="E91" s="13" t="s">
+        <v>349</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:S72"/>
+  <autoFilter ref="A4:S73"/>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="R6:R7 R9:R11 R13:R15 R17:R19 R22:R27 R30:R32 R35:R37 R39:R40 R43:R46 R49:R50 R52 R54 R56:R59 R61:R65 R67:R69 R71:R72" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="R6:R7 R9:R11 R13:R15 R17:R19 R22:R27 R30:R32 R35:R37 R39:R40 R43:R46 R49:R50 R52 R54 R56:R59 R61:R65 R67:R70 R72:R73" type="list">
       <formula1>"Pendiente,En carrito,Comprado,No hay,No aplica"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -5532,7 +5987,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D43"/>
+  <dimension ref="A1:D40"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="70"/>
@@ -5543,7 +5998,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>301</v>
+        <v>350</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5551,268 +6006,268 @@
         <v>2</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>302</v>
+        <v>351</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>303</v>
+        <v>352</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="12" t="s">
+      <c r="A4" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="B4" s="12" t="n">
-        <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$72,A4,'BoM por modulo'!$R$5:$R$72,"&lt;&gt;No aplica",'BoM por modulo'!$R$5:$R$72,"&lt;&gt;")</f>
+      <c r="B4" s="14" t="n">
+        <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$73,A4,'BoM por modulo'!$R$5:$R$73,"&lt;&gt;No aplica",'BoM por modulo'!$R$5:$R$73,"&lt;&gt;")</f>
         <v>2</v>
       </c>
-      <c r="C4" s="12" t="n">
-        <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$72,A4,'BoM por modulo'!$R$5:$R$72,"Pendiente")</f>
+      <c r="C4" s="14" t="n">
+        <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$73,A4,'BoM por modulo'!$R$5:$R$73,"Pendiente")</f>
         <v>0</v>
       </c>
-      <c r="D4" s="13" t="n">
-        <f aca="false">SUMIF('BoM por modulo'!$A$5:$A$72,A4,'BoM por modulo'!$Q$5:$Q$72)</f>
+      <c r="D4" s="15" t="n">
+        <f aca="false">SUMIF('BoM por modulo'!$A$5:$A$73,A4,'BoM por modulo'!$Q$5:$Q$73)</f>
         <v>1744</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="12" t="s">
+      <c r="A5" s="14" t="s">
         <v>37</v>
       </c>
-      <c r="B5" s="12" t="n">
-        <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$72,A5,'BoM por modulo'!$R$5:$R$72,"&lt;&gt;No aplica",'BoM por modulo'!$R$5:$R$72,"&lt;&gt;")</f>
+      <c r="B5" s="14" t="n">
+        <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$73,A5,'BoM por modulo'!$R$5:$R$73,"&lt;&gt;No aplica",'BoM por modulo'!$R$5:$R$73,"&lt;&gt;")</f>
         <v>3</v>
       </c>
-      <c r="C5" s="12" t="n">
-        <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$72,A5,'BoM por modulo'!$R$5:$R$72,"Pendiente")</f>
+      <c r="C5" s="14" t="n">
+        <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$73,A5,'BoM por modulo'!$R$5:$R$73,"Pendiente")</f>
         <v>0</v>
       </c>
-      <c r="D5" s="13" t="n">
-        <f aca="false">SUMIF('BoM por modulo'!$A$5:$A$72,A5,'BoM por modulo'!$Q$5:$Q$72)</f>
+      <c r="D5" s="15" t="n">
+        <f aca="false">SUMIF('BoM por modulo'!$A$5:$A$73,A5,'BoM por modulo'!$Q$5:$Q$73)</f>
         <v>1200</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="12" t="s">
+      <c r="A6" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="B6" s="12" t="n">
-        <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$72,A6,'BoM por modulo'!$R$5:$R$72,"&lt;&gt;No aplica",'BoM por modulo'!$R$5:$R$72,"&lt;&gt;")</f>
+      <c r="B6" s="14" t="n">
+        <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$73,A6,'BoM por modulo'!$R$5:$R$73,"&lt;&gt;No aplica",'BoM por modulo'!$R$5:$R$73,"&lt;&gt;")</f>
         <v>3</v>
       </c>
-      <c r="C6" s="12" t="n">
-        <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$72,A6,'BoM por modulo'!$R$5:$R$72,"Pendiente")</f>
+      <c r="C6" s="14" t="n">
+        <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$73,A6,'BoM por modulo'!$R$5:$R$73,"Pendiente")</f>
         <v>0</v>
       </c>
-      <c r="D6" s="13" t="n">
-        <f aca="false">SUMIF('BoM por modulo'!$A$5:$A$72,A6,'BoM por modulo'!$Q$5:$Q$72)</f>
+      <c r="D6" s="15" t="n">
+        <f aca="false">SUMIF('BoM por modulo'!$A$5:$A$73,A6,'BoM por modulo'!$Q$5:$Q$73)</f>
         <v>27570</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="12" t="s">
+      <c r="A7" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="B7" s="12" t="n">
-        <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$72,A7,'BoM por modulo'!$R$5:$R$72,"&lt;&gt;No aplica",'BoM por modulo'!$R$5:$R$72,"&lt;&gt;")</f>
+      <c r="B7" s="14" t="n">
+        <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$73,A7,'BoM por modulo'!$R$5:$R$73,"&lt;&gt;No aplica",'BoM por modulo'!$R$5:$R$73,"&lt;&gt;")</f>
         <v>3</v>
       </c>
-      <c r="C7" s="12" t="n">
-        <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$72,A7,'BoM por modulo'!$R$5:$R$72,"Pendiente")</f>
+      <c r="C7" s="14" t="n">
+        <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$73,A7,'BoM por modulo'!$R$5:$R$73,"Pendiente")</f>
         <v>0</v>
       </c>
-      <c r="D7" s="13" t="n">
-        <f aca="false">SUMIF('BoM por modulo'!$A$5:$A$72,A7,'BoM por modulo'!$Q$5:$Q$72)</f>
+      <c r="D7" s="15" t="n">
+        <f aca="false">SUMIF('BoM por modulo'!$A$5:$A$73,A7,'BoM por modulo'!$Q$5:$Q$73)</f>
         <v>540</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="12" t="s">
+      <c r="A8" s="14" t="s">
         <v>105</v>
       </c>
-      <c r="B8" s="12" t="n">
-        <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$72,A8,'BoM por modulo'!$R$5:$R$72,"&lt;&gt;No aplica",'BoM por modulo'!$R$5:$R$72,"&lt;&gt;")</f>
+      <c r="B8" s="14" t="n">
+        <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$73,A8,'BoM por modulo'!$R$5:$R$73,"&lt;&gt;No aplica",'BoM por modulo'!$R$5:$R$73,"&lt;&gt;")</f>
         <v>6</v>
       </c>
-      <c r="C8" s="12" t="n">
-        <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$72,A8,'BoM por modulo'!$R$5:$R$72,"Pendiente")</f>
-        <v>1</v>
-      </c>
-      <c r="D8" s="13" t="n">
-        <f aca="false">SUMIF('BoM por modulo'!$A$5:$A$72,A8,'BoM por modulo'!$Q$5:$Q$72)</f>
+      <c r="C8" s="14" t="n">
+        <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$73,A8,'BoM por modulo'!$R$5:$R$73,"Pendiente")</f>
+        <v>0</v>
+      </c>
+      <c r="D8" s="15" t="n">
+        <f aca="false">SUMIF('BoM por modulo'!$A$5:$A$73,A8,'BoM por modulo'!$Q$5:$Q$73)</f>
         <v>1325</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="12" t="s">
-        <v>145</v>
-      </c>
-      <c r="B9" s="12" t="n">
-        <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$72,A9,'BoM por modulo'!$R$5:$R$72,"&lt;&gt;No aplica",'BoM por modulo'!$R$5:$R$72,"&lt;&gt;")</f>
+      <c r="A9" s="14" t="s">
+        <v>144</v>
+      </c>
+      <c r="B9" s="14" t="n">
+        <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$73,A9,'BoM por modulo'!$R$5:$R$73,"&lt;&gt;No aplica",'BoM por modulo'!$R$5:$R$73,"&lt;&gt;")</f>
         <v>3</v>
       </c>
-      <c r="C9" s="12" t="n">
-        <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$72,A9,'BoM por modulo'!$R$5:$R$72,"Pendiente")</f>
-        <v>1</v>
-      </c>
-      <c r="D9" s="13" t="n">
-        <f aca="false">SUMIF('BoM por modulo'!$A$5:$A$72,A9,'BoM por modulo'!$Q$5:$Q$72)</f>
-        <v>560</v>
+      <c r="C9" s="14" t="n">
+        <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$73,A9,'BoM por modulo'!$R$5:$R$73,"Pendiente")</f>
+        <v>1</v>
+      </c>
+      <c r="D9" s="15" t="n">
+        <f aca="false">SUMIF('BoM por modulo'!$A$5:$A$73,A9,'BoM por modulo'!$Q$5:$Q$73)</f>
+        <v>760</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="12" t="s">
+      <c r="A10" s="14" t="s">
         <v>161</v>
       </c>
-      <c r="B10" s="12" t="n">
-        <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$72,A10,'BoM por modulo'!$R$5:$R$72,"&lt;&gt;No aplica",'BoM por modulo'!$R$5:$R$72,"&lt;&gt;")</f>
+      <c r="B10" s="14" t="n">
+        <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$73,A10,'BoM por modulo'!$R$5:$R$73,"&lt;&gt;No aplica",'BoM por modulo'!$R$5:$R$73,"&lt;&gt;")</f>
         <v>3</v>
       </c>
-      <c r="C10" s="12" t="n">
-        <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$72,A10,'BoM por modulo'!$R$5:$R$72,"Pendiente")</f>
-        <v>1</v>
-      </c>
-      <c r="D10" s="13" t="n">
-        <f aca="false">SUMIF('BoM por modulo'!$A$5:$A$72,A10,'BoM por modulo'!$Q$5:$Q$72)</f>
+      <c r="C10" s="14" t="n">
+        <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$73,A10,'BoM por modulo'!$R$5:$R$73,"Pendiente")</f>
+        <v>1</v>
+      </c>
+      <c r="D10" s="15" t="n">
+        <f aca="false">SUMIF('BoM por modulo'!$A$5:$A$73,A10,'BoM por modulo'!$Q$5:$Q$73)</f>
         <v>540</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="12" t="s">
+      <c r="A11" s="14" t="s">
         <v>174</v>
       </c>
-      <c r="B11" s="12" t="n">
-        <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$72,A11,'BoM por modulo'!$R$5:$R$72,"&lt;&gt;No aplica",'BoM por modulo'!$R$5:$R$72,"&lt;&gt;")</f>
+      <c r="B11" s="14" t="n">
+        <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$73,A11,'BoM por modulo'!$R$5:$R$73,"&lt;&gt;No aplica",'BoM por modulo'!$R$5:$R$73,"&lt;&gt;")</f>
         <v>2</v>
       </c>
-      <c r="C11" s="12" t="n">
-        <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$72,A11,'BoM por modulo'!$R$5:$R$72,"Pendiente")</f>
+      <c r="C11" s="14" t="n">
+        <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$73,A11,'BoM por modulo'!$R$5:$R$73,"Pendiente")</f>
         <v>0</v>
       </c>
-      <c r="D11" s="13" t="n">
-        <f aca="false">SUMIF('BoM por modulo'!$A$5:$A$72,A11,'BoM por modulo'!$Q$5:$Q$72)</f>
+      <c r="D11" s="15" t="n">
+        <f aca="false">SUMIF('BoM por modulo'!$A$5:$A$73,A11,'BoM por modulo'!$Q$5:$Q$73)</f>
         <v>584</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="12" t="s">
+      <c r="A12" s="14" t="s">
         <v>184</v>
       </c>
-      <c r="B12" s="12" t="n">
-        <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$72,A12,'BoM por modulo'!$R$5:$R$72,"&lt;&gt;No aplica",'BoM por modulo'!$R$5:$R$72,"&lt;&gt;")</f>
+      <c r="B12" s="14" t="n">
+        <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$73,A12,'BoM por modulo'!$R$5:$R$73,"&lt;&gt;No aplica",'BoM por modulo'!$R$5:$R$73,"&lt;&gt;")</f>
         <v>4</v>
       </c>
-      <c r="C12" s="12" t="n">
-        <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$72,A12,'BoM por modulo'!$R$5:$R$72,"Pendiente")</f>
+      <c r="C12" s="14" t="n">
+        <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$73,A12,'BoM por modulo'!$R$5:$R$73,"Pendiente")</f>
         <v>0</v>
       </c>
-      <c r="D12" s="13" t="n">
-        <f aca="false">SUMIF('BoM por modulo'!$A$5:$A$72,A12,'BoM por modulo'!$Q$5:$Q$72)</f>
+      <c r="D12" s="15" t="n">
+        <f aca="false">SUMIF('BoM por modulo'!$A$5:$A$73,A12,'BoM por modulo'!$Q$5:$Q$73)</f>
         <v>420</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="12" t="s">
+      <c r="A13" s="14" t="s">
         <v>207</v>
       </c>
-      <c r="B13" s="12" t="n">
-        <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$72,A13,'BoM por modulo'!$R$5:$R$72,"&lt;&gt;No aplica",'BoM por modulo'!$R$5:$R$72,"&lt;&gt;")</f>
+      <c r="B13" s="14" t="n">
+        <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$73,A13,'BoM por modulo'!$R$5:$R$73,"&lt;&gt;No aplica",'BoM por modulo'!$R$5:$R$73,"&lt;&gt;")</f>
         <v>3</v>
       </c>
-      <c r="C13" s="12" t="n">
-        <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$72,A13,'BoM por modulo'!$R$5:$R$72,"Pendiente")</f>
+      <c r="C13" s="14" t="n">
+        <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$73,A13,'BoM por modulo'!$R$5:$R$73,"Pendiente")</f>
         <v>0</v>
       </c>
-      <c r="D13" s="13" t="n">
-        <f aca="false">SUMIF('BoM por modulo'!$A$5:$A$72,A13,'BoM por modulo'!$Q$5:$Q$72)</f>
+      <c r="D13" s="15" t="n">
+        <f aca="false">SUMIF('BoM por modulo'!$A$5:$A$73,A13,'BoM por modulo'!$Q$5:$Q$73)</f>
         <v>20660</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="12" t="s">
+      <c r="A14" s="14" t="s">
         <v>225</v>
       </c>
-      <c r="B14" s="12" t="n">
-        <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$72,A14,'BoM por modulo'!$R$5:$R$72,"&lt;&gt;No aplica",'BoM por modulo'!$R$5:$R$72,"&lt;&gt;")</f>
+      <c r="B14" s="14" t="n">
+        <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$73,A14,'BoM por modulo'!$R$5:$R$73,"&lt;&gt;No aplica",'BoM por modulo'!$R$5:$R$73,"&lt;&gt;")</f>
         <v>5</v>
       </c>
-      <c r="C14" s="12" t="n">
-        <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$72,A14,'BoM por modulo'!$R$5:$R$72,"Pendiente")</f>
+      <c r="C14" s="14" t="n">
+        <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$73,A14,'BoM por modulo'!$R$5:$R$73,"Pendiente")</f>
+        <v>1</v>
+      </c>
+      <c r="D14" s="15" t="n">
+        <f aca="false">SUMIF('BoM por modulo'!$A$5:$A$73,A14,'BoM por modulo'!$Q$5:$Q$73)</f>
+        <v>2370</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="14" t="s">
+        <v>253</v>
+      </c>
+      <c r="B15" s="14" t="n">
+        <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$73,A15,'BoM por modulo'!$R$5:$R$73,"&lt;&gt;No aplica",'BoM por modulo'!$R$5:$R$73,"&lt;&gt;")</f>
+        <v>5</v>
+      </c>
+      <c r="C15" s="14" t="n">
+        <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$73,A15,'BoM por modulo'!$R$5:$R$73,"Pendiente")</f>
+        <v>4</v>
+      </c>
+      <c r="D15" s="15" t="n">
+        <f aca="false">SUMIF('BoM por modulo'!$A$5:$A$73,A15,'BoM por modulo'!$Q$5:$Q$73)</f>
+        <v>300</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="14" t="s">
+        <v>276</v>
+      </c>
+      <c r="B16" s="14" t="n">
+        <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$73,A16,'BoM por modulo'!$R$5:$R$73,"&lt;&gt;No aplica",'BoM por modulo'!$R$5:$R$73,"&lt;&gt;")</f>
+        <v>4</v>
+      </c>
+      <c r="C16" s="14" t="n">
+        <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$73,A16,'BoM por modulo'!$R$5:$R$73,"Pendiente")</f>
+        <v>1</v>
+      </c>
+      <c r="D16" s="15" t="n">
+        <f aca="false">SUMIF('BoM por modulo'!$A$5:$A$73,A16,'BoM por modulo'!$Q$5:$Q$73)</f>
+        <v>1880</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="14" t="s">
+        <v>297</v>
+      </c>
+      <c r="B17" s="14" t="n">
+        <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$73,A17,'BoM por modulo'!$R$5:$R$73,"&lt;&gt;No aplica",'BoM por modulo'!$R$5:$R$73,"&lt;&gt;")</f>
         <v>2</v>
       </c>
-      <c r="D14" s="13" t="n">
-        <f aca="false">SUMIF('BoM por modulo'!$A$5:$A$72,A14,'BoM por modulo'!$Q$5:$Q$72)</f>
-        <v>2370</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="12" t="s">
-        <v>253</v>
-      </c>
-      <c r="B15" s="12" t="n">
-        <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$72,A15,'BoM por modulo'!$R$5:$R$72,"&lt;&gt;No aplica",'BoM por modulo'!$R$5:$R$72,"&lt;&gt;")</f>
-        <v>5</v>
-      </c>
-      <c r="C15" s="12" t="n">
-        <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$72,A15,'BoM por modulo'!$R$5:$R$72,"Pendiente")</f>
-        <v>4</v>
-      </c>
-      <c r="D15" s="13" t="n">
-        <f aca="false">SUMIF('BoM por modulo'!$A$5:$A$72,A15,'BoM por modulo'!$Q$5:$Q$72)</f>
-        <v>300</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="12" t="s">
-        <v>276</v>
-      </c>
-      <c r="B16" s="12" t="n">
-        <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$72,A16,'BoM por modulo'!$R$5:$R$72,"&lt;&gt;No aplica",'BoM por modulo'!$R$5:$R$72,"&lt;&gt;")</f>
-        <v>3</v>
-      </c>
-      <c r="C16" s="12" t="n">
-        <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$72,A16,'BoM por modulo'!$R$5:$R$72,"Pendiente")</f>
-        <v>2</v>
-      </c>
-      <c r="D16" s="13" t="n">
-        <f aca="false">SUMIF('BoM por modulo'!$A$5:$A$72,A16,'BoM por modulo'!$Q$5:$Q$72)</f>
-        <v>900</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="12" t="s">
-        <v>291</v>
-      </c>
-      <c r="B17" s="12" t="n">
-        <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$72,A17,'BoM por modulo'!$R$5:$R$72,"&lt;&gt;No aplica",'BoM por modulo'!$R$5:$R$72,"&lt;&gt;")</f>
-        <v>2</v>
-      </c>
-      <c r="C17" s="12" t="n">
-        <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$72,A17,'BoM por modulo'!$R$5:$R$72,"Pendiente")</f>
-        <v>1</v>
-      </c>
-      <c r="D17" s="13" t="n">
-        <f aca="false">SUMIF('BoM por modulo'!$A$5:$A$72,A17,'BoM por modulo'!$Q$5:$Q$72)</f>
+      <c r="C17" s="14" t="n">
+        <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$73,A17,'BoM por modulo'!$R$5:$R$73,"Pendiente")</f>
+        <v>1</v>
+      </c>
+      <c r="D17" s="15" t="n">
+        <f aca="false">SUMIF('BoM por modulo'!$A$5:$A$73,A17,'BoM por modulo'!$Q$5:$Q$73)</f>
         <v>7790</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="14" t="s">
-        <v>300</v>
-      </c>
-      <c r="B18" s="14" t="n">
+      <c r="A18" s="16" t="s">
+        <v>306</v>
+      </c>
+      <c r="B18" s="16" t="n">
         <f aca="false">SUM(B4:B17)</f>
-        <v>47</v>
-      </c>
-      <c r="C18" s="14" t="n">
+        <v>48</v>
+      </c>
+      <c r="C18" s="16" t="n">
         <f aca="false">SUM(C4:C17)</f>
-        <v>12</v>
-      </c>
-      <c r="D18" s="15" t="n">
+        <v>9</v>
+      </c>
+      <c r="D18" s="17" t="n">
         <f aca="false">SUM(D4:D17)</f>
-        <v>66503</v>
+        <v>67683</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5820,168 +6275,144 @@
         <v>14</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>304</v>
+        <v>353</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>305</v>
+        <v>354</v>
       </c>
       <c r="D20" s="3"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="16" t="s">
+      <c r="A21" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="B21" s="17" t="n">
-        <f aca="false">SUMIFS('BoM por modulo'!$Q$5:$Q$72,'BoM por modulo'!$M$5:$M$72,A21,'BoM por modulo'!$R$5:$R$72,"En carrito")</f>
-        <v>37683</v>
-      </c>
-      <c r="C21" s="17" t="n">
-        <f aca="false">SUMIFS('BoM por modulo'!$Q$5:$Q$72,'BoM por modulo'!$M$5:$M$72,A21,'BoM por modulo'!$R$5:$R$72,"Pendiente")</f>
-        <v>860</v>
+      <c r="B21" s="19" t="n">
+        <f aca="false">SUMIFS('BoM por modulo'!$Q$5:$Q$73,'BoM por modulo'!$M$5:$M$73,A21,'BoM por modulo'!$R$5:$R$73,"En carrito")</f>
+        <v>38793</v>
+      </c>
+      <c r="C21" s="19" t="n">
+        <f aca="false">SUMIFS('BoM por modulo'!$Q$5:$Q$73,'BoM por modulo'!$M$5:$M$73,A21,'BoM por modulo'!$R$5:$R$73,"Pendiente")</f>
+        <v>440</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="16" t="s">
+      <c r="A22" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="B22" s="17" t="n">
-        <f aca="false">SUMIFS('BoM por modulo'!$Q$5:$Q$72,'BoM por modulo'!$M$5:$M$72,A22,'BoM por modulo'!$R$5:$R$72,"En carrito")</f>
-        <v>27960</v>
-      </c>
-      <c r="C22" s="17" t="n">
-        <f aca="false">SUMIFS('BoM por modulo'!$Q$5:$Q$72,'BoM por modulo'!$M$5:$M$72,A22,'BoM por modulo'!$R$5:$R$72,"Pendiente")</f>
+      <c r="B22" s="19" t="n">
+        <f aca="false">SUMIFS('BoM por modulo'!$Q$5:$Q$73,'BoM por modulo'!$M$5:$M$73,A22,'BoM por modulo'!$R$5:$R$73,"En carrito")</f>
+        <v>28450</v>
+      </c>
+      <c r="C22" s="19" t="n">
+        <f aca="false">SUMIFS('BoM por modulo'!$Q$5:$Q$73,'BoM por modulo'!$M$5:$M$73,A22,'BoM por modulo'!$R$5:$R$73,"Pendiente")</f>
         <v>0</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="18" t="s">
-        <v>306</v>
+      <c r="A24" s="20" t="s">
+        <v>355</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="16" t="s">
-        <v>307</v>
-      </c>
-      <c r="B25" s="19" t="s">
-        <v>308</v>
+      <c r="A25" s="18" t="s">
+        <v>356</v>
+      </c>
+      <c r="B25" s="21" t="s">
+        <v>357</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="16" t="s">
-        <v>309</v>
-      </c>
-      <c r="B26" s="19" t="s">
-        <v>310</v>
+      <c r="A26" s="18" t="s">
+        <v>358</v>
+      </c>
+      <c r="B26" s="21" t="s">
+        <v>172</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="16" t="s">
-        <v>311</v>
-      </c>
-      <c r="B27" s="19" t="s">
-        <v>172</v>
+      <c r="A27" s="18" t="s">
+        <v>359</v>
+      </c>
+      <c r="B27" s="21" t="s">
+        <v>251</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="16" t="s">
-        <v>312</v>
-      </c>
-      <c r="B28" s="19" t="s">
-        <v>313</v>
+      <c r="A28" s="18" t="s">
+        <v>360</v>
+      </c>
+      <c r="B28" s="21" t="s">
+        <v>258</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="16" t="s">
-        <v>314</v>
-      </c>
-      <c r="B29" s="19" t="s">
+      <c r="A29" s="18" t="s">
+        <v>361</v>
+      </c>
+      <c r="B29" s="21" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="18" t="s">
+        <v>362</v>
+      </c>
+      <c r="B30" s="21" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="18" t="s">
+        <v>363</v>
+      </c>
+      <c r="B31" s="21" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="18" t="s">
+        <v>364</v>
+      </c>
+      <c r="B32" s="21" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="18" t="s">
+        <v>365</v>
+      </c>
+      <c r="B33" s="21" t="s">
         <v>251</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="16" t="s">
-        <v>315</v>
-      </c>
-      <c r="B30" s="19" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="16" t="s">
-        <v>316</v>
-      </c>
-      <c r="B31" s="19" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="16" t="s">
-        <v>317</v>
-      </c>
-      <c r="B32" s="19" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="16" t="s">
-        <v>318</v>
-      </c>
-      <c r="B33" s="19" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="16" t="s">
-        <v>319</v>
-      </c>
-      <c r="B34" s="19" t="s">
-        <v>280</v>
-      </c>
-    </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="16" t="s">
-        <v>320</v>
-      </c>
-      <c r="B35" s="19" t="s">
-        <v>284</v>
+      <c r="A35" s="10" t="s">
+        <v>366</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="16" t="s">
-        <v>321</v>
-      </c>
-      <c r="B36" s="19" t="s">
-        <v>251</v>
+      <c r="A36" s="18" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="18" t="s">
+        <v>368</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="10" t="s">
-        <v>322</v>
+      <c r="A38" s="18" t="s">
+        <v>369</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="16" t="s">
-        <v>323</v>
+      <c r="A39" s="18" t="s">
+        <v>370</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="16" t="s">
-        <v>324</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="16" t="s">
-        <v>325</v>
-      </c>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="16" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="16" t="s">
-        <v>327</v>
+      <c r="A40" s="18" t="s">
+        <v>371</v>
       </c>
     </row>
   </sheetData>
@@ -6010,398 +6441,398 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>328</v>
+        <v>372</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>329</v>
+        <v>373</v>
       </c>
       <c r="B3" s="4"/>
       <c r="C3" s="4"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>330</v>
+        <v>374</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>331</v>
+        <v>375</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>332</v>
+        <v>376</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="20" t="s">
-        <v>333</v>
-      </c>
-      <c r="B5" s="21" t="s">
-        <v>334</v>
-      </c>
-      <c r="C5" s="21" t="s">
-        <v>335</v>
+      <c r="A5" s="22" t="s">
+        <v>377</v>
+      </c>
+      <c r="B5" s="13" t="s">
+        <v>378</v>
+      </c>
+      <c r="C5" s="13" t="s">
+        <v>379</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="20" t="s">
-        <v>336</v>
-      </c>
-      <c r="B6" s="21" t="s">
-        <v>337</v>
-      </c>
-      <c r="C6" s="21" t="s">
-        <v>338</v>
+      <c r="A6" s="22" t="s">
+        <v>380</v>
+      </c>
+      <c r="B6" s="13" t="s">
+        <v>381</v>
+      </c>
+      <c r="C6" s="13" t="s">
+        <v>382</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="20" t="s">
-        <v>339</v>
-      </c>
-      <c r="B7" s="21" t="s">
-        <v>340</v>
-      </c>
-      <c r="C7" s="21" t="s">
-        <v>341</v>
+      <c r="A7" s="22" t="s">
+        <v>383</v>
+      </c>
+      <c r="B7" s="13" t="s">
+        <v>384</v>
+      </c>
+      <c r="C7" s="13" t="s">
+        <v>385</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="20" t="s">
-        <v>342</v>
-      </c>
-      <c r="B8" s="21" t="s">
-        <v>343</v>
-      </c>
-      <c r="C8" s="21" t="s">
-        <v>344</v>
+      <c r="A8" s="22" t="s">
+        <v>386</v>
+      </c>
+      <c r="B8" s="13" t="s">
+        <v>387</v>
+      </c>
+      <c r="C8" s="13" t="s">
+        <v>388</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="20" t="s">
-        <v>345</v>
-      </c>
-      <c r="B9" s="21" t="s">
-        <v>346</v>
-      </c>
-      <c r="C9" s="21" t="s">
-        <v>347</v>
+      <c r="A9" s="22" t="s">
+        <v>389</v>
+      </c>
+      <c r="B9" s="13" t="s">
+        <v>390</v>
+      </c>
+      <c r="C9" s="13" t="s">
+        <v>391</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="20" t="s">
-        <v>348</v>
-      </c>
-      <c r="B10" s="21" t="s">
-        <v>349</v>
-      </c>
-      <c r="C10" s="21" t="s">
-        <v>350</v>
+      <c r="A10" s="22" t="s">
+        <v>392</v>
+      </c>
+      <c r="B10" s="13" t="s">
+        <v>393</v>
+      </c>
+      <c r="C10" s="13" t="s">
+        <v>394</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="20" t="s">
-        <v>351</v>
-      </c>
-      <c r="B11" s="21" t="s">
-        <v>352</v>
-      </c>
-      <c r="C11" s="21" t="s">
-        <v>353</v>
+      <c r="A11" s="22" t="s">
+        <v>395</v>
+      </c>
+      <c r="B11" s="13" t="s">
+        <v>396</v>
+      </c>
+      <c r="C11" s="13" t="s">
+        <v>397</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="20" t="s">
-        <v>354</v>
-      </c>
-      <c r="B12" s="21" t="s">
-        <v>355</v>
-      </c>
-      <c r="C12" s="21" t="s">
-        <v>356</v>
+      <c r="A12" s="22" t="s">
+        <v>398</v>
+      </c>
+      <c r="B12" s="13" t="s">
+        <v>399</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>400</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="20" t="s">
-        <v>357</v>
-      </c>
-      <c r="B13" s="21" t="s">
-        <v>358</v>
-      </c>
-      <c r="C13" s="21" t="s">
-        <v>359</v>
+      <c r="A13" s="22" t="s">
+        <v>401</v>
+      </c>
+      <c r="B13" s="13" t="s">
+        <v>402</v>
+      </c>
+      <c r="C13" s="13" t="s">
+        <v>403</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="20" t="s">
-        <v>360</v>
-      </c>
-      <c r="B14" s="21" t="s">
-        <v>361</v>
-      </c>
-      <c r="C14" s="21" t="s">
+      <c r="A14" s="22" t="s">
+        <v>404</v>
+      </c>
+      <c r="B14" s="13" t="s">
+        <v>405</v>
+      </c>
+      <c r="C14" s="13" t="s">
         <v>277</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="20" t="s">
-        <v>362</v>
-      </c>
-      <c r="B15" s="21" t="s">
-        <v>363</v>
-      </c>
-      <c r="C15" s="21"/>
+      <c r="A15" s="22" t="s">
+        <v>406</v>
+      </c>
+      <c r="B15" s="13" t="s">
+        <v>407</v>
+      </c>
+      <c r="C15" s="13"/>
     </row>
     <row r="16" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="20" t="s">
-        <v>364</v>
-      </c>
-      <c r="B16" s="21" t="s">
-        <v>365</v>
-      </c>
-      <c r="C16" s="21"/>
+      <c r="A16" s="22" t="s">
+        <v>408</v>
+      </c>
+      <c r="B16" s="13" t="s">
+        <v>409</v>
+      </c>
+      <c r="C16" s="13"/>
     </row>
     <row r="17" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="20" t="s">
-        <v>366</v>
-      </c>
-      <c r="B17" s="21" t="s">
-        <v>367</v>
-      </c>
-      <c r="C17" s="21"/>
+      <c r="A17" s="22" t="s">
+        <v>410</v>
+      </c>
+      <c r="B17" s="13" t="s">
+        <v>411</v>
+      </c>
+      <c r="C17" s="13"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>368</v>
+        <v>412</v>
       </c>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>330</v>
+        <v>374</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>331</v>
+        <v>375</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>332</v>
+        <v>376</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="20" t="s">
-        <v>333</v>
-      </c>
-      <c r="B21" s="21" t="s">
-        <v>369</v>
-      </c>
-      <c r="C21" s="21" t="s">
-        <v>370</v>
+      <c r="A21" s="22" t="s">
+        <v>377</v>
+      </c>
+      <c r="B21" s="13" t="s">
+        <v>413</v>
+      </c>
+      <c r="C21" s="13" t="s">
+        <v>414</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="20" t="s">
-        <v>371</v>
-      </c>
-      <c r="B22" s="21" t="s">
-        <v>372</v>
-      </c>
-      <c r="C22" s="21" t="s">
-        <v>373</v>
+      <c r="A22" s="22" t="s">
+        <v>415</v>
+      </c>
+      <c r="B22" s="13" t="s">
+        <v>416</v>
+      </c>
+      <c r="C22" s="13" t="s">
+        <v>417</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="20" t="s">
-        <v>339</v>
-      </c>
-      <c r="B23" s="21" t="s">
-        <v>374</v>
-      </c>
-      <c r="C23" s="21" t="s">
-        <v>375</v>
+      <c r="A23" s="22" t="s">
+        <v>383</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>418</v>
+      </c>
+      <c r="C23" s="13" t="s">
+        <v>419</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="20" t="s">
-        <v>376</v>
-      </c>
-      <c r="B24" s="21" t="s">
-        <v>377</v>
-      </c>
-      <c r="C24" s="21" t="s">
-        <v>378</v>
+      <c r="A24" s="22" t="s">
+        <v>420</v>
+      </c>
+      <c r="B24" s="13" t="s">
+        <v>421</v>
+      </c>
+      <c r="C24" s="13" t="s">
+        <v>422</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="20" t="s">
-        <v>379</v>
-      </c>
-      <c r="B25" s="21" t="s">
-        <v>380</v>
-      </c>
-      <c r="C25" s="21" t="s">
-        <v>381</v>
+      <c r="A25" s="22" t="s">
+        <v>423</v>
+      </c>
+      <c r="B25" s="13" t="s">
+        <v>424</v>
+      </c>
+      <c r="C25" s="13" t="s">
+        <v>425</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="20" t="s">
-        <v>382</v>
-      </c>
-      <c r="B26" s="21" t="s">
-        <v>383</v>
-      </c>
-      <c r="C26" s="21" t="s">
-        <v>384</v>
+      <c r="A26" s="22" t="s">
+        <v>426</v>
+      </c>
+      <c r="B26" s="13" t="s">
+        <v>427</v>
+      </c>
+      <c r="C26" s="13" t="s">
+        <v>428</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="20" t="s">
-        <v>348</v>
-      </c>
-      <c r="B27" s="21" t="s">
-        <v>385</v>
-      </c>
-      <c r="C27" s="21" t="s">
-        <v>386</v>
+      <c r="A27" s="22" t="s">
+        <v>392</v>
+      </c>
+      <c r="B27" s="13" t="s">
+        <v>429</v>
+      </c>
+      <c r="C27" s="13" t="s">
+        <v>430</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="20" t="s">
-        <v>354</v>
-      </c>
-      <c r="B28" s="21" t="s">
-        <v>387</v>
-      </c>
-      <c r="C28" s="21" t="s">
-        <v>388</v>
+      <c r="A28" s="22" t="s">
+        <v>398</v>
+      </c>
+      <c r="B28" s="13" t="s">
+        <v>431</v>
+      </c>
+      <c r="C28" s="13" t="s">
+        <v>432</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="20" t="s">
-        <v>389</v>
-      </c>
-      <c r="B29" s="21" t="s">
-        <v>390</v>
-      </c>
-      <c r="C29" s="21" t="s">
-        <v>391</v>
+      <c r="A29" s="22" t="s">
+        <v>433</v>
+      </c>
+      <c r="B29" s="13" t="s">
+        <v>434</v>
+      </c>
+      <c r="C29" s="13" t="s">
+        <v>435</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="20" t="s">
-        <v>360</v>
-      </c>
-      <c r="B30" s="21" t="s">
-        <v>392</v>
-      </c>
-      <c r="C30" s="21" t="s">
+      <c r="A30" s="22" t="s">
+        <v>404</v>
+      </c>
+      <c r="B30" s="13" t="s">
+        <v>436</v>
+      </c>
+      <c r="C30" s="13" t="s">
         <v>277</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="20" t="s">
-        <v>362</v>
-      </c>
-      <c r="B31" s="21" t="s">
-        <v>393</v>
-      </c>
-      <c r="C31" s="21"/>
+      <c r="A31" s="22" t="s">
+        <v>406</v>
+      </c>
+      <c r="B31" s="13" t="s">
+        <v>437</v>
+      </c>
+      <c r="C31" s="13"/>
     </row>
     <row r="32" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="20" t="s">
-        <v>364</v>
-      </c>
-      <c r="B32" s="21" t="s">
-        <v>394</v>
-      </c>
-      <c r="C32" s="21" t="s">
-        <v>395</v>
+      <c r="A32" s="22" t="s">
+        <v>408</v>
+      </c>
+      <c r="B32" s="13" t="s">
+        <v>438</v>
+      </c>
+      <c r="C32" s="13" t="s">
+        <v>439</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="20" t="s">
-        <v>366</v>
-      </c>
-      <c r="B33" s="21" t="s">
-        <v>396</v>
-      </c>
-      <c r="C33" s="21"/>
+      <c r="A33" s="22" t="s">
+        <v>410</v>
+      </c>
+      <c r="B33" s="13" t="s">
+        <v>440</v>
+      </c>
+      <c r="C33" s="13"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="s">
-        <v>397</v>
+        <v>441</v>
       </c>
       <c r="B35" s="4"/>
       <c r="C35" s="4"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="3" t="s">
-        <v>330</v>
+        <v>374</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>331</v>
+        <v>375</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>332</v>
+        <v>376</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="20" t="s">
-        <v>371</v>
-      </c>
-      <c r="B37" s="21" t="s">
-        <v>398</v>
-      </c>
-      <c r="C37" s="21" t="s">
-        <v>399</v>
+      <c r="A37" s="22" t="s">
+        <v>415</v>
+      </c>
+      <c r="B37" s="13" t="s">
+        <v>442</v>
+      </c>
+      <c r="C37" s="13" t="s">
+        <v>443</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="20" t="s">
-        <v>400</v>
-      </c>
-      <c r="B38" s="21" t="s">
-        <v>401</v>
-      </c>
-      <c r="C38" s="21" t="s">
-        <v>402</v>
+      <c r="A38" s="22" t="s">
+        <v>444</v>
+      </c>
+      <c r="B38" s="13" t="s">
+        <v>445</v>
+      </c>
+      <c r="C38" s="13" t="s">
+        <v>446</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="20" t="s">
-        <v>403</v>
-      </c>
-      <c r="B39" s="21" t="s">
-        <v>404</v>
-      </c>
-      <c r="C39" s="21"/>
+      <c r="A39" s="22" t="s">
+        <v>447</v>
+      </c>
+      <c r="B39" s="13" t="s">
+        <v>448</v>
+      </c>
+      <c r="C39" s="13"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="20" t="s">
-        <v>362</v>
-      </c>
-      <c r="B40" s="21" t="s">
-        <v>405</v>
-      </c>
-      <c r="C40" s="21" t="s">
+      <c r="A40" s="22" t="s">
         <v>406</v>
       </c>
+      <c r="B40" s="13" t="s">
+        <v>449</v>
+      </c>
+      <c r="C40" s="13" t="s">
+        <v>450</v>
+      </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="20" t="s">
-        <v>364</v>
-      </c>
-      <c r="B41" s="21" t="s">
-        <v>407</v>
-      </c>
-      <c r="C41" s="21"/>
+      <c r="A41" s="22" t="s">
+        <v>408</v>
+      </c>
+      <c r="B41" s="13" t="s">
+        <v>451</v>
+      </c>
+      <c r="C41" s="13"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="20" t="s">
-        <v>408</v>
-      </c>
-      <c r="B42" s="21" t="s">
-        <v>409</v>
-      </c>
-      <c r="C42" s="21"/>
+      <c r="A42" s="22" t="s">
+        <v>452</v>
+      </c>
+      <c r="B42" s="13" t="s">
+        <v>453</v>
+      </c>
+      <c r="C42" s="13"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -6431,7 +6862,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>410</v>
+        <v>454</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6439,186 +6870,186 @@
         <v>14</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>411</v>
+        <v>455</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>412</v>
+        <v>456</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>413</v>
+        <v>457</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>414</v>
+        <v>458</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="21" t="s">
+      <c r="A4" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="B4" s="21" t="s">
-        <v>415</v>
-      </c>
-      <c r="C4" s="21" t="s">
-        <v>416</v>
-      </c>
-      <c r="D4" s="21" t="s">
-        <v>417</v>
-      </c>
-      <c r="E4" s="21" t="s">
-        <v>418</v>
+      <c r="B4" s="13" t="s">
+        <v>459</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>460</v>
+      </c>
+      <c r="D4" s="13" t="s">
+        <v>461</v>
+      </c>
+      <c r="E4" s="13" t="s">
+        <v>462</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="21" t="s">
-        <v>419</v>
-      </c>
-      <c r="B5" s="21" t="s">
-        <v>420</v>
-      </c>
-      <c r="C5" s="21" t="s">
-        <v>421</v>
-      </c>
-      <c r="D5" s="21" t="s">
-        <v>422</v>
-      </c>
-      <c r="E5" s="21" t="s">
-        <v>423</v>
+      <c r="A5" s="13" t="s">
+        <v>463</v>
+      </c>
+      <c r="B5" s="13" t="s">
+        <v>464</v>
+      </c>
+      <c r="C5" s="13" t="s">
+        <v>465</v>
+      </c>
+      <c r="D5" s="13" t="s">
+        <v>466</v>
+      </c>
+      <c r="E5" s="13" t="s">
+        <v>467</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="21" t="s">
-        <v>424</v>
-      </c>
-      <c r="B6" s="21" t="s">
-        <v>415</v>
-      </c>
-      <c r="C6" s="21" t="s">
-        <v>425</v>
-      </c>
-      <c r="D6" s="21" t="s">
-        <v>426</v>
-      </c>
-      <c r="E6" s="21" t="s">
-        <v>427</v>
+      <c r="A6" s="13" t="s">
+        <v>468</v>
+      </c>
+      <c r="B6" s="13" t="s">
+        <v>459</v>
+      </c>
+      <c r="C6" s="13" t="s">
+        <v>469</v>
+      </c>
+      <c r="D6" s="13" t="s">
+        <v>470</v>
+      </c>
+      <c r="E6" s="13" t="s">
+        <v>471</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="21" t="s">
-        <v>428</v>
-      </c>
-      <c r="B7" s="21" t="s">
-        <v>415</v>
-      </c>
-      <c r="C7" s="21" t="s">
-        <v>429</v>
-      </c>
-      <c r="D7" s="21" t="s">
-        <v>430</v>
-      </c>
-      <c r="E7" s="21" t="s">
-        <v>431</v>
+      <c r="A7" s="13" t="s">
+        <v>472</v>
+      </c>
+      <c r="B7" s="13" t="s">
+        <v>459</v>
+      </c>
+      <c r="C7" s="13" t="s">
+        <v>473</v>
+      </c>
+      <c r="D7" s="13" t="s">
+        <v>474</v>
+      </c>
+      <c r="E7" s="13" t="s">
+        <v>475</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="21" t="s">
-        <v>432</v>
-      </c>
-      <c r="B8" s="21" t="s">
-        <v>415</v>
-      </c>
-      <c r="C8" s="21" t="s">
-        <v>433</v>
-      </c>
-      <c r="D8" s="21" t="s">
-        <v>434</v>
-      </c>
-      <c r="E8" s="21" t="s">
-        <v>435</v>
+      <c r="A8" s="13" t="s">
+        <v>476</v>
+      </c>
+      <c r="B8" s="13" t="s">
+        <v>459</v>
+      </c>
+      <c r="C8" s="13" t="s">
+        <v>477</v>
+      </c>
+      <c r="D8" s="13" t="s">
+        <v>478</v>
+      </c>
+      <c r="E8" s="13" t="s">
+        <v>479</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="21" t="s">
+      <c r="A9" s="13" t="s">
         <v>43</v>
       </c>
-      <c r="B9" s="21" t="s">
-        <v>436</v>
-      </c>
-      <c r="C9" s="21" t="s">
-        <v>437</v>
-      </c>
-      <c r="D9" s="21" t="s">
-        <v>438</v>
-      </c>
-      <c r="E9" s="21" t="s">
-        <v>439</v>
+      <c r="B9" s="13" t="s">
+        <v>480</v>
+      </c>
+      <c r="C9" s="13" t="s">
+        <v>481</v>
+      </c>
+      <c r="D9" s="13" t="s">
+        <v>482</v>
+      </c>
+      <c r="E9" s="13" t="s">
+        <v>483</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="21" t="s">
-        <v>440</v>
-      </c>
-      <c r="B10" s="21" t="s">
+      <c r="A10" s="13" t="s">
+        <v>484</v>
+      </c>
+      <c r="B10" s="13" t="s">
         <v>102</v>
       </c>
-      <c r="C10" s="21" t="s">
-        <v>441</v>
-      </c>
-      <c r="D10" s="21" t="s">
-        <v>442</v>
-      </c>
-      <c r="E10" s="21" t="s">
-        <v>443</v>
+      <c r="C10" s="13" t="s">
+        <v>485</v>
+      </c>
+      <c r="D10" s="13" t="s">
+        <v>486</v>
+      </c>
+      <c r="E10" s="13" t="s">
+        <v>487</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="21" t="s">
-        <v>444</v>
-      </c>
-      <c r="B11" s="21" t="s">
+      <c r="A11" s="13" t="s">
+        <v>488</v>
+      </c>
+      <c r="B11" s="13" t="s">
         <v>102</v>
       </c>
-      <c r="C11" s="21" t="s">
-        <v>445</v>
-      </c>
-      <c r="D11" s="21" t="s">
-        <v>446</v>
-      </c>
-      <c r="E11" s="21" t="s">
-        <v>447</v>
+      <c r="C11" s="13" t="s">
+        <v>489</v>
+      </c>
+      <c r="D11" s="13" t="s">
+        <v>490</v>
+      </c>
+      <c r="E11" s="13" t="s">
+        <v>491</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="21" t="s">
-        <v>448</v>
-      </c>
-      <c r="B12" s="21" t="s">
-        <v>415</v>
-      </c>
-      <c r="C12" s="21" t="s">
-        <v>449</v>
-      </c>
-      <c r="D12" s="21" t="s">
-        <v>450</v>
-      </c>
-      <c r="E12" s="21" t="s">
-        <v>451</v>
+      <c r="A12" s="13" t="s">
+        <v>492</v>
+      </c>
+      <c r="B12" s="13" t="s">
+        <v>459</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>493</v>
+      </c>
+      <c r="D12" s="13" t="s">
+        <v>494</v>
+      </c>
+      <c r="E12" s="13" t="s">
+        <v>495</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="21" t="s">
-        <v>452</v>
-      </c>
-      <c r="B13" s="21" t="s">
-        <v>453</v>
-      </c>
-      <c r="C13" s="21" t="s">
-        <v>454</v>
-      </c>
-      <c r="D13" s="21" t="s">
-        <v>455</v>
-      </c>
-      <c r="E13" s="21" t="s">
-        <v>456</v>
+      <c r="A13" s="13" t="s">
+        <v>496</v>
+      </c>
+      <c r="B13" s="13" t="s">
+        <v>497</v>
+      </c>
+      <c r="C13" s="13" t="s">
+        <v>498</v>
+      </c>
+      <c r="D13" s="13" t="s">
+        <v>499</v>
+      </c>
+      <c r="E13" s="13" t="s">
+        <v>500</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
BoM: C21 y tiras Dupont en carrito; perfboard e insumos ya disponibles; falta solo electrodos, cables y alcohol
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V5Cz1Wb6HSRhqzouEW9mso
</commit_message>
<xml_diff>
--- a/docs/afe-emg/BoM_AFE_AuraVox.xlsx
+++ b/docs/afe-emg/BoM_AFE_AuraVox.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="871" uniqueCount="501">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="830" uniqueCount="469">
   <si>
     <t xml:space="preserve">BoM AFE sEMG AuraVox: 3 canales (submentoniano, labio inferior, laringe), 7 electrodos, RLD. Ordenada por modulo, igual que los recuadros del esquematico LTspice (sim/ltspice).</t>
   </si>
@@ -490,321 +490,330 @@
     <t xml:space="preserve">2A103J poliester 10nF 100V + 2A472K poliester 4.7nF 100V, en paralelo (par)</t>
   </si>
   <si>
+    <t xml:space="preserve">15 nF agotado (2A153J en Global; tampoco en MechatronicStore): 10n + 4.7n en paralelo = 14.7 nF (f0 +1 %, Q -1 %). Cantidad en pares; precio del par ($50 + $60)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.2n</t>
+  </si>
+  <si>
+    <t xml:space="preserve">condensador poliester 2.2nF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C222NPO05D disco NPO 2.2nF 50V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">XLB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7 BUCKET + SALIDA AL ADC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rbk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resistencia del bucket</t>
+  </si>
+  <si>
+    <t xml:space="preserve">100</t>
+  </si>
+  <si>
+    <t xml:space="preserve">resistencia 100 ohm 1%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R1W100 carbon 1 W 100 ohm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cbk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Condensador del bucket</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ADCk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cable a Arduino A1..A3 del STM32N6570-DK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">jumper Dupont M-H</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cable dupont macho-hembra (tira de 40)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Por confirmar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tira de 40 jumpers Dupont M-H (compartida: A1-A3, 5 V/GND, microfono)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Llenar tienda y precio de la tira. CH1-A1 (PA9), CH2-A2 (PA10), CH3-A3 (PA12). Mas 1 cable de GND. A0 no: comparte ADC con USB1 ISENSE (UM3300)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8 VREF 1.65 V (compartido)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">compartido</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RA1, RA2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Divisor de VREF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">resistencia 100k 1%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Condensador del divisor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ceramico X7R o electrolitico</t>
+  </si>
+  <si>
+    <t xml:space="preserve">condensador 10uF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">XVR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9 RLD (compartido)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RSM1..RSM3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sensado de modo comun (punto medio de RG)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">604k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">620k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">resistencia 620k 1%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">291-620K carbon 1/4 W 5 %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CINT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Condensador del integrador</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Si oscila en banco: 2.2n</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RPAR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resistencia en paralelo al integrador</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pelicula 5 %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">resistencia 10M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">291-10M carbon 1/4 W 5 %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RLIM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resistencia de seguridad al electrodo RLD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">390k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">resistencia 390k 1%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">293-390K carbon 1/2 W 5 %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Limita la corriente al paciente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">XRLD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10 OP-AMPS (paquetes)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">XHP, XMF, XLB x3, XRLD, XVR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Op-amp doble TS922AIYDT (Global 001-TS922)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TS922</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TS922AIYDT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SOIC-8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11 secciones = 3 por canal x 3 + RLD + VREF (1 libre). Solo habia 6 en stock</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adaptador SOIC-8 a DIP-8 (S08D8, Global; trae PCB y 2 headers de 4)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S08D8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PCB adaptador</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S08D8 adaptador SOIC 8 a DIP 8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">En el carrito hay 12; bastan 7 (sobran 5 = $1.250). Solo para los TS922 (SOIC-8, 1.27 mm). NO sirve para el TLV757 (SOT-23) ni para el INA333 (MSOP). Soldar con flux y probar antes de montar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zocalo DIP-8 (opcional)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DIP-8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">zocalo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">zocalo DIP 8 pines</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Opcional: soldar los pines del S08D8 directo a la perfboard, o usar tira hembra 2.54 como zocalo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Desacople de cada op-amp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11 ALIMENTACION (5 V USB / powerbank -&gt; 3.3 V)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">XLDO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Regulador LDO 3.3 V TLV75733PDBVR (Global 014-75733)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TLV75733P</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TLV75733PDBVR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SOT-23-5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entrada 5 V desde el pin +5V del STM32N6570-DK (Arduino CN8). EN unido a IN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Montaje del TLV757 sin adaptador (dead bug)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pegado boca arriba en la perfboard, hilo fino a cada pata. Pines: 1 IN, 2 GND, 3 EN (a IN), 4 NC, 5 OUT. El SOT23S3 de Global es de 3 pines: no sirve</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CLDOI, CLDOO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Condensadores del LDO (entrada y salida)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1u</t>
+  </si>
+  <si>
+    <t xml:space="preserve">condensador ceramico 1uF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CE50102 electrolitico 1uF 50V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ver la fila CLDOO cer.: a la salida hace falta ademas un ceramico. Pegados a los pines del LDO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CLDOO cer.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Condensador ceramico de salida del LDO (en paralelo con el electrolitico)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1u X7R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MLCC X7R 16 V o mas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MLCC THD 1uF X7R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CM105 MLCC THD 1uF 50V X7R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El TLV757 esta pensado para ceramico a la salida (&gt;= 0.47 uF efectivos); un electrolitico solo puede oscilar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CBULK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Condensador bulk del riel 3.3 V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ceramico o electrolitico</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cable 5 V y GND desde el DK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cable dupont macho-hembra</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tira de 40 jumpers Dupont M-H (compartida)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Usar powerbank o PC a bateria mientras haya electrodos puestos (ver Notas de seguridad)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12 ELECTRODOS Y CONECTORES (7)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">XE1P..XE3N, XER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Electrodo Ag/AgCl con broche 4 mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Skintact FS-RG1/10 32x41</t>
+  </si>
+  <si>
+    <t xml:space="preserve">desechable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Skintact FS-RG1/10 / Kendall Arbo H124SG 24 mm</t>
+  </si>
+  <si>
     <t xml:space="preserve">Pendiente</t>
   </si>
   <si>
-    <t xml:space="preserve">AGREGAR AL CARRITO DE GLOBAL. 15 nF agotado (2A153J en Global; tampoco en MechatronicStore): 10n + 4.7n en paralelo = 14.7 nF (f0 +1 %, Q -1 %). Stock al 4-oct: 2A103J 22 u, 2A472K 122 u. Cantidad en pares; precio del par ($50 + $60)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C22</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.2n</t>
-  </si>
-  <si>
-    <t xml:space="preserve">condensador poliester 2.2nF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C222NPO05D disco NPO 2.2nF 50V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">XLB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7 BUCKET + SALIDA AL ADC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rbk</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Resistencia del bucket</t>
-  </si>
-  <si>
-    <t xml:space="preserve">100</t>
-  </si>
-  <si>
-    <t xml:space="preserve">resistencia 100 ohm 1%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R1W100 carbon 1 W 100 ohm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cbk</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Condensador del bucket</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ADCk</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cable a Arduino A1..A3 del STM32N6570-DK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">jumper Dupont M-H</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cable dupont macho-hembra (tira de 40)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FALTA EN EL CARRITO. CH1-A1 (PA9), CH2-A2 (PA10), CH3-A3 (PA12). Mas 1 cable de GND. A0 no: comparte ADC con USB1 ISENSE (UM3300)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8 VREF 1.65 V (compartido)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">compartido</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RA1, RA2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Divisor de VREF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">resistencia 100k 1%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Condensador del divisor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ceramico X7R o electrolitico</t>
-  </si>
-  <si>
-    <t xml:space="preserve">condensador 10uF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">XVR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9 RLD (compartido)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RSM1..RSM3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sensado de modo comun (punto medio de RG)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">604k</t>
-  </si>
-  <si>
-    <t xml:space="preserve">620k</t>
-  </si>
-  <si>
-    <t xml:space="preserve">resistencia 620k 1%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">291-620K carbon 1/4 W 5 %</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CINT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Condensador del integrador</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Si oscila en banco: 2.2n</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RPAR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Resistencia en paralelo al integrador</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10M</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pelicula 5 %</t>
-  </si>
-  <si>
-    <t xml:space="preserve">resistencia 10M</t>
-  </si>
-  <si>
-    <t xml:space="preserve">291-10M carbon 1/4 W 5 %</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RLIM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Resistencia de seguridad al electrodo RLD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">390k</t>
-  </si>
-  <si>
-    <t xml:space="preserve">resistencia 390k 1%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">293-390K carbon 1/2 W 5 %</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Limita la corriente al paciente</t>
-  </si>
-  <si>
-    <t xml:space="preserve">XRLD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10 OP-AMPS (paquetes)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">XHP, XMF, XLB x3, XRLD, XVR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Op-amp doble TS922AIYDT (Global 001-TS922)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TS922</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TS922AIYDT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SOIC-8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">11 secciones = 3 por canal x 3 + RLD + VREF (1 libre). Solo habia 6 en stock</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Adaptador SOIC-8 a DIP-8 (S08D8, Global; trae PCB y 2 headers de 4)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S08D8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PCB adaptador</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S08D8 adaptador SOIC 8 a DIP 8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">En el carrito hay 12; bastan 7 (sobran 5 = $1.250). Solo para los TS922 (SOIC-8, 1.27 mm). NO sirve para el TLV757 (SOT-23) ni para el INA333 (MSOP). Soldar con flux y probar antes de montar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Zocalo DIP-8 (opcional)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DIP-8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">zocalo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">zocalo DIP 8 pines</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Opcional: soldar los pines del S08D8 directo a la perfboard, o usar tira hembra 2.54 como zocalo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Desacople de cada op-amp</t>
-  </si>
-  <si>
-    <t xml:space="preserve">11 ALIMENTACION (5 V USB / powerbank -&gt; 3.3 V)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">XLDO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Regulador LDO 3.3 V TLV75733PDBVR (Global 014-75733)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TLV75733P</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TLV75733PDBVR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SOT-23-5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Entrada 5 V desde el pin +5V del STM32N6570-DK (Arduino CN8). EN unido a IN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Montaje del TLV757 sin adaptador (dead bug)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pegado boca arriba en la perfboard, hilo fino a cada pata. Pines: 1 IN, 2 GND, 3 EN (a IN), 4 NC, 5 OUT. El SOT23S3 de Global es de 3 pines: no sirve</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CLDOI, CLDOO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Condensadores del LDO (entrada y salida)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1u</t>
-  </si>
-  <si>
-    <t xml:space="preserve">condensador ceramico 1uF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CE50102 electrolitico 1uF 50V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ver la fila CLDOO cer.: a la salida hace falta ademas un ceramico. Pegados a los pines del LDO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CLDOO cer.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Condensador ceramico de salida del LDO (en paralelo con el electrolitico)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1u X7R</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MLCC X7R 16 V o mas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MLCC THD 1uF X7R</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CM105 MLCC THD 1uF 50V X7R</t>
-  </si>
-  <si>
-    <t xml:space="preserve">El TLV757 esta pensado para ceramico a la salida (&gt;= 0.47 uF efectivos); un electrolitico solo puede oscilar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBULK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Condensador bulk del riel 3.3 V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ceramico o electrolitico</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cable 5 V y GND desde el DK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cable dupont macho-hembra</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FALTA EN EL CARRITO. Usar powerbank o PC a bateria mientras haya electrodos puestos (ver Notas de seguridad)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">12 ELECTRODOS Y CONECTORES (7)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">XE1P..XE3N, XER</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Electrodo Ag/AgCl con broche 4 mm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Skintact FS-RG1/10 32x41</t>
-  </si>
-  <si>
-    <t xml:space="preserve">desechable</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Skintact FS-RG1/10 / Kendall Arbo H124SG 24 mm</t>
-  </si>
-  <si>
     <t xml:space="preserve">FALTA EN EL CARRITO. 7 por sesion (6 de senal + 1 RLD); caja de 50. Skintact para CH1, CH3 y RLD. CH2: Arbo H124SG (24 mm) o par sobre el menton. ISIMED 55x55 solo como RLD</t>
   </si>
   <si>
@@ -844,7 +853,10 @@
     <t xml:space="preserve">cable dupont macho-macho 20 cm tira 40</t>
   </si>
   <si>
-    <t xml:space="preserve">FALTA EN EL CARRITO. Lado macho al conector 2x8; el otro extremo se une a los cables de electrodo (soldado + termorretractil o enchufado)</t>
+    <t xml:space="preserve">Tira de 40 jumpers Dupont M-M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Llenar tienda y precio de la tira. Lado macho al conector 2x8; el otro extremo se une a los cables de electrodo (soldado + termorretractil o enchufado)</t>
   </si>
   <si>
     <t xml:space="preserve">Alcohol isopropilico / gel</t>
@@ -871,7 +883,7 @@
     <t xml:space="preserve">placa perforada 10x15</t>
   </si>
   <si>
-    <t xml:space="preserve">FALTA EN EL CARRITO</t>
+    <t xml:space="preserve">Ya lo tengo</t>
   </si>
   <si>
     <t xml:space="preserve">Tira de header macho 1x40 2.54 THT</t>
@@ -943,7 +955,7 @@
     <t xml:space="preserve">Cables Dupont para el microfono</t>
   </si>
   <si>
-    <t xml:space="preserve">FALTA EN EL CARRITO. VDD 3.3V, GND, SCK, WS, SD, L/R (L/R a GND)</t>
+    <t xml:space="preserve">VDD 3.3V, GND, SCK, WS, SD, L/R (L/R a GND)</t>
   </si>
   <si>
     <t xml:space="preserve">TOTAL</t>
@@ -961,33 +973,6 @@
     <t xml:space="preserve">Donde</t>
   </si>
   <si>
-    <t xml:space="preserve">15n Condensador de realimentacion</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Global (agregar al carrito)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">15 nF agotado (2A153J en Global; tampoco en MechatronicStore): 10n + 4.7n en paralelo = 14.7 nF (f0 +1 %, Q -1 %). Stock al 4-oct: 2A103J 22 u, 2A472K 122 u. Cantidad en pares; precio del par ($50 + $60)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">jumper Dupont M-H Cable a Arduino A1..A3 del STM32N6570-DK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MechatronicStore / Global. 1 tira de 40 M-H cubre las 3 filas M-H (14 cables)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CH1-A1 (PA9), CH2-A2 (PA10), CH3-A3 (PA12). Mas 1 cable de GND. A0 no: comparte ADC con USB1 ISENSE (UM3300)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">jumper Dupont M-H Cable 5 V y GND desde el DK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MechatronicStore / Global (misma tira M-H)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Usar powerbank o PC a bateria mientras haya electrodos puestos (ver Notas de seguridad)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Skintact FS-RG1/10 32x41 Electrodo Ag/AgCl con broche 4 mm</t>
   </si>
   <si>
@@ -1006,78 +991,12 @@
     <t xml:space="preserve">Uno por electrodo; trenzar los dos de cada par. REVISAR EL TERMINAL antes de comprar: debe calzar en header hembra 2.54 mm. Si termina en DIN 1.5 mm touchproof (DIN 42802), cortar y crimpar terminal Dupont hembra o comprar bases touchproof. Alternativa: cable de 3 electrodos con jack 3.5 mm (el de los kits AD8232) + jack hembra 3.5 mm TRS en la placa</t>
   </si>
   <si>
-    <t xml:space="preserve">jumper Dupont M-M Bus de 8 cables Dupont macho (separado de una tira de 40)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MechatronicStore / Global. 1 tira de 40 M-M</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lado macho al conector 2x8; el otro extremo se une a los cables de electrodo (soldado + termorretractil o enchufado)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Farmacia / ferreteria</t>
   </si>
   <si>
     <t xml:space="preserve">Preparar la piel</t>
   </si>
   <si>
-    <t xml:space="preserve">10 x 15 cm Perfboard</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Global (tarjetas para prototipos) / MechatronicStore</t>
-  </si>
-  <si>
-    <t xml:space="preserve">jumper Dupont M-H Cables Dupont para el microfono</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VDD 3.3V, GND, SCK, WS, SD, L/R (L/R a GND)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Estano 0.5-0.8 mm con nucleo de flux</t>
-  </si>
-  <si>
-    <t xml:space="preserve">soldadura estano 0.8 mm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Global (soldadura)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">insumo, no esta en el esquematico</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Flux (lapiz o pasta)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">flux</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Global (flux y mallas)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Imprescindible para soldar los TS922 en los S08D8 (insumo, no esta en el esquematico)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Malla desoldadora</t>
-  </si>
-  <si>
-    <t xml:space="preserve">malla desoldadora</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Para sacar los trimmers de los modulos INA333 (insumo, no esta en el esquematico)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Termorretractil 2-3 mm (surtido)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tubo termo retractil</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Global</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Uniones bus Dupont - cable de electrodo (insumo, no esta en el esquematico)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Resumen por modulo</t>
   </si>
   <si>
@@ -1096,43 +1015,28 @@
     <t xml:space="preserve">Faltan en los carritos</t>
   </si>
   <si>
-    <t xml:space="preserve">4 x 15n  Condensador de realimentacion</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Global: 2A103J poliester 10nF 100V + 2A472K poliester 4.7nF 100V, en paralelo (par)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5 x jumper Dupont M-H  Cable a Arduino A1..A3 del STM32N6570-DK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3 x jumper Dupont M-H  Cable 5 V y GND desde el DK</t>
-  </si>
-  <si>
     <t xml:space="preserve">50 x Skintact FS-RG1/10 32x41  Electrodo Ag/AgCl con broche 4 mm</t>
   </si>
   <si>
     <t xml:space="preserve">8 x broche 4 mm a pin  Cable de electrodo con broche (snap) 4 mm, idealmente apantallado</t>
   </si>
   <si>
-    <t xml:space="preserve">8 x jumper Dupont M-M  Bus de 8 cables Dupont macho (separado de una tira de 40)</t>
-  </si>
-  <si>
     <t xml:space="preserve">1 x   Alcohol isopropilico / gel</t>
   </si>
   <si>
     <t xml:space="preserve">2 x 10 x 15 cm  Perfboard</t>
   </si>
   <si>
-    <t xml:space="preserve">6 x jumper Dupont M-H  Cables Dupont para el microfono</t>
-  </si>
-  <si>
     <t xml:space="preserve">Avisos de la compra</t>
   </si>
   <si>
-    <t xml:space="preserve">AGREGAR al carrito de Global: 4 x 2A103J (10n poliester) + 4 x 2A472K (4.7n poliester) para C21 (10n + 4.7n en paralelo = 14.7 nF; el 15 nF esta agotado).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pendiente (otra tienda): electrodos, cables de electrodo, jumpers Dupont (tira M-H y tira M-M), perfboard, tiras de header 1x40 y alcohol.</t>
+    <t xml:space="preserve">Cm1 = 100n + 47n poliester en paralelo (147 nF) y C21 = 10n + 4.7n poliester en paralelo (14.7 nF): no habia 150 nF y el 15 nF estaba agotado.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Falta: electrodos, cables de electrodo y alcohol (ver FALTA COMPRAR). Perfboard e insumos de soldadura: ya los tienes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiras Dupont M-H y M-M: llenar tienda y precio en la hoja BoM por modulo.</t>
   </si>
   <si>
     <t xml:space="preserve">Resistencias de carbon 5 % en vez de pelicula metalica 1 %: aceptado para la demo (ganancia por canal +-7 %, se normaliza en firmware). Para produccion: 1 %.</t>
@@ -2124,7 +2028,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:S91"/>
+  <dimension ref="A1:S81"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
@@ -3546,7 +3450,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="5" t="s">
         <v>144</v>
       </c>
@@ -3601,11 +3505,11 @@
         <f aca="false">IF(P31="","",IF(O31="",K31,O31)*P31)</f>
         <v>440</v>
       </c>
-      <c r="R31" s="9" t="s">
+      <c r="R31" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="S31" s="5" t="s">
         <v>154</v>
-      </c>
-      <c r="S31" s="5" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3613,16 +3517,16 @@
         <v>144</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C32" s="5" t="s">
         <v>130</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="F32" s="5" t="s">
         <v>151</v>
@@ -3645,13 +3549,13 @@
         <v>4</v>
       </c>
       <c r="L32" s="5" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="M32" s="6" t="s">
         <v>28</v>
       </c>
       <c r="N32" s="6" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="O32" s="6" t="n">
         <v>4</v>
@@ -3673,7 +3577,7 @@
         <v>144</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C33" s="5" t="s">
         <v>101</v>
@@ -3707,7 +3611,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B34" s="4"/>
       <c r="C34" s="4" t="s">
@@ -3732,19 +3636,19 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="B35" s="5" t="s">
         <v>161</v>
       </c>
-      <c r="B35" s="5" t="s">
+      <c r="C35" s="5" t="s">
         <v>162</v>
       </c>
-      <c r="C35" s="5" t="s">
+      <c r="D35" s="5" t="s">
         <v>163</v>
       </c>
-      <c r="D35" s="5" t="s">
-        <v>164</v>
-      </c>
       <c r="E35" s="5" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="F35" s="5" t="s">
         <v>41</v>
@@ -3767,13 +3671,13 @@
         <v>4</v>
       </c>
       <c r="L35" s="5" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="M35" s="6" t="s">
         <v>28</v>
       </c>
       <c r="N35" s="6" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="O35" s="6" t="n">
         <v>6</v>
@@ -3792,13 +3696,13 @@
     </row>
     <row r="36" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="5" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B36" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="C36" s="5" t="s">
         <v>167</v>
-      </c>
-      <c r="C36" s="5" t="s">
-        <v>168</v>
       </c>
       <c r="D36" s="5" t="s">
         <v>138</v>
@@ -3850,21 +3754,21 @@
       </c>
       <c r="S36" s="5"/>
     </row>
-    <row r="37" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="5" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B37" s="5" t="s">
+        <v>168</v>
+      </c>
+      <c r="C37" s="5" t="s">
         <v>169</v>
-      </c>
-      <c r="C37" s="5" t="s">
-        <v>170</v>
       </c>
       <c r="D37" s="5" t="s">
         <v>102</v>
       </c>
       <c r="E37" s="5" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="F37" s="5" t="s">
         <v>102</v>
@@ -3887,30 +3791,36 @@
         <v>5</v>
       </c>
       <c r="L37" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="M37" s="6" t="s">
         <v>172</v>
       </c>
-      <c r="M37" s="6"/>
-      <c r="N37" s="6"/>
-      <c r="O37" s="6"/>
+      <c r="N37" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="O37" s="6" t="n">
+        <v>5</v>
+      </c>
       <c r="P37" s="7"/>
       <c r="Q37" s="8" t="str">
         <f aca="false">IF(P37="","",IF(O37="",K37,O37)*P37)</f>
         <v/>
       </c>
-      <c r="R37" s="9" t="s">
-        <v>154</v>
+      <c r="R37" s="6" t="s">
+        <v>30</v>
       </c>
       <c r="S37" s="5" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="4" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B38" s="4"/>
       <c r="C38" s="4" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D38" s="4"/>
       <c r="E38" s="4"/>
@@ -3931,13 +3841,13 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="5" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="D39" s="5" t="s">
         <v>25</v>
@@ -3966,7 +3876,7 @@
         <v>2</v>
       </c>
       <c r="L39" s="5" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="M39" s="6" t="s">
         <v>28</v>
@@ -3991,13 +3901,13 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="5" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D40" s="5" t="s">
         <v>108</v>
@@ -4006,7 +3916,7 @@
         <v>108</v>
       </c>
       <c r="F40" s="5" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="G40" s="5" t="n">
         <v>1</v>
@@ -4026,7 +3936,7 @@
         <v>1</v>
       </c>
       <c r="L40" s="5" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="M40" s="6" t="s">
         <v>28</v>
@@ -4051,10 +3961,10 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="5" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C41" s="5" t="s">
         <v>101</v>
@@ -4088,11 +3998,11 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="4" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B42" s="4"/>
       <c r="C42" s="4" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D42" s="4"/>
       <c r="E42" s="4"/>
@@ -4113,19 +4023,19 @@
     </row>
     <row r="43" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="5" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D43" s="5" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="E43" s="5" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="F43" s="5" t="s">
         <v>41</v>
@@ -4148,13 +4058,13 @@
         <v>4</v>
       </c>
       <c r="L43" s="5" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="M43" s="6" t="s">
         <v>28</v>
       </c>
       <c r="N43" s="6" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="O43" s="6" t="n">
         <v>6</v>
@@ -4173,13 +4083,13 @@
     </row>
     <row r="44" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="5" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="D44" s="5" t="s">
         <v>138</v>
@@ -4230,27 +4140,27 @@
         <v>30</v>
       </c>
       <c r="S44" s="5" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="5" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="D45" s="5" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="E45" s="5" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="F45" s="5" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="G45" s="5" t="n">
         <v>1</v>
@@ -4270,13 +4180,13 @@
         <v>2</v>
       </c>
       <c r="L45" s="5" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="M45" s="6" t="s">
         <v>28</v>
       </c>
       <c r="N45" s="6" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="O45" s="6" t="n">
         <v>4</v>
@@ -4295,19 +4205,19 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="5" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="D46" s="5" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="E46" s="5" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="F46" s="5" t="s">
         <v>41</v>
@@ -4330,13 +4240,13 @@
         <v>2</v>
       </c>
       <c r="L46" s="5" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="M46" s="6" t="s">
         <v>28</v>
       </c>
       <c r="N46" s="6" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="O46" s="6" t="n">
         <v>4</v>
@@ -4352,15 +4262,15 @@
         <v>30</v>
       </c>
       <c r="S46" s="5" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="5" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B47" s="5" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="C47" s="5" t="s">
         <v>101</v>
@@ -4394,11 +4304,11 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="4" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B48" s="4"/>
       <c r="C48" s="4" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D48" s="4"/>
       <c r="E48" s="4"/>
@@ -4419,22 +4329,22 @@
     </row>
     <row r="49" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="5" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B49" s="5" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C49" s="5" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="D49" s="5" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="E49" s="5" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="F49" s="5" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="G49" s="5" t="n">
         <v>6</v>
@@ -4454,13 +4364,13 @@
         <v>6</v>
       </c>
       <c r="L49" s="5" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="M49" s="6" t="s">
         <v>28</v>
       </c>
       <c r="N49" s="6" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="O49" s="6" t="n">
         <v>6</v>
@@ -4476,27 +4386,27 @@
         <v>30</v>
       </c>
       <c r="S49" s="5" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="5" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B50" s="5" t="s">
         <v>102</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D50" s="5" t="s">
         <v>102</v>
       </c>
       <c r="E50" s="5" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="F50" s="5" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="G50" s="5" t="n">
         <v>6</v>
@@ -4516,13 +4426,13 @@
         <v>7</v>
       </c>
       <c r="L50" s="5" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="M50" s="6" t="s">
         <v>28</v>
       </c>
       <c r="N50" s="6" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="O50" s="6" t="n">
         <v>12</v>
@@ -4538,27 +4448,27 @@
         <v>30</v>
       </c>
       <c r="S50" s="5" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="5" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B51" s="5" t="s">
         <v>102</v>
       </c>
       <c r="C51" s="5" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="D51" s="5" t="s">
         <v>102</v>
       </c>
       <c r="E51" s="5" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="F51" s="5" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="G51" s="5"/>
       <c r="H51" s="5"/>
@@ -4566,7 +4476,7 @@
       <c r="J51" s="5"/>
       <c r="K51" s="5"/>
       <c r="L51" s="5" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="M51" s="5"/>
       <c r="N51" s="5"/>
@@ -4577,18 +4487,18 @@
         <v>103</v>
       </c>
       <c r="S51" s="5" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="5" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B52" s="5" t="s">
         <v>102</v>
       </c>
       <c r="C52" s="5" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="D52" s="5" t="s">
         <v>76</v>
@@ -4644,11 +4554,11 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="4" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B53" s="4"/>
       <c r="C53" s="4" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D53" s="4"/>
       <c r="E53" s="4"/>
@@ -4669,22 +4579,22 @@
     </row>
     <row r="54" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="5" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B54" s="5" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="C54" s="5" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="D54" s="5" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="E54" s="5" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="F54" s="5" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="G54" s="5" t="n">
         <v>1</v>
@@ -4704,13 +4614,13 @@
         <v>2</v>
       </c>
       <c r="L54" s="5" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="M54" s="6" t="s">
         <v>28</v>
       </c>
       <c r="N54" s="6" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="O54" s="6" t="n">
         <v>2</v>
@@ -4726,18 +4636,18 @@
         <v>30</v>
       </c>
       <c r="S54" s="5" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="5" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B55" s="5" t="s">
         <v>102</v>
       </c>
       <c r="C55" s="5" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="D55" s="5" t="s">
         <v>102</v>
@@ -4763,24 +4673,24 @@
         <v>103</v>
       </c>
       <c r="S55" s="5" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="5" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B56" s="5" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C56" s="5" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D56" s="5" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="E56" s="5" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="F56" s="5" t="s">
         <v>77</v>
@@ -4803,13 +4713,13 @@
         <v>3</v>
       </c>
       <c r="L56" s="5" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="M56" s="6" t="s">
         <v>28</v>
       </c>
       <c r="N56" s="6" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="O56" s="6" t="n">
         <v>3</v>
@@ -4825,27 +4735,27 @@
         <v>30</v>
       </c>
       <c r="S56" s="5" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="5" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B57" s="5" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C57" s="5" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="D57" s="5" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="E57" s="5" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="F57" s="5" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="G57" s="5" t="n">
         <v>1</v>
@@ -4865,13 +4775,13 @@
         <v>2</v>
       </c>
       <c r="L57" s="5" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="M57" s="6" t="s">
         <v>28</v>
       </c>
       <c r="N57" s="6" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="O57" s="6" t="n">
         <v>2</v>
@@ -4887,18 +4797,18 @@
         <v>30</v>
       </c>
       <c r="S57" s="5" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="5" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B58" s="5" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C58" s="5" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="D58" s="5" t="s">
         <v>108</v>
@@ -4907,7 +4817,7 @@
         <v>108</v>
       </c>
       <c r="F58" s="5" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="G58" s="5" t="n">
         <v>1</v>
@@ -4927,7 +4837,7 @@
         <v>2</v>
       </c>
       <c r="L58" s="5" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="M58" s="6" t="s">
         <v>28</v>
@@ -4952,19 +4862,19 @@
     </row>
     <row r="59" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="5" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B59" s="5" t="s">
         <v>102</v>
       </c>
       <c r="C59" s="5" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="D59" s="5" t="s">
         <v>102</v>
       </c>
       <c r="E59" s="5" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="F59" s="5" t="s">
         <v>102</v>
@@ -4987,30 +4897,36 @@
         <v>3</v>
       </c>
       <c r="L59" s="5" t="s">
-        <v>251</v>
-      </c>
-      <c r="M59" s="6"/>
-      <c r="N59" s="6"/>
-      <c r="O59" s="6"/>
+        <v>252</v>
+      </c>
+      <c r="M59" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="N59" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="O59" s="6" t="n">
+        <v>3</v>
+      </c>
       <c r="P59" s="7"/>
       <c r="Q59" s="8" t="str">
         <f aca="false">IF(P59="","",IF(O59="",K59,O59)*P59)</f>
         <v/>
       </c>
-      <c r="R59" s="9" t="s">
-        <v>154</v>
+      <c r="R59" s="6" t="s">
+        <v>30</v>
       </c>
       <c r="S59" s="5" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="4" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B60" s="4"/>
       <c r="C60" s="4" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D60" s="4"/>
       <c r="E60" s="4"/>
@@ -5031,22 +4947,22 @@
     </row>
     <row r="61" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="5" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B61" s="5" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="C61" s="5" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="D61" s="5" t="s">
         <v>102</v>
       </c>
       <c r="E61" s="5" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="F61" s="5" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="G61" s="5" t="n">
         <v>7</v>
@@ -5066,7 +4982,7 @@
         <v>50</v>
       </c>
       <c r="L61" s="5" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="M61" s="6"/>
       <c r="N61" s="6"/>
@@ -5077,27 +4993,27 @@
         <v/>
       </c>
       <c r="R61" s="9" t="s">
-        <v>154</v>
+        <v>261</v>
       </c>
       <c r="S61" s="5" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="5" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B62" s="5" t="s">
         <v>102</v>
       </c>
       <c r="C62" s="5" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="D62" s="5" t="s">
         <v>102</v>
       </c>
       <c r="E62" s="5" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="F62" s="5" t="s">
         <v>102</v>
@@ -5120,7 +5036,7 @@
         <v>8</v>
       </c>
       <c r="L62" s="5" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="M62" s="6"/>
       <c r="N62" s="6"/>
@@ -5131,27 +5047,27 @@
         <v/>
       </c>
       <c r="R62" s="9" t="s">
-        <v>154</v>
+        <v>261</v>
       </c>
       <c r="S62" s="5" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="5" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B63" s="5" t="s">
         <v>102</v>
       </c>
       <c r="C63" s="5" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="D63" s="5" t="s">
         <v>102</v>
       </c>
       <c r="E63" s="5" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="F63" s="5" t="s">
         <v>102</v>
@@ -5174,13 +5090,13 @@
         <v>2</v>
       </c>
       <c r="L63" s="5" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="M63" s="6" t="s">
         <v>28</v>
       </c>
       <c r="N63" s="6" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="O63" s="6" t="n">
         <v>2</v>
@@ -5196,24 +5112,24 @@
         <v>30</v>
       </c>
       <c r="S63" s="5" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="5" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B64" s="5" t="s">
         <v>102</v>
       </c>
       <c r="C64" s="5" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="D64" s="5" t="s">
         <v>102</v>
       </c>
       <c r="E64" s="5" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="F64" s="5" t="s">
         <v>102</v>
@@ -5236,32 +5152,38 @@
         <v>8</v>
       </c>
       <c r="L64" s="5" t="s">
-        <v>271</v>
-      </c>
-      <c r="M64" s="6"/>
-      <c r="N64" s="6"/>
-      <c r="O64" s="6"/>
+        <v>274</v>
+      </c>
+      <c r="M64" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="N64" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="O64" s="6" t="n">
+        <v>8</v>
+      </c>
       <c r="P64" s="7"/>
       <c r="Q64" s="8" t="str">
         <f aca="false">IF(P64="","",IF(O64="",K64,O64)*P64)</f>
         <v/>
       </c>
-      <c r="R64" s="9" t="s">
-        <v>154</v>
+      <c r="R64" s="6" t="s">
+        <v>30</v>
       </c>
       <c r="S64" s="5" t="s">
-        <v>272</v>
+        <v>276</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="5" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B65" s="5" t="s">
         <v>102</v>
       </c>
       <c r="C65" s="5" t="s">
-        <v>273</v>
+        <v>277</v>
       </c>
       <c r="D65" s="5" t="s">
         <v>102</v>
@@ -5290,7 +5212,7 @@
         <v>1</v>
       </c>
       <c r="L65" s="5" t="s">
-        <v>274</v>
+        <v>278</v>
       </c>
       <c r="M65" s="6"/>
       <c r="N65" s="6"/>
@@ -5301,19 +5223,19 @@
         <v/>
       </c>
       <c r="R65" s="9" t="s">
-        <v>154</v>
+        <v>261</v>
       </c>
       <c r="S65" s="5" t="s">
-        <v>275</v>
+        <v>279</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="4" t="s">
-        <v>276</v>
+        <v>280</v>
       </c>
       <c r="B66" s="4"/>
       <c r="C66" s="4" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D66" s="4"/>
       <c r="E66" s="4"/>
@@ -5334,22 +5256,22 @@
     </row>
     <row r="67" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="5" t="s">
-        <v>276</v>
+        <v>280</v>
       </c>
       <c r="B67" s="5" t="s">
         <v>102</v>
       </c>
       <c r="C67" s="5" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="D67" s="5" t="s">
         <v>102</v>
       </c>
       <c r="E67" s="5" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
       <c r="F67" s="5" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
       <c r="G67" s="5" t="n">
         <v>1</v>
@@ -5369,7 +5291,7 @@
         <v>2</v>
       </c>
       <c r="L67" s="5" t="s">
-        <v>280</v>
+        <v>284</v>
       </c>
       <c r="M67" s="6"/>
       <c r="N67" s="6"/>
@@ -5379,28 +5301,26 @@
         <f aca="false">IF(P67="","",IF(O67="",K67,O67)*P67)</f>
         <v/>
       </c>
-      <c r="R67" s="9" t="s">
-        <v>154</v>
-      </c>
-      <c r="S67" s="5" t="s">
-        <v>281</v>
-      </c>
+      <c r="R67" s="6" t="s">
+        <v>285</v>
+      </c>
+      <c r="S67" s="5"/>
     </row>
     <row r="68" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="5" t="s">
-        <v>276</v>
+        <v>280</v>
       </c>
       <c r="B68" s="5" t="s">
         <v>102</v>
       </c>
       <c r="C68" s="5" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="D68" s="5" t="s">
         <v>102</v>
       </c>
       <c r="E68" s="5" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="F68" s="5" t="s">
         <v>102</v>
@@ -5423,13 +5343,13 @@
         <v>1</v>
       </c>
       <c r="L68" s="5" t="s">
-        <v>284</v>
+        <v>288</v>
       </c>
       <c r="M68" s="6" t="s">
         <v>28</v>
       </c>
       <c r="N68" s="6" t="s">
-        <v>285</v>
+        <v>289</v>
       </c>
       <c r="O68" s="6" t="n">
         <v>1</v>
@@ -5445,24 +5365,24 @@
         <v>30</v>
       </c>
       <c r="S68" s="5" t="s">
-        <v>286</v>
+        <v>290</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="5" t="s">
-        <v>276</v>
+        <v>280</v>
       </c>
       <c r="B69" s="5" t="s">
         <v>102</v>
       </c>
       <c r="C69" s="5" t="s">
-        <v>287</v>
+        <v>291</v>
       </c>
       <c r="D69" s="5" t="s">
         <v>102</v>
       </c>
       <c r="E69" s="5" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="F69" s="5" t="s">
         <v>102</v>
@@ -5485,13 +5405,13 @@
         <v>1</v>
       </c>
       <c r="L69" s="5" t="s">
-        <v>289</v>
+        <v>293</v>
       </c>
       <c r="M69" s="6" t="s">
         <v>43</v>
       </c>
       <c r="N69" s="6" t="s">
-        <v>290</v>
+        <v>294</v>
       </c>
       <c r="O69" s="6" t="n">
         <v>1</v>
@@ -5507,24 +5427,24 @@
         <v>30</v>
       </c>
       <c r="S69" s="5" t="s">
-        <v>291</v>
+        <v>295</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="5" t="s">
-        <v>276</v>
+        <v>280</v>
       </c>
       <c r="B70" s="5" t="s">
         <v>102</v>
       </c>
       <c r="C70" s="5" t="s">
-        <v>292</v>
+        <v>296</v>
       </c>
       <c r="D70" s="5" t="s">
         <v>102</v>
       </c>
       <c r="E70" s="5" t="s">
-        <v>293</v>
+        <v>297</v>
       </c>
       <c r="F70" s="5" t="s">
         <v>102</v>
@@ -5547,13 +5467,13 @@
         <v>1</v>
       </c>
       <c r="L70" s="5" t="s">
-        <v>294</v>
+        <v>298</v>
       </c>
       <c r="M70" s="6" t="s">
         <v>28</v>
       </c>
       <c r="N70" s="6" t="s">
-        <v>295</v>
+        <v>299</v>
       </c>
       <c r="O70" s="6" t="n">
         <v>3</v>
@@ -5569,16 +5489,16 @@
         <v>30</v>
       </c>
       <c r="S70" s="5" t="s">
-        <v>296</v>
+        <v>300</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="4" t="s">
-        <v>297</v>
+        <v>301</v>
       </c>
       <c r="B71" s="4"/>
       <c r="C71" s="4" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D71" s="4"/>
       <c r="E71" s="4"/>
@@ -5599,22 +5519,22 @@
     </row>
     <row r="72" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="5" t="s">
-        <v>297</v>
+        <v>301</v>
       </c>
       <c r="B72" s="5" t="s">
         <v>102</v>
       </c>
       <c r="C72" s="5" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="D72" s="5" t="s">
         <v>102</v>
       </c>
       <c r="E72" s="5" t="s">
-        <v>299</v>
+        <v>303</v>
       </c>
       <c r="F72" s="5" t="s">
-        <v>300</v>
+        <v>304</v>
       </c>
       <c r="G72" s="5" t="n">
         <v>1</v>
@@ -5634,13 +5554,13 @@
         <v>2</v>
       </c>
       <c r="L72" s="5" t="s">
-        <v>301</v>
+        <v>305</v>
       </c>
       <c r="M72" s="6" t="s">
         <v>28</v>
       </c>
       <c r="N72" s="6" t="s">
-        <v>302</v>
+        <v>306</v>
       </c>
       <c r="O72" s="6" t="n">
         <v>1</v>
@@ -5656,24 +5576,24 @@
         <v>30</v>
       </c>
       <c r="S72" s="5" t="s">
-        <v>303</v>
+        <v>307</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="5" t="s">
-        <v>297</v>
+        <v>301</v>
       </c>
       <c r="B73" s="5" t="s">
         <v>102</v>
       </c>
       <c r="C73" s="5" t="s">
-        <v>304</v>
+        <v>308</v>
       </c>
       <c r="D73" s="5" t="s">
         <v>102</v>
       </c>
       <c r="E73" s="5" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="F73" s="5" t="s">
         <v>102</v>
@@ -5696,26 +5616,32 @@
         <v>6</v>
       </c>
       <c r="L73" s="5" t="s">
-        <v>251</v>
-      </c>
-      <c r="M73" s="6"/>
-      <c r="N73" s="6"/>
-      <c r="O73" s="6"/>
+        <v>252</v>
+      </c>
+      <c r="M73" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="N73" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="O73" s="6" t="n">
+        <v>6</v>
+      </c>
       <c r="P73" s="7"/>
       <c r="Q73" s="8" t="str">
         <f aca="false">IF(P73="","",IF(O73="",K73,O73)*P73)</f>
         <v/>
       </c>
-      <c r="R73" s="9" t="s">
-        <v>154</v>
+      <c r="R73" s="6" t="s">
+        <v>30</v>
       </c>
       <c r="S73" s="5" t="s">
-        <v>305</v>
+        <v>309</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="P75" s="10" t="s">
-        <v>306</v>
+        <v>310</v>
       </c>
       <c r="Q75" s="11" t="n">
         <f aca="false">SUM(Q5:Q73)</f>
@@ -5724,250 +5650,82 @@
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="12" t="s">
-        <v>307</v>
+        <v>311</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="3" t="s">
-        <v>308</v>
+        <v>312</v>
       </c>
       <c r="B78" s="3" t="s">
-        <v>309</v>
+        <v>313</v>
       </c>
       <c r="C78" s="3" t="s">
         <v>13</v>
       </c>
       <c r="D78" s="3" t="s">
-        <v>310</v>
+        <v>314</v>
       </c>
       <c r="E78" s="3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="79" customFormat="false" ht="115.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="79" customFormat="false" ht="90.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="13" t="n">
-        <v>4</v>
+        <v>50</v>
       </c>
       <c r="B79" s="13" t="s">
-        <v>311</v>
+        <v>315</v>
       </c>
       <c r="C79" s="13" t="s">
-        <v>153</v>
+        <v>260</v>
       </c>
       <c r="D79" s="13" t="s">
-        <v>312</v>
+        <v>316</v>
       </c>
       <c r="E79" s="13" t="s">
-        <v>313</v>
-      </c>
-    </row>
-    <row r="80" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="80" customFormat="false" ht="191.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="13" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="B80" s="13" t="s">
-        <v>314</v>
+        <v>318</v>
       </c>
       <c r="C80" s="13" t="s">
-        <v>172</v>
+        <v>265</v>
       </c>
       <c r="D80" s="13" t="s">
-        <v>315</v>
+        <v>319</v>
       </c>
       <c r="E80" s="13" t="s">
-        <v>316</v>
-      </c>
-    </row>
-    <row r="81" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="81" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="13" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B81" s="13" t="s">
-        <v>317</v>
+        <v>277</v>
       </c>
       <c r="C81" s="13" t="s">
-        <v>251</v>
+        <v>278</v>
       </c>
       <c r="D81" s="13" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="E81" s="13" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="82" customFormat="false" ht="90.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A82" s="13" t="n">
-        <v>50</v>
-      </c>
-      <c r="B82" s="13" t="s">
-        <v>320</v>
-      </c>
-      <c r="C82" s="13" t="s">
-        <v>258</v>
-      </c>
-      <c r="D82" s="13" t="s">
-        <v>321</v>
-      </c>
-      <c r="E82" s="13" t="s">
         <v>322</v>
-      </c>
-    </row>
-    <row r="83" customFormat="false" ht="191.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A83" s="13" t="n">
-        <v>8</v>
-      </c>
-      <c r="B83" s="13" t="s">
-        <v>323</v>
-      </c>
-      <c r="C83" s="13" t="s">
-        <v>262</v>
-      </c>
-      <c r="D83" s="13" t="s">
-        <v>324</v>
-      </c>
-      <c r="E83" s="13" t="s">
-        <v>325</v>
-      </c>
-    </row>
-    <row r="84" customFormat="false" ht="77.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A84" s="13" t="n">
-        <v>8</v>
-      </c>
-      <c r="B84" s="13" t="s">
-        <v>326</v>
-      </c>
-      <c r="C84" s="13" t="s">
-        <v>271</v>
-      </c>
-      <c r="D84" s="13" t="s">
-        <v>327</v>
-      </c>
-      <c r="E84" s="13" t="s">
-        <v>328</v>
-      </c>
-    </row>
-    <row r="85" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A85" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="B85" s="13" t="s">
-        <v>273</v>
-      </c>
-      <c r="C85" s="13" t="s">
-        <v>274</v>
-      </c>
-      <c r="D85" s="13" t="s">
-        <v>329</v>
-      </c>
-      <c r="E85" s="13" t="s">
-        <v>330</v>
-      </c>
-    </row>
-    <row r="86" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A86" s="13" t="n">
-        <v>2</v>
-      </c>
-      <c r="B86" s="13" t="s">
-        <v>331</v>
-      </c>
-      <c r="C86" s="13" t="s">
-        <v>280</v>
-      </c>
-      <c r="D86" s="13" t="s">
-        <v>332</v>
-      </c>
-      <c r="E86" s="13"/>
-    </row>
-    <row r="87" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A87" s="13" t="n">
-        <v>6</v>
-      </c>
-      <c r="B87" s="13" t="s">
-        <v>333</v>
-      </c>
-      <c r="C87" s="13" t="s">
-        <v>251</v>
-      </c>
-      <c r="D87" s="13" t="s">
-        <v>318</v>
-      </c>
-      <c r="E87" s="13" t="s">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="88" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A88" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="B88" s="13" t="s">
-        <v>335</v>
-      </c>
-      <c r="C88" s="13" t="s">
-        <v>336</v>
-      </c>
-      <c r="D88" s="13" t="s">
-        <v>337</v>
-      </c>
-      <c r="E88" s="13" t="s">
-        <v>338</v>
-      </c>
-    </row>
-    <row r="89" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A89" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="B89" s="13" t="s">
-        <v>339</v>
-      </c>
-      <c r="C89" s="13" t="s">
-        <v>340</v>
-      </c>
-      <c r="D89" s="13" t="s">
-        <v>341</v>
-      </c>
-      <c r="E89" s="13" t="s">
-        <v>342</v>
-      </c>
-    </row>
-    <row r="90" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A90" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="B90" s="13" t="s">
-        <v>343</v>
-      </c>
-      <c r="C90" s="13" t="s">
-        <v>344</v>
-      </c>
-      <c r="D90" s="13" t="s">
-        <v>341</v>
-      </c>
-      <c r="E90" s="13" t="s">
-        <v>345</v>
-      </c>
-    </row>
-    <row r="91" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A91" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="B91" s="13" t="s">
-        <v>346</v>
-      </c>
-      <c r="C91" s="13" t="s">
-        <v>347</v>
-      </c>
-      <c r="D91" s="13" t="s">
-        <v>348</v>
-      </c>
-      <c r="E91" s="13" t="s">
-        <v>349</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A4:S73"/>
   <dataValidations count="1">
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="R6:R7 R9:R11 R13:R15 R17:R19 R22:R27 R30:R32 R35:R37 R39:R40 R43:R46 R49:R50 R52 R54 R56:R59 R61:R65 R67:R70 R72:R73" type="list">
-      <formula1>"Pendiente,En carrito,Comprado,No hay,No aplica"</formula1>
+      <formula1>"Pendiente,En carrito,Comprado,Ya lo tengo,No hay,No aplica"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -5987,7 +5745,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D40"/>
+  <dimension ref="A1:D36"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="70"/>
@@ -5998,7 +5756,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>350</v>
+        <v>323</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6006,10 +5764,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>351</v>
+        <v>324</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>352</v>
+        <v>325</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>18</v>
@@ -6110,7 +5868,7 @@
       </c>
       <c r="C9" s="14" t="n">
         <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$73,A9,'BoM por modulo'!$R$5:$R$73,"Pendiente")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D9" s="15" t="n">
         <f aca="false">SUMIF('BoM por modulo'!$A$5:$A$73,A9,'BoM por modulo'!$Q$5:$Q$73)</f>
@@ -6119,7 +5877,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B10" s="14" t="n">
         <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$73,A10,'BoM por modulo'!$R$5:$R$73,"&lt;&gt;No aplica",'BoM por modulo'!$R$5:$R$73,"&lt;&gt;")</f>
@@ -6127,7 +5885,7 @@
       </c>
       <c r="C10" s="14" t="n">
         <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$73,A10,'BoM por modulo'!$R$5:$R$73,"Pendiente")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D10" s="15" t="n">
         <f aca="false">SUMIF('BoM por modulo'!$A$5:$A$73,A10,'BoM por modulo'!$Q$5:$Q$73)</f>
@@ -6136,7 +5894,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B11" s="14" t="n">
         <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$73,A11,'BoM por modulo'!$R$5:$R$73,"&lt;&gt;No aplica",'BoM por modulo'!$R$5:$R$73,"&lt;&gt;")</f>
@@ -6153,7 +5911,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="14" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B12" s="14" t="n">
         <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$73,A12,'BoM por modulo'!$R$5:$R$73,"&lt;&gt;No aplica",'BoM por modulo'!$R$5:$R$73,"&lt;&gt;")</f>
@@ -6170,7 +5928,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="14" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B13" s="14" t="n">
         <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$73,A13,'BoM por modulo'!$R$5:$R$73,"&lt;&gt;No aplica",'BoM por modulo'!$R$5:$R$73,"&lt;&gt;")</f>
@@ -6187,7 +5945,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="14" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B14" s="14" t="n">
         <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$73,A14,'BoM por modulo'!$R$5:$R$73,"&lt;&gt;No aplica",'BoM por modulo'!$R$5:$R$73,"&lt;&gt;")</f>
@@ -6195,7 +5953,7 @@
       </c>
       <c r="C14" s="14" t="n">
         <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$73,A14,'BoM por modulo'!$R$5:$R$73,"Pendiente")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D14" s="15" t="n">
         <f aca="false">SUMIF('BoM por modulo'!$A$5:$A$73,A14,'BoM por modulo'!$Q$5:$Q$73)</f>
@@ -6204,7 +5962,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="14" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B15" s="14" t="n">
         <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$73,A15,'BoM por modulo'!$R$5:$R$73,"&lt;&gt;No aplica",'BoM por modulo'!$R$5:$R$73,"&lt;&gt;")</f>
@@ -6212,7 +5970,7 @@
       </c>
       <c r="C15" s="14" t="n">
         <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$73,A15,'BoM por modulo'!$R$5:$R$73,"Pendiente")</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D15" s="15" t="n">
         <f aca="false">SUMIF('BoM por modulo'!$A$5:$A$73,A15,'BoM por modulo'!$Q$5:$Q$73)</f>
@@ -6221,7 +5979,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="14" t="s">
-        <v>276</v>
+        <v>280</v>
       </c>
       <c r="B16" s="14" t="n">
         <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$73,A16,'BoM por modulo'!$R$5:$R$73,"&lt;&gt;No aplica",'BoM por modulo'!$R$5:$R$73,"&lt;&gt;")</f>
@@ -6229,7 +5987,7 @@
       </c>
       <c r="C16" s="14" t="n">
         <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$73,A16,'BoM por modulo'!$R$5:$R$73,"Pendiente")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D16" s="15" t="n">
         <f aca="false">SUMIF('BoM por modulo'!$A$5:$A$73,A16,'BoM por modulo'!$Q$5:$Q$73)</f>
@@ -6238,7 +5996,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="14" t="s">
-        <v>297</v>
+        <v>301</v>
       </c>
       <c r="B17" s="14" t="n">
         <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$73,A17,'BoM por modulo'!$R$5:$R$73,"&lt;&gt;No aplica",'BoM por modulo'!$R$5:$R$73,"&lt;&gt;")</f>
@@ -6246,7 +6004,7 @@
       </c>
       <c r="C17" s="14" t="n">
         <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$73,A17,'BoM por modulo'!$R$5:$R$73,"Pendiente")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D17" s="15" t="n">
         <f aca="false">SUMIF('BoM por modulo'!$A$5:$A$73,A17,'BoM por modulo'!$Q$5:$Q$73)</f>
@@ -6255,7 +6013,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="16" t="s">
-        <v>306</v>
+        <v>310</v>
       </c>
       <c r="B18" s="16" t="n">
         <f aca="false">SUM(B4:B17)</f>
@@ -6263,7 +6021,7 @@
       </c>
       <c r="C18" s="16" t="n">
         <f aca="false">SUM(C4:C17)</f>
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D18" s="17" t="n">
         <f aca="false">SUM(D4:D17)</f>
@@ -6275,10 +6033,10 @@
         <v>14</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>353</v>
+        <v>326</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>354</v>
+        <v>327</v>
       </c>
       <c r="D20" s="3"/>
     </row>
@@ -6288,11 +6046,11 @@
       </c>
       <c r="B21" s="19" t="n">
         <f aca="false">SUMIFS('BoM por modulo'!$Q$5:$Q$73,'BoM por modulo'!$M$5:$M$73,A21,'BoM por modulo'!$R$5:$R$73,"En carrito")</f>
-        <v>38793</v>
+        <v>39233</v>
       </c>
       <c r="C21" s="19" t="n">
         <f aca="false">SUMIFS('BoM por modulo'!$Q$5:$Q$73,'BoM por modulo'!$M$5:$M$73,A21,'BoM por modulo'!$R$5:$R$73,"Pendiente")</f>
-        <v>440</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6310,109 +6068,74 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="20" t="s">
-        <v>355</v>
+        <v>328</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="18" t="s">
-        <v>356</v>
+        <v>329</v>
       </c>
       <c r="B25" s="21" t="s">
-        <v>357</v>
+        <v>260</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="18" t="s">
-        <v>358</v>
+        <v>330</v>
       </c>
       <c r="B26" s="21" t="s">
-        <v>172</v>
+        <v>265</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="18" t="s">
-        <v>359</v>
+        <v>331</v>
       </c>
       <c r="B27" s="21" t="s">
-        <v>251</v>
+        <v>278</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="18" t="s">
-        <v>360</v>
+        <v>332</v>
       </c>
       <c r="B28" s="21" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="18" t="s">
-        <v>361</v>
-      </c>
-      <c r="B29" s="21" t="s">
-        <v>262</v>
+        <v>284</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="18" t="s">
-        <v>362</v>
-      </c>
-      <c r="B30" s="21" t="s">
-        <v>271</v>
+      <c r="A30" s="10" t="s">
+        <v>333</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="18" t="s">
-        <v>363</v>
-      </c>
-      <c r="B31" s="21" t="s">
-        <v>274</v>
+        <v>334</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="18" t="s">
-        <v>364</v>
-      </c>
-      <c r="B32" s="21" t="s">
-        <v>280</v>
+        <v>335</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="18" t="s">
-        <v>365</v>
-      </c>
-      <c r="B33" s="21" t="s">
-        <v>251</v>
+        <v>336</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="18" t="s">
+        <v>337</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="10" t="s">
-        <v>366</v>
+      <c r="A35" s="18" t="s">
+        <v>338</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="18" t="s">
-        <v>367</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="18" t="s">
-        <v>368</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="18" t="s">
-        <v>369</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="18" t="s">
-        <v>370</v>
-      </c>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="18" t="s">
-        <v>371</v>
+        <v>339</v>
       </c>
     </row>
   </sheetData>
@@ -6441,396 +6164,396 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>372</v>
+        <v>340</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>373</v>
+        <v>341</v>
       </c>
       <c r="B3" s="4"/>
       <c r="C3" s="4"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>374</v>
+        <v>342</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>375</v>
+        <v>343</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>376</v>
+        <v>344</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="22" t="s">
-        <v>377</v>
+        <v>345</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>378</v>
+        <v>346</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>379</v>
+        <v>347</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="22" t="s">
-        <v>380</v>
+        <v>348</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>381</v>
+        <v>349</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>382</v>
+        <v>350</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="22" t="s">
-        <v>383</v>
+        <v>351</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>384</v>
+        <v>352</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>385</v>
+        <v>353</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="22" t="s">
-        <v>386</v>
+        <v>354</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>387</v>
+        <v>355</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>388</v>
+        <v>356</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="22" t="s">
-        <v>389</v>
+        <v>357</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>390</v>
+        <v>358</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>391</v>
+        <v>359</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="22" t="s">
-        <v>392</v>
+        <v>360</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>393</v>
+        <v>361</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>394</v>
+        <v>362</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="22" t="s">
-        <v>395</v>
+        <v>363</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>396</v>
+        <v>364</v>
       </c>
       <c r="C11" s="13" t="s">
-        <v>397</v>
+        <v>365</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="22" t="s">
-        <v>398</v>
+        <v>366</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>399</v>
+        <v>367</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>400</v>
+        <v>368</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="22" t="s">
-        <v>401</v>
+        <v>369</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>402</v>
+        <v>370</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>403</v>
+        <v>371</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="22" t="s">
-        <v>404</v>
+        <v>372</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>405</v>
+        <v>373</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="22" t="s">
-        <v>406</v>
+        <v>374</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>407</v>
+        <v>375</v>
       </c>
       <c r="C15" s="13"/>
     </row>
     <row r="16" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="22" t="s">
-        <v>408</v>
+        <v>376</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>409</v>
+        <v>377</v>
       </c>
       <c r="C16" s="13"/>
     </row>
     <row r="17" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="22" t="s">
-        <v>410</v>
+        <v>378</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>411</v>
+        <v>379</v>
       </c>
       <c r="C17" s="13"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>412</v>
+        <v>380</v>
       </c>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>374</v>
+        <v>342</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>375</v>
+        <v>343</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>376</v>
+        <v>344</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="22" t="s">
-        <v>377</v>
+        <v>345</v>
       </c>
       <c r="B21" s="13" t="s">
-        <v>413</v>
+        <v>381</v>
       </c>
       <c r="C21" s="13" t="s">
-        <v>414</v>
+        <v>382</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="22" t="s">
-        <v>415</v>
+        <v>383</v>
       </c>
       <c r="B22" s="13" t="s">
-        <v>416</v>
+        <v>384</v>
       </c>
       <c r="C22" s="13" t="s">
-        <v>417</v>
+        <v>385</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="22" t="s">
-        <v>383</v>
+        <v>351</v>
       </c>
       <c r="B23" s="13" t="s">
-        <v>418</v>
+        <v>386</v>
       </c>
       <c r="C23" s="13" t="s">
-        <v>419</v>
+        <v>387</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="22" t="s">
-        <v>420</v>
+        <v>388</v>
       </c>
       <c r="B24" s="13" t="s">
-        <v>421</v>
+        <v>389</v>
       </c>
       <c r="C24" s="13" t="s">
-        <v>422</v>
+        <v>390</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="22" t="s">
-        <v>423</v>
+        <v>391</v>
       </c>
       <c r="B25" s="13" t="s">
-        <v>424</v>
+        <v>392</v>
       </c>
       <c r="C25" s="13" t="s">
-        <v>425</v>
+        <v>393</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="22" t="s">
-        <v>426</v>
+        <v>394</v>
       </c>
       <c r="B26" s="13" t="s">
-        <v>427</v>
+        <v>395</v>
       </c>
       <c r="C26" s="13" t="s">
-        <v>428</v>
+        <v>396</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="22" t="s">
-        <v>392</v>
+        <v>360</v>
       </c>
       <c r="B27" s="13" t="s">
-        <v>429</v>
+        <v>397</v>
       </c>
       <c r="C27" s="13" t="s">
-        <v>430</v>
+        <v>398</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="22" t="s">
-        <v>398</v>
+        <v>366</v>
       </c>
       <c r="B28" s="13" t="s">
-        <v>431</v>
+        <v>399</v>
       </c>
       <c r="C28" s="13" t="s">
-        <v>432</v>
+        <v>400</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="22" t="s">
-        <v>433</v>
+        <v>401</v>
       </c>
       <c r="B29" s="13" t="s">
-        <v>434</v>
+        <v>402</v>
       </c>
       <c r="C29" s="13" t="s">
-        <v>435</v>
+        <v>403</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="22" t="s">
+        <v>372</v>
+      </c>
+      <c r="B30" s="13" t="s">
         <v>404</v>
       </c>
-      <c r="B30" s="13" t="s">
-        <v>436</v>
-      </c>
       <c r="C30" s="13" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="22" t="s">
-        <v>406</v>
+        <v>374</v>
       </c>
       <c r="B31" s="13" t="s">
-        <v>437</v>
+        <v>405</v>
       </c>
       <c r="C31" s="13"/>
     </row>
     <row r="32" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="22" t="s">
-        <v>408</v>
+        <v>376</v>
       </c>
       <c r="B32" s="13" t="s">
-        <v>438</v>
+        <v>406</v>
       </c>
       <c r="C32" s="13" t="s">
-        <v>439</v>
+        <v>407</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="22" t="s">
-        <v>410</v>
+        <v>378</v>
       </c>
       <c r="B33" s="13" t="s">
-        <v>440</v>
+        <v>408</v>
       </c>
       <c r="C33" s="13"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="s">
-        <v>441</v>
+        <v>409</v>
       </c>
       <c r="B35" s="4"/>
       <c r="C35" s="4"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="3" t="s">
-        <v>374</v>
+        <v>342</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>375</v>
+        <v>343</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>376</v>
+        <v>344</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="22" t="s">
-        <v>415</v>
+        <v>383</v>
       </c>
       <c r="B37" s="13" t="s">
-        <v>442</v>
+        <v>410</v>
       </c>
       <c r="C37" s="13" t="s">
-        <v>443</v>
+        <v>411</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="22" t="s">
-        <v>444</v>
+        <v>412</v>
       </c>
       <c r="B38" s="13" t="s">
-        <v>445</v>
+        <v>413</v>
       </c>
       <c r="C38" s="13" t="s">
-        <v>446</v>
+        <v>414</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="22" t="s">
-        <v>447</v>
+        <v>415</v>
       </c>
       <c r="B39" s="13" t="s">
-        <v>448</v>
+        <v>416</v>
       </c>
       <c r="C39" s="13"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="22" t="s">
-        <v>406</v>
+        <v>374</v>
       </c>
       <c r="B40" s="13" t="s">
-        <v>449</v>
+        <v>417</v>
       </c>
       <c r="C40" s="13" t="s">
-        <v>450</v>
+        <v>418</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="22" t="s">
-        <v>408</v>
+        <v>376</v>
       </c>
       <c r="B41" s="13" t="s">
-        <v>451</v>
+        <v>419</v>
       </c>
       <c r="C41" s="13"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="22" t="s">
-        <v>452</v>
+        <v>420</v>
       </c>
       <c r="B42" s="13" t="s">
-        <v>453</v>
+        <v>421</v>
       </c>
       <c r="C42" s="13"/>
     </row>
@@ -6862,7 +6585,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>454</v>
+        <v>422</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6870,16 +6593,16 @@
         <v>14</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>455</v>
+        <v>423</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>456</v>
+        <v>424</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>457</v>
+        <v>425</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>458</v>
+        <v>426</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6887,84 +6610,84 @@
         <v>28</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>459</v>
+        <v>427</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>460</v>
+        <v>428</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>461</v>
+        <v>429</v>
       </c>
       <c r="E4" s="13" t="s">
-        <v>462</v>
+        <v>430</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>463</v>
+        <v>431</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>464</v>
+        <v>432</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>465</v>
+        <v>433</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>466</v>
+        <v>434</v>
       </c>
       <c r="E5" s="13" t="s">
-        <v>467</v>
+        <v>435</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>468</v>
+        <v>436</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>459</v>
+        <v>427</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>469</v>
+        <v>437</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>470</v>
+        <v>438</v>
       </c>
       <c r="E6" s="13" t="s">
-        <v>471</v>
+        <v>439</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>472</v>
+        <v>440</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>459</v>
+        <v>427</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>473</v>
+        <v>441</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>474</v>
+        <v>442</v>
       </c>
       <c r="E7" s="13" t="s">
-        <v>475</v>
+        <v>443</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>476</v>
+        <v>444</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>459</v>
+        <v>427</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>477</v>
+        <v>445</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>478</v>
+        <v>446</v>
       </c>
       <c r="E8" s="13" t="s">
-        <v>479</v>
+        <v>447</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6972,84 +6695,84 @@
         <v>43</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>480</v>
+        <v>448</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>481</v>
+        <v>449</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>482</v>
+        <v>450</v>
       </c>
       <c r="E9" s="13" t="s">
-        <v>483</v>
+        <v>451</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>484</v>
+        <v>452</v>
       </c>
       <c r="B10" s="13" t="s">
         <v>102</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>485</v>
+        <v>453</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>486</v>
+        <v>454</v>
       </c>
       <c r="E10" s="13" t="s">
-        <v>487</v>
+        <v>455</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
-        <v>488</v>
+        <v>456</v>
       </c>
       <c r="B11" s="13" t="s">
         <v>102</v>
       </c>
       <c r="C11" s="13" t="s">
-        <v>489</v>
+        <v>457</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>490</v>
+        <v>458</v>
       </c>
       <c r="E11" s="13" t="s">
-        <v>491</v>
+        <v>459</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>492</v>
+        <v>460</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>459</v>
+        <v>427</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>493</v>
+        <v>461</v>
       </c>
       <c r="D12" s="13" t="s">
-        <v>494</v>
+        <v>462</v>
       </c>
       <c r="E12" s="13" t="s">
-        <v>495</v>
+        <v>463</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>496</v>
+        <v>464</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>497</v>
+        <v>465</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>498</v>
+        <v>466</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>499</v>
+        <v>467</v>
       </c>
       <c r="E13" s="13" t="s">
-        <v>500</v>
+        <v>468</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
BoM: pedidos Global y MechatronicStore comprados; Dupont sueltos (faltan 12 M-H, 6 M-M); armado de Cm1 = 100n||47n y C21 = 10n||4.7n
- esquematico con los valores armados (CM1 147n, C21 14.7n) y notas de armado en los recuadros
- README: seccion Armado

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V5Cz1Wb6HSRhqzouEW9mso
</commit_message>
<xml_diff>
--- a/docs/afe-emg/BoM_AFE_AuraVox.xlsx
+++ b/docs/afe-emg/BoM_AFE_AuraVox.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="830" uniqueCount="469">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="854" uniqueCount="494">
   <si>
     <t xml:space="preserve">BoM AFE sEMG AuraVox: 3 canales (submentoniano, labio inferior, laringe), 7 electrodos, RLD. Ordenada por modulo, igual que los recuadros del esquematico LTspice (sim/ltspice).</t>
   </si>
@@ -118,7 +118,7 @@
     <t xml:space="preserve">R2W100K carbon 2 W 5 % 100k</t>
   </si>
   <si>
-    <t xml:space="preserve">En carrito</t>
+    <t xml:space="preserve">Comprado</t>
   </si>
   <si>
     <t xml:space="preserve">2 W en vez de 1/4 W: funciona, pero es grande y caro (11 x $178). Si hay 100k 1/4 W, cambiarla. Limita la corriente de falla hacia el paciente y hacia el INA</t>
@@ -418,87 +418,102 @@
     <t xml:space="preserve">Cm1</t>
   </si>
   <si>
+    <t xml:space="preserve">Condensador a GND = 2 condensadores EN PARALELO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">150n</t>
+  </si>
+  <si>
+    <t xml:space="preserve">100n + 47n en paralelo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">poliester 100 V (2A104K + 2A473J)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">condensador poliester 100nF + 47nF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2A104K poliester 100nF 100V + 2A473J poliester 47nF 100V, en paralelo (par)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No hay 150 nF en Global: 100n + 47n en paralelo = 147 nF (f0 +1 %, Q -1 %). Cantidad en pares; precio del par ($70 + $60). ARMADO: soldar el 100n y el 47n entre los mismos dos puntos (nodo MA del MFB y GND), patas cortas. 147 nF: f0 +1 %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cm2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Condensador de realimentacion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1n</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ceramico C0G/NP0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">condensador ceramico 1nF NP0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RPE110X7R102K050V MLCC X7R 1nF 50V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">X7R en vez de C0G: aceptado para la demo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">XMF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6 LPF Sallen-Key 500 Hz (Q 1.31)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rlb1, Rlb2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resistencia del LPF B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">54.9k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Con 56k: f0 = 495 Hz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Condensador de realimentacion = 2 condensadores EN PARALELO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15n</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10n + 4.7n en paralelo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">poliester 100 V (2A103J + 2A472K)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">condensador poliester 10nF + 4.7nF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2A103J poliester 10nF 100V + 2A472K poliester 4.7nF 100V, en paralelo (par)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15 nF agotado (2A153J en Global; tampoco en MechatronicStore): 10n + 4.7n en paralelo = 14.7 nF (f0 +1 %, Q -1 %). Cantidad en pares; precio del par ($50 + $60). ARMADO: soldar el 10n y el 4.7n entre los mismos dos puntos (union de Rlb1-Rlb2 y la salida del op-amp del SK), patas cortas. 14.7 nF: f0 +1 %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C22</t>
+  </si>
+  <si>
     <t xml:space="preserve">Condensador a GND</t>
   </si>
   <si>
-    <t xml:space="preserve">150n</t>
-  </si>
-  <si>
-    <t xml:space="preserve">poliester 5 %</t>
-  </si>
-  <si>
-    <t xml:space="preserve">condensador poliester 150nF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2A104K poliester 100nF 100V + 2A473J poliester 47nF 100V, en paralelo (par)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No hay 150 nF en Global: 100n + 47n en paralelo = 147 nF (f0 +1 %, Q -1 %). Cantidad en pares; precio del par ($70 + $60)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cm2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Condensador de realimentacion</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1n</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ceramico C0G/NP0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">condensador ceramico 1nF NP0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RPE110X7R102K050V MLCC X7R 1nF 50V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">X7R en vez de C0G: aceptado para la demo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">XMF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6 LPF Sallen-Key 500 Hz (Q 1.31)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rlb1, Rlb2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Resistencia del LPF B</t>
-  </si>
-  <si>
-    <t xml:space="preserve">54.9k</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Con 56k: f0 = 495 Hz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C21</t>
-  </si>
-  <si>
-    <t xml:space="preserve">15n</t>
+    <t xml:space="preserve">2.2n</t>
   </si>
   <si>
     <t xml:space="preserve">poliester 5 % o C0G</t>
   </si>
   <si>
-    <t xml:space="preserve">condensador poliester 15nF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2A103J poliester 10nF 100V + 2A472K poliester 4.7nF 100V, en paralelo (par)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">15 nF agotado (2A153J en Global; tampoco en MechatronicStore): 10n + 4.7n en paralelo = 14.7 nF (f0 +1 %, Q -1 %). Cantidad en pares; precio del par ($50 + $60)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C22</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.2n</t>
-  </si>
-  <si>
     <t xml:space="preserve">condensador poliester 2.2nF</t>
   </si>
   <si>
@@ -544,13 +559,13 @@
     <t xml:space="preserve">cable dupont macho-hembra (tira de 40)</t>
   </si>
   <si>
-    <t xml:space="preserve">Por confirmar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tira de 40 jumpers Dupont M-H (compartida: A1-A3, 5 V/GND, microfono)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Llenar tienda y precio de la tira. CH1-A1 (PA9), CH2-A2 (PA10), CH3-A3 (PA12). Mas 1 cable de GND. A0 no: comparte ADC con USB1 ISENSE (UM3300)</t>
+    <t xml:space="preserve">JPMH20 cable Dupont M-H 20 cm (1 unidad)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Parcial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Son cables sueltos, no una tira de 40. FALTAN 3. CH1-A1 (PA9), CH2-A2 (PA10), CH3-A3 (PA12). Mas 1 cable de GND. A0 no: comparte ADC con USB1 ISENSE (UM3300)</t>
   </si>
   <si>
     <t xml:space="preserve">8 VREF 1.65 V (compartido)</t>
@@ -787,216 +802,246 @@
     <t xml:space="preserve">cable dupont macho-hembra</t>
   </si>
   <si>
-    <t xml:space="preserve">Tira de 40 jumpers Dupont M-H (compartida)</t>
+    <t xml:space="preserve">Pendiente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FALTA EN EL CARRITO. Usar powerbank o PC a bateria mientras haya electrodos puestos (ver Notas de seguridad)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12 ELECTRODOS Y CONECTORES (7)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">XE1P..XE3N, XER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Electrodo Ag/AgCl con broche 4 mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Skintact FS-RG1/10 32x41</t>
+  </si>
+  <si>
+    <t xml:space="preserve">desechable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Skintact FS-RG1/10 / Kendall Arbo H124SG 24 mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FALTA EN EL CARRITO. 7 por sesion (6 de senal + 1 RLD); caja de 50. Skintact para CH1, CH3 y RLD. CH2: Arbo H124SG (24 mm) o par sobre el menton. ISIMED 55x55 solo como RLD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cable de electrodo con broche (snap) 4 mm, idealmente apantallado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">broche 4 mm a pin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cable electrodo snap 4 mm / cable ECG broche</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FALTA EN EL CARRITO. Uno por electrodo; trenzar los dos de cada par. REVISAR EL TERMINAL antes de comprar: debe calzar en header hembra 2.54 mm. Si termina en DIN 1.5 mm touchproof (DIN 42802), cortar y crimpar terminal Dupont hembra o comprar bases touchproof. Alternativa: cable de 3 electrodos con jack 3.5 mm (el de los kits AD8232) + jack hembra 3.5 mm TRS en la placa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Conector de la placa para los 7 electrodos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hembra 2x8 2.54 THT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1105-8X2 conector hembra doble fila 16 vias</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1105-8X2 hembra doble fila 16 vias 2.54</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Una fila: CH1+ CH1- CH2+ CH2- CH3+ CH3- RLD GND(malla). Se enchufa el bus Dupont macho</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bus de 8 cables Dupont macho (separado de una tira de 40)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">jumper Dupont M-M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cable dupont macho-macho 20 cm tira 40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JPMM20 cable Dupont M-M 20 cm (1 unidad)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Son cables sueltos, no una tira de 40. FALTAN 6. Lado macho al conector 2x8; el otro extremo se une a los cables de electrodo (soldado + termorretractil o enchufado)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alcohol isopropilico / gel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">alcohol isopropilico</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FALTA EN EL CARRITO. Preparar la piel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13 MECANICA E INTERCONEXION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Perfboard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10 x 15 cm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fibra de vidrio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">placa perforada 10x15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ya lo tengo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tira de header macho 1x40 2.54 THT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">macho 1x40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tira poste recto una fila 40 pines</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1109-40L tira poste recto una fila 40 pines, pin largo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Salidas A1-A3 + GND, 5 V/GND y microfono</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tira de header hembra 1x40 2.54 THT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hembra 1x40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tira 40 pines header hembra 2.54</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fila de 40 pines header hembra 2.54 (GD2-3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zocalo de los 3 modulos INA333 (se cambian sin desoldar)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cable para puentes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24 AWG rigido</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cable UTP Cat6 24 AWG unifilar (por metro)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6UNI UTP Cat6 4 pares 24 AWG unifilar (m)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3 m. UTP: 8 hilos rigidos por metro. Rigido: no usarlo para los cables de electrodo (se corta al doblarse)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14 MICROFONO DE REFERENCIA (I2S)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Modulo microfono digital INMP441 (I2S)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INMP441</t>
+  </si>
+  <si>
+    <t xml:space="preserve">modulo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">modulo microfono INMP441</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INMP441 sensor microfono omnidireccional (pagina 5044)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A SAI/I2S del STM32N6570-DK (pines por definir en CubeMX). Alternativa sin cableado: microfono MEMS PDM que trae el DK (U13)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cables Dupont para el microfono</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FALTA EN EL CARRITO. VDD 3.3V, GND, SCK, WS, SD, L/R (L/R a GND)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOTAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FALTA COMPRAR (no esta en los carritos del 4-oct-2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cant.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Que</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Donde</t>
+  </si>
+  <si>
+    <t xml:space="preserve">jumper Dupont M-H Cable a Arduino A1..A3 del STM32N6570-DK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MechatronicStore / Global. 1 tira de 40 M-H cubre las 3 filas M-H (14 cables)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compraste 2 de 5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">jumper Dupont M-H Cable 5 V y GND desde el DK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MechatronicStore / Global (misma tira M-H)</t>
   </si>
   <si>
     <t xml:space="preserve">Usar powerbank o PC a bateria mientras haya electrodos puestos (ver Notas de seguridad)</t>
   </si>
   <si>
-    <t xml:space="preserve">12 ELECTRODOS Y CONECTORES (7)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">XE1P..XE3N, XER</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Electrodo Ag/AgCl con broche 4 mm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Skintact FS-RG1/10 32x41</t>
-  </si>
-  <si>
-    <t xml:space="preserve">desechable</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Skintact FS-RG1/10 / Kendall Arbo H124SG 24 mm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pendiente</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FALTA EN EL CARRITO. 7 por sesion (6 de senal + 1 RLD); caja de 50. Skintact para CH1, CH3 y RLD. CH2: Arbo H124SG (24 mm) o par sobre el menton. ISIMED 55x55 solo como RLD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cable de electrodo con broche (snap) 4 mm, idealmente apantallado</t>
-  </si>
-  <si>
-    <t xml:space="preserve">broche 4 mm a pin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cable electrodo snap 4 mm / cable ECG broche</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FALTA EN EL CARRITO. Uno por electrodo; trenzar los dos de cada par. REVISAR EL TERMINAL antes de comprar: debe calzar en header hembra 2.54 mm. Si termina en DIN 1.5 mm touchproof (DIN 42802), cortar y crimpar terminal Dupont hembra o comprar bases touchproof. Alternativa: cable de 3 electrodos con jack 3.5 mm (el de los kits AD8232) + jack hembra 3.5 mm TRS en la placa</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Conector de la placa para los 7 electrodos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">hembra 2x8 2.54 THT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1105-8X2 conector hembra doble fila 16 vias</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1105-8X2 hembra doble fila 16 vias 2.54</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Una fila: CH1+ CH1- CH2+ CH2- CH3+ CH3- RLD GND(malla). Se enchufa el bus Dupont macho</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bus de 8 cables Dupont macho (separado de una tira de 40)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">jumper Dupont M-M</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cable dupont macho-macho 20 cm tira 40</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tira de 40 jumpers Dupont M-M</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Llenar tienda y precio de la tira. Lado macho al conector 2x8; el otro extremo se une a los cables de electrodo (soldado + termorretractil o enchufado)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alcohol isopropilico / gel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">alcohol isopropilico</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FALTA EN EL CARRITO. Preparar la piel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">13 MECANICA E INTERCONEXION</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Perfboard</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10 x 15 cm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fibra de vidrio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">placa perforada 10x15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ya lo tengo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tira de header macho 1x40 2.54 THT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">macho 1x40</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tira poste recto una fila 40 pines</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1109-40L tira poste recto una fila 40 pines, pin largo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Salidas A1-A3 + GND, 5 V/GND y microfono</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tira de header hembra 1x40 2.54 THT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">hembra 1x40</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tira 40 pines header hembra 2.54</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fila de 40 pines header hembra 2.54 (GD2-3)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Zocalo de los 3 modulos INA333 (se cambian sin desoldar)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cable para puentes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">24 AWG rigido</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cable UTP Cat6 24 AWG unifilar (por metro)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6UNI UTP Cat6 4 pares 24 AWG unifilar (m)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3 m. UTP: 8 hilos rigidos por metro. Rigido: no usarlo para los cables de electrodo (se corta al doblarse)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">14 MICROFONO DE REFERENCIA (I2S)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Modulo microfono digital INMP441 (I2S)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">INMP441</t>
-  </si>
-  <si>
-    <t xml:space="preserve">modulo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">modulo microfono INMP441</t>
-  </si>
-  <si>
-    <t xml:space="preserve">INMP441 sensor microfono omnidireccional (pagina 5044)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A SAI/I2S del STM32N6570-DK (pines por definir en CubeMX). Alternativa sin cableado: microfono MEMS PDM que trae el DK (U13)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cables Dupont para el microfono</t>
+    <t xml:space="preserve">Skintact FS-RG1/10 32x41 Electrodo Ag/AgCl con broche 4 mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiendas de insumos medicos / Mercado Libre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7 por sesion (6 de senal + 1 RLD); caja de 50. Skintact para CH1, CH3 y RLD. CH2: Arbo H124SG (24 mm) o par sobre el menton. ISIMED 55x55 solo como RLD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">broche 4 mm a pin Cable de electrodo con broche (snap) 4 mm, idealmente apantallado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MechatronicStore ("cable de electrodos AD8232") / tiendas medicas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Uno por electrodo; trenzar los dos de cada par. REVISAR EL TERMINAL antes de comprar: debe calzar en header hembra 2.54 mm. Si termina en DIN 1.5 mm touchproof (DIN 42802), cortar y crimpar terminal Dupont hembra o comprar bases touchproof. Alternativa: cable de 3 electrodos con jack 3.5 mm (el de los kits AD8232) + jack hembra 3.5 mm TRS en la placa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">jumper Dupont M-M Bus de 8 cables Dupont macho (separado de una tira de 40)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MechatronicStore / Global. 1 tira de 40 M-M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compraste 2 de 8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Farmacia / ferreteria</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Preparar la piel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">jumper Dupont M-H Cables Dupont para el microfono</t>
   </si>
   <si>
     <t xml:space="preserve">VDD 3.3V, GND, SCK, WS, SD, L/R (L/R a GND)</t>
   </si>
   <si>
-    <t xml:space="preserve">TOTAL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FALTA COMPRAR (no esta en los carritos del 4-oct-2026)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cant.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Que</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Donde</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Skintact FS-RG1/10 32x41 Electrodo Ag/AgCl con broche 4 mm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tiendas de insumos medicos / Mercado Libre</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7 por sesion (6 de senal + 1 RLD); caja de 50. Skintact para CH1, CH3 y RLD. CH2: Arbo H124SG (24 mm) o par sobre el menton. ISIMED 55x55 solo como RLD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">broche 4 mm a pin Cable de electrodo con broche (snap) 4 mm, idealmente apantallado</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MechatronicStore ("cable de electrodos AD8232") / tiendas medicas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Uno por electrodo; trenzar los dos de cada par. REVISAR EL TERMINAL antes de comprar: debe calzar en header hembra 2.54 mm. Si termina en DIN 1.5 mm touchproof (DIN 42802), cortar y crimpar terminal Dupont hembra o comprar bases touchproof. Alternativa: cable de 3 electrodos con jack 3.5 mm (el de los kits AD8232) + jack hembra 3.5 mm TRS en la placa</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Farmacia / ferreteria</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Preparar la piel</t>
-  </si>
-  <si>
     <t xml:space="preserve">Resumen por modulo</t>
   </si>
   <si>
@@ -1006,15 +1051,18 @@
     <t xml:space="preserve">Pendientes</t>
   </si>
   <si>
-    <t xml:space="preserve">En carrito (CLP)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Por agregar (CLP)</t>
+    <t xml:space="preserve">Comprado (CLP)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">En carrito / por agregar (CLP)</t>
   </si>
   <si>
     <t xml:space="preserve">Faltan en los carritos</t>
   </si>
   <si>
+    <t xml:space="preserve">3 x jumper Dupont M-H  Cable 5 V y GND desde el DK</t>
+  </si>
+  <si>
     <t xml:space="preserve">50 x Skintact FS-RG1/10 32x41  Electrodo Ag/AgCl con broche 4 mm</t>
   </si>
   <si>
@@ -1027,25 +1075,52 @@
     <t xml:space="preserve">2 x 10 x 15 cm  Perfboard</t>
   </si>
   <si>
+    <t xml:space="preserve">6 x jumper Dupont M-H  Cables Dupont para el microfono</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pedidos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Global Electronica: Pedido BVGDHKTGU (4-oct-2026), retiro en tienda Global (Vina del Mar). Total $39.433</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MechatronicStore: Pedido del 4-oct-2026, despacho Bluexpress (gratis). Total $28.450</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARMADO: condensadores en paralelo y polaridades</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cm1 (MFB, x3 canales) = 100 nF (2A104K) EN PARALELO con 47 nF (2A473J): los dos entre el nodo MA (union Rm1-Rm2-Rm3) y GND.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C21 (Sallen-Key, x3 canales) = 10 nF (2A103J) EN PARALELO con 4.7 nF (2A472K): los dos entre la union Rlb1-Rlb2 y la salida del op-amp del SK.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cm0 (10 uF electrolitico): entre sus patas hay ~0 V DC; cualquier orientacion sirve. Por convencion: + hacia la salida del HPF.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LDO: CM105 (1 uF ceramico) en paralelo con el CE50102 (1 uF electrolitico) a la salida, pegados a los pines OUT y GND.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La simulacion ya usa los valores armados: CM1 = 147n y C21 = 14.7n.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Avisos de la compra</t>
   </si>
   <si>
-    <t xml:space="preserve">Cm1 = 100n + 47n poliester en paralelo (147 nF) y C21 = 10n + 4.7n poliester en paralelo (14.7 nF): no habia 150 nF y el 15 nF estaba agotado.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Falta: electrodos, cables de electrodo y alcohol (ver FALTA COMPRAR). Perfboard e insumos de soldadura: ya los tienes.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tiras Dupont M-H y M-M: llenar tienda y precio en la hoja BoM por modulo.</t>
+    <t xml:space="preserve">Pedidos hechos el 4-oct-2026: Global $39.433 (retiro en tienda) + MechatronicStore $28.450 (Bluexpress) = $67.883.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dupont: JPMH20/JPMM20 son cables SUELTOS. Tienes 2 M-H y 2 M-M; el diseno usa 14 M-H y 8 M-M (faltan 12 M-H y 6 M-M; Global tiene stock, $50 c/u).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Falta: electrodos, cables de electrodo y alcohol (ver FALTA COMPRAR).</t>
   </si>
   <si>
     <t xml:space="preserve">Resistencias de carbon 5 % en vez de pelicula metalica 1 %: aceptado para la demo (ganancia por canal +-7 %, se normaliza en firmware). Para produccion: 1 %.</t>
   </si>
   <si>
-    <t xml:space="preserve">Ajustes opcionales: S08D8 12 -&gt; 7 (ahorro $1.250); 100k 2 W -&gt; 1/4 W si hay stock (ahorro ~$1.700).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Precios con IVA, sin despacho.</t>
+    <t xml:space="preserve">Precios con IVA.</t>
   </si>
   <si>
     <t xml:space="preserve">Condiciones que debe cumplir cada circuito integrado (para elegir reemplazos)</t>
@@ -1443,7 +1518,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="\$#,##0;&quot;($&quot;#,##0\);\-"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="15">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1538,6 +1613,14 @@
       <family val="0"/>
       <charset val="1"/>
     </font>
+    <font>
+      <b val="true"/>
+      <sz val="11"/>
+      <color rgb="FF1F3A5F"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -1614,7 +1697,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1700,6 +1783,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2028,7 +2115,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:S81"/>
+  <dimension ref="A1:S85"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
@@ -3202,7 +3289,7 @@
       </c>
       <c r="S25" s="5"/>
     </row>
-    <row r="26" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="s">
         <v>105</v>
       </c>
@@ -3216,10 +3303,10 @@
         <v>131</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="G26" s="5" t="n">
         <v>1</v>
@@ -3239,13 +3326,13 @@
         <v>4</v>
       </c>
       <c r="L26" s="5" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="M26" s="6" t="s">
         <v>28</v>
       </c>
       <c r="N26" s="6" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="O26" s="6" t="n">
         <v>4</v>
@@ -3261,7 +3348,7 @@
         <v>30</v>
       </c>
       <c r="S26" s="5" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3269,19 +3356,19 @@
         <v>105</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="G27" s="5" t="n">
         <v>1</v>
@@ -3301,13 +3388,13 @@
         <v>4</v>
       </c>
       <c r="L27" s="5" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="M27" s="6" t="s">
         <v>28</v>
       </c>
       <c r="N27" s="6" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="O27" s="6" t="n">
         <v>4</v>
@@ -3323,7 +3410,7 @@
         <v>30</v>
       </c>
       <c r="S27" s="5" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3331,7 +3418,7 @@
         <v>105</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C28" s="5" t="s">
         <v>101</v>
@@ -3365,7 +3452,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B29" s="4"/>
       <c r="C29" s="4" t="s">
@@ -3390,16 +3477,16 @@
     </row>
     <row r="30" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="5" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E30" s="5" t="s">
         <v>90</v>
@@ -3447,27 +3534,27 @@
         <v>30</v>
       </c>
       <c r="S30" s="5" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="5" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>137</v>
+        <v>151</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="F31" s="5" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="G31" s="5" t="n">
         <v>1</v>
@@ -3487,13 +3574,13 @@
         <v>4</v>
       </c>
       <c r="L31" s="5" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="M31" s="6" t="s">
         <v>28</v>
       </c>
       <c r="N31" s="6" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="O31" s="6" t="n">
         <v>4</v>
@@ -3509,27 +3596,27 @@
         <v>30</v>
       </c>
       <c r="S31" s="5" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="5" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>130</v>
+        <v>159</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="F32" s="5" t="s">
-        <v>151</v>
+        <v>161</v>
       </c>
       <c r="G32" s="5" t="n">
         <v>1</v>
@@ -3549,13 +3636,13 @@
         <v>4</v>
       </c>
       <c r="L32" s="5" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="M32" s="6" t="s">
         <v>28</v>
       </c>
       <c r="N32" s="6" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="O32" s="6" t="n">
         <v>4</v>
@@ -3574,10 +3661,10 @@
     </row>
     <row r="33" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="5" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="C33" s="5" t="s">
         <v>101</v>
@@ -3611,7 +3698,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="B34" s="4"/>
       <c r="C34" s="4" t="s">
@@ -3636,19 +3723,19 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="5" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="F35" s="5" t="s">
         <v>41</v>
@@ -3671,13 +3758,13 @@
         <v>4</v>
       </c>
       <c r="L35" s="5" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="M35" s="6" t="s">
         <v>28</v>
       </c>
       <c r="N35" s="6" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="O35" s="6" t="n">
         <v>6</v>
@@ -3696,22 +3783,22 @@
     </row>
     <row r="36" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="5" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="E36" s="5" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F36" s="5" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="G36" s="5" t="n">
         <v>1</v>
@@ -3731,13 +3818,13 @@
         <v>4</v>
       </c>
       <c r="L36" s="5" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="M36" s="6" t="s">
         <v>28</v>
       </c>
       <c r="N36" s="6" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="O36" s="6" t="n">
         <v>4</v>
@@ -3756,19 +3843,19 @@
     </row>
     <row r="37" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="5" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="D37" s="5" t="s">
         <v>102</v>
       </c>
       <c r="E37" s="5" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="F37" s="5" t="s">
         <v>102</v>
@@ -3791,36 +3878,38 @@
         <v>5</v>
       </c>
       <c r="L37" s="5" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="M37" s="6" t="s">
-        <v>172</v>
+        <v>28</v>
       </c>
       <c r="N37" s="6" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="O37" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="P37" s="7"/>
-      <c r="Q37" s="8" t="str">
+        <v>2</v>
+      </c>
+      <c r="P37" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="Q37" s="8" t="n">
         <f aca="false">IF(P37="","",IF(O37="",K37,O37)*P37)</f>
-        <v/>
-      </c>
-      <c r="R37" s="6" t="s">
-        <v>30</v>
+        <v>100</v>
+      </c>
+      <c r="R37" s="9" t="s">
+        <v>178</v>
       </c>
       <c r="S37" s="5" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="4" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="B38" s="4"/>
       <c r="C38" s="4" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="D38" s="4"/>
       <c r="E38" s="4"/>
@@ -3841,13 +3930,13 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="5" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="D39" s="5" t="s">
         <v>25</v>
@@ -3876,7 +3965,7 @@
         <v>2</v>
       </c>
       <c r="L39" s="5" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="M39" s="6" t="s">
         <v>28</v>
@@ -3901,13 +3990,13 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="5" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="D40" s="5" t="s">
         <v>108</v>
@@ -3916,7 +4005,7 @@
         <v>108</v>
       </c>
       <c r="F40" s="5" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="G40" s="5" t="n">
         <v>1</v>
@@ -3936,7 +4025,7 @@
         <v>1</v>
       </c>
       <c r="L40" s="5" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
       <c r="M40" s="6" t="s">
         <v>28</v>
@@ -3961,10 +4050,10 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="5" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="C41" s="5" t="s">
         <v>101</v>
@@ -3998,11 +4087,11 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="4" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="B42" s="4"/>
       <c r="C42" s="4" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="D42" s="4"/>
       <c r="E42" s="4"/>
@@ -4023,19 +4112,19 @@
     </row>
     <row r="43" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="5" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
       <c r="D43" s="5" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="E43" s="5" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
       <c r="F43" s="5" t="s">
         <v>41</v>
@@ -4058,13 +4147,13 @@
         <v>4</v>
       </c>
       <c r="L43" s="5" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
       <c r="M43" s="6" t="s">
         <v>28</v>
       </c>
       <c r="N43" s="6" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="O43" s="6" t="n">
         <v>6</v>
@@ -4083,22 +4172,22 @@
     </row>
     <row r="44" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="5" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>192</v>
+        <v>197</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="D44" s="5" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="E44" s="5" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F44" s="5" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="G44" s="5" t="n">
         <v>1</v>
@@ -4118,13 +4207,13 @@
         <v>2</v>
       </c>
       <c r="L44" s="5" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="M44" s="6" t="s">
         <v>28</v>
       </c>
       <c r="N44" s="6" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="O44" s="6" t="n">
         <v>2</v>
@@ -4140,27 +4229,27 @@
         <v>30</v>
       </c>
       <c r="S44" s="5" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="5" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>196</v>
+        <v>201</v>
       </c>
       <c r="D45" s="5" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="E45" s="5" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="F45" s="5" t="s">
-        <v>198</v>
+        <v>203</v>
       </c>
       <c r="G45" s="5" t="n">
         <v>1</v>
@@ -4180,13 +4269,13 @@
         <v>2</v>
       </c>
       <c r="L45" s="5" t="s">
-        <v>199</v>
+        <v>204</v>
       </c>
       <c r="M45" s="6" t="s">
         <v>28</v>
       </c>
       <c r="N45" s="6" t="s">
-        <v>200</v>
+        <v>205</v>
       </c>
       <c r="O45" s="6" t="n">
         <v>4</v>
@@ -4205,19 +4294,19 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="5" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
       <c r="D46" s="5" t="s">
-        <v>203</v>
+        <v>208</v>
       </c>
       <c r="E46" s="5" t="s">
-        <v>203</v>
+        <v>208</v>
       </c>
       <c r="F46" s="5" t="s">
         <v>41</v>
@@ -4240,13 +4329,13 @@
         <v>2</v>
       </c>
       <c r="L46" s="5" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
       <c r="M46" s="6" t="s">
         <v>28</v>
       </c>
       <c r="N46" s="6" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="O46" s="6" t="n">
         <v>4</v>
@@ -4262,15 +4351,15 @@
         <v>30</v>
       </c>
       <c r="S46" s="5" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="5" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="B47" s="5" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="C47" s="5" t="s">
         <v>101</v>
@@ -4304,11 +4393,11 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="4" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
       <c r="B48" s="4"/>
       <c r="C48" s="4" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="D48" s="4"/>
       <c r="E48" s="4"/>
@@ -4329,22 +4418,22 @@
     </row>
     <row r="49" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="5" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
       <c r="B49" s="5" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="C49" s="5" t="s">
-        <v>210</v>
+        <v>215</v>
       </c>
       <c r="D49" s="5" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
       <c r="E49" s="5" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="F49" s="5" t="s">
-        <v>213</v>
+        <v>218</v>
       </c>
       <c r="G49" s="5" t="n">
         <v>6</v>
@@ -4364,13 +4453,13 @@
         <v>6</v>
       </c>
       <c r="L49" s="5" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="M49" s="6" t="s">
         <v>28</v>
       </c>
       <c r="N49" s="6" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="O49" s="6" t="n">
         <v>6</v>
@@ -4386,27 +4475,27 @@
         <v>30</v>
       </c>
       <c r="S49" s="5" t="s">
-        <v>214</v>
+        <v>219</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="5" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
       <c r="B50" s="5" t="s">
         <v>102</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
       <c r="D50" s="5" t="s">
         <v>102</v>
       </c>
       <c r="E50" s="5" t="s">
-        <v>216</v>
+        <v>221</v>
       </c>
       <c r="F50" s="5" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
       <c r="G50" s="5" t="n">
         <v>6</v>
@@ -4426,13 +4515,13 @@
         <v>7</v>
       </c>
       <c r="L50" s="5" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
       <c r="M50" s="6" t="s">
         <v>28</v>
       </c>
       <c r="N50" s="6" t="s">
-        <v>216</v>
+        <v>221</v>
       </c>
       <c r="O50" s="6" t="n">
         <v>12</v>
@@ -4448,27 +4537,27 @@
         <v>30</v>
       </c>
       <c r="S50" s="5" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="5" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
       <c r="B51" s="5" t="s">
         <v>102</v>
       </c>
       <c r="C51" s="5" t="s">
-        <v>220</v>
+        <v>225</v>
       </c>
       <c r="D51" s="5" t="s">
         <v>102</v>
       </c>
       <c r="E51" s="5" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="F51" s="5" t="s">
-        <v>222</v>
+        <v>227</v>
       </c>
       <c r="G51" s="5"/>
       <c r="H51" s="5"/>
@@ -4476,7 +4565,7 @@
       <c r="J51" s="5"/>
       <c r="K51" s="5"/>
       <c r="L51" s="5" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
       <c r="M51" s="5"/>
       <c r="N51" s="5"/>
@@ -4487,18 +4576,18 @@
         <v>103</v>
       </c>
       <c r="S51" s="5" t="s">
-        <v>224</v>
+        <v>229</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="5" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
       <c r="B52" s="5" t="s">
         <v>102</v>
       </c>
       <c r="C52" s="5" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
       <c r="D52" s="5" t="s">
         <v>76</v>
@@ -4554,11 +4643,11 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="4" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
       <c r="B53" s="4"/>
       <c r="C53" s="4" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="D53" s="4"/>
       <c r="E53" s="4"/>
@@ -4579,22 +4668,22 @@
     </row>
     <row r="54" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="5" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
       <c r="B54" s="5" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
       <c r="C54" s="5" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="D54" s="5" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="E54" s="5" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="F54" s="5" t="s">
-        <v>231</v>
+        <v>236</v>
       </c>
       <c r="G54" s="5" t="n">
         <v>1</v>
@@ -4614,13 +4703,13 @@
         <v>2</v>
       </c>
       <c r="L54" s="5" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="M54" s="6" t="s">
         <v>28</v>
       </c>
       <c r="N54" s="6" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="O54" s="6" t="n">
         <v>2</v>
@@ -4636,18 +4725,18 @@
         <v>30</v>
       </c>
       <c r="S54" s="5" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="5" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
       <c r="B55" s="5" t="s">
         <v>102</v>
       </c>
       <c r="C55" s="5" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
       <c r="D55" s="5" t="s">
         <v>102</v>
@@ -4673,24 +4762,24 @@
         <v>103</v>
       </c>
       <c r="S55" s="5" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="5" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
       <c r="B56" s="5" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="C56" s="5" t="s">
-        <v>236</v>
+        <v>241</v>
       </c>
       <c r="D56" s="5" t="s">
-        <v>237</v>
+        <v>242</v>
       </c>
       <c r="E56" s="5" t="s">
-        <v>237</v>
+        <v>242</v>
       </c>
       <c r="F56" s="5" t="s">
         <v>77</v>
@@ -4713,13 +4802,13 @@
         <v>3</v>
       </c>
       <c r="L56" s="5" t="s">
-        <v>238</v>
+        <v>243</v>
       </c>
       <c r="M56" s="6" t="s">
         <v>28</v>
       </c>
       <c r="N56" s="6" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="O56" s="6" t="n">
         <v>3</v>
@@ -4735,27 +4824,27 @@
         <v>30</v>
       </c>
       <c r="S56" s="5" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="5" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
       <c r="B57" s="5" t="s">
-        <v>241</v>
+        <v>246</v>
       </c>
       <c r="C57" s="5" t="s">
+        <v>247</v>
+      </c>
+      <c r="D57" s="5" t="s">
         <v>242</v>
       </c>
-      <c r="D57" s="5" t="s">
-        <v>237</v>
-      </c>
       <c r="E57" s="5" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="F57" s="5" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="G57" s="5" t="n">
         <v>1</v>
@@ -4775,13 +4864,13 @@
         <v>2</v>
       </c>
       <c r="L57" s="5" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="M57" s="6" t="s">
         <v>28</v>
       </c>
       <c r="N57" s="6" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="O57" s="6" t="n">
         <v>2</v>
@@ -4797,18 +4886,18 @@
         <v>30</v>
       </c>
       <c r="S57" s="5" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="5" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
       <c r="B58" s="5" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="C58" s="5" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="D58" s="5" t="s">
         <v>108</v>
@@ -4817,7 +4906,7 @@
         <v>108</v>
       </c>
       <c r="F58" s="5" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
       <c r="G58" s="5" t="n">
         <v>1</v>
@@ -4837,7 +4926,7 @@
         <v>2</v>
       </c>
       <c r="L58" s="5" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
       <c r="M58" s="6" t="s">
         <v>28</v>
@@ -4862,19 +4951,19 @@
     </row>
     <row r="59" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="5" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
       <c r="B59" s="5" t="s">
         <v>102</v>
       </c>
       <c r="C59" s="5" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="D59" s="5" t="s">
         <v>102</v>
       </c>
       <c r="E59" s="5" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="F59" s="5" t="s">
         <v>102</v>
@@ -4897,36 +4986,30 @@
         <v>3</v>
       </c>
       <c r="L59" s="5" t="s">
-        <v>252</v>
-      </c>
-      <c r="M59" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="N59" s="6" t="s">
-        <v>253</v>
-      </c>
-      <c r="O59" s="6" t="n">
-        <v>3</v>
-      </c>
+        <v>257</v>
+      </c>
+      <c r="M59" s="6"/>
+      <c r="N59" s="6"/>
+      <c r="O59" s="6"/>
       <c r="P59" s="7"/>
       <c r="Q59" s="8" t="str">
         <f aca="false">IF(P59="","",IF(O59="",K59,O59)*P59)</f>
         <v/>
       </c>
-      <c r="R59" s="6" t="s">
-        <v>30</v>
+      <c r="R59" s="9" t="s">
+        <v>258</v>
       </c>
       <c r="S59" s="5" t="s">
-        <v>254</v>
+        <v>259</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="4" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="B60" s="4"/>
       <c r="C60" s="4" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="D60" s="4"/>
       <c r="E60" s="4"/>
@@ -4947,22 +5030,22 @@
     </row>
     <row r="61" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="5" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="B61" s="5" t="s">
-        <v>256</v>
+        <v>261</v>
       </c>
       <c r="C61" s="5" t="s">
-        <v>257</v>
+        <v>262</v>
       </c>
       <c r="D61" s="5" t="s">
         <v>102</v>
       </c>
       <c r="E61" s="5" t="s">
-        <v>258</v>
+        <v>263</v>
       </c>
       <c r="F61" s="5" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
       <c r="G61" s="5" t="n">
         <v>7</v>
@@ -4982,7 +5065,7 @@
         <v>50</v>
       </c>
       <c r="L61" s="5" t="s">
-        <v>260</v>
+        <v>265</v>
       </c>
       <c r="M61" s="6"/>
       <c r="N61" s="6"/>
@@ -4993,27 +5076,27 @@
         <v/>
       </c>
       <c r="R61" s="9" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="S61" s="5" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="5" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="B62" s="5" t="s">
         <v>102</v>
       </c>
       <c r="C62" s="5" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="D62" s="5" t="s">
         <v>102</v>
       </c>
       <c r="E62" s="5" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="F62" s="5" t="s">
         <v>102</v>
@@ -5036,7 +5119,7 @@
         <v>8</v>
       </c>
       <c r="L62" s="5" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="M62" s="6"/>
       <c r="N62" s="6"/>
@@ -5047,27 +5130,27 @@
         <v/>
       </c>
       <c r="R62" s="9" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="S62" s="5" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="5" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="B63" s="5" t="s">
         <v>102</v>
       </c>
       <c r="C63" s="5" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
       <c r="D63" s="5" t="s">
         <v>102</v>
       </c>
       <c r="E63" s="5" t="s">
-        <v>268</v>
+        <v>272</v>
       </c>
       <c r="F63" s="5" t="s">
         <v>102</v>
@@ -5090,13 +5173,13 @@
         <v>2</v>
       </c>
       <c r="L63" s="5" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
       <c r="M63" s="6" t="s">
         <v>28</v>
       </c>
       <c r="N63" s="6" t="s">
-        <v>270</v>
+        <v>274</v>
       </c>
       <c r="O63" s="6" t="n">
         <v>2</v>
@@ -5112,24 +5195,24 @@
         <v>30</v>
       </c>
       <c r="S63" s="5" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="5" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="B64" s="5" t="s">
         <v>102</v>
       </c>
       <c r="C64" s="5" t="s">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="D64" s="5" t="s">
         <v>102</v>
       </c>
       <c r="E64" s="5" t="s">
-        <v>273</v>
+        <v>277</v>
       </c>
       <c r="F64" s="5" t="s">
         <v>102</v>
@@ -5152,38 +5235,40 @@
         <v>8</v>
       </c>
       <c r="L64" s="5" t="s">
-        <v>274</v>
+        <v>278</v>
       </c>
       <c r="M64" s="6" t="s">
-        <v>172</v>
+        <v>28</v>
       </c>
       <c r="N64" s="6" t="s">
-        <v>275</v>
+        <v>279</v>
       </c>
       <c r="O64" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="P64" s="7"/>
-      <c r="Q64" s="8" t="str">
+        <v>2</v>
+      </c>
+      <c r="P64" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="Q64" s="8" t="n">
         <f aca="false">IF(P64="","",IF(O64="",K64,O64)*P64)</f>
-        <v/>
-      </c>
-      <c r="R64" s="6" t="s">
-        <v>30</v>
+        <v>100</v>
+      </c>
+      <c r="R64" s="9" t="s">
+        <v>178</v>
       </c>
       <c r="S64" s="5" t="s">
-        <v>276</v>
+        <v>280</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="5" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="B65" s="5" t="s">
         <v>102</v>
       </c>
       <c r="C65" s="5" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="D65" s="5" t="s">
         <v>102</v>
@@ -5212,7 +5297,7 @@
         <v>1</v>
       </c>
       <c r="L65" s="5" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
       <c r="M65" s="6"/>
       <c r="N65" s="6"/>
@@ -5223,19 +5308,19 @@
         <v/>
       </c>
       <c r="R65" s="9" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="S65" s="5" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="4" t="s">
-        <v>280</v>
+        <v>284</v>
       </c>
       <c r="B66" s="4"/>
       <c r="C66" s="4" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="D66" s="4"/>
       <c r="E66" s="4"/>
@@ -5256,22 +5341,22 @@
     </row>
     <row r="67" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="5" t="s">
-        <v>280</v>
+        <v>284</v>
       </c>
       <c r="B67" s="5" t="s">
         <v>102</v>
       </c>
       <c r="C67" s="5" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="D67" s="5" t="s">
         <v>102</v>
       </c>
       <c r="E67" s="5" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="F67" s="5" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="G67" s="5" t="n">
         <v>1</v>
@@ -5291,7 +5376,7 @@
         <v>2</v>
       </c>
       <c r="L67" s="5" t="s">
-        <v>284</v>
+        <v>288</v>
       </c>
       <c r="M67" s="6"/>
       <c r="N67" s="6"/>
@@ -5302,25 +5387,25 @@
         <v/>
       </c>
       <c r="R67" s="6" t="s">
-        <v>285</v>
+        <v>289</v>
       </c>
       <c r="S67" s="5"/>
     </row>
     <row r="68" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="5" t="s">
-        <v>280</v>
+        <v>284</v>
       </c>
       <c r="B68" s="5" t="s">
         <v>102</v>
       </c>
       <c r="C68" s="5" t="s">
-        <v>286</v>
+        <v>290</v>
       </c>
       <c r="D68" s="5" t="s">
         <v>102</v>
       </c>
       <c r="E68" s="5" t="s">
-        <v>287</v>
+        <v>291</v>
       </c>
       <c r="F68" s="5" t="s">
         <v>102</v>
@@ -5343,13 +5428,13 @@
         <v>1</v>
       </c>
       <c r="L68" s="5" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="M68" s="6" t="s">
         <v>28</v>
       </c>
       <c r="N68" s="6" t="s">
-        <v>289</v>
+        <v>293</v>
       </c>
       <c r="O68" s="6" t="n">
         <v>1</v>
@@ -5365,24 +5450,24 @@
         <v>30</v>
       </c>
       <c r="S68" s="5" t="s">
-        <v>290</v>
+        <v>294</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="5" t="s">
-        <v>280</v>
+        <v>284</v>
       </c>
       <c r="B69" s="5" t="s">
         <v>102</v>
       </c>
       <c r="C69" s="5" t="s">
-        <v>291</v>
+        <v>295</v>
       </c>
       <c r="D69" s="5" t="s">
         <v>102</v>
       </c>
       <c r="E69" s="5" t="s">
-        <v>292</v>
+        <v>296</v>
       </c>
       <c r="F69" s="5" t="s">
         <v>102</v>
@@ -5405,13 +5490,13 @@
         <v>1</v>
       </c>
       <c r="L69" s="5" t="s">
-        <v>293</v>
+        <v>297</v>
       </c>
       <c r="M69" s="6" t="s">
         <v>43</v>
       </c>
       <c r="N69" s="6" t="s">
-        <v>294</v>
+        <v>298</v>
       </c>
       <c r="O69" s="6" t="n">
         <v>1</v>
@@ -5427,24 +5512,24 @@
         <v>30</v>
       </c>
       <c r="S69" s="5" t="s">
-        <v>295</v>
+        <v>299</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="5" t="s">
-        <v>280</v>
+        <v>284</v>
       </c>
       <c r="B70" s="5" t="s">
         <v>102</v>
       </c>
       <c r="C70" s="5" t="s">
-        <v>296</v>
+        <v>300</v>
       </c>
       <c r="D70" s="5" t="s">
         <v>102</v>
       </c>
       <c r="E70" s="5" t="s">
-        <v>297</v>
+        <v>301</v>
       </c>
       <c r="F70" s="5" t="s">
         <v>102</v>
@@ -5467,13 +5552,13 @@
         <v>1</v>
       </c>
       <c r="L70" s="5" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="M70" s="6" t="s">
         <v>28</v>
       </c>
       <c r="N70" s="6" t="s">
-        <v>299</v>
+        <v>303</v>
       </c>
       <c r="O70" s="6" t="n">
         <v>3</v>
@@ -5489,16 +5574,16 @@
         <v>30</v>
       </c>
       <c r="S70" s="5" t="s">
-        <v>300</v>
+        <v>304</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="4" t="s">
-        <v>301</v>
+        <v>305</v>
       </c>
       <c r="B71" s="4"/>
       <c r="C71" s="4" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="D71" s="4"/>
       <c r="E71" s="4"/>
@@ -5519,22 +5604,22 @@
     </row>
     <row r="72" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="5" t="s">
-        <v>301</v>
+        <v>305</v>
       </c>
       <c r="B72" s="5" t="s">
         <v>102</v>
       </c>
       <c r="C72" s="5" t="s">
-        <v>302</v>
+        <v>306</v>
       </c>
       <c r="D72" s="5" t="s">
         <v>102</v>
       </c>
       <c r="E72" s="5" t="s">
-        <v>303</v>
+        <v>307</v>
       </c>
       <c r="F72" s="5" t="s">
-        <v>304</v>
+        <v>308</v>
       </c>
       <c r="G72" s="5" t="n">
         <v>1</v>
@@ -5547,20 +5632,20 @@
         <v>1</v>
       </c>
       <c r="J72" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K72" s="5" t="n">
         <f aca="false">I72+J72</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L72" s="5" t="s">
-        <v>305</v>
+        <v>309</v>
       </c>
       <c r="M72" s="6" t="s">
         <v>28</v>
       </c>
       <c r="N72" s="6" t="s">
-        <v>306</v>
+        <v>310</v>
       </c>
       <c r="O72" s="6" t="n">
         <v>1</v>
@@ -5576,24 +5661,24 @@
         <v>30</v>
       </c>
       <c r="S72" s="5" t="s">
-        <v>307</v>
+        <v>311</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="5" t="s">
-        <v>301</v>
+        <v>305</v>
       </c>
       <c r="B73" s="5" t="s">
         <v>102</v>
       </c>
       <c r="C73" s="5" t="s">
-        <v>308</v>
+        <v>312</v>
       </c>
       <c r="D73" s="5" t="s">
         <v>102</v>
       </c>
       <c r="E73" s="5" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="F73" s="5" t="s">
         <v>102</v>
@@ -5616,116 +5701,178 @@
         <v>6</v>
       </c>
       <c r="L73" s="5" t="s">
-        <v>252</v>
-      </c>
-      <c r="M73" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="N73" s="6" t="s">
-        <v>253</v>
-      </c>
-      <c r="O73" s="6" t="n">
-        <v>6</v>
-      </c>
+        <v>257</v>
+      </c>
+      <c r="M73" s="6"/>
+      <c r="N73" s="6"/>
+      <c r="O73" s="6"/>
       <c r="P73" s="7"/>
       <c r="Q73" s="8" t="str">
         <f aca="false">IF(P73="","",IF(O73="",K73,O73)*P73)</f>
         <v/>
       </c>
-      <c r="R73" s="6" t="s">
-        <v>30</v>
+      <c r="R73" s="9" t="s">
+        <v>258</v>
       </c>
       <c r="S73" s="5" t="s">
-        <v>309</v>
+        <v>313</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="P75" s="10" t="s">
-        <v>310</v>
+        <v>314</v>
       </c>
       <c r="Q75" s="11" t="n">
         <f aca="false">SUM(Q5:Q73)</f>
-        <v>67683</v>
+        <v>67883</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="12" t="s">
-        <v>311</v>
+        <v>315</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="3" t="s">
-        <v>312</v>
+        <v>316</v>
       </c>
       <c r="B78" s="3" t="s">
-        <v>313</v>
+        <v>317</v>
       </c>
       <c r="C78" s="3" t="s">
         <v>13</v>
       </c>
       <c r="D78" s="3" t="s">
-        <v>314</v>
+        <v>318</v>
       </c>
       <c r="E78" s="3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="79" customFormat="false" ht="90.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="79" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="B79" s="13" t="s">
+        <v>319</v>
+      </c>
+      <c r="C79" s="13" t="s">
+        <v>176</v>
+      </c>
+      <c r="D79" s="13" t="s">
+        <v>320</v>
+      </c>
+      <c r="E79" s="13" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="80" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="B80" s="13" t="s">
+        <v>322</v>
+      </c>
+      <c r="C80" s="13" t="s">
+        <v>257</v>
+      </c>
+      <c r="D80" s="13" t="s">
+        <v>323</v>
+      </c>
+      <c r="E80" s="13" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="81" customFormat="false" ht="90.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="13" t="n">
         <v>50</v>
       </c>
-      <c r="B79" s="13" t="s">
-        <v>315</v>
-      </c>
-      <c r="C79" s="13" t="s">
-        <v>260</v>
-      </c>
-      <c r="D79" s="13" t="s">
-        <v>316</v>
-      </c>
-      <c r="E79" s="13" t="s">
-        <v>317</v>
-      </c>
-    </row>
-    <row r="80" customFormat="false" ht="191.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A80" s="13" t="n">
+      <c r="B81" s="13" t="s">
+        <v>325</v>
+      </c>
+      <c r="C81" s="13" t="s">
+        <v>265</v>
+      </c>
+      <c r="D81" s="13" t="s">
+        <v>326</v>
+      </c>
+      <c r="E81" s="13" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="82" customFormat="false" ht="191.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A82" s="13" t="n">
         <v>8</v>
       </c>
-      <c r="B80" s="13" t="s">
-        <v>318</v>
-      </c>
-      <c r="C80" s="13" t="s">
-        <v>265</v>
-      </c>
-      <c r="D80" s="13" t="s">
-        <v>319</v>
-      </c>
-      <c r="E80" s="13" t="s">
-        <v>320</v>
-      </c>
-    </row>
-    <row r="81" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A81" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="B81" s="13" t="s">
-        <v>277</v>
-      </c>
-      <c r="C81" s="13" t="s">
+      <c r="B82" s="13" t="s">
+        <v>328</v>
+      </c>
+      <c r="C82" s="13" t="s">
+        <v>269</v>
+      </c>
+      <c r="D82" s="13" t="s">
+        <v>329</v>
+      </c>
+      <c r="E82" s="13" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="83" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A83" s="13" t="n">
+        <v>6</v>
+      </c>
+      <c r="B83" s="13" t="s">
+        <v>331</v>
+      </c>
+      <c r="C83" s="13" t="s">
         <v>278</v>
       </c>
-      <c r="D81" s="13" t="s">
-        <v>321</v>
-      </c>
-      <c r="E81" s="13" t="s">
-        <v>322</v>
+      <c r="D83" s="13" t="s">
+        <v>332</v>
+      </c>
+      <c r="E83" s="13" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="84" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="B84" s="13" t="s">
+        <v>281</v>
+      </c>
+      <c r="C84" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="D84" s="13" t="s">
+        <v>334</v>
+      </c>
+      <c r="E84" s="13" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="85" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A85" s="13" t="n">
+        <v>6</v>
+      </c>
+      <c r="B85" s="13" t="s">
+        <v>336</v>
+      </c>
+      <c r="C85" s="13" t="s">
+        <v>257</v>
+      </c>
+      <c r="D85" s="13" t="s">
+        <v>323</v>
+      </c>
+      <c r="E85" s="13" t="s">
+        <v>337</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A4:S73"/>
   <dataValidations count="1">
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="R6:R7 R9:R11 R13:R15 R17:R19 R22:R27 R30:R32 R35:R37 R39:R40 R43:R46 R49:R50 R52 R54 R56:R59 R61:R65 R67:R70 R72:R73" type="list">
-      <formula1>"Pendiente,En carrito,Comprado,Ya lo tengo,No hay,No aplica"</formula1>
+      <formula1>"Pendiente,En carrito,Comprado,Parcial,Ya lo tengo,No hay,No aplica"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -5745,7 +5892,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D36"/>
+  <dimension ref="A1:D48"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="70"/>
@@ -5756,7 +5903,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>323</v>
+        <v>338</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5764,10 +5911,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>324</v>
+        <v>339</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>325</v>
+        <v>340</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>18</v>
@@ -5860,7 +6007,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B9" s="14" t="n">
         <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$73,A9,'BoM por modulo'!$R$5:$R$73,"&lt;&gt;No aplica",'BoM por modulo'!$R$5:$R$73,"&lt;&gt;")</f>
@@ -5877,7 +6024,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="B10" s="14" t="n">
         <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$73,A10,'BoM por modulo'!$R$5:$R$73,"&lt;&gt;No aplica",'BoM por modulo'!$R$5:$R$73,"&lt;&gt;")</f>
@@ -5889,12 +6036,12 @@
       </c>
       <c r="D10" s="15" t="n">
         <f aca="false">SUMIF('BoM por modulo'!$A$5:$A$73,A10,'BoM por modulo'!$Q$5:$Q$73)</f>
-        <v>540</v>
+        <v>640</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="B11" s="14" t="n">
         <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$73,A11,'BoM por modulo'!$R$5:$R$73,"&lt;&gt;No aplica",'BoM por modulo'!$R$5:$R$73,"&lt;&gt;")</f>
@@ -5911,7 +6058,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="14" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="B12" s="14" t="n">
         <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$73,A12,'BoM por modulo'!$R$5:$R$73,"&lt;&gt;No aplica",'BoM por modulo'!$R$5:$R$73,"&lt;&gt;")</f>
@@ -5928,7 +6075,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="14" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
       <c r="B13" s="14" t="n">
         <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$73,A13,'BoM por modulo'!$R$5:$R$73,"&lt;&gt;No aplica",'BoM por modulo'!$R$5:$R$73,"&lt;&gt;")</f>
@@ -5945,7 +6092,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="14" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
       <c r="B14" s="14" t="n">
         <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$73,A14,'BoM por modulo'!$R$5:$R$73,"&lt;&gt;No aplica",'BoM por modulo'!$R$5:$R$73,"&lt;&gt;")</f>
@@ -5953,7 +6100,7 @@
       </c>
       <c r="C14" s="14" t="n">
         <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$73,A14,'BoM por modulo'!$R$5:$R$73,"Pendiente")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D14" s="15" t="n">
         <f aca="false">SUMIF('BoM por modulo'!$A$5:$A$73,A14,'BoM por modulo'!$Q$5:$Q$73)</f>
@@ -5962,7 +6109,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="14" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="B15" s="14" t="n">
         <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$73,A15,'BoM por modulo'!$R$5:$R$73,"&lt;&gt;No aplica",'BoM por modulo'!$R$5:$R$73,"&lt;&gt;")</f>
@@ -5974,12 +6121,12 @@
       </c>
       <c r="D15" s="15" t="n">
         <f aca="false">SUMIF('BoM por modulo'!$A$5:$A$73,A15,'BoM por modulo'!$Q$5:$Q$73)</f>
-        <v>300</v>
+        <v>400</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="14" t="s">
-        <v>280</v>
+        <v>284</v>
       </c>
       <c r="B16" s="14" t="n">
         <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$73,A16,'BoM por modulo'!$R$5:$R$73,"&lt;&gt;No aplica",'BoM por modulo'!$R$5:$R$73,"&lt;&gt;")</f>
@@ -5996,7 +6143,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="14" t="s">
-        <v>301</v>
+        <v>305</v>
       </c>
       <c r="B17" s="14" t="n">
         <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$73,A17,'BoM por modulo'!$R$5:$R$73,"&lt;&gt;No aplica",'BoM por modulo'!$R$5:$R$73,"&lt;&gt;")</f>
@@ -6004,7 +6151,7 @@
       </c>
       <c r="C17" s="14" t="n">
         <f aca="false">COUNTIFS('BoM por modulo'!$A$5:$A$73,A17,'BoM por modulo'!$R$5:$R$73,"Pendiente")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D17" s="15" t="n">
         <f aca="false">SUMIF('BoM por modulo'!$A$5:$A$73,A17,'BoM por modulo'!$Q$5:$Q$73)</f>
@@ -6013,7 +6160,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="16" t="s">
-        <v>310</v>
+        <v>314</v>
       </c>
       <c r="B18" s="16" t="n">
         <f aca="false">SUM(B4:B17)</f>
@@ -6021,22 +6168,22 @@
       </c>
       <c r="C18" s="16" t="n">
         <f aca="false">SUM(C4:C17)</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D18" s="17" t="n">
         <f aca="false">SUM(D4:D17)</f>
-        <v>67683</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>67883</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
         <v>14</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>326</v>
+        <v>341</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>327</v>
+        <v>342</v>
       </c>
       <c r="D20" s="3"/>
     </row>
@@ -6045,11 +6192,11 @@
         <v>28</v>
       </c>
       <c r="B21" s="19" t="n">
-        <f aca="false">SUMIFS('BoM por modulo'!$Q$5:$Q$73,'BoM por modulo'!$M$5:$M$73,A21,'BoM por modulo'!$R$5:$R$73,"En carrito")</f>
-        <v>39233</v>
+        <f aca="false">SUMIFS('BoM por modulo'!$Q$5:$Q$73,'BoM por modulo'!$M$5:$M$73,A21,'BoM por modulo'!$R$5:$R$73,"Comprado")+SUMIFS('BoM por modulo'!$Q$5:$Q$73,'BoM por modulo'!$M$5:$M$73,A21,'BoM por modulo'!$R$5:$R$73,"Parcial")</f>
+        <v>39433</v>
       </c>
       <c r="C21" s="19" t="n">
-        <f aca="false">SUMIFS('BoM por modulo'!$Q$5:$Q$73,'BoM por modulo'!$M$5:$M$73,A21,'BoM por modulo'!$R$5:$R$73,"Pendiente")</f>
+        <f aca="false">SUMIFS('BoM por modulo'!$Q$5:$Q$73,'BoM por modulo'!$M$5:$M$73,A21,'BoM por modulo'!$R$5:$R$73,"En carrito")+SUMIFS('BoM por modulo'!$Q$5:$Q$73,'BoM por modulo'!$M$5:$M$73,A21,'BoM por modulo'!$R$5:$R$73,"Pendiente")</f>
         <v>0</v>
       </c>
     </row>
@@ -6058,30 +6205,30 @@
         <v>43</v>
       </c>
       <c r="B22" s="19" t="n">
-        <f aca="false">SUMIFS('BoM por modulo'!$Q$5:$Q$73,'BoM por modulo'!$M$5:$M$73,A22,'BoM por modulo'!$R$5:$R$73,"En carrito")</f>
+        <f aca="false">SUMIFS('BoM por modulo'!$Q$5:$Q$73,'BoM por modulo'!$M$5:$M$73,A22,'BoM por modulo'!$R$5:$R$73,"Comprado")+SUMIFS('BoM por modulo'!$Q$5:$Q$73,'BoM por modulo'!$M$5:$M$73,A22,'BoM por modulo'!$R$5:$R$73,"Parcial")</f>
         <v>28450</v>
       </c>
       <c r="C22" s="19" t="n">
-        <f aca="false">SUMIFS('BoM por modulo'!$Q$5:$Q$73,'BoM por modulo'!$M$5:$M$73,A22,'BoM por modulo'!$R$5:$R$73,"Pendiente")</f>
+        <f aca="false">SUMIFS('BoM por modulo'!$Q$5:$Q$73,'BoM por modulo'!$M$5:$M$73,A22,'BoM por modulo'!$R$5:$R$73,"En carrito")+SUMIFS('BoM por modulo'!$Q$5:$Q$73,'BoM por modulo'!$M$5:$M$73,A22,'BoM por modulo'!$R$5:$R$73,"Pendiente")</f>
         <v>0</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="20" t="s">
-        <v>328</v>
+        <v>343</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="18" t="s">
-        <v>329</v>
+        <v>344</v>
       </c>
       <c r="B25" s="21" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="18" t="s">
-        <v>330</v>
+        <v>345</v>
       </c>
       <c r="B26" s="21" t="s">
         <v>265</v>
@@ -6089,53 +6236,109 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="18" t="s">
-        <v>331</v>
+        <v>346</v>
       </c>
       <c r="B27" s="21" t="s">
-        <v>278</v>
+        <v>269</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="18" t="s">
-        <v>332</v>
+        <v>347</v>
       </c>
       <c r="B28" s="21" t="s">
-        <v>284</v>
+        <v>282</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="18" t="s">
+        <v>348</v>
+      </c>
+      <c r="B29" s="21" t="s">
+        <v>288</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="10" t="s">
-        <v>333</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="18" t="s">
-        <v>334</v>
+      <c r="A30" s="18" t="s">
+        <v>349</v>
+      </c>
+      <c r="B30" s="21" t="s">
+        <v>257</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="18" t="s">
-        <v>335</v>
+      <c r="A32" s="10" t="s">
+        <v>350</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="18" t="s">
-        <v>336</v>
+        <v>351</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="18" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="18" t="s">
-        <v>338</v>
+        <v>352</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="18" t="s">
-        <v>339</v>
+      <c r="A36" s="22" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="18" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="18" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="18" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="18" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="18" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="10" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="18" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="18" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="18" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="18" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="18" t="s">
+        <v>364</v>
       </c>
     </row>
   </sheetData>
@@ -6164,396 +6367,396 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>340</v>
+        <v>365</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>341</v>
+        <v>366</v>
       </c>
       <c r="B3" s="4"/>
       <c r="C3" s="4"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>342</v>
+        <v>367</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>343</v>
+        <v>368</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>344</v>
+        <v>369</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="22" t="s">
-        <v>345</v>
+      <c r="A5" s="23" t="s">
+        <v>370</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>346</v>
+        <v>371</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>347</v>
+        <v>372</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="22" t="s">
-        <v>348</v>
+      <c r="A6" s="23" t="s">
+        <v>373</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>349</v>
+        <v>374</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>350</v>
+        <v>375</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="22" t="s">
-        <v>351</v>
+      <c r="A7" s="23" t="s">
+        <v>376</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>352</v>
+        <v>377</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>353</v>
+        <v>378</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="22" t="s">
-        <v>354</v>
+      <c r="A8" s="23" t="s">
+        <v>379</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>355</v>
+        <v>380</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>356</v>
+        <v>381</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="22" t="s">
-        <v>357</v>
+      <c r="A9" s="23" t="s">
+        <v>382</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>358</v>
+        <v>383</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>359</v>
+        <v>384</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="22" t="s">
-        <v>360</v>
+      <c r="A10" s="23" t="s">
+        <v>385</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>361</v>
+        <v>386</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>362</v>
+        <v>387</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="22" t="s">
-        <v>363</v>
+      <c r="A11" s="23" t="s">
+        <v>388</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>364</v>
+        <v>389</v>
       </c>
       <c r="C11" s="13" t="s">
-        <v>365</v>
+        <v>390</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="22" t="s">
-        <v>366</v>
+      <c r="A12" s="23" t="s">
+        <v>391</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>367</v>
+        <v>392</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>368</v>
+        <v>393</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="22" t="s">
-        <v>369</v>
+      <c r="A13" s="23" t="s">
+        <v>394</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>370</v>
+        <v>395</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>371</v>
+        <v>396</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="22" t="s">
-        <v>372</v>
+      <c r="A14" s="23" t="s">
+        <v>397</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>373</v>
+        <v>398</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="22" t="s">
-        <v>374</v>
+      <c r="A15" s="23" t="s">
+        <v>399</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>375</v>
+        <v>400</v>
       </c>
       <c r="C15" s="13"/>
     </row>
     <row r="16" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="22" t="s">
-        <v>376</v>
+      <c r="A16" s="23" t="s">
+        <v>401</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>377</v>
+        <v>402</v>
       </c>
       <c r="C16" s="13"/>
     </row>
     <row r="17" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="22" t="s">
-        <v>378</v>
+      <c r="A17" s="23" t="s">
+        <v>403</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>379</v>
+        <v>404</v>
       </c>
       <c r="C17" s="13"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>380</v>
+        <v>405</v>
       </c>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>342</v>
+        <v>367</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>343</v>
+        <v>368</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>344</v>
+        <v>369</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="22" t="s">
-        <v>345</v>
+      <c r="A21" s="23" t="s">
+        <v>370</v>
       </c>
       <c r="B21" s="13" t="s">
-        <v>381</v>
+        <v>406</v>
       </c>
       <c r="C21" s="13" t="s">
-        <v>382</v>
+        <v>407</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="22" t="s">
-        <v>383</v>
+      <c r="A22" s="23" t="s">
+        <v>408</v>
       </c>
       <c r="B22" s="13" t="s">
-        <v>384</v>
+        <v>409</v>
       </c>
       <c r="C22" s="13" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="23" t="s">
+        <v>376</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>411</v>
+      </c>
+      <c r="C23" s="13" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="23" t="s">
+        <v>413</v>
+      </c>
+      <c r="B24" s="13" t="s">
+        <v>414</v>
+      </c>
+      <c r="C24" s="13" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="23" t="s">
+        <v>416</v>
+      </c>
+      <c r="B25" s="13" t="s">
+        <v>417</v>
+      </c>
+      <c r="C25" s="13" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="23" t="s">
+        <v>419</v>
+      </c>
+      <c r="B26" s="13" t="s">
+        <v>420</v>
+      </c>
+      <c r="C26" s="13" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="23" t="s">
         <v>385</v>
       </c>
-    </row>
-    <row r="23" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="22" t="s">
-        <v>351</v>
-      </c>
-      <c r="B23" s="13" t="s">
-        <v>386</v>
-      </c>
-      <c r="C23" s="13" t="s">
-        <v>387</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="22" t="s">
-        <v>388</v>
-      </c>
-      <c r="B24" s="13" t="s">
-        <v>389</v>
-      </c>
-      <c r="C24" s="13" t="s">
-        <v>390</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="22" t="s">
+      <c r="B27" s="13" t="s">
+        <v>422</v>
+      </c>
+      <c r="C27" s="13" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="23" t="s">
         <v>391</v>
       </c>
-      <c r="B25" s="13" t="s">
-        <v>392</v>
-      </c>
-      <c r="C25" s="13" t="s">
-        <v>393</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="22" t="s">
-        <v>394</v>
-      </c>
-      <c r="B26" s="13" t="s">
-        <v>395</v>
-      </c>
-      <c r="C26" s="13" t="s">
-        <v>396</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="22" t="s">
-        <v>360</v>
-      </c>
-      <c r="B27" s="13" t="s">
+      <c r="B28" s="13" t="s">
+        <v>424</v>
+      </c>
+      <c r="C28" s="13" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="23" t="s">
+        <v>426</v>
+      </c>
+      <c r="B29" s="13" t="s">
+        <v>427</v>
+      </c>
+      <c r="C29" s="13" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="23" t="s">
         <v>397</v>
       </c>
-      <c r="C27" s="13" t="s">
-        <v>398</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="22" t="s">
-        <v>366</v>
-      </c>
-      <c r="B28" s="13" t="s">
+      <c r="B30" s="13" t="s">
+        <v>429</v>
+      </c>
+      <c r="C30" s="13" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="23" t="s">
         <v>399</v>
       </c>
-      <c r="C28" s="13" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="22" t="s">
+      <c r="B31" s="13" t="s">
+        <v>430</v>
+      </c>
+      <c r="C31" s="13"/>
+    </row>
+    <row r="32" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="23" t="s">
         <v>401</v>
       </c>
-      <c r="B29" s="13" t="s">
-        <v>402</v>
-      </c>
-      <c r="C29" s="13" t="s">
+      <c r="B32" s="13" t="s">
+        <v>431</v>
+      </c>
+      <c r="C32" s="13" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="23" t="s">
         <v>403</v>
       </c>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="22" t="s">
-        <v>372</v>
-      </c>
-      <c r="B30" s="13" t="s">
-        <v>404</v>
-      </c>
-      <c r="C30" s="13" t="s">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="22" t="s">
-        <v>374</v>
-      </c>
-      <c r="B31" s="13" t="s">
-        <v>405</v>
-      </c>
-      <c r="C31" s="13"/>
-    </row>
-    <row r="32" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="22" t="s">
-        <v>376</v>
-      </c>
-      <c r="B32" s="13" t="s">
-        <v>406</v>
-      </c>
-      <c r="C32" s="13" t="s">
-        <v>407</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="22" t="s">
-        <v>378</v>
-      </c>
       <c r="B33" s="13" t="s">
-        <v>408</v>
+        <v>433</v>
       </c>
       <c r="C33" s="13"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="s">
-        <v>409</v>
+        <v>434</v>
       </c>
       <c r="B35" s="4"/>
       <c r="C35" s="4"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="3" t="s">
-        <v>342</v>
+        <v>367</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>343</v>
+        <v>368</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>344</v>
+        <v>369</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="22" t="s">
-        <v>383</v>
+      <c r="A37" s="23" t="s">
+        <v>408</v>
       </c>
       <c r="B37" s="13" t="s">
-        <v>410</v>
+        <v>435</v>
       </c>
       <c r="C37" s="13" t="s">
-        <v>411</v>
+        <v>436</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="22" t="s">
-        <v>412</v>
+      <c r="A38" s="23" t="s">
+        <v>437</v>
       </c>
       <c r="B38" s="13" t="s">
-        <v>413</v>
+        <v>438</v>
       </c>
       <c r="C38" s="13" t="s">
-        <v>414</v>
+        <v>439</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="22" t="s">
-        <v>415</v>
+      <c r="A39" s="23" t="s">
+        <v>440</v>
       </c>
       <c r="B39" s="13" t="s">
-        <v>416</v>
+        <v>441</v>
       </c>
       <c r="C39" s="13"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="22" t="s">
-        <v>374</v>
+      <c r="A40" s="23" t="s">
+        <v>399</v>
       </c>
       <c r="B40" s="13" t="s">
-        <v>417</v>
+        <v>442</v>
       </c>
       <c r="C40" s="13" t="s">
-        <v>418</v>
+        <v>443</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="22" t="s">
-        <v>376</v>
+      <c r="A41" s="23" t="s">
+        <v>401</v>
       </c>
       <c r="B41" s="13" t="s">
-        <v>419</v>
+        <v>444</v>
       </c>
       <c r="C41" s="13"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="22" t="s">
-        <v>420</v>
+      <c r="A42" s="23" t="s">
+        <v>445</v>
       </c>
       <c r="B42" s="13" t="s">
-        <v>421</v>
+        <v>446</v>
       </c>
       <c r="C42" s="13"/>
     </row>
@@ -6585,7 +6788,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>422</v>
+        <v>447</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6593,16 +6796,16 @@
         <v>14</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>423</v>
+        <v>448</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>424</v>
+        <v>449</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>425</v>
+        <v>450</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>426</v>
+        <v>451</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6610,84 +6813,84 @@
         <v>28</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>427</v>
+        <v>452</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>428</v>
+        <v>453</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>429</v>
+        <v>454</v>
       </c>
       <c r="E4" s="13" t="s">
-        <v>430</v>
+        <v>455</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>431</v>
+        <v>456</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>432</v>
+        <v>457</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>433</v>
+        <v>458</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>434</v>
+        <v>459</v>
       </c>
       <c r="E5" s="13" t="s">
-        <v>435</v>
+        <v>460</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>436</v>
+        <v>461</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>427</v>
+        <v>452</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>437</v>
+        <v>462</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>438</v>
+        <v>463</v>
       </c>
       <c r="E6" s="13" t="s">
-        <v>439</v>
+        <v>464</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>440</v>
+        <v>465</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>427</v>
+        <v>452</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>441</v>
+        <v>466</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>442</v>
+        <v>467</v>
       </c>
       <c r="E7" s="13" t="s">
-        <v>443</v>
+        <v>468</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>444</v>
+        <v>469</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>427</v>
+        <v>452</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>445</v>
+        <v>470</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>446</v>
+        <v>471</v>
       </c>
       <c r="E8" s="13" t="s">
-        <v>447</v>
+        <v>472</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6695,84 +6898,84 @@
         <v>43</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>448</v>
+        <v>473</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>449</v>
+        <v>474</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>450</v>
+        <v>475</v>
       </c>
       <c r="E9" s="13" t="s">
-        <v>451</v>
+        <v>476</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>452</v>
+        <v>477</v>
       </c>
       <c r="B10" s="13" t="s">
         <v>102</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>453</v>
+        <v>478</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>454</v>
+        <v>479</v>
       </c>
       <c r="E10" s="13" t="s">
-        <v>455</v>
+        <v>480</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
-        <v>456</v>
+        <v>481</v>
       </c>
       <c r="B11" s="13" t="s">
         <v>102</v>
       </c>
       <c r="C11" s="13" t="s">
-        <v>457</v>
+        <v>482</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>458</v>
+        <v>483</v>
       </c>
       <c r="E11" s="13" t="s">
-        <v>459</v>
+        <v>484</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>460</v>
+        <v>485</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>427</v>
+        <v>452</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>461</v>
+        <v>486</v>
       </c>
       <c r="D12" s="13" t="s">
-        <v>462</v>
+        <v>487</v>
       </c>
       <c r="E12" s="13" t="s">
-        <v>463</v>
+        <v>488</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>464</v>
+        <v>489</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>465</v>
+        <v>490</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>466</v>
+        <v>491</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>467</v>
+        <v>492</v>
       </c>
       <c r="E13" s="13" t="s">
-        <v>468</v>
+        <v>493</v>
       </c>
     </row>
   </sheetData>

</xml_diff>